<commit_message>
some modifications to the set up
</commit_message>
<xml_diff>
--- a/EconJM_status.xlsx
+++ b/EconJM_status.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/jjgecon_dat/Dropbox/Work/Job Search/2025 EconJM/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A616927B-FF54-2A4B-A2B5-B8A8F6A959A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44A5C9A7-34AD-1A45-AE23-FA855FF4BF5E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="38400" windowHeight="21100" xr2:uid="{6FE48536-7E5C-BF4C-9490-2A6392576298}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="sum" sheetId="1" r:id="rId1"/>
+    <sheet name="timeline" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -36,14 +37,11 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="32">
   <si>
     <t>add_id</t>
   </si>
   <si>
-    <t>add_title</t>
-  </si>
-  <si>
     <t>add_category</t>
   </si>
   <si>
@@ -65,40 +63,103 @@
     <t>WOO_letter_status</t>
   </si>
   <si>
-    <t>add_description_file</t>
-  </si>
-  <si>
     <t>app_status</t>
   </si>
   <si>
-    <t>institution_mission</t>
-  </si>
-  <si>
-    <t>collab_name</t>
-  </si>
-  <si>
-    <t>collab_reason</t>
-  </si>
-  <si>
-    <t>add_url</t>
-  </si>
-  <si>
     <t>add_how_apply</t>
   </si>
   <si>
     <t>institution</t>
+  </si>
+  <si>
+    <t>date</t>
+  </si>
+  <si>
+    <t>app_id</t>
+  </si>
+  <si>
+    <t>comment</t>
+  </si>
+  <si>
+    <t>simon_frazer_1</t>
+  </si>
+  <si>
+    <t>location</t>
+  </si>
+  <si>
+    <t>Burnaby, Canada</t>
+  </si>
+  <si>
+    <t>deadline_target</t>
+  </si>
+  <si>
+    <t>add_rank</t>
+  </si>
+  <si>
+    <t>assistant</t>
+  </si>
+  <si>
+    <t>add_field</t>
+  </si>
+  <si>
+    <t>Simon Fraser University</t>
+  </si>
+  <si>
+    <t>add_posting</t>
+  </si>
+  <si>
+    <t>EJM</t>
+  </si>
+  <si>
+    <t>McMaster University</t>
+  </si>
+  <si>
+    <t>macmaster_1</t>
+  </si>
+  <si>
+    <t>Hamilton, Canada</t>
+  </si>
+  <si>
+    <t>applied micro</t>
+  </si>
+  <si>
+    <t>research</t>
+  </si>
+  <si>
+    <t>teaching</t>
+  </si>
+  <si>
+    <t>gathering info</t>
+  </si>
+  <si>
+    <t>prep docs</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="12"/>
+      <color theme="10"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="16"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -119,13 +180,20 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -458,76 +526,206 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F7772053-9363-CA4A-A53F-040B7C700753}">
-  <dimension ref="A1:Q1"/>
+  <dimension ref="A1:P3"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
+    <col min="1" max="1" width="19.6640625" customWidth="1"/>
     <col min="2" max="2" width="18.33203125" customWidth="1"/>
     <col min="3" max="3" width="37.33203125" customWidth="1"/>
-    <col min="4" max="4" width="19.33203125" customWidth="1"/>
-    <col min="5" max="5" width="39.33203125" customWidth="1"/>
-    <col min="6" max="6" width="17.6640625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="13.5" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="18" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="14.33203125" customWidth="1"/>
-    <col min="11" max="11" width="19.83203125" customWidth="1"/>
-    <col min="12" max="13" width="17.5" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="16.83203125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="16.6640625" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="26.1640625" customWidth="1"/>
-    <col min="17" max="17" width="32.6640625" customWidth="1"/>
+    <col min="4" max="6" width="19.5" customWidth="1"/>
+    <col min="7" max="8" width="19.33203125" customWidth="1"/>
+    <col min="9" max="9" width="14.5" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="18.1640625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="23.5" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="13.33203125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="13" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="22.6640625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="23.33203125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="21.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A1" t="s">
+    <row r="1" spans="1:16" s="3" customFormat="1" ht="22" x14ac:dyDescent="0.3">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C1" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="I1" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="J1" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="L1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="M1" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="N1" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="O1" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="P1" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B2" t="s">
+        <v>31</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D2" t="s">
         <v>16</v>
       </c>
-      <c r="D1" t="s">
-        <v>2</v>
-      </c>
-      <c r="E1" t="s">
+      <c r="E2" t="s">
+        <v>19</v>
+      </c>
+      <c r="F2" t="s">
+        <v>27</v>
+      </c>
+      <c r="G2" t="s">
+        <v>28</v>
+      </c>
+      <c r="H2" s="1">
+        <v>45931</v>
+      </c>
+      <c r="I2" t="s">
+        <v>23</v>
+      </c>
+      <c r="J2" t="s">
+        <v>23</v>
+      </c>
+      <c r="K2">
         <v>1</v>
       </c>
-      <c r="F1" t="s">
-        <v>9</v>
-      </c>
-      <c r="G1" t="s">
+      <c r="L2">
+        <v>1</v>
+      </c>
+      <c r="M2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>25</v>
+      </c>
+      <c r="B3" t="s">
+        <v>31</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="D3" t="s">
+        <v>26</v>
+      </c>
+      <c r="E3" t="s">
+        <v>19</v>
+      </c>
+      <c r="F3" t="s">
+        <v>27</v>
+      </c>
+      <c r="G3" t="s">
+        <v>29</v>
+      </c>
+      <c r="H3" s="1">
+        <v>45931</v>
+      </c>
+      <c r="I3" t="s">
+        <v>23</v>
+      </c>
+      <c r="J3" t="s">
+        <v>23</v>
+      </c>
+      <c r="K3">
+        <v>1</v>
+      </c>
+      <c r="L3">
+        <v>1</v>
+      </c>
+      <c r="M3">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="C2" r:id="rId1" xr:uid="{2FD67E99-97D4-6F4F-9C23-F094A4E233EB}"/>
+    <hyperlink ref="C3" r:id="rId2" xr:uid="{C466BD2C-2D71-FD47-B267-C9470B42EAAE}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{923E81FA-B875-3C4E-A189-1A21268FA086}">
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="32.83203125" customWidth="1"/>
+    <col min="2" max="2" width="33" customWidth="1"/>
+    <col min="3" max="3" width="25.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" s="3" customFormat="1" ht="22" x14ac:dyDescent="0.3">
+      <c r="A1" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A2" s="1">
+        <v>45909</v>
+      </c>
+      <c r="B2" t="s">
         <v>14</v>
       </c>
-      <c r="H1" t="s">
-        <v>15</v>
-      </c>
-      <c r="I1" t="s">
-        <v>3</v>
-      </c>
-      <c r="J1" t="s">
-        <v>4</v>
-      </c>
-      <c r="K1" t="s">
-        <v>5</v>
-      </c>
-      <c r="L1" t="s">
-        <v>6</v>
-      </c>
-      <c r="M1" t="s">
-        <v>7</v>
-      </c>
-      <c r="N1" t="s">
-        <v>8</v>
-      </c>
-      <c r="O1" t="s">
-        <v>11</v>
-      </c>
-      <c r="P1" t="s">
-        <v>12</v>
-      </c>
-      <c r="Q1" t="s">
-        <v>13</v>
+      <c r="C2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A3" s="1">
+        <v>45909</v>
+      </c>
+      <c r="B3" t="s">
+        <v>25</v>
+      </c>
+      <c r="C3" t="s">
+        <v>30</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
another day another life
</commit_message>
<xml_diff>
--- a/EconJM_status.xlsx
+++ b/EconJM_status.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/jjgecon_dat/Dropbox/Work/Job Search/2025 EconJM/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E04F9107-138F-F349-A1FB-AB9A66B90C8E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A67BBC1-4C1F-3742-90BA-108A88963698}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="38400" windowHeight="21100" xr2:uid="{6FE48536-7E5C-BF4C-9490-2A6392576298}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="38400" windowHeight="21100" activeTab="2" xr2:uid="{6FE48536-7E5C-BF4C-9490-2A6392576298}"/>
   </bookViews>
   <sheets>
     <sheet name="sum" sheetId="1" r:id="rId1"/>
     <sheet name="timeline" sheetId="2" r:id="rId2"/>
+    <sheet name="stats" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">sum!$A$1:$Y$19</definedName>
@@ -682,7 +683,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1030" uniqueCount="408">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1058" uniqueCount="417">
   <si>
     <t>add_id</t>
   </si>
@@ -1940,12 +1941,39 @@
   <si>
     <t>Florian Scheuer by email (florian.scheuer@uzh.ch)</t>
   </si>
+  <si>
+    <t>Total apps</t>
+  </si>
+  <si>
+    <t>good match</t>
+  </si>
+  <si>
+    <t>top ranked</t>
+  </si>
+  <si>
+    <t>Outcomes</t>
+  </si>
+  <si>
+    <t>no news</t>
+  </si>
+  <si>
+    <t>rejected</t>
+  </si>
+  <si>
+    <t>interview</t>
+  </si>
+  <si>
+    <t>fly out</t>
+  </si>
+  <si>
+    <t>offer</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -1996,6 +2024,20 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="20"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -2020,11 +2062,12 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
@@ -2043,19 +2086,41 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="9" fontId="7" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="3">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Percent" xfId="2" builtinId="5"/>
   </cellStyles>
-  <dxfs count="62">
+  <dxfs count="63">
     <dxf>
       <font>
-        <color rgb="FF006100"/>
+        <color rgb="FF9C0006"/>
       </font>
       <fill>
         <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
+          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2071,25 +2136,43 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF006100"/>
+        <color rgb="FF9C0006"/>
       </font>
       <fill>
         <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
+          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <font>
-        <b val="0"/>
-        <i/>
-        <color theme="0" tint="-0.24994659260841701"/>
+        <color rgb="FF9C0006"/>
       </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
     </dxf>
     <dxf>
       <font>
-        <color theme="5" tint="0.79998168889431442"/>
+        <color rgb="FF9C0006"/>
       </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
     </dxf>
     <dxf>
       <font>
@@ -24262,7 +24345,7 @@
         <v>372</v>
       </c>
       <c r="D16" t="s">
-        <v>28</v>
+        <v>104</v>
       </c>
       <c r="H16" t="s">
         <v>371</v>
@@ -24850,7 +24933,7 @@
         <v>350</v>
       </c>
       <c r="D30" t="s">
-        <v>28</v>
+        <v>104</v>
       </c>
       <c r="H30" t="s">
         <v>349</v>
@@ -25355,7 +25438,7 @@
         <v>377</v>
       </c>
       <c r="D42" t="s">
-        <v>28</v>
+        <v>104</v>
       </c>
       <c r="H42" t="s">
         <v>378</v>
@@ -25393,7 +25476,7 @@
         <v>381</v>
       </c>
       <c r="D43" t="s">
-        <v>28</v>
+        <v>104</v>
       </c>
       <c r="H43" t="s">
         <v>380</v>
@@ -26234,7 +26317,7 @@
         <v>97</v>
       </c>
       <c r="D63" t="s">
-        <v>28</v>
+        <v>104</v>
       </c>
       <c r="H63" s="2" t="s">
         <v>98</v>
@@ -26276,7 +26359,7 @@
         <v>101</v>
       </c>
       <c r="D64" t="s">
-        <v>28</v>
+        <v>104</v>
       </c>
       <c r="H64" s="2" t="s">
         <v>102</v>
@@ -26365,7 +26448,7 @@
         <v>374</v>
       </c>
       <c r="D66" t="s">
-        <v>28</v>
+        <v>104</v>
       </c>
       <c r="H66" t="s">
         <v>375</v>
@@ -28242,7 +28325,7 @@
         <v>389</v>
       </c>
       <c r="D109" t="s">
-        <v>28</v>
+        <v>104</v>
       </c>
       <c r="H109" t="s">
         <v>388</v>
@@ -29148,32 +29231,32 @@
     </sortState>
   </autoFilter>
   <conditionalFormatting sqref="A1:B1048576">
-    <cfRule type="duplicateValues" dxfId="61" priority="8"/>
+    <cfRule type="duplicateValues" dxfId="62" priority="8"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A2:B22">
-    <cfRule type="duplicateValues" dxfId="60" priority="9"/>
+    <cfRule type="duplicateValues" dxfId="61" priority="9"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A61:B61">
-    <cfRule type="duplicateValues" dxfId="59" priority="7"/>
+    <cfRule type="duplicateValues" dxfId="60" priority="7"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D1:D1048576">
-    <cfRule type="containsText" dxfId="58" priority="1" operator="containsText" text="abandoned">
+    <cfRule type="containsText" dxfId="59" priority="1" operator="containsText" text="abandoned">
       <formula>NOT(ISERROR(SEARCH("abandoned",D1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="57" priority="3" operator="containsText" text="late app">
+    <cfRule type="containsText" dxfId="58" priority="3" operator="containsText" text="late app">
       <formula>NOT(ISERROR(SEARCH("late app",D1)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J78:J80 J83:J89 D1:E1 J92:J112 D2:G1048576 J115:J124 J126:J128 J130:J131 L87:L131">
-    <cfRule type="containsText" dxfId="56" priority="6" operator="containsText" text="completed">
+    <cfRule type="containsText" dxfId="57" priority="6" operator="containsText" text="completed">
       <formula>NOT(ISERROR(SEARCH("completed",D1)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J78:J80 J83:J89 J92:J112 F1:G1048576 J115:J124 J126:J128 J130:J131 L87:L131">
-    <cfRule type="containsText" dxfId="55" priority="4" operator="containsText" text="NO">
+    <cfRule type="containsText" dxfId="56" priority="4" operator="containsText" text="NO">
       <formula>NOT(ISERROR(SEARCH("NO",F1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="54" priority="5" operator="containsText" text="YES">
+    <cfRule type="containsText" dxfId="55" priority="5" operator="containsText" text="YES">
       <formula>NOT(ISERROR(SEARCH("YES",F1)))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -29272,7 +29355,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{923E81FA-B875-3C4E-A189-1A21268FA086}">
-  <dimension ref="A1:C66"/>
+  <dimension ref="A1:C77"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="32.83203125" customWidth="1"/>
@@ -29964,129 +30047,394 @@
     </row>
     <row r="66" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A66" s="1">
-        <v>45952</v>
+        <v>45953</v>
+      </c>
+      <c r="B66" t="s">
+        <v>389</v>
       </c>
       <c r="C66" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="67" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A67" s="1">
+        <v>45953</v>
+      </c>
+      <c r="B67" t="s">
+        <v>372</v>
+      </c>
+      <c r="C67" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="68" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A68" s="1">
+        <v>45953</v>
+      </c>
+      <c r="B68" t="s">
+        <v>350</v>
+      </c>
+      <c r="C68" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="69" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A69" s="1">
+        <v>45953</v>
+      </c>
+      <c r="B69" t="s">
+        <v>377</v>
+      </c>
+      <c r="C69" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="70" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A70" s="1">
+        <v>45953</v>
+      </c>
+      <c r="B70" t="s">
+        <v>381</v>
+      </c>
+      <c r="C70" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="71" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A71" s="1">
+        <v>45953</v>
+      </c>
+      <c r="B71" s="7" t="s">
+        <v>97</v>
+      </c>
+      <c r="C71" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="72" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A72" s="1">
+        <v>45953</v>
+      </c>
+      <c r="B72" t="s">
+        <v>101</v>
+      </c>
+      <c r="C72" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="73" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A73" s="1">
+        <v>45953</v>
+      </c>
+      <c r="B73" t="s">
+        <v>374</v>
+      </c>
+      <c r="C73" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="74" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A74" s="1">
+        <v>45953</v>
+      </c>
+      <c r="C74" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="75" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A75" s="1">
+        <v>45953</v>
+      </c>
+      <c r="C75" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="76" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A76" s="1">
+        <v>45953</v>
+      </c>
+      <c r="C76" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="77" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A77" s="1">
+        <v>45953</v>
+      </c>
+      <c r="C77" t="s">
         <v>105</v>
       </c>
     </row>
   </sheetData>
   <conditionalFormatting sqref="B5">
-    <cfRule type="duplicateValues" dxfId="53" priority="48"/>
-    <cfRule type="duplicateValues" dxfId="52" priority="49"/>
+    <cfRule type="duplicateValues" dxfId="54" priority="57"/>
+    <cfRule type="duplicateValues" dxfId="53" priority="58"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B10">
-    <cfRule type="duplicateValues" dxfId="51" priority="46"/>
-    <cfRule type="duplicateValues" dxfId="50" priority="47"/>
+    <cfRule type="duplicateValues" dxfId="52" priority="55"/>
+    <cfRule type="duplicateValues" dxfId="51" priority="56"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B11">
-    <cfRule type="duplicateValues" dxfId="49" priority="44"/>
-    <cfRule type="duplicateValues" dxfId="48" priority="45"/>
+    <cfRule type="duplicateValues" dxfId="50" priority="53"/>
+    <cfRule type="duplicateValues" dxfId="49" priority="54"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B12">
-    <cfRule type="duplicateValues" dxfId="47" priority="42"/>
-    <cfRule type="duplicateValues" dxfId="46" priority="43"/>
+    <cfRule type="duplicateValues" dxfId="48" priority="51"/>
+    <cfRule type="duplicateValues" dxfId="47" priority="52"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B15">
-    <cfRule type="duplicateValues" dxfId="45" priority="40"/>
-    <cfRule type="duplicateValues" dxfId="44" priority="41"/>
+    <cfRule type="duplicateValues" dxfId="46" priority="49"/>
+    <cfRule type="duplicateValues" dxfId="45" priority="50"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B16">
-    <cfRule type="duplicateValues" dxfId="43" priority="39"/>
+    <cfRule type="duplicateValues" dxfId="44" priority="48"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B17">
-    <cfRule type="duplicateValues" dxfId="42" priority="37"/>
-    <cfRule type="duplicateValues" dxfId="41" priority="38"/>
+    <cfRule type="duplicateValues" dxfId="43" priority="46"/>
+    <cfRule type="duplicateValues" dxfId="42" priority="47"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B18">
-    <cfRule type="duplicateValues" dxfId="40" priority="35"/>
-    <cfRule type="duplicateValues" dxfId="39" priority="36"/>
+    <cfRule type="duplicateValues" dxfId="41" priority="44"/>
+    <cfRule type="duplicateValues" dxfId="40" priority="45"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B19">
-    <cfRule type="duplicateValues" dxfId="38" priority="34"/>
+    <cfRule type="duplicateValues" dxfId="39" priority="43"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B22:B23">
-    <cfRule type="duplicateValues" dxfId="37" priority="32"/>
-    <cfRule type="duplicateValues" dxfId="36" priority="33"/>
+    <cfRule type="duplicateValues" dxfId="38" priority="41"/>
+    <cfRule type="duplicateValues" dxfId="37" priority="42"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B24">
-    <cfRule type="duplicateValues" dxfId="35" priority="30"/>
-    <cfRule type="duplicateValues" dxfId="34" priority="31"/>
+    <cfRule type="duplicateValues" dxfId="36" priority="39"/>
+    <cfRule type="duplicateValues" dxfId="35" priority="40"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B27">
-    <cfRule type="duplicateValues" dxfId="33" priority="28"/>
-    <cfRule type="duplicateValues" dxfId="32" priority="29"/>
+    <cfRule type="duplicateValues" dxfId="34" priority="37"/>
+    <cfRule type="duplicateValues" dxfId="33" priority="38"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B28">
-    <cfRule type="duplicateValues" dxfId="31" priority="27"/>
+    <cfRule type="duplicateValues" dxfId="32" priority="36"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B29">
-    <cfRule type="duplicateValues" dxfId="30" priority="25"/>
-    <cfRule type="duplicateValues" dxfId="29" priority="26"/>
+    <cfRule type="duplicateValues" dxfId="31" priority="34"/>
+    <cfRule type="duplicateValues" dxfId="30" priority="35"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B30">
-    <cfRule type="duplicateValues" dxfId="28" priority="24"/>
+    <cfRule type="duplicateValues" dxfId="29" priority="33"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B31">
-    <cfRule type="duplicateValues" dxfId="27" priority="23"/>
+    <cfRule type="duplicateValues" dxfId="28" priority="32"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B32">
-    <cfRule type="duplicateValues" dxfId="26" priority="22"/>
+    <cfRule type="duplicateValues" dxfId="27" priority="31"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B33">
-    <cfRule type="duplicateValues" dxfId="25" priority="21"/>
+    <cfRule type="duplicateValues" dxfId="26" priority="30"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B34">
-    <cfRule type="duplicateValues" dxfId="24" priority="20"/>
+    <cfRule type="duplicateValues" dxfId="25" priority="29"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B35">
-    <cfRule type="duplicateValues" dxfId="23" priority="19"/>
+    <cfRule type="duplicateValues" dxfId="24" priority="28"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B37">
-    <cfRule type="duplicateValues" dxfId="22" priority="18"/>
+    <cfRule type="duplicateValues" dxfId="23" priority="27"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B38">
-    <cfRule type="duplicateValues" dxfId="21" priority="17"/>
+    <cfRule type="duplicateValues" dxfId="22" priority="26"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B42">
-    <cfRule type="duplicateValues" dxfId="20" priority="16"/>
+    <cfRule type="duplicateValues" dxfId="21" priority="25"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B43">
-    <cfRule type="duplicateValues" dxfId="19" priority="15"/>
+    <cfRule type="duplicateValues" dxfId="20" priority="24"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B44:B45">
-    <cfRule type="duplicateValues" dxfId="18" priority="14"/>
+    <cfRule type="duplicateValues" dxfId="19" priority="23"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B46">
-    <cfRule type="duplicateValues" dxfId="17" priority="13"/>
+    <cfRule type="duplicateValues" dxfId="18" priority="22"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B48">
-    <cfRule type="duplicateValues" dxfId="16" priority="12"/>
+    <cfRule type="duplicateValues" dxfId="17" priority="21"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B49">
-    <cfRule type="duplicateValues" dxfId="15" priority="11"/>
+    <cfRule type="duplicateValues" dxfId="16" priority="20"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B51">
-    <cfRule type="duplicateValues" dxfId="14" priority="10"/>
+    <cfRule type="duplicateValues" dxfId="15" priority="19"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B52">
-    <cfRule type="duplicateValues" dxfId="13" priority="9"/>
+    <cfRule type="duplicateValues" dxfId="14" priority="18"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B58">
-    <cfRule type="duplicateValues" dxfId="12" priority="7"/>
+    <cfRule type="duplicateValues" dxfId="13" priority="16"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B59">
-    <cfRule type="duplicateValues" dxfId="11" priority="5"/>
+    <cfRule type="duplicateValues" dxfId="12" priority="14"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B63">
-    <cfRule type="duplicateValues" dxfId="10" priority="4"/>
+    <cfRule type="duplicateValues" dxfId="11" priority="13"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B64">
-    <cfRule type="duplicateValues" dxfId="9" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="10" priority="11"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B66">
-    <cfRule type="duplicateValues" dxfId="8" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="9" priority="10"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B67">
+    <cfRule type="duplicateValues" dxfId="8" priority="8"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B67">
+    <cfRule type="duplicateValues" dxfId="7" priority="9"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B68">
+    <cfRule type="duplicateValues" dxfId="6" priority="7"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B69">
+    <cfRule type="duplicateValues" dxfId="5" priority="6"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B70">
+    <cfRule type="duplicateValues" dxfId="3" priority="4"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B72">
+    <cfRule type="duplicateValues" dxfId="2" priority="3"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B73">
+    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{852B2CA5-879F-3640-8AF9-56395EF3FA0F}">
+  <dimension ref="A1:C10"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="15.83203125" style="14" customWidth="1"/>
+    <col min="2" max="2" width="10.83203125" style="18"/>
+    <col min="3" max="3" width="10.83203125" style="12"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" ht="27" x14ac:dyDescent="0.35">
+      <c r="A1" s="13" t="s">
+        <v>408</v>
+      </c>
+      <c r="B1" s="17">
+        <f>COUNTA(sum!A:A) -1</f>
+        <v>130</v>
+      </c>
+      <c r="C1" s="16">
+        <f>COUNTIF(sum!D:D, "completed")/B1</f>
+        <v>0.47692307692307695</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" ht="22" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="15" t="s">
+        <v>409</v>
+      </c>
+      <c r="B2" s="18">
+        <f>COUNTA(sum!C:C) -1</f>
+        <v>40</v>
+      </c>
+      <c r="C2" s="12">
+        <f>COUNTIFS(sum!D:D,"completed", sum!C:C, "&lt;&gt;") / B2</f>
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="15" t="s">
+        <v>410</v>
+      </c>
+      <c r="B3" s="18">
+        <f>COUNTA(sum!F:F) -1</f>
+        <v>28</v>
+      </c>
+      <c r="C3" s="12">
+        <f>COUNTIFS(sum!D:D,"completed", sum!F:F, "&lt;&gt;") / B3</f>
+        <v>0.35714285714285715</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" ht="27" x14ac:dyDescent="0.35">
+      <c r="A5" s="13" t="s">
+        <v>411</v>
+      </c>
+      <c r="B5" s="17">
+        <f>COUNTA(sum!E:E) -1</f>
+        <v>0</v>
+      </c>
+      <c r="C5" s="16">
+        <f>B5/B1</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A6" s="15" t="s">
+        <v>412</v>
+      </c>
+      <c r="B6" s="18">
+        <f>COUNTIFS(sum!E:E,"no news")</f>
+        <v>0</v>
+      </c>
+      <c r="C6" s="12" t="e">
+        <f>B6/$B$5</f>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A7" s="15" t="s">
+        <v>413</v>
+      </c>
+      <c r="B7" s="18">
+        <f>COUNTIFS(sum!E:E,"rejected")</f>
+        <v>0</v>
+      </c>
+      <c r="C7" s="12" t="e">
+        <f t="shared" ref="C7:C10" si="0">B7/$B$5</f>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A8" s="15" t="s">
+        <v>414</v>
+      </c>
+      <c r="B8" s="18">
+        <f>COUNTIFS(sum!E:E,"interview")</f>
+        <v>0</v>
+      </c>
+      <c r="C8" s="12" t="e">
+        <f t="shared" si="0"/>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A9" s="15" t="s">
+        <v>415</v>
+      </c>
+      <c r="B9" s="18">
+        <f>COUNTIFS(sum!E:E,"fly out")</f>
+        <v>0</v>
+      </c>
+      <c r="C9" s="12" t="e">
+        <f t="shared" si="0"/>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A10" s="15" t="s">
+        <v>416</v>
+      </c>
+      <c r="B10" s="18">
+        <f>COUNTIFS(sum!E:E,"offer")</f>
+        <v>0</v>
+      </c>
+      <c r="C10" s="12" t="e">
+        <f t="shared" si="0"/>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
before try it in my windows pc
</commit_message>
<xml_diff>
--- a/EconJM_status.xlsx
+++ b/EconJM_status.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/jjgecon_dat/Dropbox/Work/Job Search/2025 EconJM/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4EE6198-228B-5C4D-98F2-B7C0D018765D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C0B354BB-FD4A-5D47-8FB7-C4F872B51FE7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="38400" windowHeight="21100" xr2:uid="{6FE48536-7E5C-BF4C-9490-2A6392576298}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="38400" windowHeight="21100" activeTab="1" xr2:uid="{6FE48536-7E5C-BF4C-9490-2A6392576298}"/>
   </bookViews>
   <sheets>
     <sheet name="sum" sheetId="1" r:id="rId1"/>
@@ -943,7 +943,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1436" uniqueCount="569">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1437" uniqueCount="570">
   <si>
     <t>add_id</t>
   </si>
@@ -2602,6 +2602,9 @@
   </si>
   <si>
     <t>University of Toledo</t>
+  </si>
+  <si>
+    <t>gatehred 10 more from JOE</t>
   </si>
   <si>
     <t>gatehred 10 more from JOE, trying to make up for 31st</t>
@@ -31645,19 +31648,19 @@
     </row>
     <row r="17" spans="1:21" ht="17" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
       <c r="C17" s="1">
         <v>45945</v>
       </c>
       <c r="D17" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
       <c r="H17" t="s">
         <v>25</v>
       </c>
       <c r="L17" s="17" t="s">
-        <v>544</v>
+        <v>545</v>
       </c>
       <c r="M17" t="e" vm="12">
         <v>#VALUE!</v>
@@ -33013,13 +33016,13 @@
         <v>45955</v>
       </c>
       <c r="D50" t="s">
-        <v>551</v>
+        <v>552</v>
       </c>
       <c r="H50" t="s">
         <v>25</v>
       </c>
       <c r="L50" t="s">
-        <v>550</v>
+        <v>551</v>
       </c>
       <c r="M50" t="e" vm="34">
         <v>#VALUE!</v>
@@ -33045,19 +33048,19 @@
     </row>
     <row r="51" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
-        <v>552</v>
+        <v>553</v>
       </c>
       <c r="C51" s="1">
         <v>45955</v>
       </c>
       <c r="D51" t="s">
-        <v>553</v>
+        <v>554</v>
       </c>
       <c r="H51" t="s">
         <v>25</v>
       </c>
       <c r="L51" t="s">
-        <v>554</v>
+        <v>555</v>
       </c>
       <c r="M51" t="e" vm="35">
         <v>#VALUE!</v>
@@ -33083,19 +33086,19 @@
     </row>
     <row r="52" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
-        <v>560</v>
+        <v>561</v>
       </c>
       <c r="C52" s="1">
         <v>45955</v>
       </c>
       <c r="D52" t="s">
-        <v>559</v>
+        <v>560</v>
       </c>
       <c r="H52" t="s">
         <v>25</v>
       </c>
       <c r="L52" t="s">
-        <v>561</v>
+        <v>562</v>
       </c>
       <c r="M52" t="e" vm="36">
         <v>#VALUE!</v>
@@ -33623,19 +33626,19 @@
     </row>
     <row r="65" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
-        <v>566</v>
+        <v>567</v>
       </c>
       <c r="C65" s="1">
         <v>45962</v>
       </c>
       <c r="D65" t="s">
-        <v>567</v>
+        <v>568</v>
       </c>
       <c r="H65" t="s">
         <v>25</v>
       </c>
       <c r="L65" t="s">
-        <v>568</v>
+        <v>569</v>
       </c>
       <c r="M65" t="e" vm="22">
         <v>#VALUE!</v>
@@ -37001,10 +37004,10 @@
     </row>
     <row r="144" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A144" t="s">
-        <v>556</v>
+        <v>557</v>
       </c>
       <c r="B144" t="s">
-        <v>557</v>
+        <v>558</v>
       </c>
       <c r="C144" s="1">
         <v>45976</v>
@@ -37013,13 +37016,13 @@
         <v>42</v>
       </c>
       <c r="E144" t="s">
-        <v>558</v>
+        <v>559</v>
       </c>
       <c r="H144" t="s">
         <v>25</v>
       </c>
       <c r="L144" t="s">
-        <v>555</v>
+        <v>556</v>
       </c>
       <c r="M144" t="e" vm="36">
         <v>#VALUE!</v>
@@ -37045,7 +37048,7 @@
     </row>
     <row r="145" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A145" t="s">
-        <v>562</v>
+        <v>563</v>
       </c>
       <c r="C145" s="1">
         <v>45976</v>
@@ -37057,7 +37060,7 @@
         <v>25</v>
       </c>
       <c r="L145" t="s">
-        <v>563</v>
+        <v>564</v>
       </c>
       <c r="M145" t="e" vm="76">
         <v>#VALUE!</v>
@@ -37083,7 +37086,7 @@
     </row>
     <row r="146" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A146" t="s">
-        <v>565</v>
+        <v>566</v>
       </c>
       <c r="C146" s="1">
         <v>45976</v>
@@ -37095,7 +37098,7 @@
         <v>25</v>
       </c>
       <c r="L146" t="s">
-        <v>564</v>
+        <v>565</v>
       </c>
       <c r="M146" t="e" vm="36">
         <v>#VALUE!</v>
@@ -38321,7 +38324,7 @@
     </row>
     <row r="177" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A177" t="s">
-        <v>542</v>
+        <v>543</v>
       </c>
       <c r="C177" s="1">
         <v>45986</v>
@@ -38333,7 +38336,7 @@
         <v>25</v>
       </c>
       <c r="L177" t="s">
-        <v>543</v>
+        <v>544</v>
       </c>
       <c r="M177" t="e" vm="22">
         <v>#VALUE!</v>
@@ -38359,19 +38362,19 @@
     </row>
     <row r="178" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A178" t="s">
-        <v>549</v>
+        <v>550</v>
       </c>
       <c r="C178" s="1">
         <v>45986</v>
       </c>
       <c r="D178" t="s">
-        <v>548</v>
+        <v>549</v>
       </c>
       <c r="H178" t="s">
         <v>25</v>
       </c>
       <c r="L178" t="s">
-        <v>547</v>
+        <v>548</v>
       </c>
       <c r="M178" t="e" vm="12">
         <v>#VALUE!</v>
@@ -38643,7 +38646,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{923E81FA-B875-3C4E-A189-1A21268FA086}">
-  <dimension ref="A1:C102"/>
+  <dimension ref="A1:C103"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="32.83203125" customWidth="1"/>
@@ -39725,6 +39728,14 @@
         <v>45962</v>
       </c>
       <c r="C102" t="s">
+        <v>542</v>
+      </c>
+    </row>
+    <row r="103" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A103" s="1">
+        <v>45962</v>
+      </c>
+      <c r="C103" t="s">
         <v>541</v>
       </c>
     </row>

</xml_diff>

<commit_message>
finished the big start of the application season
</commit_message>
<xml_diff>
--- a/EconJM_status.xlsx
+++ b/EconJM_status.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\javie\Dropbox\Work\Job Search\2025 EconJM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6BECE46-260F-430F-9FA4-C278874CD683}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{818DAC6E-E42D-4253-9031-FD3B496FCE97}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="14620" xr2:uid="{6FE48536-7E5C-BF4C-9490-2A6392576298}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="14620" activeTab="2" xr2:uid="{6FE48536-7E5C-BF4C-9490-2A6392576298}"/>
   </bookViews>
   <sheets>
     <sheet name="sum" sheetId="1" r:id="rId1"/>
@@ -18,7 +18,7 @@
     <sheet name="stats" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">sum!$A$1:$V$19</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">sum!$A$1:$V$248</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -1083,7 +1083,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2463" uniqueCount="784">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2496" uniqueCount="789">
   <si>
     <t>add_id</t>
   </si>
@@ -3471,6 +3471,21 @@
   </si>
   <si>
     <t>great fit with the department? (a bunch of new PhD have graduated with media + AI)</t>
+  </si>
+  <si>
+    <t>dartmouth_post</t>
+  </si>
+  <si>
+    <t>https://apply.interfolio.com/176743</t>
+  </si>
+  <si>
+    <t>Dartmouth</t>
+  </si>
+  <si>
+    <t>eca</t>
+  </si>
+  <si>
+    <t>E.CA Economics</t>
   </si>
 </sst>
 </file>
@@ -3598,7 +3613,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
@@ -3644,13 +3659,16 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="10" fontId="7" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Percent" xfId="2" builtinId="5"/>
   </cellStyles>
-  <dxfs count="191">
+  <dxfs count="194">
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -3658,46 +3676,6 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -5455,6 +5433,66 @@
       <font>
         <color rgb="FF9C0006"/>
       </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
     </dxf>
     <dxf>
       <font>
@@ -5505,6 +5543,16 @@
       <fill>
         <patternFill patternType="none">
           <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -36926,7 +36974,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F7772053-9363-CA4A-A53F-040B7C700753}">
-  <dimension ref="A1:V247"/>
+  <dimension ref="A1:V249"/>
   <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="16" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="19.6640625" customWidth="1"/>
@@ -38659,7 +38707,7 @@
       <c r="A38" s="4" t="s">
         <v>122</v>
       </c>
-      <c r="B38" s="19"/>
+      <c r="B38" s="22"/>
       <c r="D38" s="1">
         <v>45955</v>
       </c>
@@ -40095,6 +40143,7 @@
       <c r="A71" s="4" t="s">
         <v>314</v>
       </c>
+      <c r="B71" s="19"/>
       <c r="C71" t="s">
         <v>315</v>
       </c>
@@ -40199,7 +40248,7 @@
       <c r="A73" s="4" t="s">
         <v>116</v>
       </c>
-      <c r="B73" s="19"/>
+      <c r="B73" s="22"/>
       <c r="C73" t="s">
         <v>407</v>
       </c>
@@ -40911,9 +40960,10 @@
       </c>
     </row>
     <row r="89" spans="1:22" x14ac:dyDescent="0.4">
-      <c r="A89" t="s">
+      <c r="A89" s="4" t="s">
         <v>327</v>
       </c>
+      <c r="B89" s="19"/>
       <c r="D89" s="1">
         <v>45966</v>
       </c>
@@ -42087,7 +42137,7 @@
       <c r="A113" s="4" t="s">
         <v>388</v>
       </c>
-      <c r="B113" s="19"/>
+      <c r="B113" s="22"/>
       <c r="C113" t="s">
         <v>390</v>
       </c>
@@ -42192,7 +42242,7 @@
       <c r="A115" s="4" t="s">
         <v>342</v>
       </c>
-      <c r="B115" s="19"/>
+      <c r="B115" s="22"/>
       <c r="C115" t="s">
         <v>346</v>
       </c>
@@ -43991,6 +44041,7 @@
       <c r="A155" s="4" t="s">
         <v>140</v>
       </c>
+      <c r="B155" s="19"/>
       <c r="C155" t="s">
         <v>633</v>
       </c>
@@ -45960,7 +46011,7 @@
         <v>96</v>
       </c>
       <c r="J198" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="M198" t="s">
         <v>376</v>
@@ -46394,7 +46445,7 @@
         <v>96</v>
       </c>
       <c r="J208" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="M208" t="s">
         <v>651</v>
@@ -47422,7 +47473,7 @@
       </c>
     </row>
     <row r="232" spans="1:22" x14ac:dyDescent="0.4">
-      <c r="A232" s="22" t="s">
+      <c r="A232" t="s">
         <v>760</v>
       </c>
       <c r="D232" s="1">
@@ -47676,7 +47727,7 @@
         <v>40</v>
       </c>
       <c r="I237" t="s">
-        <v>23</v>
+        <v>96</v>
       </c>
       <c r="J237" t="s">
         <v>402</v>
@@ -47805,7 +47856,7 @@
         <v>715</v>
       </c>
       <c r="I240" t="s">
-        <v>23</v>
+        <v>96</v>
       </c>
       <c r="J240" t="s">
         <v>402</v>
@@ -47846,7 +47897,7 @@
         <v>569</v>
       </c>
       <c r="I241" t="s">
-        <v>23</v>
+        <v>96</v>
       </c>
       <c r="J241" t="s">
         <v>402</v>
@@ -47934,7 +47985,7 @@
         <v>721</v>
       </c>
       <c r="I243" t="s">
-        <v>23</v>
+        <v>96</v>
       </c>
       <c r="J243" t="s">
         <v>402</v>
@@ -47968,6 +48019,7 @@
       <c r="A244" s="4" t="s">
         <v>719</v>
       </c>
+      <c r="B244" s="19"/>
       <c r="C244" t="s">
         <v>783</v>
       </c>
@@ -47981,7 +48033,7 @@
         <v>3</v>
       </c>
       <c r="I244" t="s">
-        <v>23</v>
+        <v>96</v>
       </c>
       <c r="J244" t="s">
         <v>402</v>
@@ -48031,7 +48083,7 @@
         <v>529</v>
       </c>
       <c r="I245" t="s">
-        <v>23</v>
+        <v>96</v>
       </c>
       <c r="J245" t="s">
         <v>402</v>
@@ -48140,59 +48192,147 @@
         <v>0</v>
       </c>
     </row>
+    <row r="248" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A248" t="s">
+        <v>784</v>
+      </c>
+      <c r="D248" s="1">
+        <v>45992</v>
+      </c>
+      <c r="E248" t="s">
+        <v>40</v>
+      </c>
+      <c r="F248" t="s">
+        <v>785</v>
+      </c>
+      <c r="I248" t="s">
+        <v>23</v>
+      </c>
+      <c r="J248" t="s">
+        <v>402</v>
+      </c>
+      <c r="K248" t="s">
+        <v>244</v>
+      </c>
+      <c r="L248" s="1">
+        <v>46027</v>
+      </c>
+      <c r="M248" t="s">
+        <v>786</v>
+      </c>
+      <c r="N248" t="e" vm="35">
+        <v>#VALUE!</v>
+      </c>
+      <c r="O248" t="s">
+        <v>26</v>
+      </c>
+      <c r="Q248" t="s">
+        <v>776</v>
+      </c>
+      <c r="R248" s="1">
+        <v>46026</v>
+      </c>
+      <c r="T248">
+        <v>1</v>
+      </c>
+      <c r="U248">
+        <v>0</v>
+      </c>
+      <c r="V248">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="249" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A249" t="s">
+        <v>787</v>
+      </c>
+      <c r="D249" s="1">
+        <v>46016</v>
+      </c>
+      <c r="E249" t="s">
+        <v>15</v>
+      </c>
+      <c r="I249" t="s">
+        <v>96</v>
+      </c>
+      <c r="J249" t="s">
+        <v>402</v>
+      </c>
+      <c r="M249" t="s">
+        <v>788</v>
+      </c>
+      <c r="N249" t="e" vm="29">
+        <v>#VALUE!</v>
+      </c>
+      <c r="Q249" t="s">
+        <v>776</v>
+      </c>
+      <c r="R249" s="1">
+        <v>45992</v>
+      </c>
+      <c r="T249">
+        <v>0</v>
+      </c>
+      <c r="U249">
+        <v>0</v>
+      </c>
+      <c r="V249">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:V19" xr:uid="{F7772053-9363-CA4A-A53F-040B7C700753}">
+  <autoFilter ref="A1:V248" xr:uid="{F7772053-9363-CA4A-A53F-040B7C700753}">
     <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:V247">
       <sortCondition ref="D1:D19"/>
     </sortState>
   </autoFilter>
   <conditionalFormatting sqref="A1:B208 A210:B1048576">
-    <cfRule type="duplicateValues" dxfId="190" priority="14"/>
+    <cfRule type="duplicateValues" dxfId="193" priority="14"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A2:B22">
-    <cfRule type="duplicateValues" dxfId="189" priority="15"/>
+    <cfRule type="duplicateValues" dxfId="192" priority="15"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A61:B61">
-    <cfRule type="duplicateValues" dxfId="188" priority="13"/>
+    <cfRule type="duplicateValues" dxfId="191" priority="13"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="I1:I1048576">
-    <cfRule type="containsText" dxfId="187" priority="6" operator="containsText" text="closed">
+    <cfRule type="containsText" dxfId="190" priority="6" operator="containsText" text="closed">
       <formula>NOT(ISERROR(SEARCH("closed",I1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="186" priority="7" operator="containsText" text="abandoned">
+    <cfRule type="containsText" dxfId="189" priority="7" operator="containsText" text="abandoned">
       <formula>NOT(ISERROR(SEARCH("abandoned",I1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="185" priority="9" operator="containsText" text="late app">
+    <cfRule type="containsText" dxfId="188" priority="9" operator="containsText" text="late app">
       <formula>NOT(ISERROR(SEARCH("late app",I1)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I2:L223 O78:O80 O83:O89 O92:O112 O115:O124 O126:O181 R136 R153 R159 R166 R173 R178 O183:O205 O208:O211 O213:O218 O220:O233 I224:K224 R225 O235:O237 O239:O247 I1:J1 I225:L1048576">
-    <cfRule type="containsText" dxfId="4" priority="12" operator="containsText" text="completed">
+  <conditionalFormatting sqref="I2:L223 O78:O80 O83:O89 O92:O112 O115:O124 O126:O181 R136 R153 R159 R166 R173 R178 O183:O205 O208:O211 O213:O218 O220:O233 I224:K224 R225 I225:L1048576 O235:O237 I1:J1 M248 O239:O248">
+    <cfRule type="containsText" dxfId="187" priority="12" operator="containsText" text="completed">
       <formula>NOT(ISERROR(SEARCH("completed",I1)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J1:J1048576">
-    <cfRule type="containsText" dxfId="184" priority="1" operator="containsText" text="no news">
+    <cfRule type="containsText" dxfId="186" priority="1" operator="containsText" text="no news">
       <formula>NOT(ISERROR(SEARCH("no news",J1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="183" priority="2" operator="containsText" text="offer">
+    <cfRule type="containsText" dxfId="185" priority="2" operator="containsText" text="offer">
       <formula>NOT(ISERROR(SEARCH("offer",J1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="182" priority="3" operator="containsText" text="fly out">
+    <cfRule type="containsText" dxfId="184" priority="3" operator="containsText" text="fly out">
       <formula>NOT(ISERROR(SEARCH("fly out",J1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="181" priority="4" operator="containsText" text="interview">
+    <cfRule type="containsText" dxfId="183" priority="4" operator="containsText" text="interview">
       <formula>NOT(ISERROR(SEARCH("interview",J1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="180" priority="5" operator="containsText" text="rejected">
+    <cfRule type="containsText" dxfId="182" priority="5" operator="containsText" text="rejected">
       <formula>NOT(ISERROR(SEARCH("rejected",J1)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K1:L223 O78:O80 O83:O89 O92:O112 O115:O124 O126:O181 R136 R153 R159 R166 R173 R178 O183:O205 O208:O211 O213:O218 O220:O233 K224 R225 O235:O237 O239:O247 K225:L1048576">
-    <cfRule type="containsText" dxfId="3" priority="10" operator="containsText" text="NO">
+  <conditionalFormatting sqref="K1:L223 O78:O80 O83:O89 O92:O112 O115:O124 O126:O181 R136 R153 R159 R166 R173 R178 O183:O205 O208:O211 O213:O218 O220:O233 K224 R225 K225:L1048576 O235:O237 M248 O239:O248">
+    <cfRule type="containsText" dxfId="181" priority="10" operator="containsText" text="NO">
       <formula>NOT(ISERROR(SEARCH("NO",K1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="2" priority="11" operator="containsText" text="YES">
+    <cfRule type="containsText" dxfId="180" priority="11" operator="containsText" text="YES">
       <formula>NOT(ISERROR(SEARCH("YES",K1)))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -48305,7 +48445,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{923E81FA-B875-3C4E-A189-1A21268FA086}">
-  <dimension ref="A1:C252"/>
+  <dimension ref="A1:C261"/>
   <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="16" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="32.83203125" customWidth="1"/>
@@ -51022,507 +51162,618 @@
         <v>97</v>
       </c>
     </row>
+    <row r="253" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A253" s="1">
+        <v>45983</v>
+      </c>
+      <c r="B253" t="s">
+        <v>648</v>
+      </c>
+      <c r="C253" t="s">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="254" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A254" s="1">
+        <v>45983</v>
+      </c>
+      <c r="B254" t="s">
+        <v>719</v>
+      </c>
+      <c r="C254" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="255" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A255" s="1">
+        <v>45985</v>
+      </c>
+      <c r="B255" t="s">
+        <v>414</v>
+      </c>
+      <c r="C255" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="256" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A256" s="1">
+        <v>45985</v>
+      </c>
+      <c r="B256" t="s">
+        <v>377</v>
+      </c>
+      <c r="C256" t="s">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="257" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A257" s="1">
+        <v>45985</v>
+      </c>
+      <c r="B257" t="s">
+        <v>714</v>
+      </c>
+      <c r="C257" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="258" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A258" s="1">
+        <v>45985</v>
+      </c>
+      <c r="B258" t="s">
+        <v>568</v>
+      </c>
+      <c r="C258" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="259" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A259" s="1">
+        <v>45985</v>
+      </c>
+      <c r="B259" t="s">
+        <v>787</v>
+      </c>
+      <c r="C259" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="260" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A260" s="1">
+        <v>45985</v>
+      </c>
+      <c r="B260" t="s">
+        <v>722</v>
+      </c>
+      <c r="C260" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="261" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A261" s="1">
+        <v>45985</v>
+      </c>
+      <c r="B261" t="s">
+        <v>528</v>
+      </c>
+      <c r="C261" t="s">
+        <v>97</v>
+      </c>
+    </row>
   </sheetData>
   <conditionalFormatting sqref="B5">
-    <cfRule type="duplicateValues" dxfId="179" priority="182"/>
-    <cfRule type="duplicateValues" dxfId="178" priority="183"/>
+    <cfRule type="duplicateValues" dxfId="179" priority="186"/>
+    <cfRule type="duplicateValues" dxfId="178" priority="187"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B10">
-    <cfRule type="duplicateValues" dxfId="177" priority="181"/>
-    <cfRule type="duplicateValues" dxfId="176" priority="180"/>
+    <cfRule type="duplicateValues" dxfId="177" priority="185"/>
+    <cfRule type="duplicateValues" dxfId="176" priority="184"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B11">
-    <cfRule type="duplicateValues" dxfId="175" priority="179"/>
-    <cfRule type="duplicateValues" dxfId="174" priority="178"/>
+    <cfRule type="duplicateValues" dxfId="175" priority="183"/>
+    <cfRule type="duplicateValues" dxfId="174" priority="182"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B12">
-    <cfRule type="duplicateValues" dxfId="173" priority="177"/>
-    <cfRule type="duplicateValues" dxfId="172" priority="176"/>
+    <cfRule type="duplicateValues" dxfId="173" priority="181"/>
+    <cfRule type="duplicateValues" dxfId="172" priority="180"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B15">
-    <cfRule type="duplicateValues" dxfId="171" priority="175"/>
-    <cfRule type="duplicateValues" dxfId="170" priority="174"/>
+    <cfRule type="duplicateValues" dxfId="171" priority="179"/>
+    <cfRule type="duplicateValues" dxfId="170" priority="178"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B16">
-    <cfRule type="duplicateValues" dxfId="169" priority="173"/>
+    <cfRule type="duplicateValues" dxfId="169" priority="177"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B17">
-    <cfRule type="duplicateValues" dxfId="168" priority="172"/>
-    <cfRule type="duplicateValues" dxfId="167" priority="171"/>
+    <cfRule type="duplicateValues" dxfId="168" priority="176"/>
+    <cfRule type="duplicateValues" dxfId="167" priority="175"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B18">
-    <cfRule type="duplicateValues" dxfId="166" priority="170"/>
-    <cfRule type="duplicateValues" dxfId="165" priority="169"/>
+    <cfRule type="duplicateValues" dxfId="166" priority="174"/>
+    <cfRule type="duplicateValues" dxfId="165" priority="173"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B19">
-    <cfRule type="duplicateValues" dxfId="164" priority="168"/>
+    <cfRule type="duplicateValues" dxfId="164" priority="172"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B22:B23">
-    <cfRule type="duplicateValues" dxfId="163" priority="167"/>
-    <cfRule type="duplicateValues" dxfId="162" priority="166"/>
+    <cfRule type="duplicateValues" dxfId="163" priority="171"/>
+    <cfRule type="duplicateValues" dxfId="162" priority="170"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B24">
-    <cfRule type="duplicateValues" dxfId="161" priority="165"/>
-    <cfRule type="duplicateValues" dxfId="160" priority="164"/>
+    <cfRule type="duplicateValues" dxfId="161" priority="169"/>
+    <cfRule type="duplicateValues" dxfId="160" priority="168"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B27">
-    <cfRule type="duplicateValues" dxfId="159" priority="163"/>
-    <cfRule type="duplicateValues" dxfId="158" priority="162"/>
+    <cfRule type="duplicateValues" dxfId="159" priority="167"/>
+    <cfRule type="duplicateValues" dxfId="158" priority="166"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B28">
-    <cfRule type="duplicateValues" dxfId="157" priority="161"/>
+    <cfRule type="duplicateValues" dxfId="157" priority="165"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B29">
-    <cfRule type="duplicateValues" dxfId="156" priority="160"/>
-    <cfRule type="duplicateValues" dxfId="155" priority="159"/>
+    <cfRule type="duplicateValues" dxfId="156" priority="164"/>
+    <cfRule type="duplicateValues" dxfId="155" priority="163"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B30">
-    <cfRule type="duplicateValues" dxfId="154" priority="158"/>
+    <cfRule type="duplicateValues" dxfId="154" priority="162"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B31">
-    <cfRule type="duplicateValues" dxfId="153" priority="157"/>
+    <cfRule type="duplicateValues" dxfId="153" priority="161"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B32">
-    <cfRule type="duplicateValues" dxfId="152" priority="156"/>
+    <cfRule type="duplicateValues" dxfId="152" priority="160"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B33">
-    <cfRule type="duplicateValues" dxfId="151" priority="155"/>
+    <cfRule type="duplicateValues" dxfId="151" priority="159"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B34">
-    <cfRule type="duplicateValues" dxfId="150" priority="154"/>
+    <cfRule type="duplicateValues" dxfId="150" priority="158"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B35">
-    <cfRule type="duplicateValues" dxfId="149" priority="153"/>
+    <cfRule type="duplicateValues" dxfId="149" priority="157"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B37">
-    <cfRule type="duplicateValues" dxfId="148" priority="152"/>
+    <cfRule type="duplicateValues" dxfId="148" priority="156"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B38">
-    <cfRule type="duplicateValues" dxfId="147" priority="151"/>
+    <cfRule type="duplicateValues" dxfId="147" priority="155"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B42">
-    <cfRule type="duplicateValues" dxfId="146" priority="150"/>
+    <cfRule type="duplicateValues" dxfId="146" priority="154"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B43">
-    <cfRule type="duplicateValues" dxfId="145" priority="149"/>
+    <cfRule type="duplicateValues" dxfId="145" priority="153"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B44:B45">
-    <cfRule type="duplicateValues" dxfId="144" priority="148"/>
+    <cfRule type="duplicateValues" dxfId="144" priority="152"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B46">
-    <cfRule type="duplicateValues" dxfId="143" priority="147"/>
+    <cfRule type="duplicateValues" dxfId="143" priority="151"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B48">
-    <cfRule type="duplicateValues" dxfId="142" priority="146"/>
+    <cfRule type="duplicateValues" dxfId="142" priority="150"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B49">
-    <cfRule type="duplicateValues" dxfId="141" priority="145"/>
+    <cfRule type="duplicateValues" dxfId="141" priority="149"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B51">
-    <cfRule type="duplicateValues" dxfId="140" priority="144"/>
+    <cfRule type="duplicateValues" dxfId="140" priority="148"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B52">
-    <cfRule type="duplicateValues" dxfId="139" priority="143"/>
+    <cfRule type="duplicateValues" dxfId="139" priority="147"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B58">
-    <cfRule type="duplicateValues" dxfId="138" priority="141"/>
+    <cfRule type="duplicateValues" dxfId="138" priority="145"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B59">
-    <cfRule type="duplicateValues" dxfId="137" priority="139"/>
+    <cfRule type="duplicateValues" dxfId="137" priority="143"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B63">
-    <cfRule type="duplicateValues" dxfId="136" priority="138"/>
+    <cfRule type="duplicateValues" dxfId="136" priority="142"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B64">
-    <cfRule type="duplicateValues" dxfId="135" priority="136"/>
+    <cfRule type="duplicateValues" dxfId="135" priority="140"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B66">
-    <cfRule type="duplicateValues" dxfId="134" priority="135"/>
+    <cfRule type="duplicateValues" dxfId="134" priority="139"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B67">
-    <cfRule type="duplicateValues" dxfId="133" priority="134"/>
-    <cfRule type="duplicateValues" dxfId="132" priority="133"/>
+    <cfRule type="duplicateValues" dxfId="133" priority="138"/>
+    <cfRule type="duplicateValues" dxfId="132" priority="137"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B68">
-    <cfRule type="duplicateValues" dxfId="131" priority="132"/>
+    <cfRule type="duplicateValues" dxfId="131" priority="136"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B69">
-    <cfRule type="duplicateValues" dxfId="130" priority="131"/>
+    <cfRule type="duplicateValues" dxfId="130" priority="135"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B70">
-    <cfRule type="duplicateValues" dxfId="129" priority="129"/>
+    <cfRule type="duplicateValues" dxfId="129" priority="133"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B72">
-    <cfRule type="duplicateValues" dxfId="128" priority="128"/>
+    <cfRule type="duplicateValues" dxfId="128" priority="132"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B73">
-    <cfRule type="duplicateValues" dxfId="127" priority="126"/>
+    <cfRule type="duplicateValues" dxfId="127" priority="130"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B74">
-    <cfRule type="duplicateValues" dxfId="126" priority="125"/>
+    <cfRule type="duplicateValues" dxfId="126" priority="129"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B75">
-    <cfRule type="duplicateValues" dxfId="125" priority="124"/>
+    <cfRule type="duplicateValues" dxfId="125" priority="128"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B76">
-    <cfRule type="duplicateValues" dxfId="124" priority="123"/>
+    <cfRule type="duplicateValues" dxfId="124" priority="127"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B77">
-    <cfRule type="duplicateValues" dxfId="123" priority="121"/>
+    <cfRule type="duplicateValues" dxfId="123" priority="125"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B78">
-    <cfRule type="duplicateValues" dxfId="122" priority="120"/>
+    <cfRule type="duplicateValues" dxfId="122" priority="124"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B83">
-    <cfRule type="duplicateValues" dxfId="121" priority="119"/>
+    <cfRule type="duplicateValues" dxfId="121" priority="123"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B84">
-    <cfRule type="duplicateValues" dxfId="120" priority="118"/>
+    <cfRule type="duplicateValues" dxfId="120" priority="122"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B85">
-    <cfRule type="duplicateValues" dxfId="119" priority="117"/>
+    <cfRule type="duplicateValues" dxfId="119" priority="121"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B87">
-    <cfRule type="duplicateValues" dxfId="118" priority="116"/>
+    <cfRule type="duplicateValues" dxfId="118" priority="120"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B88">
-    <cfRule type="duplicateValues" dxfId="117" priority="115"/>
+    <cfRule type="duplicateValues" dxfId="117" priority="119"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B89">
-    <cfRule type="duplicateValues" dxfId="116" priority="114"/>
+    <cfRule type="duplicateValues" dxfId="116" priority="118"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B90">
-    <cfRule type="duplicateValues" dxfId="115" priority="113"/>
+    <cfRule type="duplicateValues" dxfId="115" priority="117"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B91">
-    <cfRule type="duplicateValues" dxfId="114" priority="112"/>
+    <cfRule type="duplicateValues" dxfId="114" priority="116"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B92">
-    <cfRule type="duplicateValues" dxfId="113" priority="111"/>
+    <cfRule type="duplicateValues" dxfId="113" priority="115"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B93">
-    <cfRule type="duplicateValues" dxfId="112" priority="110"/>
+    <cfRule type="duplicateValues" dxfId="112" priority="114"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B94">
-    <cfRule type="duplicateValues" dxfId="111" priority="109"/>
+    <cfRule type="duplicateValues" dxfId="111" priority="113"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B95">
-    <cfRule type="duplicateValues" dxfId="110" priority="108"/>
+    <cfRule type="duplicateValues" dxfId="110" priority="112"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B96">
-    <cfRule type="duplicateValues" dxfId="109" priority="107"/>
+    <cfRule type="duplicateValues" dxfId="109" priority="111"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B97">
-    <cfRule type="duplicateValues" dxfId="108" priority="106"/>
+    <cfRule type="duplicateValues" dxfId="108" priority="110"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B98">
-    <cfRule type="duplicateValues" dxfId="107" priority="105"/>
+    <cfRule type="duplicateValues" dxfId="107" priority="109"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B99">
-    <cfRule type="duplicateValues" dxfId="106" priority="104"/>
+    <cfRule type="duplicateValues" dxfId="106" priority="108"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B100">
-    <cfRule type="duplicateValues" dxfId="105" priority="103"/>
+    <cfRule type="duplicateValues" dxfId="105" priority="107"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B101">
-    <cfRule type="duplicateValues" dxfId="104" priority="102"/>
+    <cfRule type="duplicateValues" dxfId="104" priority="106"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B104">
-    <cfRule type="duplicateValues" dxfId="103" priority="101"/>
-    <cfRule type="duplicateValues" dxfId="102" priority="100"/>
+    <cfRule type="duplicateValues" dxfId="103" priority="105"/>
+    <cfRule type="duplicateValues" dxfId="102" priority="104"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B105:B106">
-    <cfRule type="duplicateValues" dxfId="101" priority="99"/>
+    <cfRule type="duplicateValues" dxfId="101" priority="103"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B107">
-    <cfRule type="duplicateValues" dxfId="100" priority="98"/>
+    <cfRule type="duplicateValues" dxfId="100" priority="102"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B108">
-    <cfRule type="duplicateValues" dxfId="99" priority="97"/>
+    <cfRule type="duplicateValues" dxfId="99" priority="101"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B109">
-    <cfRule type="duplicateValues" dxfId="98" priority="96"/>
+    <cfRule type="duplicateValues" dxfId="98" priority="100"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B110">
-    <cfRule type="duplicateValues" dxfId="97" priority="95"/>
+    <cfRule type="duplicateValues" dxfId="97" priority="99"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B111">
-    <cfRule type="duplicateValues" dxfId="96" priority="94"/>
+    <cfRule type="duplicateValues" dxfId="96" priority="98"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B112">
-    <cfRule type="duplicateValues" dxfId="95" priority="93"/>
+    <cfRule type="duplicateValues" dxfId="95" priority="97"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B113">
-    <cfRule type="duplicateValues" dxfId="94" priority="92"/>
+    <cfRule type="duplicateValues" dxfId="94" priority="96"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B114">
-    <cfRule type="duplicateValues" dxfId="93" priority="91"/>
+    <cfRule type="duplicateValues" dxfId="93" priority="95"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B115">
-    <cfRule type="duplicateValues" dxfId="92" priority="90"/>
+    <cfRule type="duplicateValues" dxfId="92" priority="94"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B116">
-    <cfRule type="duplicateValues" dxfId="91" priority="89"/>
+    <cfRule type="duplicateValues" dxfId="91" priority="93"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B117">
-    <cfRule type="duplicateValues" dxfId="90" priority="88"/>
+    <cfRule type="duplicateValues" dxfId="90" priority="92"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B118">
-    <cfRule type="duplicateValues" dxfId="89" priority="87"/>
+    <cfRule type="duplicateValues" dxfId="89" priority="91"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B119">
-    <cfRule type="duplicateValues" dxfId="88" priority="86"/>
+    <cfRule type="duplicateValues" dxfId="88" priority="90"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B120">
-    <cfRule type="duplicateValues" dxfId="87" priority="85"/>
+    <cfRule type="duplicateValues" dxfId="87" priority="89"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B121">
-    <cfRule type="duplicateValues" dxfId="86" priority="84"/>
+    <cfRule type="duplicateValues" dxfId="86" priority="88"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B122">
-    <cfRule type="duplicateValues" dxfId="85" priority="83"/>
+    <cfRule type="duplicateValues" dxfId="85" priority="87"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B126">
-    <cfRule type="duplicateValues" dxfId="84" priority="82"/>
+    <cfRule type="duplicateValues" dxfId="84" priority="86"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B127">
-    <cfRule type="duplicateValues" dxfId="83" priority="81"/>
+    <cfRule type="duplicateValues" dxfId="83" priority="85"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B128">
-    <cfRule type="duplicateValues" dxfId="82" priority="80"/>
+    <cfRule type="duplicateValues" dxfId="82" priority="84"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B129">
-    <cfRule type="duplicateValues" dxfId="81" priority="79"/>
+    <cfRule type="duplicateValues" dxfId="81" priority="83"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B130">
-    <cfRule type="duplicateValues" dxfId="80" priority="78"/>
+    <cfRule type="duplicateValues" dxfId="80" priority="82"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B131">
-    <cfRule type="duplicateValues" dxfId="79" priority="77"/>
+    <cfRule type="duplicateValues" dxfId="79" priority="81"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B132">
-    <cfRule type="duplicateValues" dxfId="78" priority="76"/>
+    <cfRule type="duplicateValues" dxfId="78" priority="80"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B133">
-    <cfRule type="duplicateValues" dxfId="77" priority="75"/>
+    <cfRule type="duplicateValues" dxfId="77" priority="79"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B136">
-    <cfRule type="duplicateValues" dxfId="76" priority="74"/>
+    <cfRule type="duplicateValues" dxfId="76" priority="78"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B137">
-    <cfRule type="duplicateValues" dxfId="75" priority="73"/>
+    <cfRule type="duplicateValues" dxfId="75" priority="77"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B138">
-    <cfRule type="duplicateValues" dxfId="74" priority="72"/>
+    <cfRule type="duplicateValues" dxfId="74" priority="76"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B139">
-    <cfRule type="duplicateValues" dxfId="73" priority="71"/>
+    <cfRule type="duplicateValues" dxfId="73" priority="75"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B140">
-    <cfRule type="duplicateValues" dxfId="72" priority="70"/>
+    <cfRule type="duplicateValues" dxfId="72" priority="74"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B141">
-    <cfRule type="duplicateValues" dxfId="71" priority="69"/>
+    <cfRule type="duplicateValues" dxfId="71" priority="73"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B142">
-    <cfRule type="duplicateValues" dxfId="70" priority="68"/>
+    <cfRule type="duplicateValues" dxfId="70" priority="72"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B143">
-    <cfRule type="duplicateValues" dxfId="69" priority="67"/>
+    <cfRule type="duplicateValues" dxfId="69" priority="71"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B144">
-    <cfRule type="duplicateValues" dxfId="68" priority="66"/>
+    <cfRule type="duplicateValues" dxfId="68" priority="70"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B145">
-    <cfRule type="duplicateValues" dxfId="67" priority="65"/>
+    <cfRule type="duplicateValues" dxfId="67" priority="69"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B147">
-    <cfRule type="duplicateValues" dxfId="66" priority="64"/>
+    <cfRule type="duplicateValues" dxfId="66" priority="68"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B148">
-    <cfRule type="duplicateValues" dxfId="65" priority="63"/>
+    <cfRule type="duplicateValues" dxfId="65" priority="67"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B149">
-    <cfRule type="duplicateValues" dxfId="64" priority="62"/>
+    <cfRule type="duplicateValues" dxfId="64" priority="66"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B150">
-    <cfRule type="duplicateValues" dxfId="63" priority="61"/>
+    <cfRule type="duplicateValues" dxfId="63" priority="65"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B151">
-    <cfRule type="duplicateValues" dxfId="62" priority="60"/>
+    <cfRule type="duplicateValues" dxfId="62" priority="64"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B152">
-    <cfRule type="duplicateValues" dxfId="61" priority="59"/>
+    <cfRule type="duplicateValues" dxfId="61" priority="63"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B153">
-    <cfRule type="duplicateValues" dxfId="60" priority="58"/>
+    <cfRule type="duplicateValues" dxfId="60" priority="62"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B154">
-    <cfRule type="duplicateValues" dxfId="59" priority="57"/>
+    <cfRule type="duplicateValues" dxfId="59" priority="61"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B155">
-    <cfRule type="duplicateValues" dxfId="58" priority="56"/>
+    <cfRule type="duplicateValues" dxfId="58" priority="60"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B156">
-    <cfRule type="duplicateValues" dxfId="57" priority="55"/>
+    <cfRule type="duplicateValues" dxfId="57" priority="59"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B157">
-    <cfRule type="duplicateValues" dxfId="56" priority="54"/>
+    <cfRule type="duplicateValues" dxfId="56" priority="58"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B171">
-    <cfRule type="duplicateValues" dxfId="55" priority="53"/>
+    <cfRule type="duplicateValues" dxfId="55" priority="57"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B172">
-    <cfRule type="duplicateValues" dxfId="54" priority="52"/>
+    <cfRule type="duplicateValues" dxfId="54" priority="56"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B174">
-    <cfRule type="duplicateValues" dxfId="53" priority="51"/>
+    <cfRule type="duplicateValues" dxfId="53" priority="55"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B177:B178">
-    <cfRule type="duplicateValues" dxfId="52" priority="50"/>
+    <cfRule type="duplicateValues" dxfId="52" priority="54"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B181">
-    <cfRule type="duplicateValues" dxfId="51" priority="49"/>
+    <cfRule type="duplicateValues" dxfId="51" priority="53"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B182">
-    <cfRule type="duplicateValues" dxfId="50" priority="48"/>
+    <cfRule type="duplicateValues" dxfId="50" priority="52"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B183">
-    <cfRule type="duplicateValues" dxfId="49" priority="47"/>
+    <cfRule type="duplicateValues" dxfId="49" priority="51"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B184">
-    <cfRule type="duplicateValues" dxfId="48" priority="46"/>
+    <cfRule type="duplicateValues" dxfId="48" priority="50"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B185">
-    <cfRule type="duplicateValues" dxfId="47" priority="45"/>
+    <cfRule type="duplicateValues" dxfId="47" priority="49"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B186">
-    <cfRule type="duplicateValues" dxfId="46" priority="44"/>
+    <cfRule type="duplicateValues" dxfId="46" priority="48"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B188">
-    <cfRule type="duplicateValues" dxfId="45" priority="43"/>
+    <cfRule type="duplicateValues" dxfId="45" priority="47"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B189">
-    <cfRule type="duplicateValues" dxfId="44" priority="42"/>
+    <cfRule type="duplicateValues" dxfId="44" priority="46"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B190">
-    <cfRule type="duplicateValues" dxfId="43" priority="41"/>
+    <cfRule type="duplicateValues" dxfId="43" priority="45"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B191">
-    <cfRule type="duplicateValues" dxfId="42" priority="40"/>
+    <cfRule type="duplicateValues" dxfId="42" priority="44"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B192">
-    <cfRule type="duplicateValues" dxfId="41" priority="39"/>
+    <cfRule type="duplicateValues" dxfId="41" priority="43"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B193">
-    <cfRule type="duplicateValues" dxfId="40" priority="38"/>
+    <cfRule type="duplicateValues" dxfId="40" priority="42"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B195">
-    <cfRule type="duplicateValues" dxfId="39" priority="37"/>
+    <cfRule type="duplicateValues" dxfId="39" priority="41"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B196">
-    <cfRule type="duplicateValues" dxfId="38" priority="36"/>
+    <cfRule type="duplicateValues" dxfId="38" priority="40"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B197">
-    <cfRule type="duplicateValues" dxfId="37" priority="35"/>
+    <cfRule type="duplicateValues" dxfId="37" priority="39"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B198">
-    <cfRule type="duplicateValues" dxfId="36" priority="34"/>
+    <cfRule type="duplicateValues" dxfId="36" priority="38"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B199">
-    <cfRule type="duplicateValues" dxfId="35" priority="33"/>
+    <cfRule type="duplicateValues" dxfId="35" priority="37"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B200">
-    <cfRule type="duplicateValues" dxfId="34" priority="32"/>
+    <cfRule type="duplicateValues" dxfId="34" priority="36"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B201">
-    <cfRule type="duplicateValues" dxfId="33" priority="31"/>
+    <cfRule type="duplicateValues" dxfId="33" priority="35"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B202">
-    <cfRule type="duplicateValues" dxfId="32" priority="30"/>
+    <cfRule type="duplicateValues" dxfId="32" priority="34"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B203">
-    <cfRule type="duplicateValues" dxfId="31" priority="29"/>
+    <cfRule type="duplicateValues" dxfId="31" priority="33"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B204">
-    <cfRule type="duplicateValues" dxfId="30" priority="28"/>
+    <cfRule type="duplicateValues" dxfId="30" priority="32"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B205">
-    <cfRule type="duplicateValues" dxfId="29" priority="27"/>
+    <cfRule type="duplicateValues" dxfId="29" priority="31"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B206">
-    <cfRule type="duplicateValues" dxfId="28" priority="26"/>
+    <cfRule type="duplicateValues" dxfId="28" priority="30"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B207">
-    <cfRule type="duplicateValues" dxfId="27" priority="25"/>
+    <cfRule type="duplicateValues" dxfId="27" priority="29"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B215">
-    <cfRule type="duplicateValues" dxfId="26" priority="24"/>
+    <cfRule type="duplicateValues" dxfId="26" priority="28"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B218">
-    <cfRule type="duplicateValues" dxfId="25" priority="23"/>
+    <cfRule type="duplicateValues" dxfId="25" priority="27"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B220">
-    <cfRule type="duplicateValues" dxfId="24" priority="22"/>
+    <cfRule type="duplicateValues" dxfId="24" priority="26"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B222">
-    <cfRule type="duplicateValues" dxfId="23" priority="21"/>
+    <cfRule type="duplicateValues" dxfId="23" priority="25"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B223">
-    <cfRule type="duplicateValues" dxfId="22" priority="20"/>
+    <cfRule type="duplicateValues" dxfId="22" priority="24"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B224">
-    <cfRule type="duplicateValues" dxfId="21" priority="19"/>
+    <cfRule type="duplicateValues" dxfId="21" priority="23"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B225">
-    <cfRule type="duplicateValues" dxfId="20" priority="18"/>
+    <cfRule type="duplicateValues" dxfId="20" priority="22"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B227">
-    <cfRule type="duplicateValues" dxfId="19" priority="17"/>
+    <cfRule type="duplicateValues" dxfId="19" priority="21"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B229">
-    <cfRule type="duplicateValues" dxfId="18" priority="16"/>
+    <cfRule type="duplicateValues" dxfId="18" priority="20"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B230">
-    <cfRule type="duplicateValues" dxfId="17" priority="15"/>
+    <cfRule type="duplicateValues" dxfId="17" priority="19"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B232">
-    <cfRule type="duplicateValues" dxfId="16" priority="14"/>
+    <cfRule type="duplicateValues" dxfId="16" priority="18"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B233">
-    <cfRule type="duplicateValues" dxfId="15" priority="13"/>
+    <cfRule type="duplicateValues" dxfId="15" priority="17"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B234">
-    <cfRule type="duplicateValues" dxfId="14" priority="12"/>
+    <cfRule type="duplicateValues" dxfId="14" priority="16"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B235">
-    <cfRule type="duplicateValues" dxfId="13" priority="11"/>
+    <cfRule type="duplicateValues" dxfId="13" priority="15"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B236">
-    <cfRule type="duplicateValues" dxfId="12" priority="10"/>
+    <cfRule type="duplicateValues" dxfId="12" priority="14"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B237">
-    <cfRule type="duplicateValues" dxfId="11" priority="9"/>
+    <cfRule type="duplicateValues" dxfId="11" priority="13"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B239">
-    <cfRule type="duplicateValues" dxfId="9" priority="7"/>
+    <cfRule type="duplicateValues" dxfId="10" priority="11"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B240">
-    <cfRule type="duplicateValues" dxfId="8" priority="6"/>
+    <cfRule type="duplicateValues" dxfId="9" priority="10"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B241">
-    <cfRule type="duplicateValues" dxfId="7" priority="5"/>
+    <cfRule type="duplicateValues" dxfId="8" priority="9"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B242">
-    <cfRule type="duplicateValues" dxfId="6" priority="4"/>
+    <cfRule type="duplicateValues" dxfId="7" priority="8"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B243">
-    <cfRule type="duplicateValues" dxfId="5" priority="3"/>
+    <cfRule type="duplicateValues" dxfId="6" priority="7"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B250">
+    <cfRule type="duplicateValues" dxfId="5" priority="6"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B251">
+    <cfRule type="duplicateValues" dxfId="4" priority="5"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B253">
+    <cfRule type="duplicateValues" dxfId="3" priority="4"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B255">
+    <cfRule type="duplicateValues" dxfId="2" priority="3"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B258:B259">
     <cfRule type="duplicateValues" dxfId="1" priority="2"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B251">
+  <conditionalFormatting sqref="B260">
     <cfRule type="duplicateValues" dxfId="0" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -51536,7 +51787,7 @@
   <cols>
     <col min="1" max="1" width="15.83203125" style="12" customWidth="1"/>
     <col min="2" max="2" width="10.83203125" style="16"/>
-    <col min="3" max="3" width="10.83203125" style="10"/>
+    <col min="3" max="3" width="15.33203125" style="10" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="26" x14ac:dyDescent="0.6">
@@ -51545,15 +51796,15 @@
       </c>
       <c r="B1" s="15">
         <f>COUNTA(sum!A:A) -1</f>
-        <v>246</v>
-      </c>
-      <c r="C1" s="14">
-        <f>COUNTIF(sum!I:I, "completed")/B1</f>
-        <v>0.94715447154471544</v>
+        <v>248</v>
+      </c>
+      <c r="C1" s="23">
+        <f>COUNTIF(sum!I:I, "completed")/(B1-COUNTIF(sum!I:I, "abandoned")-COUNTIF(sum!I:I, "late app"))</f>
+        <v>0.99585062240663902</v>
       </c>
       <c r="D1" s="21">
         <f>COUNTIF(sum!I:I, "completed")</f>
-        <v>233</v>
+        <v>240</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="22" customHeight="1" x14ac:dyDescent="0.4">
@@ -51566,7 +51817,7 @@
       </c>
       <c r="C2" s="10">
         <f>COUNTIFS(sum!I:I,"completed", sum!G:G, "&lt;&gt;") / B2</f>
-        <v>0.94339622641509435</v>
+        <v>0.96226415094339623</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="21" customHeight="1" x14ac:dyDescent="0.4">
@@ -51575,11 +51826,11 @@
       </c>
       <c r="B3" s="16">
         <f>COUNTA(sum!K:K) -1</f>
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C3" s="10">
         <f>COUNTIFS(sum!I:I,"completed", sum!K:K, "&lt;&gt;") / B3</f>
-        <v>0.9821428571428571</v>
+        <v>0.98245614035087714</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="26" x14ac:dyDescent="0.6">
@@ -51588,7 +51839,7 @@
       </c>
       <c r="B5" s="15">
         <f>COUNTA(sum!J:J) -1</f>
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="C5" s="14">
         <f>B5/B1</f>
@@ -51605,7 +51856,7 @@
       </c>
       <c r="C6" s="10">
         <f>B6/$B$5</f>
-        <v>0.97967479674796742</v>
+        <v>0.97177419354838712</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.4">
@@ -51614,11 +51865,11 @@
       </c>
       <c r="B7" s="16">
         <f>COUNTIFS(sum!J:J,"rejected")</f>
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C7" s="10">
         <f t="shared" ref="C7:C10" si="0">B7/$B$5</f>
-        <v>2.032520325203252E-2</v>
+        <v>2.8225806451612902E-2</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.4">

</xml_diff>

<commit_message>
updated some stragelers in thanksgiving
</commit_message>
<xml_diff>
--- a/EconJM_status.xlsx
+++ b/EconJM_status.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\javie\Dropbox\Work\Job Search\2025 EconJM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{818DAC6E-E42D-4253-9031-FD3B496FCE97}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33AB038B-FA27-40F4-A9D7-3716430E3770}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="14620" activeTab="2" xr2:uid="{6FE48536-7E5C-BF4C-9490-2A6392576298}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="14620" activeTab="1" xr2:uid="{6FE48536-7E5C-BF4C-9490-2A6392576298}"/>
   </bookViews>
   <sheets>
     <sheet name="sum" sheetId="1" r:id="rId1"/>
@@ -1083,7 +1083,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2496" uniqueCount="789">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2538" uniqueCount="802">
   <si>
     <t>add_id</t>
   </si>
@@ -3486,6 +3486,45 @@
   </si>
   <si>
     <t>E.CA Economics</t>
+  </si>
+  <si>
+    <t>Lisbon School of Economics and Management</t>
+  </si>
+  <si>
+    <t>iseg</t>
+  </si>
+  <si>
+    <t>manhaeim</t>
+  </si>
+  <si>
+    <t>escp</t>
+  </si>
+  <si>
+    <t>ESCP Business School</t>
+  </si>
+  <si>
+    <t>submit CV to https://tinyurl.com/BerlinESCPEcon</t>
+  </si>
+  <si>
+    <t>https://tinyurl.com/BerlinESCPEcon</t>
+  </si>
+  <si>
+    <t>unidistance_post</t>
+  </si>
+  <si>
+    <t>Michael Kurschilgen: michael.kurschilgen@unidistance.ch</t>
+  </si>
+  <si>
+    <t>kings</t>
+  </si>
+  <si>
+    <t>Kings College</t>
+  </si>
+  <si>
+    <t>historical econ</t>
+  </si>
+  <si>
+    <t>added some info of stragelers in EJM and JOE</t>
   </si>
 </sst>
 </file>
@@ -3613,7 +3652,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
@@ -3658,7 +3697,6 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="10" fontId="7" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -36974,7 +37012,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F7772053-9363-CA4A-A53F-040B7C700753}">
-  <dimension ref="A1:V249"/>
+  <dimension ref="A1:V254"/>
   <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="16" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="19.6640625" customWidth="1"/>
@@ -38707,7 +38745,6 @@
       <c r="A38" s="4" t="s">
         <v>122</v>
       </c>
-      <c r="B38" s="22"/>
       <c r="D38" s="1">
         <v>45955</v>
       </c>
@@ -40143,7 +40180,6 @@
       <c r="A71" s="4" t="s">
         <v>314</v>
       </c>
-      <c r="B71" s="19"/>
       <c r="C71" t="s">
         <v>315</v>
       </c>
@@ -40248,7 +40284,6 @@
       <c r="A73" s="4" t="s">
         <v>116</v>
       </c>
-      <c r="B73" s="22"/>
       <c r="C73" t="s">
         <v>407</v>
       </c>
@@ -41396,7 +41431,6 @@
       <c r="A99" s="4" t="s">
         <v>278</v>
       </c>
-      <c r="B99" s="19"/>
       <c r="C99" t="s">
         <v>279</v>
       </c>
@@ -42137,7 +42171,6 @@
       <c r="A113" s="4" t="s">
         <v>388</v>
       </c>
-      <c r="B113" s="22"/>
       <c r="C113" t="s">
         <v>390</v>
       </c>
@@ -42242,7 +42275,7 @@
       <c r="A115" s="4" t="s">
         <v>342</v>
       </c>
-      <c r="B115" s="22"/>
+      <c r="B115" s="19"/>
       <c r="C115" t="s">
         <v>346</v>
       </c>
@@ -42629,7 +42662,7 @@
         <v>96</v>
       </c>
       <c r="J123" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="M123" t="s">
         <v>575</v>
@@ -44041,7 +44074,6 @@
       <c r="A155" s="4" t="s">
         <v>140</v>
       </c>
-      <c r="B155" s="19"/>
       <c r="C155" t="s">
         <v>633</v>
       </c>
@@ -44525,6 +44557,7 @@
       <c r="A166" s="4" t="s">
         <v>687</v>
       </c>
+      <c r="B166" s="19"/>
       <c r="D166" s="1">
         <v>45976</v>
       </c>
@@ -44714,6 +44747,7 @@
       <c r="A170" s="4" t="s">
         <v>658</v>
       </c>
+      <c r="B170" s="19"/>
       <c r="C170" t="s">
         <v>659</v>
       </c>
@@ -47926,27 +47960,33 @@
     </row>
     <row r="242" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A242" t="s">
-        <v>662</v>
+        <v>784</v>
       </c>
       <c r="D242" s="1">
-        <v>46011</v>
+        <v>45992</v>
       </c>
       <c r="E242" t="s">
-        <v>15</v>
-      </c>
-      <c r="H242" t="s">
-        <v>664</v>
+        <v>40</v>
+      </c>
+      <c r="F242" t="s">
+        <v>785</v>
       </c>
       <c r="I242" t="s">
-        <v>96</v>
+        <v>23</v>
       </c>
       <c r="J242" t="s">
         <v>402</v>
       </c>
+      <c r="K242" t="s">
+        <v>244</v>
+      </c>
+      <c r="L242" s="1">
+        <v>46027</v>
+      </c>
       <c r="M242" t="s">
-        <v>663</v>
-      </c>
-      <c r="N242" t="e" vm="45">
+        <v>786</v>
+      </c>
+      <c r="N242" t="e" vm="35">
         <v>#VALUE!</v>
       </c>
       <c r="O242" t="s">
@@ -47956,7 +47996,7 @@
         <v>776</v>
       </c>
       <c r="R242" s="1">
-        <v>46037</v>
+        <v>46026</v>
       </c>
       <c r="T242">
         <v>1</v>
@@ -47970,30 +48010,24 @@
     </row>
     <row r="243" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A243" t="s">
-        <v>722</v>
-      </c>
-      <c r="C243" t="s">
-        <v>723</v>
+        <v>791</v>
       </c>
       <c r="D243" s="1">
-        <v>46016</v>
+        <v>45992</v>
       </c>
       <c r="E243" t="s">
         <v>15</v>
       </c>
-      <c r="F243" t="s">
-        <v>721</v>
-      </c>
       <c r="I243" t="s">
-        <v>96</v>
+        <v>23</v>
       </c>
       <c r="J243" t="s">
         <v>402</v>
       </c>
       <c r="M243" t="s">
-        <v>720</v>
-      </c>
-      <c r="N243" t="e" vm="68">
+        <v>185</v>
+      </c>
+      <c r="N243" t="e" vm="29">
         <v>#VALUE!</v>
       </c>
       <c r="O243" t="s">
@@ -48003,7 +48037,7 @@
         <v>776</v>
       </c>
       <c r="R243" s="1">
-        <v>45992</v>
+        <v>46022</v>
       </c>
       <c r="T243">
         <v>1</v>
@@ -48016,48 +48050,41 @@
       </c>
     </row>
     <row r="244" spans="1:22" x14ac:dyDescent="0.4">
-      <c r="A244" s="4" t="s">
-        <v>719</v>
-      </c>
-      <c r="B244" s="19"/>
+      <c r="A244" t="s">
+        <v>792</v>
+      </c>
       <c r="C244" t="s">
-        <v>783</v>
+        <v>794</v>
       </c>
       <c r="D244" s="1">
-        <v>46016</v>
+        <v>45992</v>
       </c>
       <c r="E244" t="s">
         <v>15</v>
       </c>
-      <c r="G244">
-        <v>3</v>
+      <c r="F244" s="2" t="s">
+        <v>795</v>
       </c>
       <c r="I244" t="s">
-        <v>96</v>
+        <v>23</v>
       </c>
       <c r="J244" t="s">
         <v>402</v>
       </c>
-      <c r="K244" t="s">
-        <v>244</v>
-      </c>
-      <c r="L244" s="1">
-        <v>45992</v>
-      </c>
-      <c r="M244" s="2" t="s">
-        <v>718</v>
-      </c>
-      <c r="N244" t="e" vm="45">
+      <c r="M244" t="s">
+        <v>793</v>
+      </c>
+      <c r="N244" t="e" vm="29">
         <v>#VALUE!</v>
       </c>
       <c r="O244" t="s">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="Q244" t="s">
         <v>776</v>
       </c>
       <c r="R244" s="1">
-        <v>45996</v>
+        <v>46053</v>
       </c>
       <c r="T244">
         <v>1</v>
@@ -48071,37 +48098,37 @@
     </row>
     <row r="245" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A245" t="s">
-        <v>528</v>
-      </c>
-      <c r="C245" t="s">
-        <v>178</v>
+        <v>796</v>
       </c>
       <c r="D245" s="1">
-        <v>46023</v>
+        <v>45992</v>
       </c>
       <c r="E245" t="s">
-        <v>529</v>
+        <v>15</v>
+      </c>
+      <c r="H245" t="s">
+        <v>797</v>
       </c>
       <c r="I245" t="s">
-        <v>96</v>
+        <v>23</v>
       </c>
       <c r="J245" t="s">
         <v>402</v>
       </c>
       <c r="M245" t="s">
-        <v>530</v>
-      </c>
-      <c r="N245" t="e" vm="102">
+        <v>750</v>
+      </c>
+      <c r="N245" t="e" vm="47">
         <v>#VALUE!</v>
       </c>
       <c r="O245" t="s">
-        <v>19</v>
+        <v>26</v>
       </c>
       <c r="Q245" t="s">
         <v>776</v>
       </c>
       <c r="R245" s="1">
-        <v>46041</v>
+        <v>46054</v>
       </c>
       <c r="T245">
         <v>1</v>
@@ -48110,18 +48137,21 @@
         <v>0</v>
       </c>
       <c r="V245">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="246" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A246" t="s">
-        <v>564</v>
+        <v>662</v>
       </c>
       <c r="D246" s="1">
-        <v>46023</v>
+        <v>46011</v>
       </c>
       <c r="E246" t="s">
-        <v>565</v>
+        <v>15</v>
+      </c>
+      <c r="H246" t="s">
+        <v>664</v>
       </c>
       <c r="I246" t="s">
         <v>96</v>
@@ -48130,9 +48160,9 @@
         <v>402</v>
       </c>
       <c r="M246" t="s">
-        <v>566</v>
-      </c>
-      <c r="N246" t="e" vm="103">
+        <v>663</v>
+      </c>
+      <c r="N246" t="e" vm="45">
         <v>#VALUE!</v>
       </c>
       <c r="O246" t="s">
@@ -48142,7 +48172,7 @@
         <v>776</v>
       </c>
       <c r="R246" s="1">
-        <v>45664</v>
+        <v>46037</v>
       </c>
       <c r="T246">
         <v>1</v>
@@ -48156,13 +48186,19 @@
     </row>
     <row r="247" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A247" t="s">
-        <v>255</v>
+        <v>722</v>
+      </c>
+      <c r="C247" t="s">
+        <v>723</v>
+      </c>
+      <c r="D247" s="1">
+        <v>46016</v>
       </c>
       <c r="E247" t="s">
         <v>15</v>
       </c>
-      <c r="F247" s="2" t="s">
-        <v>257</v>
+      <c r="F247" t="s">
+        <v>721</v>
       </c>
       <c r="I247" t="s">
         <v>96</v>
@@ -48171,19 +48207,22 @@
         <v>402</v>
       </c>
       <c r="M247" t="s">
-        <v>256</v>
-      </c>
-      <c r="N247" t="e" vm="35">
+        <v>720</v>
+      </c>
+      <c r="N247" t="e" vm="68">
         <v>#VALUE!</v>
       </c>
       <c r="O247" t="s">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="Q247" t="s">
         <v>776</v>
       </c>
+      <c r="R247" s="1">
+        <v>45992</v>
+      </c>
       <c r="T247">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U247">
         <v>0</v>
@@ -48193,20 +48232,24 @@
       </c>
     </row>
     <row r="248" spans="1:22" x14ac:dyDescent="0.4">
-      <c r="A248" t="s">
-        <v>784</v>
+      <c r="A248" s="4" t="s">
+        <v>719</v>
+      </c>
+      <c r="B248" s="19"/>
+      <c r="C248" t="s">
+        <v>783</v>
       </c>
       <c r="D248" s="1">
-        <v>45992</v>
+        <v>46016</v>
       </c>
       <c r="E248" t="s">
-        <v>40</v>
-      </c>
-      <c r="F248" t="s">
-        <v>785</v>
+        <v>15</v>
+      </c>
+      <c r="G248">
+        <v>3</v>
       </c>
       <c r="I248" t="s">
-        <v>23</v>
+        <v>96</v>
       </c>
       <c r="J248" t="s">
         <v>402</v>
@@ -48215,22 +48258,22 @@
         <v>244</v>
       </c>
       <c r="L248" s="1">
-        <v>46027</v>
-      </c>
-      <c r="M248" t="s">
-        <v>786</v>
-      </c>
-      <c r="N248" t="e" vm="35">
+        <v>45992</v>
+      </c>
+      <c r="M248" s="2" t="s">
+        <v>718</v>
+      </c>
+      <c r="N248" t="e" vm="45">
         <v>#VALUE!</v>
       </c>
       <c r="O248" t="s">
-        <v>26</v>
+        <v>11</v>
       </c>
       <c r="Q248" t="s">
         <v>776</v>
       </c>
       <c r="R248" s="1">
-        <v>46026</v>
+        <v>45996</v>
       </c>
       <c r="T248">
         <v>1</v>
@@ -48280,10 +48323,218 @@
         <v>0</v>
       </c>
     </row>
+    <row r="250" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A250" t="s">
+        <v>790</v>
+      </c>
+      <c r="D250" s="1">
+        <v>46016</v>
+      </c>
+      <c r="E250" t="s">
+        <v>15</v>
+      </c>
+      <c r="I250" t="s">
+        <v>23</v>
+      </c>
+      <c r="J250" t="s">
+        <v>402</v>
+      </c>
+      <c r="M250" t="s">
+        <v>789</v>
+      </c>
+      <c r="N250" t="e" vm="75">
+        <v>#VALUE!</v>
+      </c>
+      <c r="O250" t="s">
+        <v>11</v>
+      </c>
+      <c r="Q250" t="s">
+        <v>776</v>
+      </c>
+      <c r="R250" s="1">
+        <v>45992</v>
+      </c>
+      <c r="T250">
+        <v>1</v>
+      </c>
+      <c r="U250">
+        <v>0</v>
+      </c>
+      <c r="V250">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="251" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A251" t="s">
+        <v>528</v>
+      </c>
+      <c r="C251" t="s">
+        <v>178</v>
+      </c>
+      <c r="D251" s="1">
+        <v>46023</v>
+      </c>
+      <c r="E251" t="s">
+        <v>529</v>
+      </c>
+      <c r="I251" t="s">
+        <v>96</v>
+      </c>
+      <c r="J251" t="s">
+        <v>402</v>
+      </c>
+      <c r="M251" t="s">
+        <v>530</v>
+      </c>
+      <c r="N251" t="e" vm="102">
+        <v>#VALUE!</v>
+      </c>
+      <c r="O251" t="s">
+        <v>19</v>
+      </c>
+      <c r="Q251" t="s">
+        <v>776</v>
+      </c>
+      <c r="R251" s="1">
+        <v>46041</v>
+      </c>
+      <c r="T251">
+        <v>1</v>
+      </c>
+      <c r="U251">
+        <v>0</v>
+      </c>
+      <c r="V251">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="252" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A252" t="s">
+        <v>564</v>
+      </c>
+      <c r="D252" s="1">
+        <v>46023</v>
+      </c>
+      <c r="E252" t="s">
+        <v>565</v>
+      </c>
+      <c r="I252" t="s">
+        <v>96</v>
+      </c>
+      <c r="J252" t="s">
+        <v>402</v>
+      </c>
+      <c r="M252" t="s">
+        <v>566</v>
+      </c>
+      <c r="N252" t="e" vm="103">
+        <v>#VALUE!</v>
+      </c>
+      <c r="O252" t="s">
+        <v>26</v>
+      </c>
+      <c r="Q252" t="s">
+        <v>776</v>
+      </c>
+      <c r="R252" s="1">
+        <v>45664</v>
+      </c>
+      <c r="T252">
+        <v>1</v>
+      </c>
+      <c r="U252">
+        <v>0</v>
+      </c>
+      <c r="V252">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="253" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A253" t="s">
+        <v>255</v>
+      </c>
+      <c r="E253" t="s">
+        <v>15</v>
+      </c>
+      <c r="F253" s="2" t="s">
+        <v>257</v>
+      </c>
+      <c r="I253" t="s">
+        <v>96</v>
+      </c>
+      <c r="J253" t="s">
+        <v>402</v>
+      </c>
+      <c r="M253" t="s">
+        <v>256</v>
+      </c>
+      <c r="N253" t="e" vm="35">
+        <v>#VALUE!</v>
+      </c>
+      <c r="O253" t="s">
+        <v>11</v>
+      </c>
+      <c r="Q253" t="s">
+        <v>776</v>
+      </c>
+      <c r="T253">
+        <v>0</v>
+      </c>
+      <c r="U253">
+        <v>0</v>
+      </c>
+      <c r="V253">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="254" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A254" t="s">
+        <v>798</v>
+      </c>
+      <c r="C254" t="s">
+        <v>800</v>
+      </c>
+      <c r="D254" s="1">
+        <v>45992</v>
+      </c>
+      <c r="E254" t="s">
+        <v>40</v>
+      </c>
+      <c r="I254" t="s">
+        <v>23</v>
+      </c>
+      <c r="J254" t="s">
+        <v>402</v>
+      </c>
+      <c r="M254" t="s">
+        <v>799</v>
+      </c>
+      <c r="N254" t="e" vm="70">
+        <v>#VALUE!</v>
+      </c>
+      <c r="O254" t="s">
+        <v>11</v>
+      </c>
+      <c r="Q254" t="s">
+        <v>776</v>
+      </c>
+      <c r="R254" s="1">
+        <v>46026</v>
+      </c>
+      <c r="T254">
+        <v>1</v>
+      </c>
+      <c r="U254">
+        <v>0</v>
+      </c>
+      <c r="V254">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:V248" xr:uid="{F7772053-9363-CA4A-A53F-040B7C700753}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:V247">
-      <sortCondition ref="D1:D19"/>
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:V253">
+      <sortCondition ref="D1:D248"/>
     </sortState>
   </autoFilter>
   <conditionalFormatting sqref="A1:B208 A210:B1048576">
@@ -48306,7 +48557,7 @@
       <formula>NOT(ISERROR(SEARCH("late app",I1)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I2:L223 O78:O80 O83:O89 O92:O112 O115:O124 O126:O181 R136 R153 R159 R166 R173 R178 O183:O205 O208:O211 O213:O218 O220:O233 I224:K224 R225 I225:L1048576 O235:O237 I1:J1 M248 O239:O248">
+  <conditionalFormatting sqref="I2:L223 O78:O80 O83:O89 O92:O112 O115:O124 O126:O181 R136 R153 R159 R166 R173 R178 O183:O205 O208:O211 O213:O218 O220:O233 I224:K224 R225 I225:L1048576 O235:O237 O239:O248 M248 O250:O254 I1:J1">
     <cfRule type="containsText" dxfId="187" priority="12" operator="containsText" text="completed">
       <formula>NOT(ISERROR(SEARCH("completed",I1)))</formula>
     </cfRule>
@@ -48328,7 +48579,7 @@
       <formula>NOT(ISERROR(SEARCH("rejected",J1)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K1:L223 O78:O80 O83:O89 O92:O112 O115:O124 O126:O181 R136 R153 R159 R166 R173 R178 O183:O205 O208:O211 O213:O218 O220:O233 K224 R225 K225:L1048576 O235:O237 M248 O239:O248">
+  <conditionalFormatting sqref="K1:L223 O78:O80 O83:O89 O92:O112 O115:O124 O126:O181 R136 R153 R159 R166 R173 R178 O183:O205 O208:O211 O213:O218 O220:O233 K224 R225 K225:L1048576 O235:O237 O239:O248 M248 O250:O254">
     <cfRule type="containsText" dxfId="181" priority="10" operator="containsText" text="NO">
       <formula>NOT(ISERROR(SEARCH("NO",K1)))</formula>
     </cfRule>
@@ -48418,7 +48669,7 @@
     <hyperlink ref="M17" r:id="rId79" xr:uid="{9A9A6BC9-B330-7842-A78C-4DCC88F5E19F}"/>
     <hyperlink ref="M32" r:id="rId80" xr:uid="{928CABEF-4FA6-E646-8140-7B6E43F8FB96}"/>
     <hyperlink ref="F177" r:id="rId81" xr:uid="{82BF1574-A6C6-1641-9FFE-615861E401FD}"/>
-    <hyperlink ref="F247" r:id="rId82" xr:uid="{3562807E-7FDA-F046-BA03-5DDD43072DB7}"/>
+    <hyperlink ref="F253" r:id="rId82" xr:uid="{3562807E-7FDA-F046-BA03-5DDD43072DB7}"/>
     <hyperlink ref="H215" r:id="rId83" display="mailto:ivanpaya@ua.es" xr:uid="{DEFB77A5-E57F-714C-BAB9-56DE82BA0B2E}"/>
     <hyperlink ref="H138" r:id="rId84" display="mailto:ari.hyytinen@hanken.fi" xr:uid="{7777B12A-FD99-4A43-A14B-A15661B760DC}"/>
     <hyperlink ref="H115" r:id="rId85" display="mailto:peter.haan@fu-berlin.de" xr:uid="{3D1A69ED-8F06-1246-B586-201CB349DB62}"/>
@@ -48436,16 +48687,17 @@
     <hyperlink ref="H240" r:id="rId97" display="mailto:ondrej.krcal@econ.muni.cz" xr:uid="{EDDEB1E6-5767-4FFB-A0AE-57A909D04E81}"/>
     <hyperlink ref="M218" r:id="rId98" display="https://www.ovgu.de/unimagdeburg/en/" xr:uid="{BCB3935D-2B6D-4090-86F5-762D762ED0E3}"/>
     <hyperlink ref="E152" r:id="rId99" xr:uid="{550520C0-1E25-41CD-9AEE-9A3C4D7D328C}"/>
-    <hyperlink ref="M244" r:id="rId100" xr:uid="{F0DD6D71-3FFD-4EAB-A251-AAF2DA8EF53C}"/>
+    <hyperlink ref="M248" r:id="rId100" xr:uid="{F0DD6D71-3FFD-4EAB-A251-AAF2DA8EF53C}"/>
+    <hyperlink ref="F244" r:id="rId101" xr:uid="{BDBBC2E2-C3C5-4526-A621-853D22D99CCF}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId101"/>
+  <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId102"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{923E81FA-B875-3C4E-A189-1A21268FA086}">
-  <dimension ref="A1:C261"/>
+  <dimension ref="A1:C263"/>
   <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="16" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="32.83203125" customWidth="1"/>
@@ -51259,6 +51511,25 @@
       </c>
       <c r="C261" t="s">
         <v>97</v>
+      </c>
+    </row>
+    <row r="262" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A262" s="1">
+        <v>45990</v>
+      </c>
+      <c r="C262" t="s">
+        <v>801</v>
+      </c>
+    </row>
+    <row r="263" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A263" s="1">
+        <v>45990</v>
+      </c>
+      <c r="B263" t="s">
+        <v>573</v>
+      </c>
+      <c r="C263" t="s">
+        <v>403</v>
       </c>
     </row>
   </sheetData>
@@ -51279,8 +51550,8 @@
     <cfRule type="duplicateValues" dxfId="172" priority="180"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B15">
-    <cfRule type="duplicateValues" dxfId="171" priority="179"/>
-    <cfRule type="duplicateValues" dxfId="170" priority="178"/>
+    <cfRule type="duplicateValues" dxfId="171" priority="178"/>
+    <cfRule type="duplicateValues" dxfId="170" priority="179"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B16">
     <cfRule type="duplicateValues" dxfId="169" priority="177"/>
@@ -51301,12 +51572,12 @@
     <cfRule type="duplicateValues" dxfId="162" priority="170"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B24">
-    <cfRule type="duplicateValues" dxfId="161" priority="169"/>
-    <cfRule type="duplicateValues" dxfId="160" priority="168"/>
+    <cfRule type="duplicateValues" dxfId="161" priority="168"/>
+    <cfRule type="duplicateValues" dxfId="160" priority="169"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B27">
-    <cfRule type="duplicateValues" dxfId="159" priority="167"/>
-    <cfRule type="duplicateValues" dxfId="158" priority="166"/>
+    <cfRule type="duplicateValues" dxfId="159" priority="166"/>
+    <cfRule type="duplicateValues" dxfId="158" priority="167"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B28">
     <cfRule type="duplicateValues" dxfId="157" priority="165"/>
@@ -51796,11 +52067,11 @@
       </c>
       <c r="B1" s="15">
         <f>COUNTA(sum!A:A) -1</f>
-        <v>248</v>
-      </c>
-      <c r="C1" s="23">
+        <v>253</v>
+      </c>
+      <c r="C1" s="22">
         <f>COUNTIF(sum!I:I, "completed")/(B1-COUNTIF(sum!I:I, "abandoned")-COUNTIF(sum!I:I, "late app"))</f>
-        <v>0.99585062240663902</v>
+        <v>0.97560975609756095</v>
       </c>
       <c r="D1" s="21">
         <f>COUNTIF(sum!I:I, "completed")</f>
@@ -51839,7 +52110,7 @@
       </c>
       <c r="B5" s="15">
         <f>COUNTA(sum!J:J) -1</f>
-        <v>248</v>
+        <v>253</v>
       </c>
       <c r="C5" s="14">
         <f>B5/B1</f>
@@ -51852,11 +52123,11 @@
       </c>
       <c r="B6" s="16">
         <f>COUNTIFS(sum!J:J,"no news")</f>
-        <v>241</v>
+        <v>245</v>
       </c>
       <c r="C6" s="10">
         <f>B6/$B$5</f>
-        <v>0.97177419354838712</v>
+        <v>0.96837944664031617</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.4">
@@ -51865,11 +52136,11 @@
       </c>
       <c r="B7" s="16">
         <f>COUNTIFS(sum!J:J,"rejected")</f>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C7" s="10">
         <f t="shared" ref="C7:C10" si="0">B7/$B$5</f>
-        <v>2.8225806451612902E-2</v>
+        <v>3.1620553359683792E-2</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.4">

</xml_diff>

<commit_message>
other 5 stragelers apps
</commit_message>
<xml_diff>
--- a/EconJM_status.xlsx
+++ b/EconJM_status.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\javie\Dropbox\Work\Job Search\2025 EconJM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33AB038B-FA27-40F4-A9D7-3716430E3770}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{820AC922-C742-4C7E-AD3C-B3FC9CEE83F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="14620" activeTab="1" xr2:uid="{6FE48536-7E5C-BF4C-9490-2A6392576298}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="14620" xr2:uid="{6FE48536-7E5C-BF4C-9490-2A6392576298}"/>
   </bookViews>
   <sheets>
     <sheet name="sum" sheetId="1" r:id="rId1"/>
@@ -1083,7 +1083,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2538" uniqueCount="802">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2551" uniqueCount="803">
   <si>
     <t>add_id</t>
   </si>
@@ -3525,6 +3525,9 @@
   </si>
   <si>
     <t>added some info of stragelers in EJM and JOE</t>
+  </si>
+  <si>
+    <t>Prof. Philipp Ager philipp.ager@uni-mannheim.de</t>
   </si>
 </sst>
 </file>
@@ -3706,7 +3709,27 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Percent" xfId="2" builtinId="5"/>
   </cellStyles>
-  <dxfs count="194">
+  <dxfs count="196">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -39524,7 +39547,7 @@
         <v>96</v>
       </c>
       <c r="J56" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="K56" t="s">
         <v>309</v>
@@ -48018,8 +48041,11 @@
       <c r="E243" t="s">
         <v>15</v>
       </c>
+      <c r="H243" t="s">
+        <v>802</v>
+      </c>
       <c r="I243" t="s">
-        <v>23</v>
+        <v>96</v>
       </c>
       <c r="J243" t="s">
         <v>402</v>
@@ -48066,7 +48092,7 @@
         <v>795</v>
       </c>
       <c r="I244" t="s">
-        <v>23</v>
+        <v>96</v>
       </c>
       <c r="J244" t="s">
         <v>402</v>
@@ -48110,7 +48136,7 @@
         <v>797</v>
       </c>
       <c r="I245" t="s">
-        <v>23</v>
+        <v>96</v>
       </c>
       <c r="J245" t="s">
         <v>402</v>
@@ -48334,7 +48360,7 @@
         <v>15</v>
       </c>
       <c r="I250" t="s">
-        <v>23</v>
+        <v>96</v>
       </c>
       <c r="J250" t="s">
         <v>402</v>
@@ -48501,7 +48527,7 @@
         <v>40</v>
       </c>
       <c r="I254" t="s">
-        <v>23</v>
+        <v>96</v>
       </c>
       <c r="J254" t="s">
         <v>402</v>
@@ -48538,52 +48564,52 @@
     </sortState>
   </autoFilter>
   <conditionalFormatting sqref="A1:B208 A210:B1048576">
-    <cfRule type="duplicateValues" dxfId="193" priority="14"/>
+    <cfRule type="duplicateValues" dxfId="195" priority="14"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A2:B22">
-    <cfRule type="duplicateValues" dxfId="192" priority="15"/>
+    <cfRule type="duplicateValues" dxfId="194" priority="15"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A61:B61">
-    <cfRule type="duplicateValues" dxfId="191" priority="13"/>
+    <cfRule type="duplicateValues" dxfId="193" priority="13"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="I1:I1048576">
-    <cfRule type="containsText" dxfId="190" priority="6" operator="containsText" text="closed">
+    <cfRule type="containsText" dxfId="192" priority="6" operator="containsText" text="closed">
       <formula>NOT(ISERROR(SEARCH("closed",I1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="189" priority="7" operator="containsText" text="abandoned">
+    <cfRule type="containsText" dxfId="191" priority="7" operator="containsText" text="abandoned">
       <formula>NOT(ISERROR(SEARCH("abandoned",I1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="188" priority="9" operator="containsText" text="late app">
+    <cfRule type="containsText" dxfId="190" priority="9" operator="containsText" text="late app">
       <formula>NOT(ISERROR(SEARCH("late app",I1)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I2:L223 O78:O80 O83:O89 O92:O112 O115:O124 O126:O181 R136 R153 R159 R166 R173 R178 O183:O205 O208:O211 O213:O218 O220:O233 I224:K224 R225 I225:L1048576 O235:O237 O239:O248 M248 O250:O254 I1:J1">
-    <cfRule type="containsText" dxfId="187" priority="12" operator="containsText" text="completed">
+    <cfRule type="containsText" dxfId="189" priority="12" operator="containsText" text="completed">
       <formula>NOT(ISERROR(SEARCH("completed",I1)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J1:J1048576">
-    <cfRule type="containsText" dxfId="186" priority="1" operator="containsText" text="no news">
+    <cfRule type="containsText" dxfId="188" priority="1" operator="containsText" text="no news">
       <formula>NOT(ISERROR(SEARCH("no news",J1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="185" priority="2" operator="containsText" text="offer">
+    <cfRule type="containsText" dxfId="187" priority="2" operator="containsText" text="offer">
       <formula>NOT(ISERROR(SEARCH("offer",J1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="184" priority="3" operator="containsText" text="fly out">
+    <cfRule type="containsText" dxfId="186" priority="3" operator="containsText" text="fly out">
       <formula>NOT(ISERROR(SEARCH("fly out",J1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="183" priority="4" operator="containsText" text="interview">
+    <cfRule type="containsText" dxfId="185" priority="4" operator="containsText" text="interview">
       <formula>NOT(ISERROR(SEARCH("interview",J1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="182" priority="5" operator="containsText" text="rejected">
+    <cfRule type="containsText" dxfId="184" priority="5" operator="containsText" text="rejected">
       <formula>NOT(ISERROR(SEARCH("rejected",J1)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K1:L223 O78:O80 O83:O89 O92:O112 O115:O124 O126:O181 R136 R153 R159 R166 R173 R178 O183:O205 O208:O211 O213:O218 O220:O233 K224 R225 K225:L1048576 O235:O237 O239:O248 M248 O250:O254">
-    <cfRule type="containsText" dxfId="181" priority="10" operator="containsText" text="NO">
+    <cfRule type="containsText" dxfId="183" priority="10" operator="containsText" text="NO">
       <formula>NOT(ISERROR(SEARCH("NO",K1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="180" priority="11" operator="containsText" text="YES">
+    <cfRule type="containsText" dxfId="182" priority="11" operator="containsText" text="YES">
       <formula>NOT(ISERROR(SEARCH("YES",K1)))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -48697,7 +48723,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{923E81FA-B875-3C4E-A189-1A21268FA086}">
-  <dimension ref="A1:C263"/>
+  <dimension ref="A1:C269"/>
   <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="16" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="32.83203125" customWidth="1"/>
@@ -51532,519 +51558,591 @@
         <v>403</v>
       </c>
     </row>
+    <row r="264" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A264" s="1">
+        <v>45989</v>
+      </c>
+      <c r="B264" t="s">
+        <v>144</v>
+      </c>
+      <c r="C264" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="265" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A265" s="1">
+        <v>45991</v>
+      </c>
+      <c r="B265" t="s">
+        <v>791</v>
+      </c>
+      <c r="C265" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="266" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A266" s="1">
+        <v>45991</v>
+      </c>
+      <c r="B266" t="s">
+        <v>792</v>
+      </c>
+      <c r="C266" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="267" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A267" s="1">
+        <v>45991</v>
+      </c>
+      <c r="B267" t="s">
+        <v>796</v>
+      </c>
+      <c r="C267" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="268" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A268" s="1">
+        <v>45991</v>
+      </c>
+      <c r="B268" t="s">
+        <v>790</v>
+      </c>
+      <c r="C268" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="269" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A269" s="1">
+        <v>45991</v>
+      </c>
+      <c r="B269" t="s">
+        <v>798</v>
+      </c>
+      <c r="C269" t="s">
+        <v>97</v>
+      </c>
+    </row>
   </sheetData>
   <conditionalFormatting sqref="B5">
-    <cfRule type="duplicateValues" dxfId="179" priority="186"/>
-    <cfRule type="duplicateValues" dxfId="178" priority="187"/>
+    <cfRule type="duplicateValues" dxfId="181" priority="188"/>
+    <cfRule type="duplicateValues" dxfId="180" priority="189"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B10">
+    <cfRule type="duplicateValues" dxfId="179" priority="187"/>
+    <cfRule type="duplicateValues" dxfId="178" priority="186"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B11">
     <cfRule type="duplicateValues" dxfId="177" priority="185"/>
     <cfRule type="duplicateValues" dxfId="176" priority="184"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B11">
+  <conditionalFormatting sqref="B12">
     <cfRule type="duplicateValues" dxfId="175" priority="183"/>
     <cfRule type="duplicateValues" dxfId="174" priority="182"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B12">
-    <cfRule type="duplicateValues" dxfId="173" priority="181"/>
-    <cfRule type="duplicateValues" dxfId="172" priority="180"/>
-  </conditionalFormatting>
   <conditionalFormatting sqref="B15">
-    <cfRule type="duplicateValues" dxfId="171" priority="178"/>
-    <cfRule type="duplicateValues" dxfId="170" priority="179"/>
+    <cfRule type="duplicateValues" dxfId="173" priority="180"/>
+    <cfRule type="duplicateValues" dxfId="172" priority="181"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B16">
+    <cfRule type="duplicateValues" dxfId="171" priority="179"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B17">
+    <cfRule type="duplicateValues" dxfId="170" priority="178"/>
     <cfRule type="duplicateValues" dxfId="169" priority="177"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B17">
+  <conditionalFormatting sqref="B18">
     <cfRule type="duplicateValues" dxfId="168" priority="176"/>
     <cfRule type="duplicateValues" dxfId="167" priority="175"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B18">
+  <conditionalFormatting sqref="B19">
     <cfRule type="duplicateValues" dxfId="166" priority="174"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B22:B23">
     <cfRule type="duplicateValues" dxfId="165" priority="173"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B19">
     <cfRule type="duplicateValues" dxfId="164" priority="172"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B22:B23">
-    <cfRule type="duplicateValues" dxfId="163" priority="171"/>
-    <cfRule type="duplicateValues" dxfId="162" priority="170"/>
+  <conditionalFormatting sqref="B24">
+    <cfRule type="duplicateValues" dxfId="163" priority="170"/>
+    <cfRule type="duplicateValues" dxfId="162" priority="171"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B24">
+  <conditionalFormatting sqref="B27">
     <cfRule type="duplicateValues" dxfId="161" priority="168"/>
     <cfRule type="duplicateValues" dxfId="160" priority="169"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B27">
-    <cfRule type="duplicateValues" dxfId="159" priority="166"/>
-    <cfRule type="duplicateValues" dxfId="158" priority="167"/>
+  <conditionalFormatting sqref="B28">
+    <cfRule type="duplicateValues" dxfId="159" priority="167"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B28">
+  <conditionalFormatting sqref="B29">
+    <cfRule type="duplicateValues" dxfId="158" priority="166"/>
     <cfRule type="duplicateValues" dxfId="157" priority="165"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B29">
+  <conditionalFormatting sqref="B30">
     <cfRule type="duplicateValues" dxfId="156" priority="164"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B31">
     <cfRule type="duplicateValues" dxfId="155" priority="163"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B30">
+  <conditionalFormatting sqref="B32">
     <cfRule type="duplicateValues" dxfId="154" priority="162"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B31">
+  <conditionalFormatting sqref="B33">
     <cfRule type="duplicateValues" dxfId="153" priority="161"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B32">
+  <conditionalFormatting sqref="B34">
     <cfRule type="duplicateValues" dxfId="152" priority="160"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B33">
+  <conditionalFormatting sqref="B35">
     <cfRule type="duplicateValues" dxfId="151" priority="159"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B34">
+  <conditionalFormatting sqref="B37">
     <cfRule type="duplicateValues" dxfId="150" priority="158"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B35">
+  <conditionalFormatting sqref="B38">
     <cfRule type="duplicateValues" dxfId="149" priority="157"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B37">
+  <conditionalFormatting sqref="B42">
     <cfRule type="duplicateValues" dxfId="148" priority="156"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B38">
+  <conditionalFormatting sqref="B43">
     <cfRule type="duplicateValues" dxfId="147" priority="155"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B42">
+  <conditionalFormatting sqref="B44:B45">
     <cfRule type="duplicateValues" dxfId="146" priority="154"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B43">
+  <conditionalFormatting sqref="B46">
     <cfRule type="duplicateValues" dxfId="145" priority="153"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B44:B45">
+  <conditionalFormatting sqref="B48">
     <cfRule type="duplicateValues" dxfId="144" priority="152"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B46">
+  <conditionalFormatting sqref="B49">
     <cfRule type="duplicateValues" dxfId="143" priority="151"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B48">
+  <conditionalFormatting sqref="B51">
     <cfRule type="duplicateValues" dxfId="142" priority="150"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B49">
+  <conditionalFormatting sqref="B52">
     <cfRule type="duplicateValues" dxfId="141" priority="149"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B51">
-    <cfRule type="duplicateValues" dxfId="140" priority="148"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B52">
-    <cfRule type="duplicateValues" dxfId="139" priority="147"/>
-  </conditionalFormatting>
   <conditionalFormatting sqref="B58">
-    <cfRule type="duplicateValues" dxfId="138" priority="145"/>
+    <cfRule type="duplicateValues" dxfId="140" priority="147"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B59">
-    <cfRule type="duplicateValues" dxfId="137" priority="143"/>
+    <cfRule type="duplicateValues" dxfId="139" priority="145"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B63">
-    <cfRule type="duplicateValues" dxfId="136" priority="142"/>
+    <cfRule type="duplicateValues" dxfId="138" priority="144"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B64">
-    <cfRule type="duplicateValues" dxfId="135" priority="140"/>
+    <cfRule type="duplicateValues" dxfId="137" priority="142"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B66">
+    <cfRule type="duplicateValues" dxfId="136" priority="141"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B67">
+    <cfRule type="duplicateValues" dxfId="135" priority="140"/>
     <cfRule type="duplicateValues" dxfId="134" priority="139"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B67">
+  <conditionalFormatting sqref="B68">
     <cfRule type="duplicateValues" dxfId="133" priority="138"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B69">
     <cfRule type="duplicateValues" dxfId="132" priority="137"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B68">
-    <cfRule type="duplicateValues" dxfId="131" priority="136"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B69">
-    <cfRule type="duplicateValues" dxfId="130" priority="135"/>
-  </conditionalFormatting>
   <conditionalFormatting sqref="B70">
-    <cfRule type="duplicateValues" dxfId="129" priority="133"/>
+    <cfRule type="duplicateValues" dxfId="131" priority="135"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B72">
-    <cfRule type="duplicateValues" dxfId="128" priority="132"/>
+    <cfRule type="duplicateValues" dxfId="130" priority="134"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B73">
+    <cfRule type="duplicateValues" dxfId="129" priority="132"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B74">
+    <cfRule type="duplicateValues" dxfId="128" priority="131"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B75">
     <cfRule type="duplicateValues" dxfId="127" priority="130"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B74">
+  <conditionalFormatting sqref="B76">
     <cfRule type="duplicateValues" dxfId="126" priority="129"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B75">
-    <cfRule type="duplicateValues" dxfId="125" priority="128"/>
+  <conditionalFormatting sqref="B77">
+    <cfRule type="duplicateValues" dxfId="125" priority="127"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B76">
-    <cfRule type="duplicateValues" dxfId="124" priority="127"/>
+  <conditionalFormatting sqref="B78">
+    <cfRule type="duplicateValues" dxfId="124" priority="126"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B77">
+  <conditionalFormatting sqref="B83">
     <cfRule type="duplicateValues" dxfId="123" priority="125"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B78">
+  <conditionalFormatting sqref="B84">
     <cfRule type="duplicateValues" dxfId="122" priority="124"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B83">
+  <conditionalFormatting sqref="B85">
     <cfRule type="duplicateValues" dxfId="121" priority="123"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B84">
+  <conditionalFormatting sqref="B87">
     <cfRule type="duplicateValues" dxfId="120" priority="122"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B85">
+  <conditionalFormatting sqref="B88">
     <cfRule type="duplicateValues" dxfId="119" priority="121"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B87">
+  <conditionalFormatting sqref="B89">
     <cfRule type="duplicateValues" dxfId="118" priority="120"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B88">
+  <conditionalFormatting sqref="B90">
     <cfRule type="duplicateValues" dxfId="117" priority="119"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B89">
+  <conditionalFormatting sqref="B91">
     <cfRule type="duplicateValues" dxfId="116" priority="118"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B90">
+  <conditionalFormatting sqref="B92">
     <cfRule type="duplicateValues" dxfId="115" priority="117"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B91">
+  <conditionalFormatting sqref="B93">
     <cfRule type="duplicateValues" dxfId="114" priority="116"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B92">
+  <conditionalFormatting sqref="B94">
     <cfRule type="duplicateValues" dxfId="113" priority="115"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B93">
+  <conditionalFormatting sqref="B95">
     <cfRule type="duplicateValues" dxfId="112" priority="114"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B94">
+  <conditionalFormatting sqref="B96">
     <cfRule type="duplicateValues" dxfId="111" priority="113"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B95">
+  <conditionalFormatting sqref="B97">
     <cfRule type="duplicateValues" dxfId="110" priority="112"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B96">
+  <conditionalFormatting sqref="B98">
     <cfRule type="duplicateValues" dxfId="109" priority="111"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B97">
+  <conditionalFormatting sqref="B99">
     <cfRule type="duplicateValues" dxfId="108" priority="110"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B98">
+  <conditionalFormatting sqref="B100">
     <cfRule type="duplicateValues" dxfId="107" priority="109"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B99">
+  <conditionalFormatting sqref="B101">
     <cfRule type="duplicateValues" dxfId="106" priority="108"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B100">
+  <conditionalFormatting sqref="B104">
     <cfRule type="duplicateValues" dxfId="105" priority="107"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B101">
     <cfRule type="duplicateValues" dxfId="104" priority="106"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B104">
+  <conditionalFormatting sqref="B105:B106">
     <cfRule type="duplicateValues" dxfId="103" priority="105"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B107">
     <cfRule type="duplicateValues" dxfId="102" priority="104"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B105:B106">
+  <conditionalFormatting sqref="B108">
     <cfRule type="duplicateValues" dxfId="101" priority="103"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B107">
+  <conditionalFormatting sqref="B109">
     <cfRule type="duplicateValues" dxfId="100" priority="102"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B108">
+  <conditionalFormatting sqref="B110">
     <cfRule type="duplicateValues" dxfId="99" priority="101"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B109">
+  <conditionalFormatting sqref="B111">
     <cfRule type="duplicateValues" dxfId="98" priority="100"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B110">
+  <conditionalFormatting sqref="B112">
     <cfRule type="duplicateValues" dxfId="97" priority="99"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B111">
+  <conditionalFormatting sqref="B113">
     <cfRule type="duplicateValues" dxfId="96" priority="98"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B112">
+  <conditionalFormatting sqref="B114">
     <cfRule type="duplicateValues" dxfId="95" priority="97"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B113">
+  <conditionalFormatting sqref="B115">
     <cfRule type="duplicateValues" dxfId="94" priority="96"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B114">
+  <conditionalFormatting sqref="B116">
     <cfRule type="duplicateValues" dxfId="93" priority="95"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B115">
+  <conditionalFormatting sqref="B117">
     <cfRule type="duplicateValues" dxfId="92" priority="94"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B116">
+  <conditionalFormatting sqref="B118">
     <cfRule type="duplicateValues" dxfId="91" priority="93"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B117">
+  <conditionalFormatting sqref="B119">
     <cfRule type="duplicateValues" dxfId="90" priority="92"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B118">
+  <conditionalFormatting sqref="B120">
     <cfRule type="duplicateValues" dxfId="89" priority="91"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B119">
+  <conditionalFormatting sqref="B121">
     <cfRule type="duplicateValues" dxfId="88" priority="90"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B120">
+  <conditionalFormatting sqref="B122">
     <cfRule type="duplicateValues" dxfId="87" priority="89"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B121">
+  <conditionalFormatting sqref="B126">
     <cfRule type="duplicateValues" dxfId="86" priority="88"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B122">
+  <conditionalFormatting sqref="B127">
     <cfRule type="duplicateValues" dxfId="85" priority="87"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B126">
+  <conditionalFormatting sqref="B128">
     <cfRule type="duplicateValues" dxfId="84" priority="86"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B127">
+  <conditionalFormatting sqref="B129">
     <cfRule type="duplicateValues" dxfId="83" priority="85"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B128">
+  <conditionalFormatting sqref="B130">
     <cfRule type="duplicateValues" dxfId="82" priority="84"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B129">
+  <conditionalFormatting sqref="B131">
     <cfRule type="duplicateValues" dxfId="81" priority="83"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B130">
+  <conditionalFormatting sqref="B132">
     <cfRule type="duplicateValues" dxfId="80" priority="82"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B131">
+  <conditionalFormatting sqref="B133">
     <cfRule type="duplicateValues" dxfId="79" priority="81"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B132">
+  <conditionalFormatting sqref="B136">
     <cfRule type="duplicateValues" dxfId="78" priority="80"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B133">
+  <conditionalFormatting sqref="B137">
     <cfRule type="duplicateValues" dxfId="77" priority="79"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B136">
+  <conditionalFormatting sqref="B138">
     <cfRule type="duplicateValues" dxfId="76" priority="78"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B137">
+  <conditionalFormatting sqref="B139">
     <cfRule type="duplicateValues" dxfId="75" priority="77"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B138">
+  <conditionalFormatting sqref="B140">
     <cfRule type="duplicateValues" dxfId="74" priority="76"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B139">
+  <conditionalFormatting sqref="B141">
     <cfRule type="duplicateValues" dxfId="73" priority="75"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B140">
+  <conditionalFormatting sqref="B142">
     <cfRule type="duplicateValues" dxfId="72" priority="74"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B141">
+  <conditionalFormatting sqref="B143">
     <cfRule type="duplicateValues" dxfId="71" priority="73"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B142">
+  <conditionalFormatting sqref="B144">
     <cfRule type="duplicateValues" dxfId="70" priority="72"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B143">
+  <conditionalFormatting sqref="B145">
     <cfRule type="duplicateValues" dxfId="69" priority="71"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B144">
+  <conditionalFormatting sqref="B147">
     <cfRule type="duplicateValues" dxfId="68" priority="70"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B145">
+  <conditionalFormatting sqref="B148">
     <cfRule type="duplicateValues" dxfId="67" priority="69"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B147">
+  <conditionalFormatting sqref="B149">
     <cfRule type="duplicateValues" dxfId="66" priority="68"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B148">
+  <conditionalFormatting sqref="B150">
     <cfRule type="duplicateValues" dxfId="65" priority="67"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B149">
+  <conditionalFormatting sqref="B151">
     <cfRule type="duplicateValues" dxfId="64" priority="66"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B150">
+  <conditionalFormatting sqref="B152">
     <cfRule type="duplicateValues" dxfId="63" priority="65"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B151">
+  <conditionalFormatting sqref="B153">
     <cfRule type="duplicateValues" dxfId="62" priority="64"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B152">
+  <conditionalFormatting sqref="B154">
     <cfRule type="duplicateValues" dxfId="61" priority="63"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B153">
+  <conditionalFormatting sqref="B155">
     <cfRule type="duplicateValues" dxfId="60" priority="62"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B154">
+  <conditionalFormatting sqref="B156">
     <cfRule type="duplicateValues" dxfId="59" priority="61"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B155">
+  <conditionalFormatting sqref="B157">
     <cfRule type="duplicateValues" dxfId="58" priority="60"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B156">
+  <conditionalFormatting sqref="B171">
     <cfRule type="duplicateValues" dxfId="57" priority="59"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B157">
+  <conditionalFormatting sqref="B172">
     <cfRule type="duplicateValues" dxfId="56" priority="58"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B171">
+  <conditionalFormatting sqref="B174">
     <cfRule type="duplicateValues" dxfId="55" priority="57"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B172">
+  <conditionalFormatting sqref="B177:B178">
     <cfRule type="duplicateValues" dxfId="54" priority="56"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B174">
+  <conditionalFormatting sqref="B181">
     <cfRule type="duplicateValues" dxfId="53" priority="55"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B177:B178">
+  <conditionalFormatting sqref="B182">
     <cfRule type="duplicateValues" dxfId="52" priority="54"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B181">
+  <conditionalFormatting sqref="B183">
     <cfRule type="duplicateValues" dxfId="51" priority="53"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B182">
+  <conditionalFormatting sqref="B184">
     <cfRule type="duplicateValues" dxfId="50" priority="52"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B183">
+  <conditionalFormatting sqref="B185">
     <cfRule type="duplicateValues" dxfId="49" priority="51"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B184">
+  <conditionalFormatting sqref="B186">
     <cfRule type="duplicateValues" dxfId="48" priority="50"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B185">
+  <conditionalFormatting sqref="B188">
     <cfRule type="duplicateValues" dxfId="47" priority="49"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B186">
+  <conditionalFormatting sqref="B189">
     <cfRule type="duplicateValues" dxfId="46" priority="48"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B188">
+  <conditionalFormatting sqref="B190">
     <cfRule type="duplicateValues" dxfId="45" priority="47"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B189">
+  <conditionalFormatting sqref="B191">
     <cfRule type="duplicateValues" dxfId="44" priority="46"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B190">
+  <conditionalFormatting sqref="B192">
     <cfRule type="duplicateValues" dxfId="43" priority="45"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B191">
+  <conditionalFormatting sqref="B193">
     <cfRule type="duplicateValues" dxfId="42" priority="44"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B192">
+  <conditionalFormatting sqref="B195">
     <cfRule type="duplicateValues" dxfId="41" priority="43"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B193">
+  <conditionalFormatting sqref="B196">
     <cfRule type="duplicateValues" dxfId="40" priority="42"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B195">
+  <conditionalFormatting sqref="B197">
     <cfRule type="duplicateValues" dxfId="39" priority="41"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B196">
+  <conditionalFormatting sqref="B198">
     <cfRule type="duplicateValues" dxfId="38" priority="40"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B197">
+  <conditionalFormatting sqref="B199">
     <cfRule type="duplicateValues" dxfId="37" priority="39"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B198">
+  <conditionalFormatting sqref="B200">
     <cfRule type="duplicateValues" dxfId="36" priority="38"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B199">
+  <conditionalFormatting sqref="B201">
     <cfRule type="duplicateValues" dxfId="35" priority="37"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B200">
+  <conditionalFormatting sqref="B202">
     <cfRule type="duplicateValues" dxfId="34" priority="36"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B201">
+  <conditionalFormatting sqref="B203">
     <cfRule type="duplicateValues" dxfId="33" priority="35"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B202">
+  <conditionalFormatting sqref="B204">
     <cfRule type="duplicateValues" dxfId="32" priority="34"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B203">
+  <conditionalFormatting sqref="B205">
     <cfRule type="duplicateValues" dxfId="31" priority="33"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B204">
+  <conditionalFormatting sqref="B206">
     <cfRule type="duplicateValues" dxfId="30" priority="32"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B205">
+  <conditionalFormatting sqref="B207">
     <cfRule type="duplicateValues" dxfId="29" priority="31"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B206">
+  <conditionalFormatting sqref="B215">
     <cfRule type="duplicateValues" dxfId="28" priority="30"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B207">
+  <conditionalFormatting sqref="B218">
     <cfRule type="duplicateValues" dxfId="27" priority="29"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B215">
+  <conditionalFormatting sqref="B220">
     <cfRule type="duplicateValues" dxfId="26" priority="28"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B218">
+  <conditionalFormatting sqref="B222">
     <cfRule type="duplicateValues" dxfId="25" priority="27"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B220">
+  <conditionalFormatting sqref="B223">
     <cfRule type="duplicateValues" dxfId="24" priority="26"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B222">
+  <conditionalFormatting sqref="B224">
     <cfRule type="duplicateValues" dxfId="23" priority="25"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B223">
+  <conditionalFormatting sqref="B225">
     <cfRule type="duplicateValues" dxfId="22" priority="24"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B224">
+  <conditionalFormatting sqref="B227">
     <cfRule type="duplicateValues" dxfId="21" priority="23"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B225">
+  <conditionalFormatting sqref="B229">
     <cfRule type="duplicateValues" dxfId="20" priority="22"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B227">
+  <conditionalFormatting sqref="B230">
     <cfRule type="duplicateValues" dxfId="19" priority="21"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B229">
+  <conditionalFormatting sqref="B232">
     <cfRule type="duplicateValues" dxfId="18" priority="20"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B230">
+  <conditionalFormatting sqref="B233">
     <cfRule type="duplicateValues" dxfId="17" priority="19"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B232">
+  <conditionalFormatting sqref="B234">
     <cfRule type="duplicateValues" dxfId="16" priority="18"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B233">
+  <conditionalFormatting sqref="B235">
     <cfRule type="duplicateValues" dxfId="15" priority="17"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B234">
+  <conditionalFormatting sqref="B236">
     <cfRule type="duplicateValues" dxfId="14" priority="16"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B235">
+  <conditionalFormatting sqref="B237">
     <cfRule type="duplicateValues" dxfId="13" priority="15"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B236">
-    <cfRule type="duplicateValues" dxfId="12" priority="14"/>
+  <conditionalFormatting sqref="B239">
+    <cfRule type="duplicateValues" dxfId="12" priority="13"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B237">
-    <cfRule type="duplicateValues" dxfId="11" priority="13"/>
+  <conditionalFormatting sqref="B240">
+    <cfRule type="duplicateValues" dxfId="11" priority="12"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B239">
+  <conditionalFormatting sqref="B241">
     <cfRule type="duplicateValues" dxfId="10" priority="11"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B240">
+  <conditionalFormatting sqref="B242">
     <cfRule type="duplicateValues" dxfId="9" priority="10"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B241">
+  <conditionalFormatting sqref="B243">
     <cfRule type="duplicateValues" dxfId="8" priority="9"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B242">
+  <conditionalFormatting sqref="B250">
     <cfRule type="duplicateValues" dxfId="7" priority="8"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B243">
+  <conditionalFormatting sqref="B251">
     <cfRule type="duplicateValues" dxfId="6" priority="7"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B250">
+  <conditionalFormatting sqref="B253">
     <cfRule type="duplicateValues" dxfId="5" priority="6"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B251">
+  <conditionalFormatting sqref="B255">
     <cfRule type="duplicateValues" dxfId="4" priority="5"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B253">
+  <conditionalFormatting sqref="B258:B259">
     <cfRule type="duplicateValues" dxfId="3" priority="4"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B255">
+  <conditionalFormatting sqref="B260">
     <cfRule type="duplicateValues" dxfId="2" priority="3"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B258:B259">
+  <conditionalFormatting sqref="B265:B267 B269">
     <cfRule type="duplicateValues" dxfId="1" priority="2"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B260">
+  <conditionalFormatting sqref="B268">
     <cfRule type="duplicateValues" dxfId="0" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -52071,11 +52169,11 @@
       </c>
       <c r="C1" s="22">
         <f>COUNTIF(sum!I:I, "completed")/(B1-COUNTIF(sum!I:I, "abandoned")-COUNTIF(sum!I:I, "late app"))</f>
-        <v>0.97560975609756095</v>
+        <v>0.99593495934959353</v>
       </c>
       <c r="D1" s="21">
         <f>COUNTIF(sum!I:I, "completed")</f>
-        <v>240</v>
+        <v>245</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="22" customHeight="1" x14ac:dyDescent="0.4">
@@ -52123,11 +52221,11 @@
       </c>
       <c r="B6" s="16">
         <f>COUNTIFS(sum!J:J,"no news")</f>
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="C6" s="10">
         <f>B6/$B$5</f>
-        <v>0.96837944664031617</v>
+        <v>0.96442687747035571</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.4">
@@ -52149,11 +52247,11 @@
       </c>
       <c r="B8" s="16">
         <f>COUNTIFS(sum!J:J,"interview")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C8" s="10">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>3.952569169960474E-3</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.4">

</xml_diff>

<commit_message>
added more stragalers to the database and created the docs
</commit_message>
<xml_diff>
--- a/EconJM_status.xlsx
+++ b/EconJM_status.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\javie\Dropbox\Work\Job Search\2025 EconJM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{820AC922-C742-4C7E-AD3C-B3FC9CEE83F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE209D34-6373-4EA0-B5DA-E4851DEED772}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="14620" xr2:uid="{6FE48536-7E5C-BF4C-9490-2A6392576298}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="14620" activeTab="1" xr2:uid="{6FE48536-7E5C-BF4C-9490-2A6392576298}"/>
   </bookViews>
   <sheets>
     <sheet name="sum" sheetId="1" r:id="rId1"/>
@@ -1083,7 +1083,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2551" uniqueCount="803">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2675" uniqueCount="853">
   <si>
     <t>add_id</t>
   </si>
@@ -3528,6 +3528,156 @@
   </si>
   <si>
     <t>Prof. Philipp Ager philipp.ager@uni-mannheim.de</t>
+  </si>
+  <si>
+    <t>https://postdocs.northwestern.edu/announcements/positions-at-northwestern/2025/postdoctoral-research-opportunity-global-llm-values-benchmarking-working-group.html</t>
+  </si>
+  <si>
+    <t>llm_nwest</t>
+  </si>
+  <si>
+    <t>Northwestern University</t>
+  </si>
+  <si>
+    <t>Yingdan Lu. </t>
+  </si>
+  <si>
+    <t>hec_paris</t>
+  </si>
+  <si>
+    <t>HEC Paris</t>
+  </si>
+  <si>
+    <t>monash_post_2</t>
+  </si>
+  <si>
+    <t>Ricardo Dahis, the Primary Investigator (PI)</t>
+  </si>
+  <si>
+    <t>virginia_common</t>
+  </si>
+  <si>
+    <t>Virginia Commonwealth University</t>
+  </si>
+  <si>
+    <t>https://vcujobs.com/jobs/assistant-professor-economics-vcu-main-campus-virginia-united-states</t>
+  </si>
+  <si>
+    <t>apply in JOE + internal wb</t>
+  </si>
+  <si>
+    <t>Christopher Herrington   herringtoncm@vcu.edu</t>
+  </si>
+  <si>
+    <t>bowling_state</t>
+  </si>
+  <si>
+    <t>https://www.schooljobs.com/careers/bgsu/faculty/jobs/5151499/assistant-teaching-professor-of-economics?pagetype=jobOpportunitiesJobs</t>
+  </si>
+  <si>
+    <t>Bowling Green State University</t>
+  </si>
+  <si>
+    <t>osaka_micro</t>
+  </si>
+  <si>
+    <t>https://www.econ.osaka-u.ac.jp/en/en-news/3377/</t>
+  </si>
+  <si>
+    <t>Osaka University</t>
+  </si>
+  <si>
+    <t>Duquesne University</t>
+  </si>
+  <si>
+    <t>duquesne</t>
+  </si>
+  <si>
+    <t>https://apply.interfolio.com/178305</t>
+  </si>
+  <si>
+    <t>rochester</t>
+  </si>
+  <si>
+    <t>c.massaro@rochester.edu</t>
+  </si>
+  <si>
+    <t>University of Rochester</t>
+  </si>
+  <si>
+    <t>uncarolina</t>
+  </si>
+  <si>
+    <t>The University of North Carolina, Charlotte</t>
+  </si>
+  <si>
+    <t>email rec letters to econsearch@charlotte.edu</t>
+  </si>
+  <si>
+    <t>send to email + letter of rec</t>
+  </si>
+  <si>
+    <t>https://jobs.charlotte.edu/postings/65111</t>
+  </si>
+  <si>
+    <t>fiu</t>
+  </si>
+  <si>
+    <t>Florida International University</t>
+  </si>
+  <si>
+    <t>https://pslinks.fiu.edu/psc/jobs/CUSTOMER/HRMS/c/HRS_HRAM_FL.HRS_CG_SEARCH_FL.GBL?Page=HRS_APP_SCHJOB_FL&amp;Action=U</t>
+  </si>
+  <si>
+    <t>Job Opening ID 536413</t>
+  </si>
+  <si>
+    <t>added some stragelers from JOE and EJM</t>
+  </si>
+  <si>
+    <t>rio_grande</t>
+  </si>
+  <si>
+    <t>https://careers.utrgv.edu/postings/49492</t>
+  </si>
+  <si>
+    <t>U Texas Rio Grande Valey</t>
+  </si>
+  <si>
+    <t>lund_post</t>
+  </si>
+  <si>
+    <t>Professor Jutta Bolt</t>
+  </si>
+  <si>
+    <t>University of Lund</t>
+  </si>
+  <si>
+    <t>https://lu.varbi.com/en/what:job/jobID:875828/type:job/where:4/apply:1</t>
+  </si>
+  <si>
+    <t>hse</t>
+  </si>
+  <si>
+    <t>https://iri.hse.ru/announcements/876324879.html</t>
+  </si>
+  <si>
+    <t>National Research University Higher School of Economics</t>
+  </si>
+  <si>
+    <t>warthon_media</t>
+  </si>
+  <si>
+    <t>University of Pennsylvania</t>
+  </si>
+  <si>
+    <t>https://infodem.upenn.edu/wharton-postdoc/</t>
+  </si>
+  <si>
+    <t>about media effects and LLMs</t>
+  </si>
+  <si>
+    <t>added a few more stragelers</t>
   </si>
 </sst>
 </file>
@@ -3709,7 +3859,57 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Percent" xfId="2" builtinId="5"/>
   </cellStyles>
-  <dxfs count="196">
+  <dxfs count="208">
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -5517,6 +5717,76 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -37035,7 +37305,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F7772053-9363-CA4A-A53F-040B7C700753}">
-  <dimension ref="A1:V254"/>
+  <dimension ref="A1:V268"/>
   <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="16" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="19.6640625" customWidth="1"/>
@@ -39955,7 +40225,7 @@
         <v>96</v>
       </c>
       <c r="J65" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="M65" t="s">
         <v>609</v>
@@ -40172,7 +40442,7 @@
         <v>96</v>
       </c>
       <c r="J70" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="M70" s="2" t="s">
         <v>196</v>
@@ -42213,7 +42483,7 @@
         <v>402</v>
       </c>
       <c r="K113" t="s">
-        <v>244</v>
+        <v>309</v>
       </c>
       <c r="L113" s="1">
         <v>45986</v>
@@ -42264,7 +42534,7 @@
         <v>402</v>
       </c>
       <c r="K114" t="s">
-        <v>244</v>
+        <v>309</v>
       </c>
       <c r="L114" s="1">
         <v>45986</v>
@@ -42324,7 +42594,7 @@
         <v>402</v>
       </c>
       <c r="K115" t="s">
-        <v>244</v>
+        <v>309</v>
       </c>
       <c r="L115" s="1">
         <v>45986</v>
@@ -43960,7 +44230,7 @@
         <v>402</v>
       </c>
       <c r="K152" t="s">
-        <v>244</v>
+        <v>309</v>
       </c>
       <c r="L152" s="1">
         <v>45986</v>
@@ -44013,7 +44283,7 @@
         <v>402</v>
       </c>
       <c r="K153" t="s">
-        <v>244</v>
+        <v>309</v>
       </c>
       <c r="L153" s="1">
         <v>45986</v>
@@ -44063,7 +44333,7 @@
         <v>402</v>
       </c>
       <c r="K154" t="s">
-        <v>244</v>
+        <v>309</v>
       </c>
       <c r="L154" s="1">
         <v>45986</v>
@@ -44116,7 +44386,7 @@
         <v>402</v>
       </c>
       <c r="K155" t="s">
-        <v>244</v>
+        <v>309</v>
       </c>
       <c r="L155" s="1">
         <v>45986</v>
@@ -44594,7 +44864,7 @@
         <v>402</v>
       </c>
       <c r="K166" t="s">
-        <v>244</v>
+        <v>309</v>
       </c>
       <c r="L166" s="1">
         <v>45986</v>
@@ -44736,7 +45006,7 @@
         <v>402</v>
       </c>
       <c r="K169" t="s">
-        <v>244</v>
+        <v>309</v>
       </c>
       <c r="L169" s="1">
         <v>45986</v>
@@ -44793,7 +45063,7 @@
         <v>402</v>
       </c>
       <c r="K170" t="s">
-        <v>244</v>
+        <v>309</v>
       </c>
       <c r="L170" s="1">
         <v>45992</v>
@@ -44843,7 +45113,7 @@
         <v>402</v>
       </c>
       <c r="K171" t="s">
-        <v>244</v>
+        <v>309</v>
       </c>
       <c r="L171" s="1">
         <v>45992</v>
@@ -44893,7 +45163,7 @@
         <v>402</v>
       </c>
       <c r="K172" t="s">
-        <v>244</v>
+        <v>309</v>
       </c>
       <c r="L172" s="1">
         <v>45992</v>
@@ -44946,7 +45216,7 @@
         <v>402</v>
       </c>
       <c r="K173" t="s">
-        <v>244</v>
+        <v>309</v>
       </c>
       <c r="L173" s="1">
         <v>45992</v>
@@ -44993,7 +45263,7 @@
         <v>402</v>
       </c>
       <c r="K174" t="s">
-        <v>244</v>
+        <v>309</v>
       </c>
       <c r="L174" s="1">
         <v>45992</v>
@@ -45087,7 +45357,7 @@
         <v>402</v>
       </c>
       <c r="K176" t="s">
-        <v>244</v>
+        <v>309</v>
       </c>
       <c r="L176" s="1">
         <v>45992</v>
@@ -45137,7 +45407,7 @@
         <v>402</v>
       </c>
       <c r="K177" t="s">
-        <v>244</v>
+        <v>309</v>
       </c>
       <c r="L177" s="1">
         <v>45992</v>
@@ -45234,7 +45504,7 @@
         <v>402</v>
       </c>
       <c r="K179" t="s">
-        <v>244</v>
+        <v>309</v>
       </c>
       <c r="L179" s="1">
         <v>45992</v>
@@ -45331,7 +45601,7 @@
         <v>402</v>
       </c>
       <c r="K181" t="s">
-        <v>244</v>
+        <v>309</v>
       </c>
       <c r="L181" s="1">
         <v>45992</v>
@@ -45734,7 +46004,7 @@
         <v>402</v>
       </c>
       <c r="K190" t="s">
-        <v>244</v>
+        <v>309</v>
       </c>
       <c r="L190" s="1">
         <v>45992</v>
@@ -46114,6 +46384,12 @@
       <c r="J199" t="s">
         <v>402</v>
       </c>
+      <c r="K199" t="s">
+        <v>309</v>
+      </c>
+      <c r="L199" s="1">
+        <v>45992</v>
+      </c>
       <c r="M199" t="s">
         <v>680</v>
       </c>
@@ -46282,7 +46558,7 @@
         <v>402</v>
       </c>
       <c r="K203" t="s">
-        <v>244</v>
+        <v>309</v>
       </c>
       <c r="L203" s="1">
         <v>45992</v>
@@ -46455,7 +46731,7 @@
         <v>402</v>
       </c>
       <c r="K207" t="s">
-        <v>244</v>
+        <v>309</v>
       </c>
       <c r="L207" s="1">
         <v>45992</v>
@@ -46892,7 +47168,7 @@
         <v>402</v>
       </c>
       <c r="K217" t="s">
-        <v>244</v>
+        <v>309</v>
       </c>
       <c r="L217" s="1">
         <v>45992</v>
@@ -47068,7 +47344,7 @@
         <v>402</v>
       </c>
       <c r="K221" t="s">
-        <v>244</v>
+        <v>309</v>
       </c>
       <c r="L221" s="1">
         <v>45992</v>
@@ -47199,6 +47475,12 @@
       <c r="J224" t="s">
         <v>402</v>
       </c>
+      <c r="K224" t="s">
+        <v>309</v>
+      </c>
+      <c r="L224" s="1">
+        <v>45992</v>
+      </c>
       <c r="M224" t="s">
         <v>709</v>
       </c>
@@ -47411,7 +47693,7 @@
         <v>402</v>
       </c>
       <c r="K229" t="s">
-        <v>244</v>
+        <v>309</v>
       </c>
       <c r="L229" s="1">
         <v>45992</v>
@@ -47499,7 +47781,7 @@
         <v>402</v>
       </c>
       <c r="K231" t="s">
-        <v>244</v>
+        <v>309</v>
       </c>
       <c r="L231" s="1">
         <v>45992</v>
@@ -47587,7 +47869,7 @@
         <v>402</v>
       </c>
       <c r="K233" t="s">
-        <v>244</v>
+        <v>309</v>
       </c>
       <c r="L233" s="1">
         <v>45992</v>
@@ -47637,7 +47919,7 @@
         <v>402</v>
       </c>
       <c r="K234" t="s">
-        <v>244</v>
+        <v>309</v>
       </c>
       <c r="L234" s="1">
         <v>45992</v>
@@ -47693,7 +47975,7 @@
         <v>402</v>
       </c>
       <c r="K235" t="s">
-        <v>244</v>
+        <v>309</v>
       </c>
       <c r="L235" s="1">
         <v>45992</v>
@@ -47743,7 +48025,7 @@
         <v>402</v>
       </c>
       <c r="K236" t="s">
-        <v>244</v>
+        <v>309</v>
       </c>
       <c r="L236" s="1">
         <v>45992</v>
@@ -47957,7 +48239,7 @@
         <v>96</v>
       </c>
       <c r="J241" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="M241" t="s">
         <v>570</v>
@@ -47983,33 +48265,27 @@
     </row>
     <row r="242" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A242" t="s">
-        <v>784</v>
+        <v>791</v>
       </c>
       <c r="D242" s="1">
         <v>45992</v>
       </c>
       <c r="E242" t="s">
-        <v>40</v>
-      </c>
-      <c r="F242" t="s">
-        <v>785</v>
+        <v>15</v>
+      </c>
+      <c r="H242" t="s">
+        <v>802</v>
       </c>
       <c r="I242" t="s">
-        <v>23</v>
+        <v>96</v>
       </c>
       <c r="J242" t="s">
         <v>402</v>
       </c>
-      <c r="K242" t="s">
-        <v>244</v>
-      </c>
-      <c r="L242" s="1">
-        <v>46027</v>
-      </c>
       <c r="M242" t="s">
-        <v>786</v>
-      </c>
-      <c r="N242" t="e" vm="35">
+        <v>185</v>
+      </c>
+      <c r="N242" t="e" vm="29">
         <v>#VALUE!</v>
       </c>
       <c r="O242" t="s">
@@ -48019,7 +48295,7 @@
         <v>776</v>
       </c>
       <c r="R242" s="1">
-        <v>46026</v>
+        <v>46022</v>
       </c>
       <c r="T242">
         <v>1</v>
@@ -48033,7 +48309,10 @@
     </row>
     <row r="243" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A243" t="s">
-        <v>791</v>
+        <v>792</v>
+      </c>
+      <c r="C243" t="s">
+        <v>794</v>
       </c>
       <c r="D243" s="1">
         <v>45992</v>
@@ -48041,8 +48320,8 @@
       <c r="E243" t="s">
         <v>15</v>
       </c>
-      <c r="H243" t="s">
-        <v>802</v>
+      <c r="F243" s="2" t="s">
+        <v>795</v>
       </c>
       <c r="I243" t="s">
         <v>96</v>
@@ -48051,7 +48330,7 @@
         <v>402</v>
       </c>
       <c r="M243" t="s">
-        <v>185</v>
+        <v>793</v>
       </c>
       <c r="N243" t="e" vm="29">
         <v>#VALUE!</v>
@@ -48063,7 +48342,7 @@
         <v>776</v>
       </c>
       <c r="R243" s="1">
-        <v>46022</v>
+        <v>46053</v>
       </c>
       <c r="T243">
         <v>1</v>
@@ -48077,10 +48356,7 @@
     </row>
     <row r="244" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A244" t="s">
-        <v>792</v>
-      </c>
-      <c r="C244" t="s">
-        <v>794</v>
+        <v>796</v>
       </c>
       <c r="D244" s="1">
         <v>45992</v>
@@ -48088,8 +48364,8 @@
       <c r="E244" t="s">
         <v>15</v>
       </c>
-      <c r="F244" s="2" t="s">
-        <v>795</v>
+      <c r="H244" t="s">
+        <v>797</v>
       </c>
       <c r="I244" t="s">
         <v>96</v>
@@ -48098,9 +48374,9 @@
         <v>402</v>
       </c>
       <c r="M244" t="s">
-        <v>793</v>
-      </c>
-      <c r="N244" t="e" vm="29">
+        <v>750</v>
+      </c>
+      <c r="N244" t="e" vm="47">
         <v>#VALUE!</v>
       </c>
       <c r="O244" t="s">
@@ -48110,7 +48386,7 @@
         <v>776</v>
       </c>
       <c r="R244" s="1">
-        <v>46053</v>
+        <v>46054</v>
       </c>
       <c r="T244">
         <v>1</v>
@@ -48124,16 +48400,16 @@
     </row>
     <row r="245" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A245" t="s">
-        <v>796</v>
+        <v>798</v>
+      </c>
+      <c r="C245" t="s">
+        <v>800</v>
       </c>
       <c r="D245" s="1">
         <v>45992</v>
       </c>
       <c r="E245" t="s">
-        <v>15</v>
-      </c>
-      <c r="H245" t="s">
-        <v>797</v>
+        <v>40</v>
       </c>
       <c r="I245" t="s">
         <v>96</v>
@@ -48142,19 +48418,19 @@
         <v>402</v>
       </c>
       <c r="M245" t="s">
-        <v>750</v>
-      </c>
-      <c r="N245" t="e" vm="47">
+        <v>799</v>
+      </c>
+      <c r="N245" t="e" vm="70">
         <v>#VALUE!</v>
       </c>
       <c r="O245" t="s">
-        <v>26</v>
+        <v>11</v>
       </c>
       <c r="Q245" t="s">
         <v>776</v>
       </c>
       <c r="R245" s="1">
-        <v>46054</v>
+        <v>46026</v>
       </c>
       <c r="T245">
         <v>1</v>
@@ -48168,27 +48444,33 @@
     </row>
     <row r="246" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A246" t="s">
-        <v>662</v>
+        <v>784</v>
       </c>
       <c r="D246" s="1">
-        <v>46011</v>
+        <v>46006</v>
       </c>
       <c r="E246" t="s">
-        <v>15</v>
-      </c>
-      <c r="H246" t="s">
-        <v>664</v>
+        <v>40</v>
+      </c>
+      <c r="F246" t="s">
+        <v>785</v>
       </c>
       <c r="I246" t="s">
-        <v>96</v>
+        <v>23</v>
       </c>
       <c r="J246" t="s">
         <v>402</v>
       </c>
+      <c r="K246" t="s">
+        <v>244</v>
+      </c>
+      <c r="L246" s="1">
+        <v>46027</v>
+      </c>
       <c r="M246" t="s">
-        <v>663</v>
-      </c>
-      <c r="N246" t="e" vm="45">
+        <v>786</v>
+      </c>
+      <c r="N246" t="e" vm="35">
         <v>#VALUE!</v>
       </c>
       <c r="O246" t="s">
@@ -48198,7 +48480,7 @@
         <v>776</v>
       </c>
       <c r="R246" s="1">
-        <v>46037</v>
+        <v>46026</v>
       </c>
       <c r="T246">
         <v>1</v>
@@ -48212,30 +48494,27 @@
     </row>
     <row r="247" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A247" t="s">
-        <v>722</v>
-      </c>
-      <c r="C247" t="s">
-        <v>723</v>
+        <v>841</v>
       </c>
       <c r="D247" s="1">
-        <v>46016</v>
+        <v>46006</v>
       </c>
       <c r="E247" t="s">
-        <v>15</v>
-      </c>
-      <c r="F247" t="s">
-        <v>721</v>
+        <v>844</v>
+      </c>
+      <c r="H247" t="s">
+        <v>842</v>
       </c>
       <c r="I247" t="s">
-        <v>96</v>
+        <v>23</v>
       </c>
       <c r="J247" t="s">
         <v>402</v>
       </c>
       <c r="M247" t="s">
-        <v>720</v>
-      </c>
-      <c r="N247" t="e" vm="68">
+        <v>843</v>
+      </c>
+      <c r="N247" t="e" vm="46">
         <v>#VALUE!</v>
       </c>
       <c r="O247" t="s">
@@ -48245,7 +48524,7 @@
         <v>776</v>
       </c>
       <c r="R247" s="1">
-        <v>45992</v>
+        <v>46022</v>
       </c>
       <c r="T247">
         <v>1</v>
@@ -48258,21 +48537,17 @@
       </c>
     </row>
     <row r="248" spans="1:22" x14ac:dyDescent="0.4">
-      <c r="A248" s="4" t="s">
-        <v>719</v>
-      </c>
-      <c r="B248" s="19"/>
-      <c r="C248" t="s">
-        <v>783</v>
+      <c r="A248" t="s">
+        <v>662</v>
       </c>
       <c r="D248" s="1">
-        <v>46016</v>
+        <v>46011</v>
       </c>
       <c r="E248" t="s">
         <v>15</v>
       </c>
-      <c r="G248">
-        <v>3</v>
+      <c r="H248" t="s">
+        <v>664</v>
       </c>
       <c r="I248" t="s">
         <v>96</v>
@@ -48280,26 +48555,20 @@
       <c r="J248" t="s">
         <v>402</v>
       </c>
-      <c r="K248" t="s">
-        <v>244</v>
-      </c>
-      <c r="L248" s="1">
-        <v>45992</v>
-      </c>
-      <c r="M248" s="2" t="s">
-        <v>718</v>
+      <c r="M248" t="s">
+        <v>663</v>
       </c>
       <c r="N248" t="e" vm="45">
         <v>#VALUE!</v>
       </c>
       <c r="O248" t="s">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="Q248" t="s">
         <v>776</v>
       </c>
       <c r="R248" s="1">
-        <v>45996</v>
+        <v>46037</v>
       </c>
       <c r="T248">
         <v>1</v>
@@ -48313,7 +48582,10 @@
     </row>
     <row r="249" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A249" t="s">
-        <v>787</v>
+        <v>722</v>
+      </c>
+      <c r="C249" t="s">
+        <v>723</v>
       </c>
       <c r="D249" s="1">
         <v>46016</v>
@@ -48321,6 +48593,9 @@
       <c r="E249" t="s">
         <v>15</v>
       </c>
+      <c r="F249" t="s">
+        <v>721</v>
+      </c>
       <c r="I249" t="s">
         <v>96</v>
       </c>
@@ -48328,10 +48603,13 @@
         <v>402</v>
       </c>
       <c r="M249" t="s">
-        <v>788</v>
-      </c>
-      <c r="N249" t="e" vm="29">
+        <v>720</v>
+      </c>
+      <c r="N249" t="e" vm="68">
         <v>#VALUE!</v>
+      </c>
+      <c r="O249" t="s">
+        <v>26</v>
       </c>
       <c r="Q249" t="s">
         <v>776</v>
@@ -48340,7 +48618,7 @@
         <v>45992</v>
       </c>
       <c r="T249">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U249">
         <v>0</v>
@@ -48350,8 +48628,12 @@
       </c>
     </row>
     <row r="250" spans="1:22" x14ac:dyDescent="0.4">
-      <c r="A250" t="s">
-        <v>790</v>
+      <c r="A250" s="4" t="s">
+        <v>719</v>
+      </c>
+      <c r="B250" s="19"/>
+      <c r="C250" t="s">
+        <v>783</v>
       </c>
       <c r="D250" s="1">
         <v>46016</v>
@@ -48359,16 +48641,25 @@
       <c r="E250" t="s">
         <v>15</v>
       </c>
+      <c r="G250">
+        <v>3</v>
+      </c>
       <c r="I250" t="s">
         <v>96</v>
       </c>
       <c r="J250" t="s">
         <v>402</v>
       </c>
-      <c r="M250" t="s">
-        <v>789</v>
-      </c>
-      <c r="N250" t="e" vm="75">
+      <c r="K250" t="s">
+        <v>309</v>
+      </c>
+      <c r="L250" s="1">
+        <v>45992</v>
+      </c>
+      <c r="M250" s="2" t="s">
+        <v>718</v>
+      </c>
+      <c r="N250" t="e" vm="45">
         <v>#VALUE!</v>
       </c>
       <c r="O250" t="s">
@@ -48378,7 +48669,7 @@
         <v>776</v>
       </c>
       <c r="R250" s="1">
-        <v>45992</v>
+        <v>45996</v>
       </c>
       <c r="T250">
         <v>1</v>
@@ -48392,16 +48683,13 @@
     </row>
     <row r="251" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A251" t="s">
-        <v>528</v>
-      </c>
-      <c r="C251" t="s">
-        <v>178</v>
+        <v>787</v>
       </c>
       <c r="D251" s="1">
-        <v>46023</v>
+        <v>46016</v>
       </c>
       <c r="E251" t="s">
-        <v>529</v>
+        <v>15</v>
       </c>
       <c r="I251" t="s">
         <v>96</v>
@@ -48410,39 +48698,36 @@
         <v>402</v>
       </c>
       <c r="M251" t="s">
-        <v>530</v>
-      </c>
-      <c r="N251" t="e" vm="102">
+        <v>788</v>
+      </c>
+      <c r="N251" t="e" vm="29">
         <v>#VALUE!</v>
-      </c>
-      <c r="O251" t="s">
-        <v>19</v>
       </c>
       <c r="Q251" t="s">
         <v>776</v>
       </c>
       <c r="R251" s="1">
-        <v>46041</v>
+        <v>45992</v>
       </c>
       <c r="T251">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U251">
         <v>0</v>
       </c>
       <c r="V251">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="252" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A252" t="s">
-        <v>564</v>
+        <v>790</v>
       </c>
       <c r="D252" s="1">
-        <v>46023</v>
+        <v>46016</v>
       </c>
       <c r="E252" t="s">
-        <v>565</v>
+        <v>15</v>
       </c>
       <c r="I252" t="s">
         <v>96</v>
@@ -48451,19 +48736,19 @@
         <v>402</v>
       </c>
       <c r="M252" t="s">
-        <v>566</v>
-      </c>
-      <c r="N252" t="e" vm="103">
+        <v>789</v>
+      </c>
+      <c r="N252" t="e" vm="75">
         <v>#VALUE!</v>
       </c>
       <c r="O252" t="s">
-        <v>26</v>
+        <v>11</v>
       </c>
       <c r="Q252" t="s">
         <v>776</v>
       </c>
       <c r="R252" s="1">
-        <v>45664</v>
+        <v>45992</v>
       </c>
       <c r="T252">
         <v>1</v>
@@ -48477,13 +48762,16 @@
     </row>
     <row r="253" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A253" t="s">
-        <v>255</v>
+        <v>528</v>
+      </c>
+      <c r="C253" t="s">
+        <v>178</v>
+      </c>
+      <c r="D253" s="1">
+        <v>46023</v>
       </c>
       <c r="E253" t="s">
-        <v>15</v>
-      </c>
-      <c r="F253" s="2" t="s">
-        <v>257</v>
+        <v>529</v>
       </c>
       <c r="I253" t="s">
         <v>96</v>
@@ -48492,39 +48780,39 @@
         <v>402</v>
       </c>
       <c r="M253" t="s">
-        <v>256</v>
-      </c>
-      <c r="N253" t="e" vm="35">
+        <v>530</v>
+      </c>
+      <c r="N253" t="e" vm="102">
         <v>#VALUE!</v>
       </c>
       <c r="O253" t="s">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="Q253" t="s">
         <v>776</v>
       </c>
+      <c r="R253" s="1">
+        <v>46041</v>
+      </c>
       <c r="T253">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U253">
         <v>0</v>
       </c>
       <c r="V253">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="254" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A254" t="s">
-        <v>798</v>
-      </c>
-      <c r="C254" t="s">
-        <v>800</v>
+        <v>564</v>
       </c>
       <c r="D254" s="1">
-        <v>45992</v>
+        <v>46023</v>
       </c>
       <c r="E254" t="s">
-        <v>40</v>
+        <v>565</v>
       </c>
       <c r="I254" t="s">
         <v>96</v>
@@ -48533,19 +48821,19 @@
         <v>402</v>
       </c>
       <c r="M254" t="s">
-        <v>799</v>
-      </c>
-      <c r="N254" t="e" vm="70">
+        <v>566</v>
+      </c>
+      <c r="N254" t="e" vm="103">
         <v>#VALUE!</v>
       </c>
       <c r="O254" t="s">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="Q254" t="s">
         <v>776</v>
       </c>
       <c r="R254" s="1">
-        <v>46026</v>
+        <v>45664</v>
       </c>
       <c r="T254">
         <v>1</v>
@@ -48557,60 +48845,706 @@
         <v>0</v>
       </c>
     </row>
+    <row r="255" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A255" t="s">
+        <v>804</v>
+      </c>
+      <c r="D255" s="1">
+        <v>46023</v>
+      </c>
+      <c r="E255" s="2" t="s">
+        <v>803</v>
+      </c>
+      <c r="F255" s="2" t="s">
+        <v>806</v>
+      </c>
+      <c r="I255" t="s">
+        <v>23</v>
+      </c>
+      <c r="J255" t="s">
+        <v>402</v>
+      </c>
+      <c r="M255" t="s">
+        <v>805</v>
+      </c>
+      <c r="N255" t="e" vm="35">
+        <v>#VALUE!</v>
+      </c>
+      <c r="O255" t="s">
+        <v>26</v>
+      </c>
+      <c r="Q255" t="s">
+        <v>776</v>
+      </c>
+      <c r="R255" s="1">
+        <v>46038</v>
+      </c>
+      <c r="T255">
+        <v>1</v>
+      </c>
+      <c r="U255">
+        <v>0</v>
+      </c>
+      <c r="V255">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="256" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A256" t="s">
+        <v>807</v>
+      </c>
+      <c r="D256" s="1">
+        <v>46023</v>
+      </c>
+      <c r="E256" t="s">
+        <v>15</v>
+      </c>
+      <c r="I256" t="s">
+        <v>23</v>
+      </c>
+      <c r="J256" t="s">
+        <v>402</v>
+      </c>
+      <c r="M256" t="s">
+        <v>808</v>
+      </c>
+      <c r="N256" t="e" vm="54">
+        <v>#VALUE!</v>
+      </c>
+      <c r="O256" t="s">
+        <v>11</v>
+      </c>
+      <c r="Q256" t="s">
+        <v>776</v>
+      </c>
+      <c r="R256" s="1">
+        <v>46052</v>
+      </c>
+      <c r="T256">
+        <v>1</v>
+      </c>
+      <c r="U256">
+        <v>0</v>
+      </c>
+      <c r="V256">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="257" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A257" t="s">
+        <v>809</v>
+      </c>
+      <c r="D257" s="1">
+        <v>46023</v>
+      </c>
+      <c r="E257" t="s">
+        <v>15</v>
+      </c>
+      <c r="H257" t="s">
+        <v>810</v>
+      </c>
+      <c r="I257" t="s">
+        <v>23</v>
+      </c>
+      <c r="J257" t="s">
+        <v>402</v>
+      </c>
+      <c r="M257" t="s">
+        <v>123</v>
+      </c>
+      <c r="N257" t="e" vm="25">
+        <v>#VALUE!</v>
+      </c>
+      <c r="O257" t="s">
+        <v>26</v>
+      </c>
+      <c r="Q257" t="s">
+        <v>776</v>
+      </c>
+      <c r="R257" s="1">
+        <v>46052</v>
+      </c>
+      <c r="T257">
+        <v>1</v>
+      </c>
+      <c r="U257">
+        <v>0</v>
+      </c>
+      <c r="V257">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="258" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A258" t="s">
+        <v>811</v>
+      </c>
+      <c r="C258" t="s">
+        <v>814</v>
+      </c>
+      <c r="D258" s="1">
+        <v>46023</v>
+      </c>
+      <c r="E258" t="s">
+        <v>40</v>
+      </c>
+      <c r="F258" t="s">
+        <v>813</v>
+      </c>
+      <c r="H258" t="s">
+        <v>815</v>
+      </c>
+      <c r="I258" t="s">
+        <v>23</v>
+      </c>
+      <c r="J258" t="s">
+        <v>402</v>
+      </c>
+      <c r="M258" t="s">
+        <v>812</v>
+      </c>
+      <c r="N258" t="e" vm="35">
+        <v>#VALUE!</v>
+      </c>
+      <c r="O258" t="s">
+        <v>11</v>
+      </c>
+      <c r="Q258" t="s">
+        <v>776</v>
+      </c>
+      <c r="R258" s="1">
+        <v>46037</v>
+      </c>
+      <c r="T258">
+        <v>1</v>
+      </c>
+      <c r="U258">
+        <v>0</v>
+      </c>
+      <c r="V258">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="259" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A259" t="s">
+        <v>816</v>
+      </c>
+      <c r="D259" s="1">
+        <v>46023</v>
+      </c>
+      <c r="E259" t="s">
+        <v>40</v>
+      </c>
+      <c r="F259" s="2" t="s">
+        <v>817</v>
+      </c>
+      <c r="I259" t="s">
+        <v>23</v>
+      </c>
+      <c r="J259" t="s">
+        <v>402</v>
+      </c>
+      <c r="M259" t="s">
+        <v>818</v>
+      </c>
+      <c r="N259" t="e" vm="35">
+        <v>#VALUE!</v>
+      </c>
+      <c r="O259" t="s">
+        <v>11</v>
+      </c>
+      <c r="Q259" t="s">
+        <v>776</v>
+      </c>
+      <c r="R259" s="1">
+        <v>46066</v>
+      </c>
+      <c r="T259">
+        <v>1</v>
+      </c>
+      <c r="U259">
+        <v>0</v>
+      </c>
+      <c r="V259">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="260" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A260" t="s">
+        <v>819</v>
+      </c>
+      <c r="D260" s="1">
+        <v>46023</v>
+      </c>
+      <c r="E260" t="s">
+        <v>40</v>
+      </c>
+      <c r="F260" t="s">
+        <v>820</v>
+      </c>
+      <c r="I260" t="s">
+        <v>23</v>
+      </c>
+      <c r="J260" t="s">
+        <v>402</v>
+      </c>
+      <c r="M260" t="s">
+        <v>821</v>
+      </c>
+      <c r="N260" t="e" vm="6">
+        <v>#VALUE!</v>
+      </c>
+      <c r="O260" t="s">
+        <v>11</v>
+      </c>
+      <c r="Q260" t="s">
+        <v>776</v>
+      </c>
+      <c r="R260" s="1">
+        <v>46052</v>
+      </c>
+      <c r="T260">
+        <v>1</v>
+      </c>
+      <c r="U260">
+        <v>0</v>
+      </c>
+      <c r="V260">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="261" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A261" t="s">
+        <v>823</v>
+      </c>
+      <c r="D261" s="1">
+        <v>46023</v>
+      </c>
+      <c r="E261" t="s">
+        <v>40</v>
+      </c>
+      <c r="F261" s="2" t="s">
+        <v>824</v>
+      </c>
+      <c r="I261" t="s">
+        <v>23</v>
+      </c>
+      <c r="J261" t="s">
+        <v>402</v>
+      </c>
+      <c r="M261" t="s">
+        <v>822</v>
+      </c>
+      <c r="N261" t="e" vm="35">
+        <v>#VALUE!</v>
+      </c>
+      <c r="O261" t="s">
+        <v>11</v>
+      </c>
+      <c r="Q261" t="s">
+        <v>776</v>
+      </c>
+      <c r="R261" s="1">
+        <v>46113</v>
+      </c>
+      <c r="T261">
+        <v>1</v>
+      </c>
+      <c r="U261">
+        <v>0</v>
+      </c>
+      <c r="V261">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="262" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A262" t="s">
+        <v>825</v>
+      </c>
+      <c r="C262" t="s">
+        <v>831</v>
+      </c>
+      <c r="D262" s="1">
+        <v>46023</v>
+      </c>
+      <c r="E262" t="s">
+        <v>40</v>
+      </c>
+      <c r="F262" s="2" t="s">
+        <v>826</v>
+      </c>
+      <c r="I262" t="s">
+        <v>23</v>
+      </c>
+      <c r="J262" t="s">
+        <v>402</v>
+      </c>
+      <c r="M262" t="s">
+        <v>827</v>
+      </c>
+      <c r="N262" t="e" vm="35">
+        <v>#VALUE!</v>
+      </c>
+      <c r="O262" t="s">
+        <v>26</v>
+      </c>
+      <c r="Q262" t="s">
+        <v>776</v>
+      </c>
+      <c r="R262" s="1">
+        <v>46038</v>
+      </c>
+      <c r="T262">
+        <v>1</v>
+      </c>
+      <c r="U262">
+        <v>0</v>
+      </c>
+      <c r="V262">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="263" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A263" t="s">
+        <v>828</v>
+      </c>
+      <c r="C263" t="s">
+        <v>830</v>
+      </c>
+      <c r="D263" s="1">
+        <v>46023</v>
+      </c>
+      <c r="E263" t="s">
+        <v>40</v>
+      </c>
+      <c r="F263" t="s">
+        <v>832</v>
+      </c>
+      <c r="I263" t="s">
+        <v>23</v>
+      </c>
+      <c r="J263" t="s">
+        <v>402</v>
+      </c>
+      <c r="M263" t="s">
+        <v>829</v>
+      </c>
+      <c r="N263" t="e" vm="35">
+        <v>#VALUE!</v>
+      </c>
+      <c r="O263" t="s">
+        <v>11</v>
+      </c>
+      <c r="Q263" t="s">
+        <v>776</v>
+      </c>
+      <c r="R263" s="1">
+        <v>46143</v>
+      </c>
+      <c r="T263">
+        <v>1</v>
+      </c>
+      <c r="U263">
+        <v>0</v>
+      </c>
+      <c r="V263">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="264" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A264" t="s">
+        <v>833</v>
+      </c>
+      <c r="C264" t="s">
+        <v>836</v>
+      </c>
+      <c r="D264" s="1">
+        <v>46023</v>
+      </c>
+      <c r="E264" t="s">
+        <v>40</v>
+      </c>
+      <c r="F264" s="2" t="s">
+        <v>835</v>
+      </c>
+      <c r="I264" t="s">
+        <v>23</v>
+      </c>
+      <c r="J264" t="s">
+        <v>402</v>
+      </c>
+      <c r="M264" t="s">
+        <v>834</v>
+      </c>
+      <c r="N264" t="e" vm="35">
+        <v>#VALUE!</v>
+      </c>
+      <c r="O264" t="s">
+        <v>11</v>
+      </c>
+      <c r="Q264" t="s">
+        <v>776</v>
+      </c>
+      <c r="R264" s="1">
+        <v>46027</v>
+      </c>
+      <c r="T264">
+        <v>1</v>
+      </c>
+      <c r="U264">
+        <v>0</v>
+      </c>
+      <c r="V264">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="265" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A265" t="s">
+        <v>838</v>
+      </c>
+      <c r="D265" s="1">
+        <v>46023</v>
+      </c>
+      <c r="E265" t="s">
+        <v>839</v>
+      </c>
+      <c r="I265" t="s">
+        <v>23</v>
+      </c>
+      <c r="J265" t="s">
+        <v>402</v>
+      </c>
+      <c r="M265" t="s">
+        <v>840</v>
+      </c>
+      <c r="N265" t="e" vm="35">
+        <v>#VALUE!</v>
+      </c>
+      <c r="O265" t="s">
+        <v>11</v>
+      </c>
+      <c r="Q265" t="s">
+        <v>776</v>
+      </c>
+      <c r="T265">
+        <v>1</v>
+      </c>
+      <c r="U265">
+        <v>0</v>
+      </c>
+      <c r="V265">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="266" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A266" t="s">
+        <v>845</v>
+      </c>
+      <c r="D266" s="1">
+        <v>46023</v>
+      </c>
+      <c r="E266" t="s">
+        <v>846</v>
+      </c>
+      <c r="I266" t="s">
+        <v>23</v>
+      </c>
+      <c r="J266" t="s">
+        <v>402</v>
+      </c>
+      <c r="M266" t="s">
+        <v>847</v>
+      </c>
+      <c r="N266" t="e" vm="84">
+        <v>#VALUE!</v>
+      </c>
+      <c r="O266" t="s">
+        <v>11</v>
+      </c>
+      <c r="Q266" t="s">
+        <v>776</v>
+      </c>
+      <c r="R266" s="1">
+        <v>46037</v>
+      </c>
+      <c r="T266">
+        <v>1</v>
+      </c>
+      <c r="U266">
+        <v>0</v>
+      </c>
+      <c r="V266">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="267" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A267" t="s">
+        <v>848</v>
+      </c>
+      <c r="C267" t="s">
+        <v>851</v>
+      </c>
+      <c r="D267" s="1">
+        <v>46023</v>
+      </c>
+      <c r="E267" t="s">
+        <v>850</v>
+      </c>
+      <c r="I267" t="s">
+        <v>23</v>
+      </c>
+      <c r="J267" t="s">
+        <v>402</v>
+      </c>
+      <c r="M267" t="s">
+        <v>849</v>
+      </c>
+      <c r="N267" t="e" vm="35">
+        <v>#VALUE!</v>
+      </c>
+      <c r="O267" t="s">
+        <v>26</v>
+      </c>
+      <c r="Q267" t="s">
+        <v>776</v>
+      </c>
+      <c r="R267" s="1">
+        <v>46033</v>
+      </c>
+      <c r="T267">
+        <v>1</v>
+      </c>
+      <c r="U267">
+        <v>0</v>
+      </c>
+      <c r="V267">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="268" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A268" t="s">
+        <v>255</v>
+      </c>
+      <c r="E268" t="s">
+        <v>15</v>
+      </c>
+      <c r="F268" s="2" t="s">
+        <v>257</v>
+      </c>
+      <c r="I268" t="s">
+        <v>96</v>
+      </c>
+      <c r="J268" t="s">
+        <v>402</v>
+      </c>
+      <c r="M268" t="s">
+        <v>256</v>
+      </c>
+      <c r="N268" t="e" vm="35">
+        <v>#VALUE!</v>
+      </c>
+      <c r="O268" t="s">
+        <v>11</v>
+      </c>
+      <c r="Q268" t="s">
+        <v>776</v>
+      </c>
+      <c r="T268">
+        <v>0</v>
+      </c>
+      <c r="U268">
+        <v>0</v>
+      </c>
+      <c r="V268">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:V248" xr:uid="{F7772053-9363-CA4A-A53F-040B7C700753}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:V253">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:V268">
       <sortCondition ref="D1:D248"/>
     </sortState>
   </autoFilter>
   <conditionalFormatting sqref="A1:B208 A210:B1048576">
-    <cfRule type="duplicateValues" dxfId="195" priority="14"/>
+    <cfRule type="duplicateValues" dxfId="207" priority="23"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A2:B22">
-    <cfRule type="duplicateValues" dxfId="194" priority="15"/>
+    <cfRule type="duplicateValues" dxfId="206" priority="24"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A61:B61">
-    <cfRule type="duplicateValues" dxfId="193" priority="13"/>
+    <cfRule type="duplicateValues" dxfId="205" priority="22"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="I1:I1048576">
-    <cfRule type="containsText" dxfId="192" priority="6" operator="containsText" text="closed">
+    <cfRule type="containsText" dxfId="204" priority="15" operator="containsText" text="closed">
       <formula>NOT(ISERROR(SEARCH("closed",I1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="191" priority="7" operator="containsText" text="abandoned">
+    <cfRule type="containsText" dxfId="203" priority="16" operator="containsText" text="abandoned">
       <formula>NOT(ISERROR(SEARCH("abandoned",I1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="190" priority="9" operator="containsText" text="late app">
+    <cfRule type="containsText" dxfId="202" priority="18" operator="containsText" text="late app">
       <formula>NOT(ISERROR(SEARCH("late app",I1)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I2:L223 O78:O80 O83:O89 O92:O112 O115:O124 O126:O181 R136 R153 R159 R166 R173 R178 O183:O205 O208:O211 O213:O218 O220:O233 I224:K224 R225 I225:L1048576 O235:O237 O239:O248 M248 O250:O254 I1:J1">
-    <cfRule type="containsText" dxfId="189" priority="12" operator="containsText" text="completed">
+  <conditionalFormatting sqref="I2:L1048576 O78:O80 O83:O89 O92:O112 O115:O124 O126:O181 R136 R153 R159 R166 R173 R178 O183:O205 O208:O211 O213:O218 O220:O233 R225 O235:O237 O239:O248 M248 O250:O255 I1:J1 M266 N267">
+    <cfRule type="containsText" dxfId="201" priority="21" operator="containsText" text="completed">
       <formula>NOT(ISERROR(SEARCH("completed",I1)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J1:J1048576">
-    <cfRule type="containsText" dxfId="188" priority="1" operator="containsText" text="no news">
+    <cfRule type="containsText" dxfId="200" priority="10" operator="containsText" text="no news">
       <formula>NOT(ISERROR(SEARCH("no news",J1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="187" priority="2" operator="containsText" text="offer">
+    <cfRule type="containsText" dxfId="199" priority="11" operator="containsText" text="offer">
       <formula>NOT(ISERROR(SEARCH("offer",J1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="186" priority="3" operator="containsText" text="fly out">
+    <cfRule type="containsText" dxfId="198" priority="12" operator="containsText" text="fly out">
       <formula>NOT(ISERROR(SEARCH("fly out",J1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="185" priority="4" operator="containsText" text="interview">
+    <cfRule type="containsText" dxfId="197" priority="13" operator="containsText" text="interview">
       <formula>NOT(ISERROR(SEARCH("interview",J1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="184" priority="5" operator="containsText" text="rejected">
+    <cfRule type="containsText" dxfId="196" priority="14" operator="containsText" text="rejected">
       <formula>NOT(ISERROR(SEARCH("rejected",J1)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K1:L223 O78:O80 O83:O89 O92:O112 O115:O124 O126:O181 R136 R153 R159 R166 R173 R178 O183:O205 O208:O211 O213:O218 O220:O233 K224 R225 K225:L1048576 O235:O237 O239:O248 M248 O250:O254">
-    <cfRule type="containsText" dxfId="183" priority="10" operator="containsText" text="NO">
+  <conditionalFormatting sqref="K1:L1048576 O78:O80 O83:O89 O92:O112 O115:O124 O126:O181 R136 R153 R159 R166 R173 R178 O183:O205 O208:O211 O213:O218 O220:O233 R225 O235:O237 O239:O248 M248 O250:O255 M266 N267">
+    <cfRule type="containsText" dxfId="195" priority="19" operator="containsText" text="NO">
       <formula>NOT(ISERROR(SEARCH("NO",K1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="182" priority="11" operator="containsText" text="YES">
+    <cfRule type="containsText" dxfId="194" priority="20" operator="containsText" text="YES">
       <formula>NOT(ISERROR(SEARCH("YES",K1)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="N256:O264 O265 N266:O266 O267:O268">
+    <cfRule type="containsText" dxfId="193" priority="7" operator="containsText" text="NO">
+      <formula>NOT(ISERROR(SEARCH("NO",N256)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="192" priority="8" operator="containsText" text="YES">
+      <formula>NOT(ISERROR(SEARCH("YES",N256)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="191" priority="9" operator="containsText" text="completed">
+      <formula>NOT(ISERROR(SEARCH("completed",N256)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="N265">
+    <cfRule type="containsText" dxfId="5" priority="4" operator="containsText" text="NO">
+      <formula>NOT(ISERROR(SEARCH("NO",N265)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="4" priority="5" operator="containsText" text="YES">
+      <formula>NOT(ISERROR(SEARCH("YES",N265)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="3" priority="6" operator="containsText" text="completed">
+      <formula>NOT(ISERROR(SEARCH("completed",N265)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="N268">
+    <cfRule type="containsText" dxfId="2" priority="1" operator="containsText" text="NO">
+      <formula>NOT(ISERROR(SEARCH("NO",N268)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="YES">
+      <formula>NOT(ISERROR(SEARCH("YES",N268)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="0" priority="3" operator="containsText" text="completed">
+      <formula>NOT(ISERROR(SEARCH("completed",N268)))</formula>
     </cfRule>
   </conditionalFormatting>
   <hyperlinks>
@@ -48695,7 +49629,7 @@
     <hyperlink ref="M17" r:id="rId79" xr:uid="{9A9A6BC9-B330-7842-A78C-4DCC88F5E19F}"/>
     <hyperlink ref="M32" r:id="rId80" xr:uid="{928CABEF-4FA6-E646-8140-7B6E43F8FB96}"/>
     <hyperlink ref="F177" r:id="rId81" xr:uid="{82BF1574-A6C6-1641-9FFE-615861E401FD}"/>
-    <hyperlink ref="F253" r:id="rId82" xr:uid="{3562807E-7FDA-F046-BA03-5DDD43072DB7}"/>
+    <hyperlink ref="F268" r:id="rId82" xr:uid="{3562807E-7FDA-F046-BA03-5DDD43072DB7}"/>
     <hyperlink ref="H215" r:id="rId83" display="mailto:ivanpaya@ua.es" xr:uid="{DEFB77A5-E57F-714C-BAB9-56DE82BA0B2E}"/>
     <hyperlink ref="H138" r:id="rId84" display="mailto:ari.hyytinen@hanken.fi" xr:uid="{7777B12A-FD99-4A43-A14B-A15661B760DC}"/>
     <hyperlink ref="H115" r:id="rId85" display="mailto:peter.haan@fu-berlin.de" xr:uid="{3D1A69ED-8F06-1246-B586-201CB349DB62}"/>
@@ -48713,17 +49647,23 @@
     <hyperlink ref="H240" r:id="rId97" display="mailto:ondrej.krcal@econ.muni.cz" xr:uid="{EDDEB1E6-5767-4FFB-A0AE-57A909D04E81}"/>
     <hyperlink ref="M218" r:id="rId98" display="https://www.ovgu.de/unimagdeburg/en/" xr:uid="{BCB3935D-2B6D-4090-86F5-762D762ED0E3}"/>
     <hyperlink ref="E152" r:id="rId99" xr:uid="{550520C0-1E25-41CD-9AEE-9A3C4D7D328C}"/>
-    <hyperlink ref="M248" r:id="rId100" xr:uid="{F0DD6D71-3FFD-4EAB-A251-AAF2DA8EF53C}"/>
-    <hyperlink ref="F244" r:id="rId101" xr:uid="{BDBBC2E2-C3C5-4526-A621-853D22D99CCF}"/>
+    <hyperlink ref="M250" r:id="rId100" xr:uid="{F0DD6D71-3FFD-4EAB-A251-AAF2DA8EF53C}"/>
+    <hyperlink ref="F243" r:id="rId101" xr:uid="{BDBBC2E2-C3C5-4526-A621-853D22D99CCF}"/>
+    <hyperlink ref="F255" r:id="rId102" display="mailto:comap@northwestern.edu" xr:uid="{4DD04925-4C98-401C-B09E-A61B83C23B4E}"/>
+    <hyperlink ref="E255" r:id="rId103" xr:uid="{491ECAF5-1DC5-4C3F-B1BE-621395157776}"/>
+    <hyperlink ref="F259" r:id="rId104" xr:uid="{B084E08B-44BE-4FA5-A345-8036292B3E22}"/>
+    <hyperlink ref="F261" r:id="rId105" xr:uid="{F59B1D31-814A-4100-8601-8879ABB1E739}"/>
+    <hyperlink ref="F262" r:id="rId106" xr:uid="{C4BD89A9-F3F0-4E10-BAC5-751787E6C1A9}"/>
+    <hyperlink ref="F264" r:id="rId107" xr:uid="{64E2681C-F146-4414-BBE6-9DC59E57C615}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId102"/>
+  <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId108"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{923E81FA-B875-3C4E-A189-1A21268FA086}">
-  <dimension ref="A1:C269"/>
+  <dimension ref="A1:C274"/>
   <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="16" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="32.83203125" customWidth="1"/>
@@ -51624,526 +52564,584 @@
         <v>97</v>
       </c>
     </row>
+    <row r="270" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A270" s="1">
+        <v>45992</v>
+      </c>
+      <c r="B270" t="s">
+        <v>195</v>
+      </c>
+      <c r="C270" t="s">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="271" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A271" s="1">
+        <v>45993</v>
+      </c>
+      <c r="B271" t="s">
+        <v>611</v>
+      </c>
+      <c r="C271" t="s">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="272" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A272" s="1">
+        <v>45993</v>
+      </c>
+      <c r="C272" t="s">
+        <v>837</v>
+      </c>
+    </row>
+    <row r="273" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A273" s="1">
+        <v>45993</v>
+      </c>
+      <c r="B273" t="s">
+        <v>568</v>
+      </c>
+      <c r="C273" t="s">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="274" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A274" s="1">
+        <v>45994</v>
+      </c>
+      <c r="C274" t="s">
+        <v>852</v>
+      </c>
+    </row>
   </sheetData>
   <conditionalFormatting sqref="B5">
-    <cfRule type="duplicateValues" dxfId="181" priority="188"/>
-    <cfRule type="duplicateValues" dxfId="180" priority="189"/>
+    <cfRule type="duplicateValues" dxfId="190" priority="191"/>
+    <cfRule type="duplicateValues" dxfId="189" priority="192"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B10">
-    <cfRule type="duplicateValues" dxfId="179" priority="187"/>
-    <cfRule type="duplicateValues" dxfId="178" priority="186"/>
+    <cfRule type="duplicateValues" dxfId="188" priority="190"/>
+    <cfRule type="duplicateValues" dxfId="187" priority="189"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B11">
-    <cfRule type="duplicateValues" dxfId="177" priority="185"/>
-    <cfRule type="duplicateValues" dxfId="176" priority="184"/>
+    <cfRule type="duplicateValues" dxfId="186" priority="188"/>
+    <cfRule type="duplicateValues" dxfId="185" priority="187"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B12">
-    <cfRule type="duplicateValues" dxfId="175" priority="183"/>
-    <cfRule type="duplicateValues" dxfId="174" priority="182"/>
+    <cfRule type="duplicateValues" dxfId="184" priority="186"/>
+    <cfRule type="duplicateValues" dxfId="183" priority="185"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B15">
-    <cfRule type="duplicateValues" dxfId="173" priority="180"/>
-    <cfRule type="duplicateValues" dxfId="172" priority="181"/>
+    <cfRule type="duplicateValues" dxfId="182" priority="184"/>
+    <cfRule type="duplicateValues" dxfId="181" priority="183"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B16">
-    <cfRule type="duplicateValues" dxfId="171" priority="179"/>
+    <cfRule type="duplicateValues" dxfId="180" priority="182"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B17">
-    <cfRule type="duplicateValues" dxfId="170" priority="178"/>
-    <cfRule type="duplicateValues" dxfId="169" priority="177"/>
+    <cfRule type="duplicateValues" dxfId="179" priority="181"/>
+    <cfRule type="duplicateValues" dxfId="178" priority="180"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B18">
-    <cfRule type="duplicateValues" dxfId="168" priority="176"/>
-    <cfRule type="duplicateValues" dxfId="167" priority="175"/>
+    <cfRule type="duplicateValues" dxfId="177" priority="179"/>
+    <cfRule type="duplicateValues" dxfId="176" priority="178"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B19">
-    <cfRule type="duplicateValues" dxfId="166" priority="174"/>
+    <cfRule type="duplicateValues" dxfId="175" priority="177"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B22:B23">
-    <cfRule type="duplicateValues" dxfId="165" priority="173"/>
-    <cfRule type="duplicateValues" dxfId="164" priority="172"/>
+    <cfRule type="duplicateValues" dxfId="174" priority="176"/>
+    <cfRule type="duplicateValues" dxfId="173" priority="175"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B24">
-    <cfRule type="duplicateValues" dxfId="163" priority="170"/>
-    <cfRule type="duplicateValues" dxfId="162" priority="171"/>
+    <cfRule type="duplicateValues" dxfId="172" priority="174"/>
+    <cfRule type="duplicateValues" dxfId="171" priority="173"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B27">
-    <cfRule type="duplicateValues" dxfId="161" priority="168"/>
-    <cfRule type="duplicateValues" dxfId="160" priority="169"/>
+    <cfRule type="duplicateValues" dxfId="170" priority="172"/>
+    <cfRule type="duplicateValues" dxfId="169" priority="171"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B28">
-    <cfRule type="duplicateValues" dxfId="159" priority="167"/>
+    <cfRule type="duplicateValues" dxfId="168" priority="170"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B29">
-    <cfRule type="duplicateValues" dxfId="158" priority="166"/>
-    <cfRule type="duplicateValues" dxfId="157" priority="165"/>
+    <cfRule type="duplicateValues" dxfId="167" priority="169"/>
+    <cfRule type="duplicateValues" dxfId="166" priority="168"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B30">
-    <cfRule type="duplicateValues" dxfId="156" priority="164"/>
+    <cfRule type="duplicateValues" dxfId="165" priority="167"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B31">
-    <cfRule type="duplicateValues" dxfId="155" priority="163"/>
+    <cfRule type="duplicateValues" dxfId="164" priority="166"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B32">
-    <cfRule type="duplicateValues" dxfId="154" priority="162"/>
+    <cfRule type="duplicateValues" dxfId="163" priority="165"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B33">
-    <cfRule type="duplicateValues" dxfId="153" priority="161"/>
+    <cfRule type="duplicateValues" dxfId="162" priority="164"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B34">
-    <cfRule type="duplicateValues" dxfId="152" priority="160"/>
+    <cfRule type="duplicateValues" dxfId="161" priority="163"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B35">
-    <cfRule type="duplicateValues" dxfId="151" priority="159"/>
+    <cfRule type="duplicateValues" dxfId="160" priority="162"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B37">
-    <cfRule type="duplicateValues" dxfId="150" priority="158"/>
+    <cfRule type="duplicateValues" dxfId="159" priority="161"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B38">
-    <cfRule type="duplicateValues" dxfId="149" priority="157"/>
+    <cfRule type="duplicateValues" dxfId="158" priority="160"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B42">
-    <cfRule type="duplicateValues" dxfId="148" priority="156"/>
+    <cfRule type="duplicateValues" dxfId="157" priority="159"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B43">
-    <cfRule type="duplicateValues" dxfId="147" priority="155"/>
+    <cfRule type="duplicateValues" dxfId="156" priority="158"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B44:B45">
-    <cfRule type="duplicateValues" dxfId="146" priority="154"/>
+    <cfRule type="duplicateValues" dxfId="155" priority="157"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B46">
-    <cfRule type="duplicateValues" dxfId="145" priority="153"/>
+    <cfRule type="duplicateValues" dxfId="154" priority="156"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B48">
-    <cfRule type="duplicateValues" dxfId="144" priority="152"/>
+    <cfRule type="duplicateValues" dxfId="153" priority="155"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B49">
-    <cfRule type="duplicateValues" dxfId="143" priority="151"/>
+    <cfRule type="duplicateValues" dxfId="152" priority="154"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B51">
-    <cfRule type="duplicateValues" dxfId="142" priority="150"/>
+    <cfRule type="duplicateValues" dxfId="151" priority="153"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B52">
-    <cfRule type="duplicateValues" dxfId="141" priority="149"/>
+    <cfRule type="duplicateValues" dxfId="150" priority="152"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B58">
-    <cfRule type="duplicateValues" dxfId="140" priority="147"/>
+    <cfRule type="duplicateValues" dxfId="149" priority="150"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B59">
-    <cfRule type="duplicateValues" dxfId="139" priority="145"/>
+    <cfRule type="duplicateValues" dxfId="148" priority="148"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B63">
-    <cfRule type="duplicateValues" dxfId="138" priority="144"/>
+    <cfRule type="duplicateValues" dxfId="147" priority="147"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B64">
-    <cfRule type="duplicateValues" dxfId="137" priority="142"/>
+    <cfRule type="duplicateValues" dxfId="146" priority="145"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B66">
-    <cfRule type="duplicateValues" dxfId="136" priority="141"/>
+    <cfRule type="duplicateValues" dxfId="145" priority="144"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B67">
-    <cfRule type="duplicateValues" dxfId="135" priority="140"/>
-    <cfRule type="duplicateValues" dxfId="134" priority="139"/>
+    <cfRule type="duplicateValues" dxfId="144" priority="143"/>
+    <cfRule type="duplicateValues" dxfId="143" priority="142"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B68">
-    <cfRule type="duplicateValues" dxfId="133" priority="138"/>
+    <cfRule type="duplicateValues" dxfId="142" priority="141"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B69">
-    <cfRule type="duplicateValues" dxfId="132" priority="137"/>
+    <cfRule type="duplicateValues" dxfId="141" priority="140"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B70">
-    <cfRule type="duplicateValues" dxfId="131" priority="135"/>
+    <cfRule type="duplicateValues" dxfId="140" priority="138"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B72">
-    <cfRule type="duplicateValues" dxfId="130" priority="134"/>
+    <cfRule type="duplicateValues" dxfId="139" priority="137"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B73">
-    <cfRule type="duplicateValues" dxfId="129" priority="132"/>
+    <cfRule type="duplicateValues" dxfId="138" priority="135"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B74">
-    <cfRule type="duplicateValues" dxfId="128" priority="131"/>
+    <cfRule type="duplicateValues" dxfId="137" priority="134"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B75">
-    <cfRule type="duplicateValues" dxfId="127" priority="130"/>
+    <cfRule type="duplicateValues" dxfId="136" priority="133"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B76">
-    <cfRule type="duplicateValues" dxfId="126" priority="129"/>
+    <cfRule type="duplicateValues" dxfId="135" priority="132"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B77">
-    <cfRule type="duplicateValues" dxfId="125" priority="127"/>
+    <cfRule type="duplicateValues" dxfId="134" priority="130"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B78">
-    <cfRule type="duplicateValues" dxfId="124" priority="126"/>
+    <cfRule type="duplicateValues" dxfId="133" priority="129"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B83">
-    <cfRule type="duplicateValues" dxfId="123" priority="125"/>
+    <cfRule type="duplicateValues" dxfId="132" priority="128"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B84">
-    <cfRule type="duplicateValues" dxfId="122" priority="124"/>
+    <cfRule type="duplicateValues" dxfId="131" priority="127"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B85">
-    <cfRule type="duplicateValues" dxfId="121" priority="123"/>
+    <cfRule type="duplicateValues" dxfId="130" priority="126"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B87">
-    <cfRule type="duplicateValues" dxfId="120" priority="122"/>
+    <cfRule type="duplicateValues" dxfId="129" priority="125"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B88">
-    <cfRule type="duplicateValues" dxfId="119" priority="121"/>
+    <cfRule type="duplicateValues" dxfId="128" priority="124"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B89">
-    <cfRule type="duplicateValues" dxfId="118" priority="120"/>
+    <cfRule type="duplicateValues" dxfId="127" priority="123"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B90">
-    <cfRule type="duplicateValues" dxfId="117" priority="119"/>
+    <cfRule type="duplicateValues" dxfId="126" priority="122"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B91">
-    <cfRule type="duplicateValues" dxfId="116" priority="118"/>
+    <cfRule type="duplicateValues" dxfId="125" priority="121"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B92">
-    <cfRule type="duplicateValues" dxfId="115" priority="117"/>
+    <cfRule type="duplicateValues" dxfId="124" priority="120"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B93">
-    <cfRule type="duplicateValues" dxfId="114" priority="116"/>
+    <cfRule type="duplicateValues" dxfId="123" priority="119"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B94">
-    <cfRule type="duplicateValues" dxfId="113" priority="115"/>
+    <cfRule type="duplicateValues" dxfId="122" priority="118"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B95">
-    <cfRule type="duplicateValues" dxfId="112" priority="114"/>
+    <cfRule type="duplicateValues" dxfId="121" priority="117"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B96">
-    <cfRule type="duplicateValues" dxfId="111" priority="113"/>
+    <cfRule type="duplicateValues" dxfId="120" priority="116"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B97">
-    <cfRule type="duplicateValues" dxfId="110" priority="112"/>
+    <cfRule type="duplicateValues" dxfId="119" priority="115"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B98">
-    <cfRule type="duplicateValues" dxfId="109" priority="111"/>
+    <cfRule type="duplicateValues" dxfId="118" priority="114"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B99">
-    <cfRule type="duplicateValues" dxfId="108" priority="110"/>
+    <cfRule type="duplicateValues" dxfId="117" priority="113"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B100">
-    <cfRule type="duplicateValues" dxfId="107" priority="109"/>
+    <cfRule type="duplicateValues" dxfId="116" priority="112"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B101">
-    <cfRule type="duplicateValues" dxfId="106" priority="108"/>
+    <cfRule type="duplicateValues" dxfId="115" priority="111"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B104">
-    <cfRule type="duplicateValues" dxfId="105" priority="107"/>
-    <cfRule type="duplicateValues" dxfId="104" priority="106"/>
+    <cfRule type="duplicateValues" dxfId="114" priority="110"/>
+    <cfRule type="duplicateValues" dxfId="113" priority="109"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B105:B106">
-    <cfRule type="duplicateValues" dxfId="103" priority="105"/>
+    <cfRule type="duplicateValues" dxfId="112" priority="108"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B107">
-    <cfRule type="duplicateValues" dxfId="102" priority="104"/>
+    <cfRule type="duplicateValues" dxfId="111" priority="107"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B108">
-    <cfRule type="duplicateValues" dxfId="101" priority="103"/>
+    <cfRule type="duplicateValues" dxfId="110" priority="106"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B109">
-    <cfRule type="duplicateValues" dxfId="100" priority="102"/>
+    <cfRule type="duplicateValues" dxfId="109" priority="105"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B110">
-    <cfRule type="duplicateValues" dxfId="99" priority="101"/>
+    <cfRule type="duplicateValues" dxfId="108" priority="104"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B111">
-    <cfRule type="duplicateValues" dxfId="98" priority="100"/>
+    <cfRule type="duplicateValues" dxfId="107" priority="103"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B112">
-    <cfRule type="duplicateValues" dxfId="97" priority="99"/>
+    <cfRule type="duplicateValues" dxfId="106" priority="102"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B113">
-    <cfRule type="duplicateValues" dxfId="96" priority="98"/>
+    <cfRule type="duplicateValues" dxfId="105" priority="101"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B114">
-    <cfRule type="duplicateValues" dxfId="95" priority="97"/>
+    <cfRule type="duplicateValues" dxfId="104" priority="100"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B115">
-    <cfRule type="duplicateValues" dxfId="94" priority="96"/>
+    <cfRule type="duplicateValues" dxfId="103" priority="99"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B116">
-    <cfRule type="duplicateValues" dxfId="93" priority="95"/>
+    <cfRule type="duplicateValues" dxfId="102" priority="98"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B117">
-    <cfRule type="duplicateValues" dxfId="92" priority="94"/>
+    <cfRule type="duplicateValues" dxfId="101" priority="97"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B118">
-    <cfRule type="duplicateValues" dxfId="91" priority="93"/>
+    <cfRule type="duplicateValues" dxfId="100" priority="96"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B119">
-    <cfRule type="duplicateValues" dxfId="90" priority="92"/>
+    <cfRule type="duplicateValues" dxfId="99" priority="95"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B120">
-    <cfRule type="duplicateValues" dxfId="89" priority="91"/>
+    <cfRule type="duplicateValues" dxfId="98" priority="94"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B121">
-    <cfRule type="duplicateValues" dxfId="88" priority="90"/>
+    <cfRule type="duplicateValues" dxfId="97" priority="93"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B122">
-    <cfRule type="duplicateValues" dxfId="87" priority="89"/>
+    <cfRule type="duplicateValues" dxfId="96" priority="92"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B126">
-    <cfRule type="duplicateValues" dxfId="86" priority="88"/>
+    <cfRule type="duplicateValues" dxfId="95" priority="91"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B127">
-    <cfRule type="duplicateValues" dxfId="85" priority="87"/>
+    <cfRule type="duplicateValues" dxfId="94" priority="90"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B128">
-    <cfRule type="duplicateValues" dxfId="84" priority="86"/>
+    <cfRule type="duplicateValues" dxfId="93" priority="89"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B129">
-    <cfRule type="duplicateValues" dxfId="83" priority="85"/>
+    <cfRule type="duplicateValues" dxfId="92" priority="88"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B130">
-    <cfRule type="duplicateValues" dxfId="82" priority="84"/>
+    <cfRule type="duplicateValues" dxfId="91" priority="87"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B131">
-    <cfRule type="duplicateValues" dxfId="81" priority="83"/>
+    <cfRule type="duplicateValues" dxfId="90" priority="86"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B132">
-    <cfRule type="duplicateValues" dxfId="80" priority="82"/>
+    <cfRule type="duplicateValues" dxfId="89" priority="85"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B133">
-    <cfRule type="duplicateValues" dxfId="79" priority="81"/>
+    <cfRule type="duplicateValues" dxfId="88" priority="84"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B136">
-    <cfRule type="duplicateValues" dxfId="78" priority="80"/>
+    <cfRule type="duplicateValues" dxfId="87" priority="83"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B137">
-    <cfRule type="duplicateValues" dxfId="77" priority="79"/>
+    <cfRule type="duplicateValues" dxfId="86" priority="82"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B138">
-    <cfRule type="duplicateValues" dxfId="76" priority="78"/>
+    <cfRule type="duplicateValues" dxfId="85" priority="81"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B139">
-    <cfRule type="duplicateValues" dxfId="75" priority="77"/>
+    <cfRule type="duplicateValues" dxfId="84" priority="80"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B140">
-    <cfRule type="duplicateValues" dxfId="74" priority="76"/>
+    <cfRule type="duplicateValues" dxfId="83" priority="79"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B141">
-    <cfRule type="duplicateValues" dxfId="73" priority="75"/>
+    <cfRule type="duplicateValues" dxfId="82" priority="78"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B142">
-    <cfRule type="duplicateValues" dxfId="72" priority="74"/>
+    <cfRule type="duplicateValues" dxfId="81" priority="77"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B143">
-    <cfRule type="duplicateValues" dxfId="71" priority="73"/>
+    <cfRule type="duplicateValues" dxfId="80" priority="76"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B144">
-    <cfRule type="duplicateValues" dxfId="70" priority="72"/>
+    <cfRule type="duplicateValues" dxfId="79" priority="75"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B145">
-    <cfRule type="duplicateValues" dxfId="69" priority="71"/>
+    <cfRule type="duplicateValues" dxfId="78" priority="74"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B147">
-    <cfRule type="duplicateValues" dxfId="68" priority="70"/>
+    <cfRule type="duplicateValues" dxfId="77" priority="73"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B148">
-    <cfRule type="duplicateValues" dxfId="67" priority="69"/>
+    <cfRule type="duplicateValues" dxfId="76" priority="72"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B149">
-    <cfRule type="duplicateValues" dxfId="66" priority="68"/>
+    <cfRule type="duplicateValues" dxfId="75" priority="71"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B150">
-    <cfRule type="duplicateValues" dxfId="65" priority="67"/>
+    <cfRule type="duplicateValues" dxfId="74" priority="70"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B151">
-    <cfRule type="duplicateValues" dxfId="64" priority="66"/>
+    <cfRule type="duplicateValues" dxfId="73" priority="69"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B152">
-    <cfRule type="duplicateValues" dxfId="63" priority="65"/>
+    <cfRule type="duplicateValues" dxfId="72" priority="68"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B153">
-    <cfRule type="duplicateValues" dxfId="62" priority="64"/>
+    <cfRule type="duplicateValues" dxfId="71" priority="67"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B154">
-    <cfRule type="duplicateValues" dxfId="61" priority="63"/>
+    <cfRule type="duplicateValues" dxfId="70" priority="66"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B155">
-    <cfRule type="duplicateValues" dxfId="60" priority="62"/>
+    <cfRule type="duplicateValues" dxfId="69" priority="65"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B156">
-    <cfRule type="duplicateValues" dxfId="59" priority="61"/>
+    <cfRule type="duplicateValues" dxfId="68" priority="64"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B157">
-    <cfRule type="duplicateValues" dxfId="58" priority="60"/>
+    <cfRule type="duplicateValues" dxfId="67" priority="63"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B171">
-    <cfRule type="duplicateValues" dxfId="57" priority="59"/>
+    <cfRule type="duplicateValues" dxfId="66" priority="62"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B172">
-    <cfRule type="duplicateValues" dxfId="56" priority="58"/>
+    <cfRule type="duplicateValues" dxfId="65" priority="61"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B174">
-    <cfRule type="duplicateValues" dxfId="55" priority="57"/>
+    <cfRule type="duplicateValues" dxfId="64" priority="60"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B177:B178">
-    <cfRule type="duplicateValues" dxfId="54" priority="56"/>
+    <cfRule type="duplicateValues" dxfId="63" priority="59"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B181">
-    <cfRule type="duplicateValues" dxfId="53" priority="55"/>
+    <cfRule type="duplicateValues" dxfId="62" priority="58"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B182">
-    <cfRule type="duplicateValues" dxfId="52" priority="54"/>
+    <cfRule type="duplicateValues" dxfId="61" priority="57"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B183">
-    <cfRule type="duplicateValues" dxfId="51" priority="53"/>
+    <cfRule type="duplicateValues" dxfId="60" priority="56"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B184">
-    <cfRule type="duplicateValues" dxfId="50" priority="52"/>
+    <cfRule type="duplicateValues" dxfId="59" priority="55"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B185">
-    <cfRule type="duplicateValues" dxfId="49" priority="51"/>
+    <cfRule type="duplicateValues" dxfId="58" priority="54"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B186">
-    <cfRule type="duplicateValues" dxfId="48" priority="50"/>
+    <cfRule type="duplicateValues" dxfId="57" priority="53"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B188">
-    <cfRule type="duplicateValues" dxfId="47" priority="49"/>
+    <cfRule type="duplicateValues" dxfId="56" priority="52"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B189">
-    <cfRule type="duplicateValues" dxfId="46" priority="48"/>
+    <cfRule type="duplicateValues" dxfId="55" priority="51"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B190">
-    <cfRule type="duplicateValues" dxfId="45" priority="47"/>
+    <cfRule type="duplicateValues" dxfId="54" priority="50"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B191">
-    <cfRule type="duplicateValues" dxfId="44" priority="46"/>
+    <cfRule type="duplicateValues" dxfId="53" priority="49"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B192">
-    <cfRule type="duplicateValues" dxfId="43" priority="45"/>
+    <cfRule type="duplicateValues" dxfId="52" priority="48"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B193">
-    <cfRule type="duplicateValues" dxfId="42" priority="44"/>
+    <cfRule type="duplicateValues" dxfId="51" priority="47"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B195">
-    <cfRule type="duplicateValues" dxfId="41" priority="43"/>
+    <cfRule type="duplicateValues" dxfId="50" priority="46"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B196">
-    <cfRule type="duplicateValues" dxfId="40" priority="42"/>
+    <cfRule type="duplicateValues" dxfId="49" priority="45"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B197">
-    <cfRule type="duplicateValues" dxfId="39" priority="41"/>
+    <cfRule type="duplicateValues" dxfId="48" priority="44"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B198">
-    <cfRule type="duplicateValues" dxfId="38" priority="40"/>
+    <cfRule type="duplicateValues" dxfId="47" priority="43"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B199">
-    <cfRule type="duplicateValues" dxfId="37" priority="39"/>
+    <cfRule type="duplicateValues" dxfId="46" priority="42"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B200">
-    <cfRule type="duplicateValues" dxfId="36" priority="38"/>
+    <cfRule type="duplicateValues" dxfId="45" priority="41"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B201">
-    <cfRule type="duplicateValues" dxfId="35" priority="37"/>
+    <cfRule type="duplicateValues" dxfId="44" priority="40"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B202">
-    <cfRule type="duplicateValues" dxfId="34" priority="36"/>
+    <cfRule type="duplicateValues" dxfId="43" priority="39"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B203">
-    <cfRule type="duplicateValues" dxfId="33" priority="35"/>
+    <cfRule type="duplicateValues" dxfId="42" priority="38"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B204">
-    <cfRule type="duplicateValues" dxfId="32" priority="34"/>
+    <cfRule type="duplicateValues" dxfId="41" priority="37"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B205">
-    <cfRule type="duplicateValues" dxfId="31" priority="33"/>
+    <cfRule type="duplicateValues" dxfId="40" priority="36"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B206">
-    <cfRule type="duplicateValues" dxfId="30" priority="32"/>
+    <cfRule type="duplicateValues" dxfId="39" priority="35"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B207">
-    <cfRule type="duplicateValues" dxfId="29" priority="31"/>
+    <cfRule type="duplicateValues" dxfId="38" priority="34"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B215">
-    <cfRule type="duplicateValues" dxfId="28" priority="30"/>
+    <cfRule type="duplicateValues" dxfId="37" priority="33"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B218">
-    <cfRule type="duplicateValues" dxfId="27" priority="29"/>
+    <cfRule type="duplicateValues" dxfId="36" priority="32"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B220">
-    <cfRule type="duplicateValues" dxfId="26" priority="28"/>
+    <cfRule type="duplicateValues" dxfId="35" priority="31"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B222">
-    <cfRule type="duplicateValues" dxfId="25" priority="27"/>
+    <cfRule type="duplicateValues" dxfId="34" priority="30"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B223">
-    <cfRule type="duplicateValues" dxfId="24" priority="26"/>
+    <cfRule type="duplicateValues" dxfId="33" priority="29"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B224">
-    <cfRule type="duplicateValues" dxfId="23" priority="25"/>
+    <cfRule type="duplicateValues" dxfId="32" priority="28"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B225">
-    <cfRule type="duplicateValues" dxfId="22" priority="24"/>
+    <cfRule type="duplicateValues" dxfId="31" priority="27"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B227">
-    <cfRule type="duplicateValues" dxfId="21" priority="23"/>
+    <cfRule type="duplicateValues" dxfId="30" priority="26"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B229">
-    <cfRule type="duplicateValues" dxfId="20" priority="22"/>
+    <cfRule type="duplicateValues" dxfId="29" priority="25"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B230">
-    <cfRule type="duplicateValues" dxfId="19" priority="21"/>
+    <cfRule type="duplicateValues" dxfId="28" priority="24"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B232">
-    <cfRule type="duplicateValues" dxfId="18" priority="20"/>
+    <cfRule type="duplicateValues" dxfId="27" priority="23"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B233">
-    <cfRule type="duplicateValues" dxfId="17" priority="19"/>
+    <cfRule type="duplicateValues" dxfId="26" priority="22"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B234">
-    <cfRule type="duplicateValues" dxfId="16" priority="18"/>
+    <cfRule type="duplicateValues" dxfId="25" priority="21"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B235">
-    <cfRule type="duplicateValues" dxfId="15" priority="17"/>
+    <cfRule type="duplicateValues" dxfId="24" priority="20"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B236">
-    <cfRule type="duplicateValues" dxfId="14" priority="16"/>
+    <cfRule type="duplicateValues" dxfId="23" priority="19"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B237">
-    <cfRule type="duplicateValues" dxfId="13" priority="15"/>
+    <cfRule type="duplicateValues" dxfId="22" priority="18"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B239">
-    <cfRule type="duplicateValues" dxfId="12" priority="13"/>
+    <cfRule type="duplicateValues" dxfId="21" priority="16"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B240">
-    <cfRule type="duplicateValues" dxfId="11" priority="12"/>
+    <cfRule type="duplicateValues" dxfId="20" priority="15"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B241">
-    <cfRule type="duplicateValues" dxfId="10" priority="11"/>
+    <cfRule type="duplicateValues" dxfId="19" priority="14"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B242">
-    <cfRule type="duplicateValues" dxfId="9" priority="10"/>
+    <cfRule type="duplicateValues" dxfId="18" priority="13"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B243">
-    <cfRule type="duplicateValues" dxfId="8" priority="9"/>
+    <cfRule type="duplicateValues" dxfId="17" priority="12"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B250">
-    <cfRule type="duplicateValues" dxfId="7" priority="8"/>
+    <cfRule type="duplicateValues" dxfId="16" priority="11"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B251">
-    <cfRule type="duplicateValues" dxfId="6" priority="7"/>
+    <cfRule type="duplicateValues" dxfId="15" priority="10"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B253">
-    <cfRule type="duplicateValues" dxfId="5" priority="6"/>
+    <cfRule type="duplicateValues" dxfId="14" priority="9"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B255">
-    <cfRule type="duplicateValues" dxfId="4" priority="5"/>
+    <cfRule type="duplicateValues" dxfId="13" priority="8"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B258:B259">
-    <cfRule type="duplicateValues" dxfId="3" priority="4"/>
+    <cfRule type="duplicateValues" dxfId="12" priority="7"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B260">
-    <cfRule type="duplicateValues" dxfId="2" priority="3"/>
+    <cfRule type="duplicateValues" dxfId="11" priority="6"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B265:B267 B269">
-    <cfRule type="duplicateValues" dxfId="1" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="10" priority="5"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B268">
-    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="9" priority="4"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B270">
+    <cfRule type="duplicateValues" dxfId="8" priority="3"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B271">
+    <cfRule type="duplicateValues" dxfId="7" priority="2"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B273">
+    <cfRule type="duplicateValues" dxfId="6" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -52165,11 +53163,11 @@
       </c>
       <c r="B1" s="15">
         <f>COUNTA(sum!A:A) -1</f>
-        <v>253</v>
+        <v>267</v>
       </c>
       <c r="C1" s="22">
         <f>COUNTIF(sum!I:I, "completed")/(B1-COUNTIF(sum!I:I, "abandoned")-COUNTIF(sum!I:I, "late app"))</f>
-        <v>0.99593495934959353</v>
+        <v>0.94230769230769229</v>
       </c>
       <c r="D1" s="21">
         <f>COUNTIF(sum!I:I, "completed")</f>
@@ -52195,11 +53193,11 @@
       </c>
       <c r="B3" s="16">
         <f>COUNTA(sum!K:K) -1</f>
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C3" s="10">
         <f>COUNTIFS(sum!I:I,"completed", sum!K:K, "&lt;&gt;") / B3</f>
-        <v>0.98245614035087714</v>
+        <v>0.98305084745762716</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="26" x14ac:dyDescent="0.6">
@@ -52208,7 +53206,7 @@
       </c>
       <c r="B5" s="15">
         <f>COUNTA(sum!J:J) -1</f>
-        <v>253</v>
+        <v>267</v>
       </c>
       <c r="C5" s="14">
         <f>B5/B1</f>
@@ -52221,11 +53219,11 @@
       </c>
       <c r="B6" s="16">
         <f>COUNTIFS(sum!J:J,"no news")</f>
-        <v>244</v>
+        <v>255</v>
       </c>
       <c r="C6" s="10">
         <f>B6/$B$5</f>
-        <v>0.96442687747035571</v>
+        <v>0.9550561797752809</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.4">
@@ -52234,11 +53232,11 @@
       </c>
       <c r="B7" s="16">
         <f>COUNTIFS(sum!J:J,"rejected")</f>
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="C7" s="10">
         <f t="shared" ref="C7:C10" si="0">B7/$B$5</f>
-        <v>3.1620553359683792E-2</v>
+        <v>4.1198501872659173E-2</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.4">
@@ -52251,7 +53249,7 @@
       </c>
       <c r="C8" s="10">
         <f t="shared" si="0"/>
-        <v>3.952569169960474E-3</v>
+        <v>3.7453183520599251E-3</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.4">

</xml_diff>

<commit_message>
after flyout! some apps
</commit_message>
<xml_diff>
--- a/EconJM_status.xlsx
+++ b/EconJM_status.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\javie\Dropbox\Work\Job Search\2025 EconJM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE209D34-6373-4EA0-B5DA-E4851DEED772}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2472ACC8-6AF5-40ED-BCEE-1A327BB2778B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="14620" activeTab="1" xr2:uid="{6FE48536-7E5C-BF4C-9490-2A6392576298}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="14620" xr2:uid="{6FE48536-7E5C-BF4C-9490-2A6392576298}"/>
   </bookViews>
   <sheets>
     <sheet name="sum" sheetId="1" r:id="rId1"/>
@@ -18,7 +18,7 @@
     <sheet name="stats" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">sum!$A$1:$V$248</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">sum!$A$1:$V$267</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -45,7 +45,7 @@
   <metadataTypes count="1">
     <metadataType name="XLRICHVALUE" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1"/>
   </metadataTypes>
-  <futureMetadata name="XLRICHVALUE" count="103">
+  <futureMetadata name="XLRICHVALUE" count="104">
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
@@ -767,8 +767,15 @@
         </ext>
       </extLst>
     </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="3219"/>
+        </ext>
+      </extLst>
+    </bk>
   </futureMetadata>
-  <valueMetadata count="103">
+  <valueMetadata count="104">
     <bk>
       <rc t="1" v="0"/>
     </bk>
@@ -1078,12 +1085,15 @@
     <bk>
       <rc t="1" v="102"/>
     </bk>
+    <bk>
+      <rc t="1" v="103"/>
+    </bk>
   </valueMetadata>
 </metadata>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2675" uniqueCount="853">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2767" uniqueCount="872">
   <si>
     <t>add_id</t>
   </si>
@@ -3548,12 +3558,6 @@
     <t>HEC Paris</t>
   </si>
   <si>
-    <t>monash_post_2</t>
-  </si>
-  <si>
-    <t>Ricardo Dahis, the Primary Investigator (PI)</t>
-  </si>
-  <si>
     <t>virginia_common</t>
   </si>
   <si>
@@ -3626,9 +3630,6 @@
     <t>Florida International University</t>
   </si>
   <si>
-    <t>https://pslinks.fiu.edu/psc/jobs/CUSTOMER/HRMS/c/HRS_HRAM_FL.HRS_CG_SEARCH_FL.GBL?Page=HRS_APP_SCHJOB_FL&amp;Action=U</t>
-  </si>
-  <si>
     <t>Job Opening ID 536413</t>
   </si>
   <si>
@@ -3678,6 +3679,72 @@
   </si>
   <si>
     <t>added a few more stragelers</t>
+  </si>
+  <si>
+    <t>sloan</t>
+  </si>
+  <si>
+    <t>https://sloan.org/about/careers</t>
+  </si>
+  <si>
+    <t>Alfred P. Sloan Foundation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cover letter and resume/CV via email to HR@sloan.org with “LAST NAME – Program Associate, Economics” </t>
+  </si>
+  <si>
+    <t>urbana_champ_post</t>
+  </si>
+  <si>
+    <t>https://illinois.csod.com/ux/ats/careersite/1/home/requisition/15669?c=illinois</t>
+  </si>
+  <si>
+    <t>st_andrews</t>
+  </si>
+  <si>
+    <t>https://www.vacancies.st-andrews.ac.uk/Vacancies/W/4445/0/461020/889/senior-lecturer-or-reader-in-economics-microeconomics-ac2400</t>
+  </si>
+  <si>
+    <t>University of St Andrews</t>
+  </si>
+  <si>
+    <t>Professor Conny Wollbrant, Head of Department (conny.wollbrant@st-andrews.ac.uk) or Professor Mark Brewer, Dean of the Business School (BSchoolDean@st-andrews.ac.uk).</t>
+  </si>
+  <si>
+    <t>namur</t>
+  </si>
+  <si>
+    <t>University of Namur</t>
+  </si>
+  <si>
+    <t>app form (https://www.unamur.be/en/university/work/forms)</t>
+  </si>
+  <si>
+    <t>https://jobs.unamur.be/emploi.2025-12-02.1636013715</t>
+  </si>
+  <si>
+    <t>coppen_post2</t>
+  </si>
+  <si>
+    <t>https://candidate.hr-manager.net/ApplicationForm/SinglePageApplicationForm.aspx?cid=3010&amp;departmentId=19853&amp;ProjectId=152721&amp;MediaId=5105</t>
+  </si>
+  <si>
+    <t>zurich_dev</t>
+  </si>
+  <si>
+    <t>kyev</t>
+  </si>
+  <si>
+    <t>Kyiv School of Economics</t>
+  </si>
+  <si>
+    <t>san_andres</t>
+  </si>
+  <si>
+    <t>Universidad de San Andrés</t>
+  </si>
+  <si>
+    <t>https://careers.fiu.edu/</t>
   </si>
 </sst>
 </file>
@@ -3859,24 +3926,14 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Percent" xfId="2" builtinId="5"/>
   </cellStyles>
-  <dxfs count="208">
+  <dxfs count="214">
     <dxf>
       <font>
-        <color rgb="FF006100"/>
+        <color rgb="FF9C0006"/>
       </font>
       <fill>
         <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
+          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -3892,21 +3949,91 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF006100"/>
+        <color rgb="FF9C0006"/>
       </font>
       <fill>
         <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
+          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF006100"/>
+        <color rgb="FF9C0006"/>
       </font>
       <fill>
         <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -6512,11 +6639,15 @@
     <address r:id="rId203"/>
     <moreImagesAddress r:id="rId204"/>
   </webImageSrd>
+  <webImageSrd>
+    <address r:id="rId205"/>
+    <moreImagesAddress r:id="rId206"/>
+  </webImageSrd>
 </webImagesSrd>
 </file>
 
 <file path=xl/richData/rdarray.xml><?xml version="1.0" encoding="utf-8"?>
-<arrayData xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" count="192">
+<arrayData xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" count="196">
   <a r="1">
     <v t="r">6</v>
   </a>
@@ -7964,11 +8095,51 @@
   <a r="1">
     <v t="r">3213</v>
   </a>
+  <a r="3">
+    <v t="r">3239</v>
+    <v t="r">3240</v>
+    <v t="r">3241</v>
+  </a>
+  <a r="1">
+    <v t="s">Ukrainian language</v>
+  </a>
+  <a r="27">
+    <v t="r">3225</v>
+    <v t="r">3253</v>
+    <v t="r">3254</v>
+    <v t="r">3255</v>
+    <v t="r">3256</v>
+    <v t="r">3257</v>
+    <v t="r">3258</v>
+    <v t="r">3259</v>
+    <v t="r">3260</v>
+    <v t="r">3261</v>
+    <v t="r">3262</v>
+    <v t="r">3263</v>
+    <v t="r">3264</v>
+    <v t="r">3265</v>
+    <v t="r">3266</v>
+    <v t="r">3267</v>
+    <v t="r">3268</v>
+    <v t="r">3269</v>
+    <v t="r">3270</v>
+    <v t="r">3271</v>
+    <v t="r">3272</v>
+    <v t="r">3273</v>
+    <v t="r">3274</v>
+    <v t="r">3275</v>
+    <v t="r">3276</v>
+    <v t="r">3277</v>
+    <v t="r">2725</v>
+  </a>
+  <a r="1">
+    <v t="s">Eastern European Time</v>
+  </a>
 </arrayData>
 </file>
 
 <file path=xl/richData/rdrichvalue.xml><?xml version="1.0" encoding="utf-8"?>
-<rvData xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="3219">
+<rvData xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="3285">
   <rv s="0">
     <v>536870912</v>
     <v>New York City</v>
@@ -28762,6 +28933,423 @@
     <v>11</v>
     <v>Baltimore</v>
     <v>mdp/vdpid/5490064267963006978</v>
+  </rv>
+  <rv s="0">
+    <v>536870912</v>
+    <v>Ukraine</v>
+    <v>ad599477-9e6d-4a0e-bab5-0edf9db7115a</v>
+    <v>en-US</v>
+    <v>Map</v>
+  </rv>
+  <rv s="1">
+    <fb>0.71665314436637995</fb>
+    <v>19</v>
+  </rv>
+  <rv s="1">
+    <fb>603550</fb>
+    <v>8</v>
+  </rv>
+  <rv s="1">
+    <fb>297000</fb>
+    <v>8</v>
+  </rv>
+  <rv s="1">
+    <fb>8.6999999999999993</fb>
+    <v>18</v>
+  </rv>
+  <rv s="1">
+    <fb>380</fb>
+    <v>39</v>
+  </rv>
+  <rv s="0">
+    <v>536870912</v>
+    <v>Kyiv</v>
+    <v>79c78723-042d-4572-bc87-599fa1203134</v>
+    <v>en-US</v>
+    <v>Map</v>
+  </rv>
+  <rv s="1">
+    <fb>202249.71799999999</fb>
+    <v>8</v>
+  </rv>
+  <rv s="1">
+    <fb>281.658595641646</fb>
+    <v>40</v>
+  </rv>
+  <rv s="1">
+    <fb>7.8867174561113002E-2</fb>
+    <v>19</v>
+  </rv>
+  <rv s="1">
+    <fb>3418.56924154441</fb>
+    <v>8</v>
+  </rv>
+  <rv s="1">
+    <fb>1.3009999999999999</fb>
+    <v>18</v>
+  </rv>
+  <rv s="1">
+    <fb>0.167080388142165</fb>
+    <v>19</v>
+  </rv>
+  <rv s="1">
+    <fb>75.3495057807649</fb>
+    <v>41</v>
+  </rv>
+  <rv s="1">
+    <fb>0.83</fb>
+    <v>42</v>
+  </rv>
+  <rv s="1">
+    <fb>153781069118.14801</fb>
+    <v>17</v>
+  </rv>
+  <rv s="1">
+    <fb>0.99040940000000011</fb>
+    <v>19</v>
+  </rv>
+  <rv s="1">
+    <fb>0.82671180000000011</fb>
+    <v>19</v>
+  </rv>
+  <rv s="2">
+    <v>102</v>
+    <v>6</v>
+    <v>470</v>
+    <v>7</v>
+    <v>0</v>
+    <v>Image of Ukraine</v>
+  </rv>
+  <rv s="1">
+    <fb>7.5</fb>
+    <v>41</v>
+  </rv>
+  <rv s="0">
+    <v>805306368</v>
+    <v>Volodymyr Zelenskyy (President)</v>
+    <v>9bae3411-f7b7-35a0-00a8-57f94c361da9</v>
+    <v>en-US</v>
+    <v>Generic</v>
+  </rv>
+  <rv s="0">
+    <v>805306368</v>
+    <v>Denys Shmyhal (Prime minister)</v>
+    <v>be5cbc70-24e7-afe9-a0b1-49d91b73bd1a</v>
+    <v>en-US</v>
+    <v>Generic</v>
+  </rv>
+  <rv s="0">
+    <v>805306368</v>
+    <v>Ruslan Stefanchuk (Chairman)</v>
+    <v>f285b81d-480f-2679-16cf-096a649d7b5e</v>
+    <v>en-US</v>
+    <v>Generic</v>
+  </rv>
+  <rv s="3">
+    <v>192</v>
+  </rv>
+  <rv s="4">
+    <v>https://www.bing.com/search?q=ukraine&amp;form=skydnc</v>
+    <v>Learn more on Bing</v>
+  </rv>
+  <rv s="1">
+    <fb>71.582682926829307</fb>
+    <v>41</v>
+  </rv>
+  <rv s="1">
+    <fb>4415440000</fb>
+    <v>17</v>
+  </rv>
+  <rv s="1">
+    <fb>0.84</fb>
+    <v>42</v>
+  </rv>
+  <rv s="3">
+    <v>193</v>
+  </rv>
+  <rv s="1">
+    <fb>0.47811215909999999</fb>
+    <v>19</v>
+  </rv>
+  <rv s="1">
+    <fb>2.9923000000000002</fb>
+    <v>18</v>
+  </rv>
+  <rv s="1">
+    <fb>38000000</fb>
+    <v>8</v>
+  </rv>
+  <rv s="1">
+    <fb>0.36099999999999999</fb>
+    <v>19</v>
+  </rv>
+  <rv s="1">
+    <fb>0.54151000976562502</fb>
+    <v>19</v>
+  </rv>
+  <rv s="0">
+    <v>536870912</v>
+    <v>Cherkasy Oblast</v>
+    <v>c9976b82-1310-ef4d-b0c9-a9afe6a1007f</v>
+    <v>en-US</v>
+    <v>Map</v>
+  </rv>
+  <rv s="0">
+    <v>536870912</v>
+    <v>Chernihiv Oblast</v>
+    <v>4d3c108d-9f83-97bb-6c45-e5206908c9ba</v>
+    <v>en-US</v>
+    <v>Map</v>
+  </rv>
+  <rv s="0">
+    <v>536870912</v>
+    <v>Chernivtsi Oblast</v>
+    <v>2b816ee4-0e8d-8ada-257c-6b9b23a72ad0</v>
+    <v>en-US</v>
+    <v>Map</v>
+  </rv>
+  <rv s="0">
+    <v>536870912</v>
+    <v>Dnipropetrovsk Oblast</v>
+    <v>83b98499-16b8-bb03-d593-dd4bdf6eca84</v>
+    <v>en-US</v>
+    <v>Map</v>
+  </rv>
+  <rv s="0">
+    <v>536870912</v>
+    <v>Donetsk Oblast</v>
+    <v>66af6664-7bd4-318e-e6c4-a5eba1b797fa</v>
+    <v>en-US</v>
+    <v>Map</v>
+  </rv>
+  <rv s="0">
+    <v>536870912</v>
+    <v>Ivano-Frankivsk Oblast</v>
+    <v>5ab8bbed-4d8c-3a6e-ce49-db79ef72183f</v>
+    <v>en-US</v>
+    <v>Map</v>
+  </rv>
+  <rv s="0">
+    <v>536870912</v>
+    <v>Kharkiv Oblast</v>
+    <v>80a0fd15-8a6f-05e0-ef8e-3ac5b137b76c</v>
+    <v>en-US</v>
+    <v>Map</v>
+  </rv>
+  <rv s="0">
+    <v>536870912</v>
+    <v>Kherson Oblast</v>
+    <v>3d03caa9-910c-b257-2449-cb94ef57e497</v>
+    <v>en-US</v>
+    <v>Map</v>
+  </rv>
+  <rv s="0">
+    <v>536870912</v>
+    <v>Khmelnytskyi Oblast</v>
+    <v>d8d2d1e1-25b5-cc8e-95a9-dd2af8f5b7a7</v>
+    <v>en-US</v>
+    <v>Map</v>
+  </rv>
+  <rv s="0">
+    <v>536870912</v>
+    <v>Kyiv Oblast</v>
+    <v>4c971681-9dca-2885-9bc5-18f1d3b975b1</v>
+    <v>en-US</v>
+    <v>Map</v>
+  </rv>
+  <rv s="0">
+    <v>536870912</v>
+    <v>Kirovohrad Oblast</v>
+    <v>ef8d4608-76c2-a832-264e-4cf51a0c5dbd</v>
+    <v>en-US</v>
+    <v>Map</v>
+  </rv>
+  <rv s="0">
+    <v>536870912</v>
+    <v>Luhansk Oblast</v>
+    <v>cccfd56b-f7a9-dd2a-d268-68084adf28b4</v>
+    <v>en-US</v>
+    <v>Map</v>
+  </rv>
+  <rv s="0">
+    <v>536870912</v>
+    <v>Lviv Oblast</v>
+    <v>aa5637b1-7fe1-a3c0-42df-6616eb84675a</v>
+    <v>en-US</v>
+    <v>Map</v>
+  </rv>
+  <rv s="0">
+    <v>536870912</v>
+    <v>Mykolaiv Oblast</v>
+    <v>11f87280-610e-7272-da94-5f8890fcf23d</v>
+    <v>en-US</v>
+    <v>Map</v>
+  </rv>
+  <rv s="0">
+    <v>536870912</v>
+    <v>Odesa Oblast</v>
+    <v>ab1bf172-10d2-6650-704b-07f524561e0c</v>
+    <v>en-US</v>
+    <v>Map</v>
+  </rv>
+  <rv s="0">
+    <v>536870912</v>
+    <v>Poltava Oblast</v>
+    <v>e5ca22a5-cbe2-e9f8-df2a-c271030dccc7</v>
+    <v>en-US</v>
+    <v>Map</v>
+  </rv>
+  <rv s="0">
+    <v>536870912</v>
+    <v>Rivne Oblast</v>
+    <v>d6cdb68d-5af6-afd9-b456-affff06b0df7</v>
+    <v>en-US</v>
+    <v>Map</v>
+  </rv>
+  <rv s="0">
+    <v>536870912</v>
+    <v>Sumy Oblast</v>
+    <v>f7532844-70f6-fa1d-38eb-23fd0dbcb818</v>
+    <v>en-US</v>
+    <v>Map</v>
+  </rv>
+  <rv s="0">
+    <v>536870912</v>
+    <v>Ternopil Oblast</v>
+    <v>8546d368-622f-6499-3510-030c076e5f17</v>
+    <v>en-US</v>
+    <v>Map</v>
+  </rv>
+  <rv s="0">
+    <v>536870912</v>
+    <v>Vinnytsia Oblast</v>
+    <v>f740bcec-499b-0dee-db2b-31a5e212bb43</v>
+    <v>en-US</v>
+    <v>Map</v>
+  </rv>
+  <rv s="0">
+    <v>536870912</v>
+    <v>Volyn Oblast</v>
+    <v>0e1b7fc3-81cf-e44d-b558-4f6a739d4ab5</v>
+    <v>en-US</v>
+    <v>Map</v>
+  </rv>
+  <rv s="0">
+    <v>536870912</v>
+    <v>Zakarpattia Oblast</v>
+    <v>2b40bf9f-f59e-2eda-4e2c-ab42a853d304</v>
+    <v>en-US</v>
+    <v>Map</v>
+  </rv>
+  <rv s="0">
+    <v>536870912</v>
+    <v>Zaporizhzhia Oblast</v>
+    <v>cfdae36e-e003-7dea-83b3-d9f416b99469</v>
+    <v>en-US</v>
+    <v>Map</v>
+  </rv>
+  <rv s="0">
+    <v>536870912</v>
+    <v>Zhytomyr Oblast</v>
+    <v>8a86953e-fa05-4b29-ba68-763eb4012703</v>
+    <v>en-US</v>
+    <v>Map</v>
+  </rv>
+  <rv s="0">
+    <v>536870912</v>
+    <v>Autonomous Republic of Crimea</v>
+    <v>79c3dba3-7806-419d-9763-6a5bc8e8e810</v>
+    <v>en-US</v>
+    <v>Map</v>
+  </rv>
+  <rv s="3">
+    <v>194</v>
+  </rv>
+  <rv s="1">
+    <fb>0.201408893342575</fb>
+    <v>19</v>
+  </rv>
+  <rv s="3">
+    <v>195</v>
+  </rv>
+  <rv s="1">
+    <fb>0.45200000000000001</fb>
+    <v>19</v>
+  </rv>
+  <rv s="1">
+    <fb>8.8819999694824195E-2</fb>
+    <v>43</v>
+  </rv>
+  <rv s="1">
+    <fb>30835699</fb>
+    <v>8</v>
+  </rv>
+  <rv s="7">
+    <v>#VALUE!</v>
+    <v>en-US</v>
+    <v>ad599477-9e6d-4a0e-bab5-0edf9db7115a</v>
+    <v>536870912</v>
+    <v>1</v>
+    <v>473</v>
+    <v>37</v>
+    <v>Ukraine</v>
+    <v>4</v>
+    <v>5</v>
+    <v>Map</v>
+    <v>6</v>
+    <v>474</v>
+    <v>UA</v>
+    <v>3220</v>
+    <v>3221</v>
+    <v>3222</v>
+    <v>3223</v>
+    <v>3224</v>
+    <v>3225</v>
+    <v>3226</v>
+    <v>3227</v>
+    <v>3228</v>
+    <v>UAH</v>
+    <v>Ukraine is a country in Eastern Europe. It is the second-largest country in Europe after Russia, which borders it to the east and northeast. Ukraine also borders Belarus to the north; Poland and Slovakia to the west; Hungary, Romania and Moldova ...</v>
+    <v>3229</v>
+    <v>3230</v>
+    <v>3231</v>
+    <v>3232</v>
+    <v>3233</v>
+    <v>3234</v>
+    <v>3235</v>
+    <v>3236</v>
+    <v>3237</v>
+    <v>3238</v>
+    <v>3225</v>
+    <v>3242</v>
+    <v>3243</v>
+    <v>3244</v>
+    <v>3245</v>
+    <v>74</v>
+    <v>3246</v>
+    <v>Ukraine</v>
+    <v>National anthem of Ukraine</v>
+    <v>3247</v>
+    <v>Україна</v>
+    <v>3248</v>
+    <v>3249</v>
+    <v>3250</v>
+    <v>786</v>
+    <v>3192</v>
+    <v>3251</v>
+    <v>175</v>
+    <v>708</v>
+    <v>178</v>
+    <v>2589</v>
+    <v>3252</v>
+    <v>3278</v>
+    <v>3279</v>
+    <v>3280</v>
+    <v>3281</v>
+    <v>3282</v>
+    <v>Ukraine</v>
+    <v>3283</v>
+    <v>mdp/vdpid/241</v>
   </rv>
 </rvData>
 </file>
@@ -30470,7 +31058,7 @@
       <v t="s">Description</v>
     </a>
   </spbArrays>
-  <spbData count="469">
+  <spbData count="475">
     <spb s="0">
       <v xml:space="preserve">Wikipedia	</v>
       <v xml:space="preserve">CC BY-SA 3.0	</v>
@@ -36335,6 +36923,113 @@
       <v>467</v>
       <v>467</v>
     </spb>
+    <spb s="0">
+      <v xml:space="preserve">Wikipedia	Cia	Youtube	</v>
+      <v xml:space="preserve">CC-BY-SA			</v>
+      <v xml:space="preserve">http://en.wikipedia.org/wiki/Ukraine	https://www.cia.gov/library/publications/the-world-factbook/geos/up.html?Transportation	https://www.youtube.com/channel/UC3ZSveaqIraw9BASEyDLYXg	</v>
+      <v xml:space="preserve">http://creativecommons.org/licenses/by-sa/3.0/			</v>
+    </spb>
+    <spb s="0">
+      <v xml:space="preserve">Wikipedia	</v>
+      <v xml:space="preserve">CC BY-SA 3.0	</v>
+      <v xml:space="preserve">https://en.wikipedia.org/wiki/Ukraine	</v>
+      <v xml:space="preserve">https://creativecommons.org/licenses/by-sa/3.0	</v>
+    </spb>
+    <spb s="0">
+      <v xml:space="preserve">Wikipedia	</v>
+      <v xml:space="preserve">CC-BY-SA	</v>
+      <v xml:space="preserve">http://en.wikipedia.org/wiki/Ukraine	</v>
+      <v xml:space="preserve">http://creativecommons.org/licenses/by-sa/3.0/	</v>
+    </spb>
+    <spb s="0">
+      <v xml:space="preserve">Cia	</v>
+      <v xml:space="preserve">	</v>
+      <v xml:space="preserve">https://www.cia.gov/library/publications/the-world-factbook/geos/up.html?Transportation	</v>
+      <v xml:space="preserve">	</v>
+    </spb>
+    <spb s="17">
+      <v>21</v>
+      <v>469</v>
+      <v>470</v>
+      <v>470</v>
+      <v>24</v>
+      <v>470</v>
+      <v>470</v>
+      <v>470</v>
+      <v>471</v>
+      <v>470</v>
+      <v>470</v>
+      <v>471</v>
+      <v>470</v>
+      <v>470</v>
+      <v>472</v>
+      <v>26</v>
+      <v>469</v>
+      <v>472</v>
+      <v>27</v>
+      <v>470</v>
+      <v>472</v>
+      <v>28</v>
+      <v>29</v>
+      <v>30</v>
+      <v>472</v>
+      <v>472</v>
+      <v>470</v>
+      <v>472</v>
+      <v>31</v>
+      <v>32</v>
+      <v>33</v>
+      <v>34</v>
+      <v>472</v>
+      <v>469</v>
+      <v>472</v>
+      <v>472</v>
+      <v>472</v>
+      <v>472</v>
+      <v>472</v>
+      <v>472</v>
+      <v>472</v>
+      <v>472</v>
+      <v>472</v>
+      <v>472</v>
+      <v>35</v>
+    </spb>
+    <spb s="12">
+      <v>2019</v>
+      <v>2019</v>
+      <v>square km</v>
+      <v>per thousand (2018)</v>
+      <v>2022</v>
+      <v>2019</v>
+      <v>2018</v>
+      <v>per liter (2016)</v>
+      <v>2019</v>
+      <v>years (2018)</v>
+      <v>2018</v>
+      <v>per thousand (2018)</v>
+      <v>2019</v>
+      <v>2017</v>
+      <v>2016</v>
+      <v>2019</v>
+      <v>2016</v>
+      <v>2014</v>
+      <v>kilotons per year (2016)</v>
+      <v>deaths per 100,000 (2017)</v>
+      <v>kWh (2014)</v>
+      <v>2014</v>
+      <v>2018</v>
+      <v>2018</v>
+      <v>2018</v>
+      <v>2018</v>
+      <v>2018</v>
+      <v>2018</v>
+      <v>2015</v>
+      <v>2018</v>
+      <v>2018</v>
+      <v>2014</v>
+      <v>2014</v>
+      <v>2019</v>
+    </spb>
   </spbData>
 </supportingPropertyBags>
 </file>
@@ -37305,7 +38000,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F7772053-9363-CA4A-A53F-040B7C700753}">
-  <dimension ref="A1:V268"/>
+  <dimension ref="A1:V275"/>
   <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="16" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="19.6640625" customWidth="1"/>
@@ -39646,7 +40341,7 @@
         <v>96</v>
       </c>
       <c r="J52" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="M52" s="2" t="s">
         <v>58</v>
@@ -39817,7 +40512,7 @@
         <v>96</v>
       </c>
       <c r="J56" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="K56" t="s">
         <v>309</v>
@@ -40489,7 +41184,7 @@
         <v>96</v>
       </c>
       <c r="J71" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="K71" t="s">
         <v>309</v>
@@ -44774,7 +45469,7 @@
         <v>96</v>
       </c>
       <c r="J164" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="M164" t="s">
         <v>558</v>
@@ -45833,7 +46528,7 @@
         <v>96</v>
       </c>
       <c r="J186" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="M186" t="s">
         <v>249</v>
@@ -47262,7 +47957,7 @@
         <v>96</v>
       </c>
       <c r="J219" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="M219" t="s">
         <v>737</v>
@@ -47972,7 +48667,7 @@
         <v>96</v>
       </c>
       <c r="J235" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="K235" t="s">
         <v>309</v>
@@ -48444,33 +49139,27 @@
     </row>
     <row r="246" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A246" t="s">
-        <v>784</v>
+        <v>864</v>
       </c>
       <c r="D246" s="1">
-        <v>46006</v>
+        <v>45996</v>
       </c>
       <c r="E246" t="s">
-        <v>40</v>
-      </c>
-      <c r="F246" t="s">
-        <v>785</v>
+        <v>15</v>
+      </c>
+      <c r="F246" s="2" t="s">
+        <v>865</v>
       </c>
       <c r="I246" t="s">
-        <v>23</v>
+        <v>96</v>
       </c>
       <c r="J246" t="s">
         <v>402</v>
       </c>
-      <c r="K246" t="s">
-        <v>244</v>
-      </c>
-      <c r="L246" s="1">
-        <v>46027</v>
-      </c>
       <c r="M246" t="s">
-        <v>786</v>
-      </c>
-      <c r="N246" t="e" vm="35">
+        <v>720</v>
+      </c>
+      <c r="N246" t="e" vm="68">
         <v>#VALUE!</v>
       </c>
       <c r="O246" t="s">
@@ -48480,7 +49169,7 @@
         <v>776</v>
       </c>
       <c r="R246" s="1">
-        <v>46026</v>
+        <v>46005</v>
       </c>
       <c r="T246">
         <v>1</v>
@@ -48494,27 +49183,24 @@
     </row>
     <row r="247" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A247" t="s">
-        <v>841</v>
+        <v>866</v>
       </c>
       <c r="D247" s="1">
-        <v>46006</v>
+        <v>45996</v>
       </c>
       <c r="E247" t="s">
-        <v>844</v>
-      </c>
-      <c r="H247" t="s">
-        <v>842</v>
+        <v>15</v>
       </c>
       <c r="I247" t="s">
-        <v>23</v>
+        <v>96</v>
       </c>
       <c r="J247" t="s">
         <v>402</v>
       </c>
       <c r="M247" t="s">
-        <v>843</v>
-      </c>
-      <c r="N247" t="e" vm="46">
+        <v>397</v>
+      </c>
+      <c r="N247" t="e" vm="47">
         <v>#VALUE!</v>
       </c>
       <c r="O247" t="s">
@@ -48524,7 +49210,7 @@
         <v>776</v>
       </c>
       <c r="R247" s="1">
-        <v>46022</v>
+        <v>46001</v>
       </c>
       <c r="T247">
         <v>1</v>
@@ -48538,27 +49224,33 @@
     </row>
     <row r="248" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A248" t="s">
-        <v>662</v>
+        <v>784</v>
       </c>
       <c r="D248" s="1">
-        <v>46011</v>
+        <v>46006</v>
       </c>
       <c r="E248" t="s">
-        <v>15</v>
-      </c>
-      <c r="H248" t="s">
-        <v>664</v>
+        <v>40</v>
+      </c>
+      <c r="F248" t="s">
+        <v>785</v>
       </c>
       <c r="I248" t="s">
-        <v>96</v>
+        <v>23</v>
       </c>
       <c r="J248" t="s">
         <v>402</v>
       </c>
+      <c r="K248" t="s">
+        <v>244</v>
+      </c>
+      <c r="L248" s="1">
+        <v>46027</v>
+      </c>
       <c r="M248" t="s">
-        <v>663</v>
-      </c>
-      <c r="N248" t="e" vm="45">
+        <v>786</v>
+      </c>
+      <c r="N248" t="e" vm="35">
         <v>#VALUE!</v>
       </c>
       <c r="O248" t="s">
@@ -48568,7 +49260,7 @@
         <v>776</v>
       </c>
       <c r="R248" s="1">
-        <v>46037</v>
+        <v>46026</v>
       </c>
       <c r="T248">
         <v>1</v>
@@ -48582,19 +49274,16 @@
     </row>
     <row r="249" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A249" t="s">
-        <v>722</v>
-      </c>
-      <c r="C249" t="s">
-        <v>723</v>
+        <v>838</v>
       </c>
       <c r="D249" s="1">
-        <v>46016</v>
+        <v>46006</v>
       </c>
       <c r="E249" t="s">
-        <v>15</v>
-      </c>
-      <c r="F249" t="s">
-        <v>721</v>
+        <v>841</v>
+      </c>
+      <c r="H249" t="s">
+        <v>839</v>
       </c>
       <c r="I249" t="s">
         <v>96</v>
@@ -48603,9 +49292,9 @@
         <v>402</v>
       </c>
       <c r="M249" t="s">
-        <v>720</v>
-      </c>
-      <c r="N249" t="e" vm="68">
+        <v>840</v>
+      </c>
+      <c r="N249" t="e" vm="46">
         <v>#VALUE!</v>
       </c>
       <c r="O249" t="s">
@@ -48615,7 +49304,7 @@
         <v>776</v>
       </c>
       <c r="R249" s="1">
-        <v>45992</v>
+        <v>46022</v>
       </c>
       <c r="T249">
         <v>1</v>
@@ -48628,21 +49317,17 @@
       </c>
     </row>
     <row r="250" spans="1:22" x14ac:dyDescent="0.4">
-      <c r="A250" s="4" t="s">
-        <v>719</v>
-      </c>
-      <c r="B250" s="19"/>
-      <c r="C250" t="s">
-        <v>783</v>
+      <c r="A250" t="s">
+        <v>662</v>
       </c>
       <c r="D250" s="1">
-        <v>46016</v>
+        <v>46011</v>
       </c>
       <c r="E250" t="s">
         <v>15</v>
       </c>
-      <c r="G250">
-        <v>3</v>
+      <c r="H250" t="s">
+        <v>664</v>
       </c>
       <c r="I250" t="s">
         <v>96</v>
@@ -48650,26 +49335,20 @@
       <c r="J250" t="s">
         <v>402</v>
       </c>
-      <c r="K250" t="s">
-        <v>309</v>
-      </c>
-      <c r="L250" s="1">
-        <v>45992</v>
-      </c>
-      <c r="M250" s="2" t="s">
-        <v>718</v>
+      <c r="M250" t="s">
+        <v>663</v>
       </c>
       <c r="N250" t="e" vm="45">
         <v>#VALUE!</v>
       </c>
       <c r="O250" t="s">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="Q250" t="s">
         <v>776</v>
       </c>
       <c r="R250" s="1">
-        <v>45996</v>
+        <v>46037</v>
       </c>
       <c r="T250">
         <v>1</v>
@@ -48683,7 +49362,10 @@
     </row>
     <row r="251" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A251" t="s">
-        <v>787</v>
+        <v>722</v>
+      </c>
+      <c r="C251" t="s">
+        <v>723</v>
       </c>
       <c r="D251" s="1">
         <v>46016</v>
@@ -48691,6 +49373,9 @@
       <c r="E251" t="s">
         <v>15</v>
       </c>
+      <c r="F251" t="s">
+        <v>721</v>
+      </c>
       <c r="I251" t="s">
         <v>96</v>
       </c>
@@ -48698,10 +49383,13 @@
         <v>402</v>
       </c>
       <c r="M251" t="s">
-        <v>788</v>
-      </c>
-      <c r="N251" t="e" vm="29">
+        <v>720</v>
+      </c>
+      <c r="N251" t="e" vm="68">
         <v>#VALUE!</v>
+      </c>
+      <c r="O251" t="s">
+        <v>26</v>
       </c>
       <c r="Q251" t="s">
         <v>776</v>
@@ -48710,7 +49398,7 @@
         <v>45992</v>
       </c>
       <c r="T251">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U251">
         <v>0</v>
@@ -48720,8 +49408,12 @@
       </c>
     </row>
     <row r="252" spans="1:22" x14ac:dyDescent="0.4">
-      <c r="A252" t="s">
-        <v>790</v>
+      <c r="A252" s="4" t="s">
+        <v>719</v>
+      </c>
+      <c r="B252" s="19"/>
+      <c r="C252" t="s">
+        <v>783</v>
       </c>
       <c r="D252" s="1">
         <v>46016</v>
@@ -48729,16 +49421,25 @@
       <c r="E252" t="s">
         <v>15</v>
       </c>
+      <c r="G252">
+        <v>3</v>
+      </c>
       <c r="I252" t="s">
         <v>96</v>
       </c>
       <c r="J252" t="s">
         <v>402</v>
       </c>
-      <c r="M252" t="s">
-        <v>789</v>
-      </c>
-      <c r="N252" t="e" vm="75">
+      <c r="K252" t="s">
+        <v>309</v>
+      </c>
+      <c r="L252" s="1">
+        <v>45992</v>
+      </c>
+      <c r="M252" s="2" t="s">
+        <v>718</v>
+      </c>
+      <c r="N252" t="e" vm="45">
         <v>#VALUE!</v>
       </c>
       <c r="O252" t="s">
@@ -48748,7 +49449,7 @@
         <v>776</v>
       </c>
       <c r="R252" s="1">
-        <v>45992</v>
+        <v>45996</v>
       </c>
       <c r="T252">
         <v>1</v>
@@ -48762,16 +49463,13 @@
     </row>
     <row r="253" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A253" t="s">
-        <v>528</v>
-      </c>
-      <c r="C253" t="s">
-        <v>178</v>
+        <v>787</v>
       </c>
       <c r="D253" s="1">
-        <v>46023</v>
+        <v>46016</v>
       </c>
       <c r="E253" t="s">
-        <v>529</v>
+        <v>15</v>
       </c>
       <c r="I253" t="s">
         <v>96</v>
@@ -48780,39 +49478,36 @@
         <v>402</v>
       </c>
       <c r="M253" t="s">
-        <v>530</v>
-      </c>
-      <c r="N253" t="e" vm="102">
+        <v>788</v>
+      </c>
+      <c r="N253" t="e" vm="29">
         <v>#VALUE!</v>
-      </c>
-      <c r="O253" t="s">
-        <v>19</v>
       </c>
       <c r="Q253" t="s">
         <v>776</v>
       </c>
       <c r="R253" s="1">
-        <v>46041</v>
+        <v>45992</v>
       </c>
       <c r="T253">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U253">
         <v>0</v>
       </c>
       <c r="V253">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="254" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A254" t="s">
-        <v>564</v>
+        <v>790</v>
       </c>
       <c r="D254" s="1">
-        <v>46023</v>
+        <v>46016</v>
       </c>
       <c r="E254" t="s">
-        <v>565</v>
+        <v>15</v>
       </c>
       <c r="I254" t="s">
         <v>96</v>
@@ -48821,19 +49516,19 @@
         <v>402</v>
       </c>
       <c r="M254" t="s">
-        <v>566</v>
-      </c>
-      <c r="N254" t="e" vm="103">
+        <v>789</v>
+      </c>
+      <c r="N254" t="e" vm="75">
         <v>#VALUE!</v>
       </c>
       <c r="O254" t="s">
-        <v>26</v>
+        <v>11</v>
       </c>
       <c r="Q254" t="s">
         <v>776</v>
       </c>
       <c r="R254" s="1">
-        <v>45664</v>
+        <v>45992</v>
       </c>
       <c r="T254">
         <v>1</v>
@@ -48847,37 +49542,37 @@
     </row>
     <row r="255" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A255" t="s">
-        <v>804</v>
+        <v>528</v>
+      </c>
+      <c r="C255" t="s">
+        <v>178</v>
       </c>
       <c r="D255" s="1">
         <v>46023</v>
       </c>
-      <c r="E255" s="2" t="s">
-        <v>803</v>
-      </c>
-      <c r="F255" s="2" t="s">
-        <v>806</v>
+      <c r="E255" t="s">
+        <v>529</v>
       </c>
       <c r="I255" t="s">
-        <v>23</v>
+        <v>96</v>
       </c>
       <c r="J255" t="s">
         <v>402</v>
       </c>
       <c r="M255" t="s">
-        <v>805</v>
-      </c>
-      <c r="N255" t="e" vm="35">
+        <v>530</v>
+      </c>
+      <c r="N255" t="e" vm="102">
         <v>#VALUE!</v>
       </c>
       <c r="O255" t="s">
-        <v>26</v>
+        <v>19</v>
       </c>
       <c r="Q255" t="s">
         <v>776</v>
       </c>
       <c r="R255" s="1">
-        <v>46038</v>
+        <v>46041</v>
       </c>
       <c r="T255">
         <v>1</v>
@@ -48886,39 +49581,39 @@
         <v>0</v>
       </c>
       <c r="V255">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="256" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A256" t="s">
-        <v>807</v>
+        <v>564</v>
       </c>
       <c r="D256" s="1">
         <v>46023</v>
       </c>
       <c r="E256" t="s">
-        <v>15</v>
+        <v>565</v>
       </c>
       <c r="I256" t="s">
-        <v>23</v>
+        <v>96</v>
       </c>
       <c r="J256" t="s">
         <v>402</v>
       </c>
       <c r="M256" t="s">
-        <v>808</v>
-      </c>
-      <c r="N256" t="e" vm="54">
+        <v>566</v>
+      </c>
+      <c r="N256" t="e" vm="103">
         <v>#VALUE!</v>
       </c>
       <c r="O256" t="s">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="Q256" t="s">
         <v>776</v>
       </c>
       <c r="R256" s="1">
-        <v>46052</v>
+        <v>45664</v>
       </c>
       <c r="T256">
         <v>1</v>
@@ -48932,27 +49627,27 @@
     </row>
     <row r="257" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A257" t="s">
-        <v>809</v>
+        <v>804</v>
       </c>
       <c r="D257" s="1">
         <v>46023</v>
       </c>
-      <c r="E257" t="s">
-        <v>15</v>
-      </c>
-      <c r="H257" t="s">
-        <v>810</v>
+      <c r="E257" s="2" t="s">
+        <v>803</v>
+      </c>
+      <c r="F257" s="2" t="s">
+        <v>806</v>
       </c>
       <c r="I257" t="s">
-        <v>23</v>
+        <v>96</v>
       </c>
       <c r="J257" t="s">
         <v>402</v>
       </c>
       <c r="M257" t="s">
-        <v>123</v>
-      </c>
-      <c r="N257" t="e" vm="25">
+        <v>805</v>
+      </c>
+      <c r="N257" t="e" vm="35">
         <v>#VALUE!</v>
       </c>
       <c r="O257" t="s">
@@ -48962,7 +49657,7 @@
         <v>776</v>
       </c>
       <c r="R257" s="1">
-        <v>46052</v>
+        <v>46038</v>
       </c>
       <c r="T257">
         <v>1</v>
@@ -48976,33 +49671,24 @@
     </row>
     <row r="258" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A258" t="s">
-        <v>811</v>
-      </c>
-      <c r="C258" t="s">
-        <v>814</v>
+        <v>807</v>
       </c>
       <c r="D258" s="1">
         <v>46023</v>
       </c>
       <c r="E258" t="s">
-        <v>40</v>
-      </c>
-      <c r="F258" t="s">
-        <v>813</v>
-      </c>
-      <c r="H258" t="s">
-        <v>815</v>
+        <v>15</v>
       </c>
       <c r="I258" t="s">
-        <v>23</v>
+        <v>96</v>
       </c>
       <c r="J258" t="s">
         <v>402</v>
       </c>
       <c r="M258" t="s">
-        <v>812</v>
-      </c>
-      <c r="N258" t="e" vm="35">
+        <v>808</v>
+      </c>
+      <c r="N258" t="e" vm="54">
         <v>#VALUE!</v>
       </c>
       <c r="O258" t="s">
@@ -49012,7 +49698,7 @@
         <v>776</v>
       </c>
       <c r="R258" s="1">
-        <v>46037</v>
+        <v>46052</v>
       </c>
       <c r="T258">
         <v>1</v>
@@ -49026,7 +49712,10 @@
     </row>
     <row r="259" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A259" t="s">
-        <v>816</v>
+        <v>809</v>
+      </c>
+      <c r="C259" t="s">
+        <v>812</v>
       </c>
       <c r="D259" s="1">
         <v>46023</v>
@@ -49034,17 +49723,20 @@
       <c r="E259" t="s">
         <v>40</v>
       </c>
-      <c r="F259" s="2" t="s">
-        <v>817</v>
+      <c r="F259" t="s">
+        <v>811</v>
+      </c>
+      <c r="H259" t="s">
+        <v>813</v>
       </c>
       <c r="I259" t="s">
-        <v>23</v>
+        <v>96</v>
       </c>
       <c r="J259" t="s">
         <v>402</v>
       </c>
       <c r="M259" t="s">
-        <v>818</v>
+        <v>810</v>
       </c>
       <c r="N259" t="e" vm="35">
         <v>#VALUE!</v>
@@ -49056,7 +49748,7 @@
         <v>776</v>
       </c>
       <c r="R259" s="1">
-        <v>46066</v>
+        <v>46037</v>
       </c>
       <c r="T259">
         <v>1</v>
@@ -49070,7 +49762,7 @@
     </row>
     <row r="260" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A260" t="s">
-        <v>819</v>
+        <v>814</v>
       </c>
       <c r="D260" s="1">
         <v>46023</v>
@@ -49078,19 +49770,19 @@
       <c r="E260" t="s">
         <v>40</v>
       </c>
-      <c r="F260" t="s">
-        <v>820</v>
+      <c r="F260" s="2" t="s">
+        <v>815</v>
       </c>
       <c r="I260" t="s">
-        <v>23</v>
+        <v>96</v>
       </c>
       <c r="J260" t="s">
         <v>402</v>
       </c>
       <c r="M260" t="s">
-        <v>821</v>
-      </c>
-      <c r="N260" t="e" vm="6">
+        <v>816</v>
+      </c>
+      <c r="N260" t="e" vm="35">
         <v>#VALUE!</v>
       </c>
       <c r="O260" t="s">
@@ -49100,7 +49792,7 @@
         <v>776</v>
       </c>
       <c r="R260" s="1">
-        <v>46052</v>
+        <v>46066</v>
       </c>
       <c r="T260">
         <v>1</v>
@@ -49114,7 +49806,7 @@
     </row>
     <row r="261" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A261" t="s">
-        <v>823</v>
+        <v>817</v>
       </c>
       <c r="D261" s="1">
         <v>46023</v>
@@ -49122,19 +49814,19 @@
       <c r="E261" t="s">
         <v>40</v>
       </c>
-      <c r="F261" s="2" t="s">
-        <v>824</v>
+      <c r="F261" t="s">
+        <v>818</v>
       </c>
       <c r="I261" t="s">
-        <v>23</v>
+        <v>96</v>
       </c>
       <c r="J261" t="s">
         <v>402</v>
       </c>
       <c r="M261" t="s">
-        <v>822</v>
-      </c>
-      <c r="N261" t="e" vm="35">
+        <v>819</v>
+      </c>
+      <c r="N261" t="e" vm="6">
         <v>#VALUE!</v>
       </c>
       <c r="O261" t="s">
@@ -49144,7 +49836,7 @@
         <v>776</v>
       </c>
       <c r="R261" s="1">
-        <v>46113</v>
+        <v>46052</v>
       </c>
       <c r="T261">
         <v>1</v>
@@ -49158,10 +49850,7 @@
     </row>
     <row r="262" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A262" t="s">
-        <v>825</v>
-      </c>
-      <c r="C262" t="s">
-        <v>831</v>
+        <v>821</v>
       </c>
       <c r="D262" s="1">
         <v>46023</v>
@@ -49170,28 +49859,28 @@
         <v>40</v>
       </c>
       <c r="F262" s="2" t="s">
-        <v>826</v>
+        <v>822</v>
       </c>
       <c r="I262" t="s">
-        <v>23</v>
+        <v>96</v>
       </c>
       <c r="J262" t="s">
         <v>402</v>
       </c>
       <c r="M262" t="s">
-        <v>827</v>
+        <v>820</v>
       </c>
       <c r="N262" t="e" vm="35">
         <v>#VALUE!</v>
       </c>
       <c r="O262" t="s">
-        <v>26</v>
+        <v>11</v>
       </c>
       <c r="Q262" t="s">
         <v>776</v>
       </c>
       <c r="R262" s="1">
-        <v>46038</v>
+        <v>46113</v>
       </c>
       <c r="T262">
         <v>1</v>
@@ -49205,10 +49894,10 @@
     </row>
     <row r="263" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A263" t="s">
-        <v>828</v>
+        <v>823</v>
       </c>
       <c r="C263" t="s">
-        <v>830</v>
+        <v>829</v>
       </c>
       <c r="D263" s="1">
         <v>46023</v>
@@ -49216,29 +49905,29 @@
       <c r="E263" t="s">
         <v>40</v>
       </c>
-      <c r="F263" t="s">
-        <v>832</v>
+      <c r="F263" s="2" t="s">
+        <v>824</v>
       </c>
       <c r="I263" t="s">
-        <v>23</v>
+        <v>96</v>
       </c>
       <c r="J263" t="s">
         <v>402</v>
       </c>
       <c r="M263" t="s">
-        <v>829</v>
+        <v>825</v>
       </c>
       <c r="N263" t="e" vm="35">
         <v>#VALUE!</v>
       </c>
       <c r="O263" t="s">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="Q263" t="s">
         <v>776</v>
       </c>
       <c r="R263" s="1">
-        <v>46143</v>
+        <v>46038</v>
       </c>
       <c r="T263">
         <v>1</v>
@@ -49252,10 +49941,10 @@
     </row>
     <row r="264" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A264" t="s">
-        <v>833</v>
+        <v>826</v>
       </c>
       <c r="C264" t="s">
-        <v>836</v>
+        <v>828</v>
       </c>
       <c r="D264" s="1">
         <v>46023</v>
@@ -49263,17 +49952,17 @@
       <c r="E264" t="s">
         <v>40</v>
       </c>
-      <c r="F264" s="2" t="s">
-        <v>835</v>
+      <c r="F264" t="s">
+        <v>830</v>
       </c>
       <c r="I264" t="s">
-        <v>23</v>
+        <v>96</v>
       </c>
       <c r="J264" t="s">
         <v>402</v>
       </c>
       <c r="M264" t="s">
-        <v>834</v>
+        <v>827</v>
       </c>
       <c r="N264" t="e" vm="35">
         <v>#VALUE!</v>
@@ -49285,7 +49974,7 @@
         <v>776</v>
       </c>
       <c r="R264" s="1">
-        <v>46027</v>
+        <v>46143</v>
       </c>
       <c r="T264">
         <v>1</v>
@@ -49299,22 +49988,28 @@
     </row>
     <row r="265" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A265" t="s">
-        <v>838</v>
+        <v>831</v>
+      </c>
+      <c r="C265" t="s">
+        <v>833</v>
       </c>
       <c r="D265" s="1">
         <v>46023</v>
       </c>
       <c r="E265" t="s">
-        <v>839</v>
+        <v>40</v>
+      </c>
+      <c r="F265" s="2" t="s">
+        <v>871</v>
       </c>
       <c r="I265" t="s">
-        <v>23</v>
+        <v>96</v>
       </c>
       <c r="J265" t="s">
         <v>402</v>
       </c>
       <c r="M265" t="s">
-        <v>840</v>
+        <v>832</v>
       </c>
       <c r="N265" t="e" vm="35">
         <v>#VALUE!</v>
@@ -49325,6 +50020,9 @@
       <c r="Q265" t="s">
         <v>776</v>
       </c>
+      <c r="R265" s="1">
+        <v>46027</v>
+      </c>
       <c r="T265">
         <v>1</v>
       </c>
@@ -49337,13 +50035,13 @@
     </row>
     <row r="266" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A266" t="s">
-        <v>845</v>
+        <v>835</v>
       </c>
       <c r="D266" s="1">
         <v>46023</v>
       </c>
       <c r="E266" t="s">
-        <v>846</v>
+        <v>836</v>
       </c>
       <c r="I266" t="s">
         <v>23</v>
@@ -49352,9 +50050,9 @@
         <v>402</v>
       </c>
       <c r="M266" t="s">
-        <v>847</v>
-      </c>
-      <c r="N266" t="e" vm="84">
+        <v>837</v>
+      </c>
+      <c r="N266" t="e" vm="35">
         <v>#VALUE!</v>
       </c>
       <c r="O266" t="s">
@@ -49363,9 +50061,6 @@
       <c r="Q266" t="s">
         <v>776</v>
       </c>
-      <c r="R266" s="1">
-        <v>46037</v>
-      </c>
       <c r="T266">
         <v>1</v>
       </c>
@@ -49378,16 +50073,13 @@
     </row>
     <row r="267" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A267" t="s">
-        <v>848</v>
-      </c>
-      <c r="C267" t="s">
-        <v>851</v>
+        <v>842</v>
       </c>
       <c r="D267" s="1">
         <v>46023</v>
       </c>
       <c r="E267" t="s">
-        <v>850</v>
+        <v>843</v>
       </c>
       <c r="I267" t="s">
         <v>23</v>
@@ -49396,19 +50088,19 @@
         <v>402</v>
       </c>
       <c r="M267" t="s">
-        <v>849</v>
-      </c>
-      <c r="N267" t="e" vm="35">
+        <v>844</v>
+      </c>
+      <c r="N267" t="e" vm="84">
         <v>#VALUE!</v>
       </c>
       <c r="O267" t="s">
-        <v>26</v>
+        <v>11</v>
       </c>
       <c r="Q267" t="s">
         <v>776</v>
       </c>
       <c r="R267" s="1">
-        <v>46033</v>
+        <v>46037</v>
       </c>
       <c r="T267">
         <v>1</v>
@@ -49422,34 +50114,40 @@
     </row>
     <row r="268" spans="1:22" x14ac:dyDescent="0.4">
       <c r="A268" t="s">
-        <v>255</v>
+        <v>845</v>
+      </c>
+      <c r="C268" t="s">
+        <v>848</v>
+      </c>
+      <c r="D268" s="1">
+        <v>46023</v>
       </c>
       <c r="E268" t="s">
-        <v>15</v>
-      </c>
-      <c r="F268" s="2" t="s">
-        <v>257</v>
+        <v>847</v>
       </c>
       <c r="I268" t="s">
-        <v>96</v>
+        <v>23</v>
       </c>
       <c r="J268" t="s">
         <v>402</v>
       </c>
       <c r="M268" t="s">
-        <v>256</v>
+        <v>846</v>
       </c>
       <c r="N268" t="e" vm="35">
         <v>#VALUE!</v>
       </c>
       <c r="O268" t="s">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="Q268" t="s">
         <v>776</v>
       </c>
+      <c r="R268" s="1">
+        <v>46033</v>
+      </c>
       <c r="T268">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U268">
         <v>0</v>
@@ -49458,93 +50156,376 @@
         <v>0</v>
       </c>
     </row>
+    <row r="269" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A269" t="s">
+        <v>850</v>
+      </c>
+      <c r="C269" t="s">
+        <v>853</v>
+      </c>
+      <c r="D269" s="1">
+        <v>46023</v>
+      </c>
+      <c r="E269" t="s">
+        <v>40</v>
+      </c>
+      <c r="F269" t="s">
+        <v>851</v>
+      </c>
+      <c r="I269" t="s">
+        <v>23</v>
+      </c>
+      <c r="J269" t="s">
+        <v>402</v>
+      </c>
+      <c r="M269" t="s">
+        <v>852</v>
+      </c>
+      <c r="N269" t="e" vm="35">
+        <v>#VALUE!</v>
+      </c>
+      <c r="O269" t="s">
+        <v>26</v>
+      </c>
+      <c r="Q269" t="s">
+        <v>776</v>
+      </c>
+      <c r="R269" s="1">
+        <v>46173</v>
+      </c>
+      <c r="T269">
+        <v>1</v>
+      </c>
+      <c r="U269">
+        <v>0</v>
+      </c>
+      <c r="V269">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="270" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A270" t="s">
+        <v>854</v>
+      </c>
+      <c r="D270" s="1">
+        <v>46023</v>
+      </c>
+      <c r="E270" t="s">
+        <v>40</v>
+      </c>
+      <c r="F270" t="s">
+        <v>855</v>
+      </c>
+      <c r="I270" t="s">
+        <v>23</v>
+      </c>
+      <c r="J270" t="s">
+        <v>402</v>
+      </c>
+      <c r="M270" t="s">
+        <v>493</v>
+      </c>
+      <c r="N270" t="e" vm="35">
+        <v>#VALUE!</v>
+      </c>
+      <c r="O270" t="s">
+        <v>26</v>
+      </c>
+      <c r="Q270" t="s">
+        <v>776</v>
+      </c>
+      <c r="R270" s="1">
+        <v>46028</v>
+      </c>
+      <c r="T270">
+        <v>1</v>
+      </c>
+      <c r="U270">
+        <v>0</v>
+      </c>
+      <c r="V270">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="271" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A271" t="s">
+        <v>856</v>
+      </c>
+      <c r="D271" s="1">
+        <v>46023</v>
+      </c>
+      <c r="E271" t="s">
+        <v>15</v>
+      </c>
+      <c r="F271" s="2" t="s">
+        <v>857</v>
+      </c>
+      <c r="H271" t="s">
+        <v>859</v>
+      </c>
+      <c r="I271" t="s">
+        <v>23</v>
+      </c>
+      <c r="J271" t="s">
+        <v>402</v>
+      </c>
+      <c r="M271" t="s">
+        <v>858</v>
+      </c>
+      <c r="N271" t="e" vm="70">
+        <v>#VALUE!</v>
+      </c>
+      <c r="O271" t="s">
+        <v>11</v>
+      </c>
+      <c r="Q271" t="s">
+        <v>776</v>
+      </c>
+      <c r="R271" s="1">
+        <v>46055</v>
+      </c>
+      <c r="T271">
+        <v>1</v>
+      </c>
+      <c r="U271">
+        <v>0</v>
+      </c>
+      <c r="V271">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="272" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A272" t="s">
+        <v>860</v>
+      </c>
+      <c r="C272" t="s">
+        <v>862</v>
+      </c>
+      <c r="D272" s="1">
+        <v>46023</v>
+      </c>
+      <c r="E272" t="s">
+        <v>15</v>
+      </c>
+      <c r="F272" s="2" t="s">
+        <v>863</v>
+      </c>
+      <c r="I272" t="s">
+        <v>23</v>
+      </c>
+      <c r="J272" t="s">
+        <v>402</v>
+      </c>
+      <c r="M272" t="s">
+        <v>861</v>
+      </c>
+      <c r="N272" t="e" vm="93">
+        <v>#VALUE!</v>
+      </c>
+      <c r="O272" t="s">
+        <v>11</v>
+      </c>
+      <c r="Q272" t="s">
+        <v>776</v>
+      </c>
+      <c r="R272" s="1">
+        <v>46026</v>
+      </c>
+      <c r="T272">
+        <v>1</v>
+      </c>
+      <c r="U272">
+        <v>0</v>
+      </c>
+      <c r="V272">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="273" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A273" t="s">
+        <v>867</v>
+      </c>
+      <c r="D273" s="1">
+        <v>46023</v>
+      </c>
+      <c r="E273" t="s">
+        <v>15</v>
+      </c>
+      <c r="I273" t="s">
+        <v>23</v>
+      </c>
+      <c r="J273" t="s">
+        <v>402</v>
+      </c>
+      <c r="M273" t="s">
+        <v>868</v>
+      </c>
+      <c r="N273" t="e" vm="104">
+        <v>#VALUE!</v>
+      </c>
+      <c r="O273" t="s">
+        <v>11</v>
+      </c>
+      <c r="Q273" t="s">
+        <v>776</v>
+      </c>
+      <c r="R273" s="1">
+        <v>46036</v>
+      </c>
+      <c r="T273">
+        <v>1</v>
+      </c>
+      <c r="U273">
+        <v>0</v>
+      </c>
+      <c r="V273">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="274" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A274" t="s">
+        <v>869</v>
+      </c>
+      <c r="D274" s="1">
+        <v>46023</v>
+      </c>
+      <c r="E274" t="s">
+        <v>15</v>
+      </c>
+      <c r="I274" t="s">
+        <v>23</v>
+      </c>
+      <c r="J274" t="s">
+        <v>402</v>
+      </c>
+      <c r="M274" t="s">
+        <v>870</v>
+      </c>
+      <c r="N274" t="e" vm="94">
+        <v>#VALUE!</v>
+      </c>
+      <c r="O274" t="s">
+        <v>11</v>
+      </c>
+      <c r="Q274" t="s">
+        <v>776</v>
+      </c>
+      <c r="R274" s="1">
+        <v>46053</v>
+      </c>
+      <c r="T274">
+        <v>1</v>
+      </c>
+      <c r="U274">
+        <v>0</v>
+      </c>
+      <c r="V274">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="275" spans="1:22" x14ac:dyDescent="0.4">
+      <c r="A275" t="s">
+        <v>255</v>
+      </c>
+      <c r="E275" t="s">
+        <v>15</v>
+      </c>
+      <c r="F275" s="2" t="s">
+        <v>257</v>
+      </c>
+      <c r="I275" t="s">
+        <v>96</v>
+      </c>
+      <c r="J275" t="s">
+        <v>402</v>
+      </c>
+      <c r="M275" t="s">
+        <v>256</v>
+      </c>
+      <c r="N275" t="e" vm="35">
+        <v>#VALUE!</v>
+      </c>
+      <c r="O275" t="s">
+        <v>11</v>
+      </c>
+      <c r="Q275" t="s">
+        <v>776</v>
+      </c>
+      <c r="T275">
+        <v>0</v>
+      </c>
+      <c r="U275">
+        <v>0</v>
+      </c>
+      <c r="V275">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:V248" xr:uid="{F7772053-9363-CA4A-A53F-040B7C700753}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:V268">
-      <sortCondition ref="D1:D248"/>
+  <autoFilter ref="A1:V267" xr:uid="{F7772053-9363-CA4A-A53F-040B7C700753}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:V275">
+      <sortCondition ref="D1:D267"/>
     </sortState>
   </autoFilter>
   <conditionalFormatting sqref="A1:B208 A210:B1048576">
-    <cfRule type="duplicateValues" dxfId="207" priority="23"/>
+    <cfRule type="duplicateValues" dxfId="213" priority="23"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A2:B22">
-    <cfRule type="duplicateValues" dxfId="206" priority="24"/>
+    <cfRule type="duplicateValues" dxfId="212" priority="24"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A61:B61">
-    <cfRule type="duplicateValues" dxfId="205" priority="22"/>
+    <cfRule type="duplicateValues" dxfId="211" priority="22"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="I1:I1048576">
-    <cfRule type="containsText" dxfId="204" priority="15" operator="containsText" text="closed">
+    <cfRule type="containsText" dxfId="210" priority="15" operator="containsText" text="closed">
       <formula>NOT(ISERROR(SEARCH("closed",I1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="203" priority="16" operator="containsText" text="abandoned">
+    <cfRule type="containsText" dxfId="209" priority="16" operator="containsText" text="abandoned">
       <formula>NOT(ISERROR(SEARCH("abandoned",I1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="202" priority="18" operator="containsText" text="late app">
+    <cfRule type="containsText" dxfId="208" priority="18" operator="containsText" text="late app">
       <formula>NOT(ISERROR(SEARCH("late app",I1)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I2:L1048576 O78:O80 O83:O89 O92:O112 O115:O124 O126:O181 R136 R153 R159 R166 R173 R178 O183:O205 O208:O211 O213:O218 O220:O233 R225 O235:O237 O239:O248 M248 O250:O255 I1:J1 M266 N267">
-    <cfRule type="containsText" dxfId="201" priority="21" operator="containsText" text="completed">
+  <conditionalFormatting sqref="I2:L1048576 O78:O80 O83:O89 O92:O112 O115:O124 O126:O181 R136 R153 R159 R166 R173 R178 O183:O205 O208:O211 O213:O218 O220:O233 R225 O235:O237 O239:O248 I1:J1">
+    <cfRule type="containsText" dxfId="207" priority="21" operator="containsText" text="completed">
       <formula>NOT(ISERROR(SEARCH("completed",I1)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J1:J1048576">
-    <cfRule type="containsText" dxfId="200" priority="10" operator="containsText" text="no news">
+    <cfRule type="containsText" dxfId="206" priority="10" operator="containsText" text="no news">
       <formula>NOT(ISERROR(SEARCH("no news",J1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="199" priority="11" operator="containsText" text="offer">
+    <cfRule type="containsText" dxfId="205" priority="11" operator="containsText" text="offer">
       <formula>NOT(ISERROR(SEARCH("offer",J1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="198" priority="12" operator="containsText" text="fly out">
+    <cfRule type="containsText" dxfId="204" priority="12" operator="containsText" text="fly out">
       <formula>NOT(ISERROR(SEARCH("fly out",J1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="197" priority="13" operator="containsText" text="interview">
+    <cfRule type="containsText" dxfId="203" priority="13" operator="containsText" text="interview">
       <formula>NOT(ISERROR(SEARCH("interview",J1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="196" priority="14" operator="containsText" text="rejected">
+    <cfRule type="containsText" dxfId="202" priority="14" operator="containsText" text="rejected">
       <formula>NOT(ISERROR(SEARCH("rejected",J1)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K1:L1048576 O78:O80 O83:O89 O92:O112 O115:O124 O126:O181 R136 R153 R159 R166 R173 R178 O183:O205 O208:O211 O213:O218 O220:O233 R225 O235:O237 O239:O248 M248 O250:O255 M266 N267">
-    <cfRule type="containsText" dxfId="195" priority="19" operator="containsText" text="NO">
+  <conditionalFormatting sqref="K1:L1048576 O78:O80 O83:O89 O92:O112 O115:O124 O126:O181 R136 R153 R159 R166 R173 R178 O183:O205 O208:O211 O213:O218 O220:O233 R225 O235:O237 O239:O248">
+    <cfRule type="containsText" dxfId="201" priority="19" operator="containsText" text="NO">
       <formula>NOT(ISERROR(SEARCH("NO",K1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="194" priority="20" operator="containsText" text="YES">
+    <cfRule type="containsText" dxfId="200" priority="20" operator="containsText" text="YES">
       <formula>NOT(ISERROR(SEARCH("YES",K1)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="N256:O264 O265 N266:O266 O267:O268">
-    <cfRule type="containsText" dxfId="193" priority="7" operator="containsText" text="NO">
-      <formula>NOT(ISERROR(SEARCH("NO",N256)))</formula>
+  <conditionalFormatting sqref="O250:O267">
+    <cfRule type="containsText" dxfId="199" priority="1" operator="containsText" text="NO">
+      <formula>NOT(ISERROR(SEARCH("NO",O250)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="192" priority="8" operator="containsText" text="YES">
-      <formula>NOT(ISERROR(SEARCH("YES",N256)))</formula>
+    <cfRule type="containsText" dxfId="198" priority="2" operator="containsText" text="YES">
+      <formula>NOT(ISERROR(SEARCH("YES",O250)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="191" priority="9" operator="containsText" text="completed">
-      <formula>NOT(ISERROR(SEARCH("completed",N256)))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="N265">
-    <cfRule type="containsText" dxfId="5" priority="4" operator="containsText" text="NO">
-      <formula>NOT(ISERROR(SEARCH("NO",N265)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="4" priority="5" operator="containsText" text="YES">
-      <formula>NOT(ISERROR(SEARCH("YES",N265)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="3" priority="6" operator="containsText" text="completed">
-      <formula>NOT(ISERROR(SEARCH("completed",N265)))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="N268">
-    <cfRule type="containsText" dxfId="2" priority="1" operator="containsText" text="NO">
-      <formula>NOT(ISERROR(SEARCH("NO",N268)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="YES">
-      <formula>NOT(ISERROR(SEARCH("YES",N268)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="0" priority="3" operator="containsText" text="completed">
-      <formula>NOT(ISERROR(SEARCH("completed",N268)))</formula>
+    <cfRule type="containsText" dxfId="197" priority="3" operator="containsText" text="completed">
+      <formula>NOT(ISERROR(SEARCH("completed",O250)))</formula>
     </cfRule>
   </conditionalFormatting>
   <hyperlinks>
@@ -49629,7 +50610,7 @@
     <hyperlink ref="M17" r:id="rId79" xr:uid="{9A9A6BC9-B330-7842-A78C-4DCC88F5E19F}"/>
     <hyperlink ref="M32" r:id="rId80" xr:uid="{928CABEF-4FA6-E646-8140-7B6E43F8FB96}"/>
     <hyperlink ref="F177" r:id="rId81" xr:uid="{82BF1574-A6C6-1641-9FFE-615861E401FD}"/>
-    <hyperlink ref="F268" r:id="rId82" xr:uid="{3562807E-7FDA-F046-BA03-5DDD43072DB7}"/>
+    <hyperlink ref="F275" r:id="rId82" xr:uid="{3562807E-7FDA-F046-BA03-5DDD43072DB7}"/>
     <hyperlink ref="H215" r:id="rId83" display="mailto:ivanpaya@ua.es" xr:uid="{DEFB77A5-E57F-714C-BAB9-56DE82BA0B2E}"/>
     <hyperlink ref="H138" r:id="rId84" display="mailto:ari.hyytinen@hanken.fi" xr:uid="{7777B12A-FD99-4A43-A14B-A15661B760DC}"/>
     <hyperlink ref="H115" r:id="rId85" display="mailto:peter.haan@fu-berlin.de" xr:uid="{3D1A69ED-8F06-1246-B586-201CB349DB62}"/>
@@ -49647,23 +50628,25 @@
     <hyperlink ref="H240" r:id="rId97" display="mailto:ondrej.krcal@econ.muni.cz" xr:uid="{EDDEB1E6-5767-4FFB-A0AE-57A909D04E81}"/>
     <hyperlink ref="M218" r:id="rId98" display="https://www.ovgu.de/unimagdeburg/en/" xr:uid="{BCB3935D-2B6D-4090-86F5-762D762ED0E3}"/>
     <hyperlink ref="E152" r:id="rId99" xr:uid="{550520C0-1E25-41CD-9AEE-9A3C4D7D328C}"/>
-    <hyperlink ref="M250" r:id="rId100" xr:uid="{F0DD6D71-3FFD-4EAB-A251-AAF2DA8EF53C}"/>
+    <hyperlink ref="M252" r:id="rId100" xr:uid="{F0DD6D71-3FFD-4EAB-A251-AAF2DA8EF53C}"/>
     <hyperlink ref="F243" r:id="rId101" xr:uid="{BDBBC2E2-C3C5-4526-A621-853D22D99CCF}"/>
-    <hyperlink ref="F255" r:id="rId102" display="mailto:comap@northwestern.edu" xr:uid="{4DD04925-4C98-401C-B09E-A61B83C23B4E}"/>
-    <hyperlink ref="E255" r:id="rId103" xr:uid="{491ECAF5-1DC5-4C3F-B1BE-621395157776}"/>
-    <hyperlink ref="F259" r:id="rId104" xr:uid="{B084E08B-44BE-4FA5-A345-8036292B3E22}"/>
-    <hyperlink ref="F261" r:id="rId105" xr:uid="{F59B1D31-814A-4100-8601-8879ABB1E739}"/>
-    <hyperlink ref="F262" r:id="rId106" xr:uid="{C4BD89A9-F3F0-4E10-BAC5-751787E6C1A9}"/>
-    <hyperlink ref="F264" r:id="rId107" xr:uid="{64E2681C-F146-4414-BBE6-9DC59E57C615}"/>
+    <hyperlink ref="F257" r:id="rId102" display="mailto:comap@northwestern.edu" xr:uid="{4DD04925-4C98-401C-B09E-A61B83C23B4E}"/>
+    <hyperlink ref="E257" r:id="rId103" xr:uid="{491ECAF5-1DC5-4C3F-B1BE-621395157776}"/>
+    <hyperlink ref="F260" r:id="rId104" xr:uid="{B084E08B-44BE-4FA5-A345-8036292B3E22}"/>
+    <hyperlink ref="F262" r:id="rId105" xr:uid="{F59B1D31-814A-4100-8601-8879ABB1E739}"/>
+    <hyperlink ref="F263" r:id="rId106" xr:uid="{C4BD89A9-F3F0-4E10-BAC5-751787E6C1A9}"/>
+    <hyperlink ref="F271" r:id="rId107" xr:uid="{A8AE6398-5E3B-44CD-895F-D20F2BEC5279}"/>
+    <hyperlink ref="F272" r:id="rId108" xr:uid="{34317180-A8EC-4C92-AB27-7AD534355822}"/>
+    <hyperlink ref="F246" r:id="rId109" xr:uid="{81F56FF4-6BEE-4876-B897-D914C7668775}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId108"/>
+  <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId110"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{923E81FA-B875-3C4E-A189-1A21268FA086}">
-  <dimension ref="A1:C274"/>
+  <dimension ref="A1:C292"/>
   <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="16" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="32.83203125" customWidth="1"/>
@@ -52591,7 +53574,7 @@
         <v>45993</v>
       </c>
       <c r="C272" t="s">
-        <v>837</v>
+        <v>834</v>
       </c>
     </row>
     <row r="273" spans="1:3" x14ac:dyDescent="0.4">
@@ -52610,538 +53593,772 @@
         <v>45994</v>
       </c>
       <c r="C274" t="s">
-        <v>852</v>
+        <v>849</v>
+      </c>
+    </row>
+    <row r="275" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A275" s="1">
+        <v>45995</v>
+      </c>
+      <c r="B275" t="s">
+        <v>735</v>
+      </c>
+      <c r="C275" t="s">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="276" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A276" s="1">
+        <v>45995</v>
+      </c>
+      <c r="B276" t="s">
+        <v>767</v>
+      </c>
+      <c r="C276" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="277" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A277" s="1">
+        <v>45998</v>
+      </c>
+      <c r="B277" t="s">
+        <v>250</v>
+      </c>
+      <c r="C277" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="278" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A278" s="1">
+        <v>45999</v>
+      </c>
+      <c r="B278" t="s">
+        <v>864</v>
+      </c>
+      <c r="C278" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="279" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A279" s="1">
+        <v>45999</v>
+      </c>
+      <c r="B279" t="s">
+        <v>472</v>
+      </c>
+      <c r="C279" t="s">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="280" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A280" s="1">
+        <v>45999</v>
+      </c>
+      <c r="B280" t="s">
+        <v>804</v>
+      </c>
+      <c r="C280" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="281" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A281" s="1">
+        <v>46000</v>
+      </c>
+      <c r="B281" t="s">
+        <v>807</v>
+      </c>
+      <c r="C281" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="282" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A282" s="1">
+        <v>46000</v>
+      </c>
+      <c r="B282" t="s">
+        <v>557</v>
+      </c>
+      <c r="C282" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="283" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A283" s="1">
+        <v>46000</v>
+      </c>
+      <c r="B283" t="s">
+        <v>54</v>
+      </c>
+      <c r="C283" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="284" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A284" s="1">
+        <v>46000</v>
+      </c>
+      <c r="B284" t="s">
+        <v>807</v>
+      </c>
+      <c r="C284" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="285" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A285" s="1">
+        <v>46000</v>
+      </c>
+      <c r="B285" t="s">
+        <v>809</v>
+      </c>
+      <c r="C285" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="286" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A286" s="1">
+        <v>46000</v>
+      </c>
+      <c r="B286" t="s">
+        <v>814</v>
+      </c>
+      <c r="C286" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="287" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A287" s="1">
+        <v>46000</v>
+      </c>
+      <c r="B287" t="s">
+        <v>817</v>
+      </c>
+      <c r="C287" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="288" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A288" s="1">
+        <v>46000</v>
+      </c>
+      <c r="B288" t="s">
+        <v>821</v>
+      </c>
+      <c r="C288" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="289" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A289" s="1">
+        <v>46001</v>
+      </c>
+      <c r="B289" t="s">
+        <v>314</v>
+      </c>
+      <c r="C289" t="s">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="290" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A290" s="1">
+        <v>46001</v>
+      </c>
+      <c r="B290" t="s">
+        <v>144</v>
+      </c>
+      <c r="C290" t="s">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="291" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A291" s="1">
+        <v>46001</v>
+      </c>
+      <c r="B291" t="s">
+        <v>823</v>
+      </c>
+      <c r="C291" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="292" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A292" s="1">
+        <v>46001</v>
+      </c>
+      <c r="B292" t="s">
+        <v>831</v>
+      </c>
+      <c r="C292" t="s">
+        <v>97</v>
       </c>
     </row>
   </sheetData>
   <conditionalFormatting sqref="B5">
-    <cfRule type="duplicateValues" dxfId="190" priority="191"/>
-    <cfRule type="duplicateValues" dxfId="189" priority="192"/>
+    <cfRule type="duplicateValues" dxfId="196" priority="204"/>
+    <cfRule type="duplicateValues" dxfId="195" priority="205"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B10">
-    <cfRule type="duplicateValues" dxfId="188" priority="190"/>
-    <cfRule type="duplicateValues" dxfId="187" priority="189"/>
+    <cfRule type="duplicateValues" dxfId="194" priority="203"/>
+    <cfRule type="duplicateValues" dxfId="193" priority="202"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B11">
-    <cfRule type="duplicateValues" dxfId="186" priority="188"/>
-    <cfRule type="duplicateValues" dxfId="185" priority="187"/>
+    <cfRule type="duplicateValues" dxfId="192" priority="201"/>
+    <cfRule type="duplicateValues" dxfId="191" priority="200"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B12">
-    <cfRule type="duplicateValues" dxfId="184" priority="186"/>
-    <cfRule type="duplicateValues" dxfId="183" priority="185"/>
+    <cfRule type="duplicateValues" dxfId="190" priority="199"/>
+    <cfRule type="duplicateValues" dxfId="189" priority="198"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B15">
-    <cfRule type="duplicateValues" dxfId="182" priority="184"/>
-    <cfRule type="duplicateValues" dxfId="181" priority="183"/>
+    <cfRule type="duplicateValues" dxfId="188" priority="196"/>
+    <cfRule type="duplicateValues" dxfId="187" priority="197"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B16">
-    <cfRule type="duplicateValues" dxfId="180" priority="182"/>
+    <cfRule type="duplicateValues" dxfId="186" priority="195"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B17">
-    <cfRule type="duplicateValues" dxfId="179" priority="181"/>
-    <cfRule type="duplicateValues" dxfId="178" priority="180"/>
+    <cfRule type="duplicateValues" dxfId="185" priority="194"/>
+    <cfRule type="duplicateValues" dxfId="184" priority="193"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B18">
-    <cfRule type="duplicateValues" dxfId="177" priority="179"/>
-    <cfRule type="duplicateValues" dxfId="176" priority="178"/>
+    <cfRule type="duplicateValues" dxfId="183" priority="192"/>
+    <cfRule type="duplicateValues" dxfId="182" priority="191"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B19">
-    <cfRule type="duplicateValues" dxfId="175" priority="177"/>
+    <cfRule type="duplicateValues" dxfId="181" priority="190"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B22:B23">
-    <cfRule type="duplicateValues" dxfId="174" priority="176"/>
-    <cfRule type="duplicateValues" dxfId="173" priority="175"/>
+    <cfRule type="duplicateValues" dxfId="180" priority="189"/>
+    <cfRule type="duplicateValues" dxfId="179" priority="188"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B24">
-    <cfRule type="duplicateValues" dxfId="172" priority="174"/>
-    <cfRule type="duplicateValues" dxfId="171" priority="173"/>
+    <cfRule type="duplicateValues" dxfId="178" priority="187"/>
+    <cfRule type="duplicateValues" dxfId="177" priority="186"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B27">
-    <cfRule type="duplicateValues" dxfId="170" priority="172"/>
-    <cfRule type="duplicateValues" dxfId="169" priority="171"/>
+    <cfRule type="duplicateValues" dxfId="176" priority="184"/>
+    <cfRule type="duplicateValues" dxfId="175" priority="185"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B28">
-    <cfRule type="duplicateValues" dxfId="168" priority="170"/>
+    <cfRule type="duplicateValues" dxfId="174" priority="183"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B29">
-    <cfRule type="duplicateValues" dxfId="167" priority="169"/>
-    <cfRule type="duplicateValues" dxfId="166" priority="168"/>
+    <cfRule type="duplicateValues" dxfId="173" priority="181"/>
+    <cfRule type="duplicateValues" dxfId="172" priority="182"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B30">
-    <cfRule type="duplicateValues" dxfId="165" priority="167"/>
+    <cfRule type="duplicateValues" dxfId="171" priority="180"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B31">
-    <cfRule type="duplicateValues" dxfId="164" priority="166"/>
+    <cfRule type="duplicateValues" dxfId="170" priority="179"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B32">
-    <cfRule type="duplicateValues" dxfId="163" priority="165"/>
+    <cfRule type="duplicateValues" dxfId="169" priority="178"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B33">
-    <cfRule type="duplicateValues" dxfId="162" priority="164"/>
+    <cfRule type="duplicateValues" dxfId="168" priority="177"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B34">
-    <cfRule type="duplicateValues" dxfId="161" priority="163"/>
+    <cfRule type="duplicateValues" dxfId="167" priority="176"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B35">
-    <cfRule type="duplicateValues" dxfId="160" priority="162"/>
+    <cfRule type="duplicateValues" dxfId="166" priority="175"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B37">
-    <cfRule type="duplicateValues" dxfId="159" priority="161"/>
+    <cfRule type="duplicateValues" dxfId="165" priority="174"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B38">
-    <cfRule type="duplicateValues" dxfId="158" priority="160"/>
+    <cfRule type="duplicateValues" dxfId="164" priority="173"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B42">
-    <cfRule type="duplicateValues" dxfId="157" priority="159"/>
+    <cfRule type="duplicateValues" dxfId="163" priority="172"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B43">
-    <cfRule type="duplicateValues" dxfId="156" priority="158"/>
+    <cfRule type="duplicateValues" dxfId="162" priority="171"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B44:B45">
-    <cfRule type="duplicateValues" dxfId="155" priority="157"/>
+    <cfRule type="duplicateValues" dxfId="161" priority="170"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B46">
-    <cfRule type="duplicateValues" dxfId="154" priority="156"/>
+    <cfRule type="duplicateValues" dxfId="160" priority="169"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B48">
-    <cfRule type="duplicateValues" dxfId="153" priority="155"/>
+    <cfRule type="duplicateValues" dxfId="159" priority="168"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B49">
-    <cfRule type="duplicateValues" dxfId="152" priority="154"/>
+    <cfRule type="duplicateValues" dxfId="158" priority="167"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B51">
-    <cfRule type="duplicateValues" dxfId="151" priority="153"/>
+    <cfRule type="duplicateValues" dxfId="157" priority="166"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B52">
-    <cfRule type="duplicateValues" dxfId="150" priority="152"/>
+    <cfRule type="duplicateValues" dxfId="156" priority="165"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B58">
-    <cfRule type="duplicateValues" dxfId="149" priority="150"/>
+    <cfRule type="duplicateValues" dxfId="155" priority="163"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B59">
-    <cfRule type="duplicateValues" dxfId="148" priority="148"/>
+    <cfRule type="duplicateValues" dxfId="154" priority="161"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B63">
-    <cfRule type="duplicateValues" dxfId="147" priority="147"/>
+    <cfRule type="duplicateValues" dxfId="153" priority="160"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B64">
-    <cfRule type="duplicateValues" dxfId="146" priority="145"/>
+    <cfRule type="duplicateValues" dxfId="152" priority="158"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B66">
-    <cfRule type="duplicateValues" dxfId="145" priority="144"/>
+    <cfRule type="duplicateValues" dxfId="151" priority="157"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B67">
-    <cfRule type="duplicateValues" dxfId="144" priority="143"/>
-    <cfRule type="duplicateValues" dxfId="143" priority="142"/>
+    <cfRule type="duplicateValues" dxfId="150" priority="155"/>
+    <cfRule type="duplicateValues" dxfId="149" priority="156"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B68">
-    <cfRule type="duplicateValues" dxfId="142" priority="141"/>
+    <cfRule type="duplicateValues" dxfId="148" priority="154"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B69">
-    <cfRule type="duplicateValues" dxfId="141" priority="140"/>
+    <cfRule type="duplicateValues" dxfId="147" priority="153"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B70">
-    <cfRule type="duplicateValues" dxfId="140" priority="138"/>
+    <cfRule type="duplicateValues" dxfId="146" priority="151"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B72">
-    <cfRule type="duplicateValues" dxfId="139" priority="137"/>
+    <cfRule type="duplicateValues" dxfId="145" priority="150"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B73">
-    <cfRule type="duplicateValues" dxfId="138" priority="135"/>
+    <cfRule type="duplicateValues" dxfId="144" priority="148"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B74">
-    <cfRule type="duplicateValues" dxfId="137" priority="134"/>
+    <cfRule type="duplicateValues" dxfId="143" priority="147"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B75">
-    <cfRule type="duplicateValues" dxfId="136" priority="133"/>
+    <cfRule type="duplicateValues" dxfId="142" priority="146"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B76">
-    <cfRule type="duplicateValues" dxfId="135" priority="132"/>
+    <cfRule type="duplicateValues" dxfId="141" priority="145"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B77">
-    <cfRule type="duplicateValues" dxfId="134" priority="130"/>
+    <cfRule type="duplicateValues" dxfId="140" priority="143"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B78">
-    <cfRule type="duplicateValues" dxfId="133" priority="129"/>
+    <cfRule type="duplicateValues" dxfId="139" priority="142"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B83">
-    <cfRule type="duplicateValues" dxfId="132" priority="128"/>
+    <cfRule type="duplicateValues" dxfId="138" priority="141"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B84">
-    <cfRule type="duplicateValues" dxfId="131" priority="127"/>
+    <cfRule type="duplicateValues" dxfId="137" priority="140"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B85">
-    <cfRule type="duplicateValues" dxfId="130" priority="126"/>
+    <cfRule type="duplicateValues" dxfId="136" priority="139"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B87">
-    <cfRule type="duplicateValues" dxfId="129" priority="125"/>
+    <cfRule type="duplicateValues" dxfId="135" priority="138"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B88">
-    <cfRule type="duplicateValues" dxfId="128" priority="124"/>
+    <cfRule type="duplicateValues" dxfId="134" priority="137"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B89">
-    <cfRule type="duplicateValues" dxfId="127" priority="123"/>
+    <cfRule type="duplicateValues" dxfId="133" priority="136"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B90">
-    <cfRule type="duplicateValues" dxfId="126" priority="122"/>
+    <cfRule type="duplicateValues" dxfId="132" priority="135"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B91">
-    <cfRule type="duplicateValues" dxfId="125" priority="121"/>
+    <cfRule type="duplicateValues" dxfId="131" priority="134"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B92">
-    <cfRule type="duplicateValues" dxfId="124" priority="120"/>
+    <cfRule type="duplicateValues" dxfId="130" priority="133"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B93">
-    <cfRule type="duplicateValues" dxfId="123" priority="119"/>
+    <cfRule type="duplicateValues" dxfId="129" priority="132"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B94">
-    <cfRule type="duplicateValues" dxfId="122" priority="118"/>
+    <cfRule type="duplicateValues" dxfId="128" priority="131"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B95">
-    <cfRule type="duplicateValues" dxfId="121" priority="117"/>
+    <cfRule type="duplicateValues" dxfId="127" priority="130"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B96">
-    <cfRule type="duplicateValues" dxfId="120" priority="116"/>
+    <cfRule type="duplicateValues" dxfId="126" priority="129"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B97">
-    <cfRule type="duplicateValues" dxfId="119" priority="115"/>
+    <cfRule type="duplicateValues" dxfId="125" priority="128"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B98">
-    <cfRule type="duplicateValues" dxfId="118" priority="114"/>
+    <cfRule type="duplicateValues" dxfId="124" priority="127"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B99">
-    <cfRule type="duplicateValues" dxfId="117" priority="113"/>
+    <cfRule type="duplicateValues" dxfId="123" priority="126"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B100">
-    <cfRule type="duplicateValues" dxfId="116" priority="112"/>
+    <cfRule type="duplicateValues" dxfId="122" priority="125"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B101">
-    <cfRule type="duplicateValues" dxfId="115" priority="111"/>
+    <cfRule type="duplicateValues" dxfId="121" priority="124"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B104">
-    <cfRule type="duplicateValues" dxfId="114" priority="110"/>
-    <cfRule type="duplicateValues" dxfId="113" priority="109"/>
+    <cfRule type="duplicateValues" dxfId="120" priority="123"/>
+    <cfRule type="duplicateValues" dxfId="119" priority="122"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B105:B106">
-    <cfRule type="duplicateValues" dxfId="112" priority="108"/>
+    <cfRule type="duplicateValues" dxfId="118" priority="121"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B107">
-    <cfRule type="duplicateValues" dxfId="111" priority="107"/>
+    <cfRule type="duplicateValues" dxfId="117" priority="120"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B108">
-    <cfRule type="duplicateValues" dxfId="110" priority="106"/>
+    <cfRule type="duplicateValues" dxfId="116" priority="119"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B109">
-    <cfRule type="duplicateValues" dxfId="109" priority="105"/>
+    <cfRule type="duplicateValues" dxfId="115" priority="118"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B110">
-    <cfRule type="duplicateValues" dxfId="108" priority="104"/>
+    <cfRule type="duplicateValues" dxfId="114" priority="117"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B111">
-    <cfRule type="duplicateValues" dxfId="107" priority="103"/>
+    <cfRule type="duplicateValues" dxfId="113" priority="116"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B112">
-    <cfRule type="duplicateValues" dxfId="106" priority="102"/>
+    <cfRule type="duplicateValues" dxfId="112" priority="115"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B113">
-    <cfRule type="duplicateValues" dxfId="105" priority="101"/>
+    <cfRule type="duplicateValues" dxfId="111" priority="114"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B114">
-    <cfRule type="duplicateValues" dxfId="104" priority="100"/>
+    <cfRule type="duplicateValues" dxfId="110" priority="113"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B115">
-    <cfRule type="duplicateValues" dxfId="103" priority="99"/>
+    <cfRule type="duplicateValues" dxfId="109" priority="112"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B116">
-    <cfRule type="duplicateValues" dxfId="102" priority="98"/>
+    <cfRule type="duplicateValues" dxfId="108" priority="111"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B117">
-    <cfRule type="duplicateValues" dxfId="101" priority="97"/>
+    <cfRule type="duplicateValues" dxfId="107" priority="110"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B118">
-    <cfRule type="duplicateValues" dxfId="100" priority="96"/>
+    <cfRule type="duplicateValues" dxfId="106" priority="109"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B119">
-    <cfRule type="duplicateValues" dxfId="99" priority="95"/>
+    <cfRule type="duplicateValues" dxfId="105" priority="108"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B120">
-    <cfRule type="duplicateValues" dxfId="98" priority="94"/>
+    <cfRule type="duplicateValues" dxfId="104" priority="107"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B121">
-    <cfRule type="duplicateValues" dxfId="97" priority="93"/>
+    <cfRule type="duplicateValues" dxfId="103" priority="106"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B122">
-    <cfRule type="duplicateValues" dxfId="96" priority="92"/>
+    <cfRule type="duplicateValues" dxfId="102" priority="105"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B126">
-    <cfRule type="duplicateValues" dxfId="95" priority="91"/>
+    <cfRule type="duplicateValues" dxfId="101" priority="104"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B127">
-    <cfRule type="duplicateValues" dxfId="94" priority="90"/>
+    <cfRule type="duplicateValues" dxfId="100" priority="103"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B128">
-    <cfRule type="duplicateValues" dxfId="93" priority="89"/>
+    <cfRule type="duplicateValues" dxfId="99" priority="102"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B129">
-    <cfRule type="duplicateValues" dxfId="92" priority="88"/>
+    <cfRule type="duplicateValues" dxfId="98" priority="101"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B130">
-    <cfRule type="duplicateValues" dxfId="91" priority="87"/>
+    <cfRule type="duplicateValues" dxfId="97" priority="100"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B131">
-    <cfRule type="duplicateValues" dxfId="90" priority="86"/>
+    <cfRule type="duplicateValues" dxfId="96" priority="99"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B132">
-    <cfRule type="duplicateValues" dxfId="89" priority="85"/>
+    <cfRule type="duplicateValues" dxfId="95" priority="98"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B133">
-    <cfRule type="duplicateValues" dxfId="88" priority="84"/>
+    <cfRule type="duplicateValues" dxfId="94" priority="97"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B136">
-    <cfRule type="duplicateValues" dxfId="87" priority="83"/>
+    <cfRule type="duplicateValues" dxfId="93" priority="96"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B137">
-    <cfRule type="duplicateValues" dxfId="86" priority="82"/>
+    <cfRule type="duplicateValues" dxfId="92" priority="95"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B138">
-    <cfRule type="duplicateValues" dxfId="85" priority="81"/>
+    <cfRule type="duplicateValues" dxfId="91" priority="94"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B139">
-    <cfRule type="duplicateValues" dxfId="84" priority="80"/>
+    <cfRule type="duplicateValues" dxfId="90" priority="93"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B140">
-    <cfRule type="duplicateValues" dxfId="83" priority="79"/>
+    <cfRule type="duplicateValues" dxfId="89" priority="92"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B141">
-    <cfRule type="duplicateValues" dxfId="82" priority="78"/>
+    <cfRule type="duplicateValues" dxfId="88" priority="91"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B142">
-    <cfRule type="duplicateValues" dxfId="81" priority="77"/>
+    <cfRule type="duplicateValues" dxfId="87" priority="90"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B143">
-    <cfRule type="duplicateValues" dxfId="80" priority="76"/>
+    <cfRule type="duplicateValues" dxfId="86" priority="89"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B144">
-    <cfRule type="duplicateValues" dxfId="79" priority="75"/>
+    <cfRule type="duplicateValues" dxfId="85" priority="88"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B145">
-    <cfRule type="duplicateValues" dxfId="78" priority="74"/>
+    <cfRule type="duplicateValues" dxfId="84" priority="87"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B147">
-    <cfRule type="duplicateValues" dxfId="77" priority="73"/>
+    <cfRule type="duplicateValues" dxfId="83" priority="86"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B148">
-    <cfRule type="duplicateValues" dxfId="76" priority="72"/>
+    <cfRule type="duplicateValues" dxfId="82" priority="85"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B149">
-    <cfRule type="duplicateValues" dxfId="75" priority="71"/>
+    <cfRule type="duplicateValues" dxfId="81" priority="84"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B150">
-    <cfRule type="duplicateValues" dxfId="74" priority="70"/>
+    <cfRule type="duplicateValues" dxfId="80" priority="83"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B151">
-    <cfRule type="duplicateValues" dxfId="73" priority="69"/>
+    <cfRule type="duplicateValues" dxfId="79" priority="82"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B152">
-    <cfRule type="duplicateValues" dxfId="72" priority="68"/>
+    <cfRule type="duplicateValues" dxfId="78" priority="81"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B153">
-    <cfRule type="duplicateValues" dxfId="71" priority="67"/>
+    <cfRule type="duplicateValues" dxfId="77" priority="80"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B154">
-    <cfRule type="duplicateValues" dxfId="70" priority="66"/>
+    <cfRule type="duplicateValues" dxfId="76" priority="79"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B155">
-    <cfRule type="duplicateValues" dxfId="69" priority="65"/>
+    <cfRule type="duplicateValues" dxfId="75" priority="78"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B156">
-    <cfRule type="duplicateValues" dxfId="68" priority="64"/>
+    <cfRule type="duplicateValues" dxfId="74" priority="77"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B157">
-    <cfRule type="duplicateValues" dxfId="67" priority="63"/>
+    <cfRule type="duplicateValues" dxfId="73" priority="76"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B171">
-    <cfRule type="duplicateValues" dxfId="66" priority="62"/>
+    <cfRule type="duplicateValues" dxfId="72" priority="75"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B172">
-    <cfRule type="duplicateValues" dxfId="65" priority="61"/>
+    <cfRule type="duplicateValues" dxfId="71" priority="74"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B174">
-    <cfRule type="duplicateValues" dxfId="64" priority="60"/>
+    <cfRule type="duplicateValues" dxfId="70" priority="73"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B177:B178">
-    <cfRule type="duplicateValues" dxfId="63" priority="59"/>
+    <cfRule type="duplicateValues" dxfId="69" priority="72"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B181">
-    <cfRule type="duplicateValues" dxfId="62" priority="58"/>
+    <cfRule type="duplicateValues" dxfId="68" priority="71"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B182">
-    <cfRule type="duplicateValues" dxfId="61" priority="57"/>
+    <cfRule type="duplicateValues" dxfId="67" priority="70"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B183">
-    <cfRule type="duplicateValues" dxfId="60" priority="56"/>
+    <cfRule type="duplicateValues" dxfId="66" priority="69"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B184">
-    <cfRule type="duplicateValues" dxfId="59" priority="55"/>
+    <cfRule type="duplicateValues" dxfId="65" priority="68"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B185">
-    <cfRule type="duplicateValues" dxfId="58" priority="54"/>
+    <cfRule type="duplicateValues" dxfId="64" priority="67"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B186">
-    <cfRule type="duplicateValues" dxfId="57" priority="53"/>
+    <cfRule type="duplicateValues" dxfId="63" priority="66"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B188">
-    <cfRule type="duplicateValues" dxfId="56" priority="52"/>
+    <cfRule type="duplicateValues" dxfId="62" priority="65"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B189">
-    <cfRule type="duplicateValues" dxfId="55" priority="51"/>
+    <cfRule type="duplicateValues" dxfId="61" priority="64"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B190">
-    <cfRule type="duplicateValues" dxfId="54" priority="50"/>
+    <cfRule type="duplicateValues" dxfId="60" priority="63"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B191">
-    <cfRule type="duplicateValues" dxfId="53" priority="49"/>
+    <cfRule type="duplicateValues" dxfId="59" priority="62"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B192">
-    <cfRule type="duplicateValues" dxfId="52" priority="48"/>
+    <cfRule type="duplicateValues" dxfId="58" priority="61"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B193">
-    <cfRule type="duplicateValues" dxfId="51" priority="47"/>
+    <cfRule type="duplicateValues" dxfId="57" priority="60"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B195">
-    <cfRule type="duplicateValues" dxfId="50" priority="46"/>
+    <cfRule type="duplicateValues" dxfId="56" priority="59"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B196">
-    <cfRule type="duplicateValues" dxfId="49" priority="45"/>
+    <cfRule type="duplicateValues" dxfId="55" priority="58"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B197">
-    <cfRule type="duplicateValues" dxfId="48" priority="44"/>
+    <cfRule type="duplicateValues" dxfId="54" priority="57"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B198">
-    <cfRule type="duplicateValues" dxfId="47" priority="43"/>
+    <cfRule type="duplicateValues" dxfId="53" priority="56"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B199">
-    <cfRule type="duplicateValues" dxfId="46" priority="42"/>
+    <cfRule type="duplicateValues" dxfId="52" priority="55"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B200">
-    <cfRule type="duplicateValues" dxfId="45" priority="41"/>
+    <cfRule type="duplicateValues" dxfId="51" priority="54"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B201">
-    <cfRule type="duplicateValues" dxfId="44" priority="40"/>
+    <cfRule type="duplicateValues" dxfId="50" priority="53"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B202">
-    <cfRule type="duplicateValues" dxfId="43" priority="39"/>
+    <cfRule type="duplicateValues" dxfId="49" priority="52"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B203">
-    <cfRule type="duplicateValues" dxfId="42" priority="38"/>
+    <cfRule type="duplicateValues" dxfId="48" priority="51"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B204">
-    <cfRule type="duplicateValues" dxfId="41" priority="37"/>
+    <cfRule type="duplicateValues" dxfId="47" priority="50"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B205">
-    <cfRule type="duplicateValues" dxfId="40" priority="36"/>
+    <cfRule type="duplicateValues" dxfId="46" priority="49"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B206">
-    <cfRule type="duplicateValues" dxfId="39" priority="35"/>
+    <cfRule type="duplicateValues" dxfId="45" priority="48"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B207">
-    <cfRule type="duplicateValues" dxfId="38" priority="34"/>
+    <cfRule type="duplicateValues" dxfId="44" priority="47"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B215">
-    <cfRule type="duplicateValues" dxfId="37" priority="33"/>
+    <cfRule type="duplicateValues" dxfId="43" priority="46"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B218">
-    <cfRule type="duplicateValues" dxfId="36" priority="32"/>
+    <cfRule type="duplicateValues" dxfId="42" priority="45"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B220">
-    <cfRule type="duplicateValues" dxfId="35" priority="31"/>
+    <cfRule type="duplicateValues" dxfId="41" priority="44"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B222">
-    <cfRule type="duplicateValues" dxfId="34" priority="30"/>
+    <cfRule type="duplicateValues" dxfId="40" priority="43"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B223">
-    <cfRule type="duplicateValues" dxfId="33" priority="29"/>
+    <cfRule type="duplicateValues" dxfId="39" priority="42"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B224">
-    <cfRule type="duplicateValues" dxfId="32" priority="28"/>
+    <cfRule type="duplicateValues" dxfId="38" priority="41"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B225">
-    <cfRule type="duplicateValues" dxfId="31" priority="27"/>
+    <cfRule type="duplicateValues" dxfId="37" priority="40"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B227">
-    <cfRule type="duplicateValues" dxfId="30" priority="26"/>
+    <cfRule type="duplicateValues" dxfId="36" priority="39"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B229">
-    <cfRule type="duplicateValues" dxfId="29" priority="25"/>
+    <cfRule type="duplicateValues" dxfId="35" priority="38"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B230">
-    <cfRule type="duplicateValues" dxfId="28" priority="24"/>
+    <cfRule type="duplicateValues" dxfId="34" priority="37"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B232">
-    <cfRule type="duplicateValues" dxfId="27" priority="23"/>
+    <cfRule type="duplicateValues" dxfId="33" priority="36"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B233">
-    <cfRule type="duplicateValues" dxfId="26" priority="22"/>
+    <cfRule type="duplicateValues" dxfId="32" priority="35"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B234">
-    <cfRule type="duplicateValues" dxfId="25" priority="21"/>
+    <cfRule type="duplicateValues" dxfId="31" priority="34"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B235">
-    <cfRule type="duplicateValues" dxfId="24" priority="20"/>
+    <cfRule type="duplicateValues" dxfId="30" priority="33"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B236">
-    <cfRule type="duplicateValues" dxfId="23" priority="19"/>
+    <cfRule type="duplicateValues" dxfId="29" priority="32"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B237">
-    <cfRule type="duplicateValues" dxfId="22" priority="18"/>
+    <cfRule type="duplicateValues" dxfId="28" priority="31"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B239">
-    <cfRule type="duplicateValues" dxfId="21" priority="16"/>
+    <cfRule type="duplicateValues" dxfId="27" priority="29"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B240">
-    <cfRule type="duplicateValues" dxfId="20" priority="15"/>
+    <cfRule type="duplicateValues" dxfId="26" priority="28"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B241">
-    <cfRule type="duplicateValues" dxfId="19" priority="14"/>
+    <cfRule type="duplicateValues" dxfId="25" priority="27"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B242">
-    <cfRule type="duplicateValues" dxfId="18" priority="13"/>
+    <cfRule type="duplicateValues" dxfId="24" priority="26"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B243">
-    <cfRule type="duplicateValues" dxfId="17" priority="12"/>
+    <cfRule type="duplicateValues" dxfId="23" priority="25"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B250">
-    <cfRule type="duplicateValues" dxfId="16" priority="11"/>
+    <cfRule type="duplicateValues" dxfId="22" priority="24"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B251">
-    <cfRule type="duplicateValues" dxfId="15" priority="10"/>
+    <cfRule type="duplicateValues" dxfId="21" priority="23"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B253">
-    <cfRule type="duplicateValues" dxfId="14" priority="9"/>
+    <cfRule type="duplicateValues" dxfId="20" priority="22"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B255">
-    <cfRule type="duplicateValues" dxfId="13" priority="8"/>
+    <cfRule type="duplicateValues" dxfId="19" priority="21"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B258:B259">
-    <cfRule type="duplicateValues" dxfId="12" priority="7"/>
+    <cfRule type="duplicateValues" dxfId="18" priority="20"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B260">
-    <cfRule type="duplicateValues" dxfId="11" priority="6"/>
+    <cfRule type="duplicateValues" dxfId="17" priority="19"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B265:B267 B269">
-    <cfRule type="duplicateValues" dxfId="10" priority="5"/>
+    <cfRule type="duplicateValues" dxfId="16" priority="18"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B268">
-    <cfRule type="duplicateValues" dxfId="9" priority="4"/>
+    <cfRule type="duplicateValues" dxfId="15" priority="17"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B270">
-    <cfRule type="duplicateValues" dxfId="8" priority="3"/>
+    <cfRule type="duplicateValues" dxfId="14" priority="16"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B271">
-    <cfRule type="duplicateValues" dxfId="7" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="13" priority="15"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B273">
-    <cfRule type="duplicateValues" dxfId="6" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="12" priority="14"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B275">
+    <cfRule type="duplicateValues" dxfId="11" priority="13"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B278">
+    <cfRule type="duplicateValues" dxfId="10" priority="12"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B279">
+    <cfRule type="duplicateValues" dxfId="9" priority="11"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B280">
+    <cfRule type="duplicateValues" dxfId="8" priority="10"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B281">
+    <cfRule type="duplicateValues" dxfId="7" priority="9"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B282">
+    <cfRule type="duplicateValues" dxfId="6" priority="8"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B283">
+    <cfRule type="duplicateValues" dxfId="5" priority="6"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B284:B286">
+    <cfRule type="duplicateValues" dxfId="4" priority="5"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B287">
+    <cfRule type="duplicateValues" dxfId="3" priority="4"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B288">
+    <cfRule type="duplicateValues" dxfId="2" priority="3"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B291">
+    <cfRule type="duplicateValues" dxfId="1" priority="2"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B292">
+    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -53163,15 +54380,15 @@
       </c>
       <c r="B1" s="15">
         <f>COUNTA(sum!A:A) -1</f>
-        <v>267</v>
+        <v>274</v>
       </c>
       <c r="C1" s="22">
         <f>COUNTIF(sum!I:I, "completed")/(B1-COUNTIF(sum!I:I, "abandoned")-COUNTIF(sum!I:I, "late app"))</f>
-        <v>0.94230769230769229</v>
+        <v>0.96254681647940077</v>
       </c>
       <c r="D1" s="21">
         <f>COUNTIF(sum!I:I, "completed")</f>
-        <v>245</v>
+        <v>257</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="22" customHeight="1" x14ac:dyDescent="0.4">
@@ -53206,7 +54423,7 @@
       </c>
       <c r="B5" s="15">
         <f>COUNTA(sum!J:J) -1</f>
-        <v>267</v>
+        <v>274</v>
       </c>
       <c r="C5" s="14">
         <f>B5/B1</f>
@@ -53219,11 +54436,11 @@
       </c>
       <c r="B6" s="16">
         <f>COUNTIFS(sum!J:J,"no news")</f>
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="C6" s="10">
         <f>B6/$B$5</f>
-        <v>0.9550561797752809</v>
+        <v>0.93430656934306566</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.4">
@@ -53232,11 +54449,11 @@
       </c>
       <c r="B7" s="16">
         <f>COUNTIFS(sum!J:J,"rejected")</f>
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="C7" s="10">
         <f t="shared" ref="C7:C10" si="0">B7/$B$5</f>
-        <v>4.1198501872659173E-2</v>
+        <v>4.7445255474452552E-2</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.4">
@@ -53244,12 +54461,12 @@
         <v>404</v>
       </c>
       <c r="B8" s="16">
-        <f>COUNTIFS(sum!J:J,"interview")</f>
-        <v>1</v>
+        <f>COUNTIFS(sum!J:J,"interview") + COUNTIFS(sum!J:J,"fly out") + COUNTIFS(sum!J:J,"offer")</f>
+        <v>5</v>
       </c>
       <c r="C8" s="10">
         <f t="shared" si="0"/>
-        <v>3.7453183520599251E-3</v>
+        <v>1.824817518248175E-2</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.4">
@@ -53257,12 +54474,12 @@
         <v>405</v>
       </c>
       <c r="B9" s="16">
-        <f>COUNTIFS(sum!J:J,"fly out")</f>
-        <v>0</v>
+        <f xml:space="preserve"> COUNTIFS(sum!J:J,"fly out") + COUNTIFS(sum!J:J,"offer")</f>
+        <v>1</v>
       </c>
       <c r="C9" s="10">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>3.6496350364963502E-3</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.4">

</xml_diff>

<commit_message>
added some tips and though I have had during this time
</commit_message>
<xml_diff>
--- a/EconJM_status.xlsx
+++ b/EconJM_status.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\javie\Dropbox\Work\Job Search\2025 EconJM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2472ACC8-6AF5-40ED-BCEE-1A327BB2778B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D80B516F-7A6D-497D-9AA7-E31BF4D26662}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="14620" xr2:uid="{6FE48536-7E5C-BF4C-9490-2A6392576298}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="14620" activeTab="1" xr2:uid="{6FE48536-7E5C-BF4C-9490-2A6392576298}"/>
   </bookViews>
   <sheets>
     <sheet name="sum" sheetId="1" r:id="rId1"/>
@@ -1093,7 +1093,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2767" uniqueCount="872">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2769" uniqueCount="872">
   <si>
     <t>add_id</t>
   </si>
@@ -3926,7 +3926,17 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Percent" xfId="2" builtinId="5"/>
   </cellStyles>
-  <dxfs count="214">
+  <dxfs count="215">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -46569,7 +46579,7 @@
         <v>96</v>
       </c>
       <c r="J187" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="M187" t="s">
         <v>683</v>
@@ -50468,63 +50478,63 @@
     </sortState>
   </autoFilter>
   <conditionalFormatting sqref="A1:B208 A210:B1048576">
-    <cfRule type="duplicateValues" dxfId="213" priority="23"/>
+    <cfRule type="duplicateValues" dxfId="214" priority="23"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A2:B22">
-    <cfRule type="duplicateValues" dxfId="212" priority="24"/>
+    <cfRule type="duplicateValues" dxfId="213" priority="24"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A61:B61">
-    <cfRule type="duplicateValues" dxfId="211" priority="22"/>
+    <cfRule type="duplicateValues" dxfId="212" priority="22"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="I1:I1048576">
-    <cfRule type="containsText" dxfId="210" priority="15" operator="containsText" text="closed">
+    <cfRule type="containsText" dxfId="211" priority="15" operator="containsText" text="closed">
       <formula>NOT(ISERROR(SEARCH("closed",I1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="209" priority="16" operator="containsText" text="abandoned">
+    <cfRule type="containsText" dxfId="210" priority="16" operator="containsText" text="abandoned">
       <formula>NOT(ISERROR(SEARCH("abandoned",I1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="208" priority="18" operator="containsText" text="late app">
+    <cfRule type="containsText" dxfId="209" priority="18" operator="containsText" text="late app">
       <formula>NOT(ISERROR(SEARCH("late app",I1)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I2:L1048576 O78:O80 O83:O89 O92:O112 O115:O124 O126:O181 R136 R153 R159 R166 R173 R178 O183:O205 O208:O211 O213:O218 O220:O233 R225 O235:O237 O239:O248 I1:J1">
-    <cfRule type="containsText" dxfId="207" priority="21" operator="containsText" text="completed">
+    <cfRule type="containsText" dxfId="208" priority="21" operator="containsText" text="completed">
       <formula>NOT(ISERROR(SEARCH("completed",I1)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J1:J1048576">
-    <cfRule type="containsText" dxfId="206" priority="10" operator="containsText" text="no news">
+    <cfRule type="containsText" dxfId="207" priority="10" operator="containsText" text="no news">
       <formula>NOT(ISERROR(SEARCH("no news",J1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="205" priority="11" operator="containsText" text="offer">
+    <cfRule type="containsText" dxfId="206" priority="11" operator="containsText" text="offer">
       <formula>NOT(ISERROR(SEARCH("offer",J1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="204" priority="12" operator="containsText" text="fly out">
+    <cfRule type="containsText" dxfId="205" priority="12" operator="containsText" text="fly out">
       <formula>NOT(ISERROR(SEARCH("fly out",J1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="203" priority="13" operator="containsText" text="interview">
+    <cfRule type="containsText" dxfId="204" priority="13" operator="containsText" text="interview">
       <formula>NOT(ISERROR(SEARCH("interview",J1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="202" priority="14" operator="containsText" text="rejected">
+    <cfRule type="containsText" dxfId="203" priority="14" operator="containsText" text="rejected">
       <formula>NOT(ISERROR(SEARCH("rejected",J1)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K1:L1048576 O78:O80 O83:O89 O92:O112 O115:O124 O126:O181 R136 R153 R159 R166 R173 R178 O183:O205 O208:O211 O213:O218 O220:O233 R225 O235:O237 O239:O248">
-    <cfRule type="containsText" dxfId="201" priority="19" operator="containsText" text="NO">
+    <cfRule type="containsText" dxfId="202" priority="19" operator="containsText" text="NO">
       <formula>NOT(ISERROR(SEARCH("NO",K1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="200" priority="20" operator="containsText" text="YES">
+    <cfRule type="containsText" dxfId="201" priority="20" operator="containsText" text="YES">
       <formula>NOT(ISERROR(SEARCH("YES",K1)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="O250:O267">
-    <cfRule type="containsText" dxfId="199" priority="1" operator="containsText" text="NO">
+    <cfRule type="containsText" dxfId="200" priority="1" operator="containsText" text="NO">
       <formula>NOT(ISERROR(SEARCH("NO",O250)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="198" priority="2" operator="containsText" text="YES">
+    <cfRule type="containsText" dxfId="199" priority="2" operator="containsText" text="YES">
       <formula>NOT(ISERROR(SEARCH("YES",O250)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="197" priority="3" operator="containsText" text="completed">
+    <cfRule type="containsText" dxfId="198" priority="3" operator="containsText" text="completed">
       <formula>NOT(ISERROR(SEARCH("completed",O250)))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -50646,7 +50656,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{923E81FA-B875-3C4E-A189-1A21268FA086}">
-  <dimension ref="A1:C292"/>
+  <dimension ref="A1:C293"/>
   <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="16" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="32.83203125" customWidth="1"/>
@@ -53794,570 +53804,584 @@
         <v>97</v>
       </c>
     </row>
+    <row r="293" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A293" s="1">
+        <v>46001</v>
+      </c>
+      <c r="B293" t="s">
+        <v>682</v>
+      </c>
+      <c r="C293" t="s">
+        <v>403</v>
+      </c>
+    </row>
   </sheetData>
   <conditionalFormatting sqref="B5">
-    <cfRule type="duplicateValues" dxfId="196" priority="204"/>
-    <cfRule type="duplicateValues" dxfId="195" priority="205"/>
+    <cfRule type="duplicateValues" dxfId="197" priority="205"/>
+    <cfRule type="duplicateValues" dxfId="196" priority="206"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B10">
+    <cfRule type="duplicateValues" dxfId="195" priority="204"/>
     <cfRule type="duplicateValues" dxfId="194" priority="203"/>
-    <cfRule type="duplicateValues" dxfId="193" priority="202"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B11">
+    <cfRule type="duplicateValues" dxfId="193" priority="202"/>
     <cfRule type="duplicateValues" dxfId="192" priority="201"/>
-    <cfRule type="duplicateValues" dxfId="191" priority="200"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B12">
+    <cfRule type="duplicateValues" dxfId="191" priority="200"/>
     <cfRule type="duplicateValues" dxfId="190" priority="199"/>
-    <cfRule type="duplicateValues" dxfId="189" priority="198"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B15">
-    <cfRule type="duplicateValues" dxfId="188" priority="196"/>
-    <cfRule type="duplicateValues" dxfId="187" priority="197"/>
+    <cfRule type="duplicateValues" dxfId="189" priority="198"/>
+    <cfRule type="duplicateValues" dxfId="188" priority="197"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B16">
-    <cfRule type="duplicateValues" dxfId="186" priority="195"/>
+    <cfRule type="duplicateValues" dxfId="187" priority="196"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B17">
-    <cfRule type="duplicateValues" dxfId="185" priority="194"/>
-    <cfRule type="duplicateValues" dxfId="184" priority="193"/>
+    <cfRule type="duplicateValues" dxfId="186" priority="194"/>
+    <cfRule type="duplicateValues" dxfId="185" priority="195"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B18">
+    <cfRule type="duplicateValues" dxfId="184" priority="193"/>
     <cfRule type="duplicateValues" dxfId="183" priority="192"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B19">
     <cfRule type="duplicateValues" dxfId="182" priority="191"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B19">
+  <conditionalFormatting sqref="B22:B23">
     <cfRule type="duplicateValues" dxfId="181" priority="190"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B22:B23">
     <cfRule type="duplicateValues" dxfId="180" priority="189"/>
-    <cfRule type="duplicateValues" dxfId="179" priority="188"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B24">
+    <cfRule type="duplicateValues" dxfId="179" priority="188"/>
     <cfRule type="duplicateValues" dxfId="178" priority="187"/>
-    <cfRule type="duplicateValues" dxfId="177" priority="186"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B27">
-    <cfRule type="duplicateValues" dxfId="176" priority="184"/>
-    <cfRule type="duplicateValues" dxfId="175" priority="185"/>
+    <cfRule type="duplicateValues" dxfId="177" priority="186"/>
+    <cfRule type="duplicateValues" dxfId="176" priority="185"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B28">
-    <cfRule type="duplicateValues" dxfId="174" priority="183"/>
+    <cfRule type="duplicateValues" dxfId="175" priority="184"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B29">
-    <cfRule type="duplicateValues" dxfId="173" priority="181"/>
-    <cfRule type="duplicateValues" dxfId="172" priority="182"/>
+    <cfRule type="duplicateValues" dxfId="174" priority="182"/>
+    <cfRule type="duplicateValues" dxfId="173" priority="183"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B30">
+    <cfRule type="duplicateValues" dxfId="172" priority="181"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B31">
     <cfRule type="duplicateValues" dxfId="171" priority="180"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B31">
+  <conditionalFormatting sqref="B32">
     <cfRule type="duplicateValues" dxfId="170" priority="179"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B32">
+  <conditionalFormatting sqref="B33">
     <cfRule type="duplicateValues" dxfId="169" priority="178"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B33">
+  <conditionalFormatting sqref="B34">
     <cfRule type="duplicateValues" dxfId="168" priority="177"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B34">
+  <conditionalFormatting sqref="B35">
     <cfRule type="duplicateValues" dxfId="167" priority="176"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B35">
+  <conditionalFormatting sqref="B37">
     <cfRule type="duplicateValues" dxfId="166" priority="175"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B37">
+  <conditionalFormatting sqref="B38">
     <cfRule type="duplicateValues" dxfId="165" priority="174"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B38">
+  <conditionalFormatting sqref="B42">
     <cfRule type="duplicateValues" dxfId="164" priority="173"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B42">
+  <conditionalFormatting sqref="B43">
     <cfRule type="duplicateValues" dxfId="163" priority="172"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B43">
+  <conditionalFormatting sqref="B44:B45">
     <cfRule type="duplicateValues" dxfId="162" priority="171"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B44:B45">
+  <conditionalFormatting sqref="B46">
     <cfRule type="duplicateValues" dxfId="161" priority="170"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B46">
+  <conditionalFormatting sqref="B48">
     <cfRule type="duplicateValues" dxfId="160" priority="169"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B48">
+  <conditionalFormatting sqref="B49">
     <cfRule type="duplicateValues" dxfId="159" priority="168"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B49">
+  <conditionalFormatting sqref="B51">
     <cfRule type="duplicateValues" dxfId="158" priority="167"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B51">
+  <conditionalFormatting sqref="B52">
     <cfRule type="duplicateValues" dxfId="157" priority="166"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B52">
-    <cfRule type="duplicateValues" dxfId="156" priority="165"/>
-  </conditionalFormatting>
   <conditionalFormatting sqref="B58">
-    <cfRule type="duplicateValues" dxfId="155" priority="163"/>
+    <cfRule type="duplicateValues" dxfId="156" priority="164"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B59">
+    <cfRule type="duplicateValues" dxfId="155" priority="162"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B63">
     <cfRule type="duplicateValues" dxfId="154" priority="161"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B63">
-    <cfRule type="duplicateValues" dxfId="153" priority="160"/>
+  <conditionalFormatting sqref="B64">
+    <cfRule type="duplicateValues" dxfId="153" priority="159"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B64">
+  <conditionalFormatting sqref="B66">
     <cfRule type="duplicateValues" dxfId="152" priority="158"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B66">
+  <conditionalFormatting sqref="B67">
     <cfRule type="duplicateValues" dxfId="151" priority="157"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B67">
-    <cfRule type="duplicateValues" dxfId="150" priority="155"/>
-    <cfRule type="duplicateValues" dxfId="149" priority="156"/>
+    <cfRule type="duplicateValues" dxfId="150" priority="156"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B68">
+    <cfRule type="duplicateValues" dxfId="149" priority="155"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B69">
     <cfRule type="duplicateValues" dxfId="148" priority="154"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B69">
-    <cfRule type="duplicateValues" dxfId="147" priority="153"/>
+  <conditionalFormatting sqref="B70">
+    <cfRule type="duplicateValues" dxfId="147" priority="152"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B70">
+  <conditionalFormatting sqref="B72">
     <cfRule type="duplicateValues" dxfId="146" priority="151"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B72">
-    <cfRule type="duplicateValues" dxfId="145" priority="150"/>
+  <conditionalFormatting sqref="B73">
+    <cfRule type="duplicateValues" dxfId="145" priority="149"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B73">
+  <conditionalFormatting sqref="B74">
     <cfRule type="duplicateValues" dxfId="144" priority="148"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B74">
+  <conditionalFormatting sqref="B75">
     <cfRule type="duplicateValues" dxfId="143" priority="147"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B75">
+  <conditionalFormatting sqref="B76">
     <cfRule type="duplicateValues" dxfId="142" priority="146"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B76">
-    <cfRule type="duplicateValues" dxfId="141" priority="145"/>
+  <conditionalFormatting sqref="B77">
+    <cfRule type="duplicateValues" dxfId="141" priority="144"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B77">
+  <conditionalFormatting sqref="B78">
     <cfRule type="duplicateValues" dxfId="140" priority="143"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B78">
+  <conditionalFormatting sqref="B83">
     <cfRule type="duplicateValues" dxfId="139" priority="142"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B83">
+  <conditionalFormatting sqref="B84">
     <cfRule type="duplicateValues" dxfId="138" priority="141"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B84">
+  <conditionalFormatting sqref="B85">
     <cfRule type="duplicateValues" dxfId="137" priority="140"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B85">
+  <conditionalFormatting sqref="B87">
     <cfRule type="duplicateValues" dxfId="136" priority="139"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B87">
+  <conditionalFormatting sqref="B88">
     <cfRule type="duplicateValues" dxfId="135" priority="138"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B88">
+  <conditionalFormatting sqref="B89">
     <cfRule type="duplicateValues" dxfId="134" priority="137"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B89">
+  <conditionalFormatting sqref="B90">
     <cfRule type="duplicateValues" dxfId="133" priority="136"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B90">
+  <conditionalFormatting sqref="B91">
     <cfRule type="duplicateValues" dxfId="132" priority="135"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B91">
+  <conditionalFormatting sqref="B92">
     <cfRule type="duplicateValues" dxfId="131" priority="134"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B92">
+  <conditionalFormatting sqref="B93">
     <cfRule type="duplicateValues" dxfId="130" priority="133"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B93">
+  <conditionalFormatting sqref="B94">
     <cfRule type="duplicateValues" dxfId="129" priority="132"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B94">
+  <conditionalFormatting sqref="B95">
     <cfRule type="duplicateValues" dxfId="128" priority="131"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B95">
+  <conditionalFormatting sqref="B96">
     <cfRule type="duplicateValues" dxfId="127" priority="130"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B96">
+  <conditionalFormatting sqref="B97">
     <cfRule type="duplicateValues" dxfId="126" priority="129"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B97">
+  <conditionalFormatting sqref="B98">
     <cfRule type="duplicateValues" dxfId="125" priority="128"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B98">
+  <conditionalFormatting sqref="B99">
     <cfRule type="duplicateValues" dxfId="124" priority="127"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B99">
+  <conditionalFormatting sqref="B100">
     <cfRule type="duplicateValues" dxfId="123" priority="126"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B100">
+  <conditionalFormatting sqref="B101">
     <cfRule type="duplicateValues" dxfId="122" priority="125"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B101">
+  <conditionalFormatting sqref="B104">
     <cfRule type="duplicateValues" dxfId="121" priority="124"/>
+    <cfRule type="duplicateValues" dxfId="120" priority="123"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B104">
-    <cfRule type="duplicateValues" dxfId="120" priority="123"/>
+  <conditionalFormatting sqref="B105:B106">
     <cfRule type="duplicateValues" dxfId="119" priority="122"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B105:B106">
+  <conditionalFormatting sqref="B107">
     <cfRule type="duplicateValues" dxfId="118" priority="121"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B107">
+  <conditionalFormatting sqref="B108">
     <cfRule type="duplicateValues" dxfId="117" priority="120"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B108">
+  <conditionalFormatting sqref="B109">
     <cfRule type="duplicateValues" dxfId="116" priority="119"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B109">
+  <conditionalFormatting sqref="B110">
     <cfRule type="duplicateValues" dxfId="115" priority="118"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B110">
+  <conditionalFormatting sqref="B111">
     <cfRule type="duplicateValues" dxfId="114" priority="117"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B111">
+  <conditionalFormatting sqref="B112">
     <cfRule type="duplicateValues" dxfId="113" priority="116"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B112">
+  <conditionalFormatting sqref="B113">
     <cfRule type="duplicateValues" dxfId="112" priority="115"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B113">
+  <conditionalFormatting sqref="B114">
     <cfRule type="duplicateValues" dxfId="111" priority="114"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B114">
+  <conditionalFormatting sqref="B115">
     <cfRule type="duplicateValues" dxfId="110" priority="113"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B115">
+  <conditionalFormatting sqref="B116">
     <cfRule type="duplicateValues" dxfId="109" priority="112"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B116">
+  <conditionalFormatting sqref="B117">
     <cfRule type="duplicateValues" dxfId="108" priority="111"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B117">
+  <conditionalFormatting sqref="B118">
     <cfRule type="duplicateValues" dxfId="107" priority="110"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B118">
+  <conditionalFormatting sqref="B119">
     <cfRule type="duplicateValues" dxfId="106" priority="109"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B119">
+  <conditionalFormatting sqref="B120">
     <cfRule type="duplicateValues" dxfId="105" priority="108"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B120">
+  <conditionalFormatting sqref="B121">
     <cfRule type="duplicateValues" dxfId="104" priority="107"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B121">
+  <conditionalFormatting sqref="B122">
     <cfRule type="duplicateValues" dxfId="103" priority="106"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B122">
+  <conditionalFormatting sqref="B126">
     <cfRule type="duplicateValues" dxfId="102" priority="105"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B126">
+  <conditionalFormatting sqref="B127">
     <cfRule type="duplicateValues" dxfId="101" priority="104"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B127">
+  <conditionalFormatting sqref="B128">
     <cfRule type="duplicateValues" dxfId="100" priority="103"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B128">
+  <conditionalFormatting sqref="B129">
     <cfRule type="duplicateValues" dxfId="99" priority="102"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B129">
+  <conditionalFormatting sqref="B130">
     <cfRule type="duplicateValues" dxfId="98" priority="101"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B130">
+  <conditionalFormatting sqref="B131">
     <cfRule type="duplicateValues" dxfId="97" priority="100"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B131">
+  <conditionalFormatting sqref="B132">
     <cfRule type="duplicateValues" dxfId="96" priority="99"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B132">
+  <conditionalFormatting sqref="B133">
     <cfRule type="duplicateValues" dxfId="95" priority="98"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B133">
+  <conditionalFormatting sqref="B136">
     <cfRule type="duplicateValues" dxfId="94" priority="97"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B136">
+  <conditionalFormatting sqref="B137">
     <cfRule type="duplicateValues" dxfId="93" priority="96"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B137">
+  <conditionalFormatting sqref="B138">
     <cfRule type="duplicateValues" dxfId="92" priority="95"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B138">
+  <conditionalFormatting sqref="B139">
     <cfRule type="duplicateValues" dxfId="91" priority="94"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B139">
+  <conditionalFormatting sqref="B140">
     <cfRule type="duplicateValues" dxfId="90" priority="93"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B140">
+  <conditionalFormatting sqref="B141">
     <cfRule type="duplicateValues" dxfId="89" priority="92"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B141">
+  <conditionalFormatting sqref="B142">
     <cfRule type="duplicateValues" dxfId="88" priority="91"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B142">
+  <conditionalFormatting sqref="B143">
     <cfRule type="duplicateValues" dxfId="87" priority="90"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B143">
+  <conditionalFormatting sqref="B144">
     <cfRule type="duplicateValues" dxfId="86" priority="89"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B144">
+  <conditionalFormatting sqref="B145">
     <cfRule type="duplicateValues" dxfId="85" priority="88"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B145">
+  <conditionalFormatting sqref="B147">
     <cfRule type="duplicateValues" dxfId="84" priority="87"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B147">
+  <conditionalFormatting sqref="B148">
     <cfRule type="duplicateValues" dxfId="83" priority="86"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B148">
+  <conditionalFormatting sqref="B149">
     <cfRule type="duplicateValues" dxfId="82" priority="85"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B149">
+  <conditionalFormatting sqref="B150">
     <cfRule type="duplicateValues" dxfId="81" priority="84"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B150">
+  <conditionalFormatting sqref="B151">
     <cfRule type="duplicateValues" dxfId="80" priority="83"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B151">
+  <conditionalFormatting sqref="B152">
     <cfRule type="duplicateValues" dxfId="79" priority="82"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B152">
+  <conditionalFormatting sqref="B153">
     <cfRule type="duplicateValues" dxfId="78" priority="81"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B153">
+  <conditionalFormatting sqref="B154">
     <cfRule type="duplicateValues" dxfId="77" priority="80"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B154">
+  <conditionalFormatting sqref="B155">
     <cfRule type="duplicateValues" dxfId="76" priority="79"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B155">
+  <conditionalFormatting sqref="B156">
     <cfRule type="duplicateValues" dxfId="75" priority="78"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B156">
+  <conditionalFormatting sqref="B157">
     <cfRule type="duplicateValues" dxfId="74" priority="77"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B157">
+  <conditionalFormatting sqref="B171">
     <cfRule type="duplicateValues" dxfId="73" priority="76"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B171">
+  <conditionalFormatting sqref="B172">
     <cfRule type="duplicateValues" dxfId="72" priority="75"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B172">
+  <conditionalFormatting sqref="B174">
     <cfRule type="duplicateValues" dxfId="71" priority="74"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B174">
+  <conditionalFormatting sqref="B177:B178">
     <cfRule type="duplicateValues" dxfId="70" priority="73"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B177:B178">
+  <conditionalFormatting sqref="B181">
     <cfRule type="duplicateValues" dxfId="69" priority="72"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B181">
+  <conditionalFormatting sqref="B182">
     <cfRule type="duplicateValues" dxfId="68" priority="71"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B182">
+  <conditionalFormatting sqref="B183">
     <cfRule type="duplicateValues" dxfId="67" priority="70"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B183">
+  <conditionalFormatting sqref="B184">
     <cfRule type="duplicateValues" dxfId="66" priority="69"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B184">
+  <conditionalFormatting sqref="B185">
     <cfRule type="duplicateValues" dxfId="65" priority="68"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B185">
+  <conditionalFormatting sqref="B186">
     <cfRule type="duplicateValues" dxfId="64" priority="67"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B186">
+  <conditionalFormatting sqref="B188">
     <cfRule type="duplicateValues" dxfId="63" priority="66"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B188">
+  <conditionalFormatting sqref="B189">
     <cfRule type="duplicateValues" dxfId="62" priority="65"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B189">
+  <conditionalFormatting sqref="B190">
     <cfRule type="duplicateValues" dxfId="61" priority="64"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B190">
+  <conditionalFormatting sqref="B191">
     <cfRule type="duplicateValues" dxfId="60" priority="63"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B191">
+  <conditionalFormatting sqref="B192">
     <cfRule type="duplicateValues" dxfId="59" priority="62"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B192">
+  <conditionalFormatting sqref="B193">
     <cfRule type="duplicateValues" dxfId="58" priority="61"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B193">
+  <conditionalFormatting sqref="B195">
     <cfRule type="duplicateValues" dxfId="57" priority="60"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B195">
+  <conditionalFormatting sqref="B196">
     <cfRule type="duplicateValues" dxfId="56" priority="59"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B196">
+  <conditionalFormatting sqref="B197">
     <cfRule type="duplicateValues" dxfId="55" priority="58"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B197">
+  <conditionalFormatting sqref="B198">
     <cfRule type="duplicateValues" dxfId="54" priority="57"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B198">
+  <conditionalFormatting sqref="B199">
     <cfRule type="duplicateValues" dxfId="53" priority="56"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B199">
+  <conditionalFormatting sqref="B200">
     <cfRule type="duplicateValues" dxfId="52" priority="55"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B200">
+  <conditionalFormatting sqref="B201">
     <cfRule type="duplicateValues" dxfId="51" priority="54"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B201">
+  <conditionalFormatting sqref="B202">
     <cfRule type="duplicateValues" dxfId="50" priority="53"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B202">
+  <conditionalFormatting sqref="B203">
     <cfRule type="duplicateValues" dxfId="49" priority="52"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B203">
+  <conditionalFormatting sqref="B204">
     <cfRule type="duplicateValues" dxfId="48" priority="51"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B204">
+  <conditionalFormatting sqref="B205">
     <cfRule type="duplicateValues" dxfId="47" priority="50"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B205">
+  <conditionalFormatting sqref="B206">
     <cfRule type="duplicateValues" dxfId="46" priority="49"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B206">
+  <conditionalFormatting sqref="B207">
     <cfRule type="duplicateValues" dxfId="45" priority="48"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B207">
+  <conditionalFormatting sqref="B215">
     <cfRule type="duplicateValues" dxfId="44" priority="47"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B215">
+  <conditionalFormatting sqref="B218">
     <cfRule type="duplicateValues" dxfId="43" priority="46"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B218">
+  <conditionalFormatting sqref="B220">
     <cfRule type="duplicateValues" dxfId="42" priority="45"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B220">
+  <conditionalFormatting sqref="B222">
     <cfRule type="duplicateValues" dxfId="41" priority="44"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B222">
+  <conditionalFormatting sqref="B223">
     <cfRule type="duplicateValues" dxfId="40" priority="43"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B223">
+  <conditionalFormatting sqref="B224">
     <cfRule type="duplicateValues" dxfId="39" priority="42"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B224">
+  <conditionalFormatting sqref="B225">
     <cfRule type="duplicateValues" dxfId="38" priority="41"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B225">
+  <conditionalFormatting sqref="B227">
     <cfRule type="duplicateValues" dxfId="37" priority="40"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B227">
+  <conditionalFormatting sqref="B229">
     <cfRule type="duplicateValues" dxfId="36" priority="39"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B229">
+  <conditionalFormatting sqref="B230">
     <cfRule type="duplicateValues" dxfId="35" priority="38"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B230">
+  <conditionalFormatting sqref="B232">
     <cfRule type="duplicateValues" dxfId="34" priority="37"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B232">
+  <conditionalFormatting sqref="B233">
     <cfRule type="duplicateValues" dxfId="33" priority="36"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B233">
+  <conditionalFormatting sqref="B234">
     <cfRule type="duplicateValues" dxfId="32" priority="35"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B234">
+  <conditionalFormatting sqref="B235">
     <cfRule type="duplicateValues" dxfId="31" priority="34"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B235">
+  <conditionalFormatting sqref="B236">
     <cfRule type="duplicateValues" dxfId="30" priority="33"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B236">
+  <conditionalFormatting sqref="B237">
     <cfRule type="duplicateValues" dxfId="29" priority="32"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B237">
-    <cfRule type="duplicateValues" dxfId="28" priority="31"/>
+  <conditionalFormatting sqref="B239">
+    <cfRule type="duplicateValues" dxfId="28" priority="30"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B239">
+  <conditionalFormatting sqref="B240">
     <cfRule type="duplicateValues" dxfId="27" priority="29"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B240">
+  <conditionalFormatting sqref="B241">
     <cfRule type="duplicateValues" dxfId="26" priority="28"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B241">
+  <conditionalFormatting sqref="B242">
     <cfRule type="duplicateValues" dxfId="25" priority="27"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B242">
+  <conditionalFormatting sqref="B243">
     <cfRule type="duplicateValues" dxfId="24" priority="26"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B243">
+  <conditionalFormatting sqref="B250">
     <cfRule type="duplicateValues" dxfId="23" priority="25"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B250">
+  <conditionalFormatting sqref="B251">
     <cfRule type="duplicateValues" dxfId="22" priority="24"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B251">
+  <conditionalFormatting sqref="B253">
     <cfRule type="duplicateValues" dxfId="21" priority="23"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B253">
+  <conditionalFormatting sqref="B255">
     <cfRule type="duplicateValues" dxfId="20" priority="22"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B255">
+  <conditionalFormatting sqref="B258:B259">
     <cfRule type="duplicateValues" dxfId="19" priority="21"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B258:B259">
+  <conditionalFormatting sqref="B260">
     <cfRule type="duplicateValues" dxfId="18" priority="20"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B260">
+  <conditionalFormatting sqref="B265:B267 B269">
     <cfRule type="duplicateValues" dxfId="17" priority="19"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B265:B267 B269">
+  <conditionalFormatting sqref="B268">
     <cfRule type="duplicateValues" dxfId="16" priority="18"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B268">
+  <conditionalFormatting sqref="B270">
     <cfRule type="duplicateValues" dxfId="15" priority="17"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B270">
+  <conditionalFormatting sqref="B271">
     <cfRule type="duplicateValues" dxfId="14" priority="16"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B271">
+  <conditionalFormatting sqref="B273">
     <cfRule type="duplicateValues" dxfId="13" priority="15"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B273">
+  <conditionalFormatting sqref="B275">
     <cfRule type="duplicateValues" dxfId="12" priority="14"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B275">
+  <conditionalFormatting sqref="B278">
     <cfRule type="duplicateValues" dxfId="11" priority="13"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B278">
+  <conditionalFormatting sqref="B279">
     <cfRule type="duplicateValues" dxfId="10" priority="12"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B279">
+  <conditionalFormatting sqref="B280">
     <cfRule type="duplicateValues" dxfId="9" priority="11"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B280">
+  <conditionalFormatting sqref="B281">
     <cfRule type="duplicateValues" dxfId="8" priority="10"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B281">
+  <conditionalFormatting sqref="B282">
     <cfRule type="duplicateValues" dxfId="7" priority="9"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B282">
-    <cfRule type="duplicateValues" dxfId="6" priority="8"/>
+  <conditionalFormatting sqref="B283">
+    <cfRule type="duplicateValues" dxfId="6" priority="7"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B283">
+  <conditionalFormatting sqref="B284:B286">
     <cfRule type="duplicateValues" dxfId="5" priority="6"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B284:B286">
+  <conditionalFormatting sqref="B287">
     <cfRule type="duplicateValues" dxfId="4" priority="5"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B287">
+  <conditionalFormatting sqref="B288">
     <cfRule type="duplicateValues" dxfId="3" priority="4"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B288">
+  <conditionalFormatting sqref="B291">
     <cfRule type="duplicateValues" dxfId="2" priority="3"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B291">
+  <conditionalFormatting sqref="B292">
     <cfRule type="duplicateValues" dxfId="1" priority="2"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B292">
+  <conditionalFormatting sqref="B293">
     <cfRule type="duplicateValues" dxfId="0" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -54436,11 +54460,11 @@
       </c>
       <c r="B6" s="16">
         <f>COUNTIFS(sum!J:J,"no news")</f>
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="C6" s="10">
         <f>B6/$B$5</f>
-        <v>0.93430656934306566</v>
+        <v>0.93065693430656937</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.4">
@@ -54449,11 +54473,11 @@
       </c>
       <c r="B7" s="16">
         <f>COUNTIFS(sum!J:J,"rejected")</f>
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C7" s="10">
         <f t="shared" ref="C7:C10" si="0">B7/$B$5</f>
-        <v>4.7445255474452552E-2</v>
+        <v>5.1094890510948905E-2</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.4">

</xml_diff>

<commit_message>
cleaned up the writing of the thoughs
</commit_message>
<xml_diff>
--- a/EconJM_status.xlsx
+++ b/EconJM_status.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\javie\Dropbox\Work\Job Search\2025 EconJM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E27037DE-BB5E-4FF5-A759-F0B52699730A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D04130B4-A7A5-4357-BA59-A6B368A572B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="14620" activeTab="2" xr2:uid="{6FE48536-7E5C-BF4C-9490-2A6392576298}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="14620" activeTab="1" xr2:uid="{6FE48536-7E5C-BF4C-9490-2A6392576298}"/>
   </bookViews>
   <sheets>
     <sheet name="sum" sheetId="1" r:id="rId1"/>
@@ -428,7 +428,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2808" uniqueCount="880">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2814" uniqueCount="880">
   <si>
     <t>add_id</t>
   </si>
@@ -3285,7 +3285,17 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Percent" xfId="2" builtinId="5"/>
   </cellStyles>
-  <dxfs count="227">
+  <dxfs count="228">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -44688,7 +44698,7 @@
         <v>96</v>
       </c>
       <c r="J179" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="K179" t="s">
         <v>309</v>
@@ -47269,7 +47279,7 @@
         <v>96</v>
       </c>
       <c r="J233" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="K233" t="s">
         <v>309</v>
@@ -49398,63 +49408,63 @@
     </sortState>
   </autoFilter>
   <conditionalFormatting sqref="A1:B208 A210:B1048576">
-    <cfRule type="duplicateValues" dxfId="226" priority="23"/>
+    <cfRule type="duplicateValues" dxfId="227" priority="23"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A2:B22">
-    <cfRule type="duplicateValues" dxfId="225" priority="24"/>
+    <cfRule type="duplicateValues" dxfId="226" priority="24"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A61:B61">
-    <cfRule type="duplicateValues" dxfId="224" priority="22"/>
+    <cfRule type="duplicateValues" dxfId="225" priority="22"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="I1:I1048576">
-    <cfRule type="containsText" dxfId="223" priority="15" operator="containsText" text="closed">
+    <cfRule type="containsText" dxfId="224" priority="15" operator="containsText" text="closed">
       <formula>NOT(ISERROR(SEARCH("closed",I1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="222" priority="16" operator="containsText" text="abandoned">
+    <cfRule type="containsText" dxfId="223" priority="16" operator="containsText" text="abandoned">
       <formula>NOT(ISERROR(SEARCH("abandoned",I1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="221" priority="18" operator="containsText" text="late app">
+    <cfRule type="containsText" dxfId="222" priority="18" operator="containsText" text="late app">
       <formula>NOT(ISERROR(SEARCH("late app",I1)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I2:L1048576 P78:P80 P83:P89 P92:P112 P115:P124 P126:P181 S136 S153 S159 S166 S173 S178 P183:P205 P208:P211 P213:P218 P220:P233 S225 P235:P237 P239:P248 P276 R276 I1:J1">
-    <cfRule type="containsText" dxfId="220" priority="21" operator="containsText" text="completed">
+    <cfRule type="containsText" dxfId="221" priority="21" operator="containsText" text="completed">
       <formula>NOT(ISERROR(SEARCH("completed",I1)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J1:J1048576">
-    <cfRule type="containsText" dxfId="219" priority="10" operator="containsText" text="no news">
+    <cfRule type="containsText" dxfId="220" priority="10" operator="containsText" text="no news">
       <formula>NOT(ISERROR(SEARCH("no news",J1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="218" priority="11" operator="containsText" text="offer">
+    <cfRule type="containsText" dxfId="219" priority="11" operator="containsText" text="offer">
       <formula>NOT(ISERROR(SEARCH("offer",J1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="217" priority="12" operator="containsText" text="fly out">
+    <cfRule type="containsText" dxfId="218" priority="12" operator="containsText" text="fly out">
       <formula>NOT(ISERROR(SEARCH("fly out",J1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="216" priority="13" operator="containsText" text="interview">
+    <cfRule type="containsText" dxfId="217" priority="13" operator="containsText" text="interview">
       <formula>NOT(ISERROR(SEARCH("interview",J1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="215" priority="14" operator="containsText" text="rejected">
+    <cfRule type="containsText" dxfId="216" priority="14" operator="containsText" text="rejected">
       <formula>NOT(ISERROR(SEARCH("rejected",J1)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K1:L1048576 P78:P80 P83:P89 P92:P112 P115:P124 P126:P181 S136 S153 S159 S166 S173 S178 P183:P205 P208:P211 P213:P218 P220:P233 S225 P235:P237 P239:P248 P276 R276">
-    <cfRule type="containsText" dxfId="214" priority="19" operator="containsText" text="NO">
+    <cfRule type="containsText" dxfId="215" priority="19" operator="containsText" text="NO">
       <formula>NOT(ISERROR(SEARCH("NO",K1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="213" priority="20" operator="containsText" text="YES">
+    <cfRule type="containsText" dxfId="214" priority="20" operator="containsText" text="YES">
       <formula>NOT(ISERROR(SEARCH("YES",K1)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="P250:P267">
-    <cfRule type="containsText" dxfId="212" priority="1" operator="containsText" text="NO">
+    <cfRule type="containsText" dxfId="213" priority="1" operator="containsText" text="NO">
       <formula>NOT(ISERROR(SEARCH("NO",P250)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="211" priority="2" operator="containsText" text="YES">
+    <cfRule type="containsText" dxfId="212" priority="2" operator="containsText" text="YES">
       <formula>NOT(ISERROR(SEARCH("YES",P250)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="210" priority="3" operator="containsText" text="completed">
+    <cfRule type="containsText" dxfId="211" priority="3" operator="containsText" text="completed">
       <formula>NOT(ISERROR(SEARCH("completed",P250)))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -49577,7 +49587,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{923E81FA-B875-3C4E-A189-1A21268FA086}">
-  <dimension ref="A1:C306"/>
+  <dimension ref="A1:C309"/>
   <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="16" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="32.83203125" customWidth="1"/>
@@ -52879,609 +52889,645 @@
         <v>403</v>
       </c>
     </row>
+    <row r="307" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A307" s="1">
+        <v>46010</v>
+      </c>
+      <c r="B307" t="s">
+        <v>578</v>
+      </c>
+      <c r="C307" t="s">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="308" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A308" s="1">
+        <v>46010</v>
+      </c>
+      <c r="B308" t="s">
+        <v>763</v>
+      </c>
+      <c r="C308" t="s">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="309" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A309" s="1">
+        <v>46010</v>
+      </c>
+      <c r="B309" t="s">
+        <v>430</v>
+      </c>
+      <c r="C309" t="s">
+        <v>403</v>
+      </c>
+    </row>
   </sheetData>
   <conditionalFormatting sqref="B5">
-    <cfRule type="duplicateValues" dxfId="209" priority="217"/>
-    <cfRule type="duplicateValues" dxfId="208" priority="218"/>
+    <cfRule type="duplicateValues" dxfId="210" priority="218"/>
+    <cfRule type="duplicateValues" dxfId="209" priority="219"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B10">
+    <cfRule type="duplicateValues" dxfId="208" priority="217"/>
     <cfRule type="duplicateValues" dxfId="207" priority="216"/>
-    <cfRule type="duplicateValues" dxfId="206" priority="215"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B11">
-    <cfRule type="duplicateValues" dxfId="205" priority="213"/>
-    <cfRule type="duplicateValues" dxfId="204" priority="214"/>
+    <cfRule type="duplicateValues" dxfId="206" priority="214"/>
+    <cfRule type="duplicateValues" dxfId="205" priority="215"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B12">
+    <cfRule type="duplicateValues" dxfId="204" priority="213"/>
     <cfRule type="duplicateValues" dxfId="203" priority="212"/>
-    <cfRule type="duplicateValues" dxfId="202" priority="211"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B15">
+    <cfRule type="duplicateValues" dxfId="202" priority="211"/>
     <cfRule type="duplicateValues" dxfId="201" priority="210"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B16">
     <cfRule type="duplicateValues" dxfId="200" priority="209"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B16">
-    <cfRule type="duplicateValues" dxfId="199" priority="208"/>
-  </conditionalFormatting>
   <conditionalFormatting sqref="B17">
-    <cfRule type="duplicateValues" dxfId="198" priority="206"/>
-    <cfRule type="duplicateValues" dxfId="197" priority="207"/>
+    <cfRule type="duplicateValues" dxfId="199" priority="207"/>
+    <cfRule type="duplicateValues" dxfId="198" priority="208"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B18">
+    <cfRule type="duplicateValues" dxfId="197" priority="206"/>
     <cfRule type="duplicateValues" dxfId="196" priority="205"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B19">
     <cfRule type="duplicateValues" dxfId="195" priority="204"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B19">
+  <conditionalFormatting sqref="B22:B23">
     <cfRule type="duplicateValues" dxfId="194" priority="203"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B22:B23">
     <cfRule type="duplicateValues" dxfId="193" priority="202"/>
-    <cfRule type="duplicateValues" dxfId="192" priority="201"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B24">
+    <cfRule type="duplicateValues" dxfId="192" priority="201"/>
     <cfRule type="duplicateValues" dxfId="191" priority="200"/>
-    <cfRule type="duplicateValues" dxfId="190" priority="199"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B27">
+    <cfRule type="duplicateValues" dxfId="190" priority="199"/>
     <cfRule type="duplicateValues" dxfId="189" priority="198"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B28">
     <cfRule type="duplicateValues" dxfId="188" priority="197"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B28">
-    <cfRule type="duplicateValues" dxfId="187" priority="196"/>
-  </conditionalFormatting>
   <conditionalFormatting sqref="B29">
-    <cfRule type="duplicateValues" dxfId="186" priority="194"/>
-    <cfRule type="duplicateValues" dxfId="185" priority="195"/>
+    <cfRule type="duplicateValues" dxfId="187" priority="195"/>
+    <cfRule type="duplicateValues" dxfId="186" priority="196"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B30">
+    <cfRule type="duplicateValues" dxfId="185" priority="194"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B31">
     <cfRule type="duplicateValues" dxfId="184" priority="193"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B31">
+  <conditionalFormatting sqref="B32">
     <cfRule type="duplicateValues" dxfId="183" priority="192"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B32">
+  <conditionalFormatting sqref="B33">
     <cfRule type="duplicateValues" dxfId="182" priority="191"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B33">
+  <conditionalFormatting sqref="B34">
     <cfRule type="duplicateValues" dxfId="181" priority="190"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B34">
+  <conditionalFormatting sqref="B35">
     <cfRule type="duplicateValues" dxfId="180" priority="189"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B35">
+  <conditionalFormatting sqref="B37">
     <cfRule type="duplicateValues" dxfId="179" priority="188"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B37">
+  <conditionalFormatting sqref="B38">
     <cfRule type="duplicateValues" dxfId="178" priority="187"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B38">
+  <conditionalFormatting sqref="B42">
     <cfRule type="duplicateValues" dxfId="177" priority="186"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B42">
+  <conditionalFormatting sqref="B43">
     <cfRule type="duplicateValues" dxfId="176" priority="185"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B43">
+  <conditionalFormatting sqref="B44:B45">
     <cfRule type="duplicateValues" dxfId="175" priority="184"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B44:B45">
+  <conditionalFormatting sqref="B46">
     <cfRule type="duplicateValues" dxfId="174" priority="183"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B46">
+  <conditionalFormatting sqref="B48">
     <cfRule type="duplicateValues" dxfId="173" priority="182"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B48">
+  <conditionalFormatting sqref="B49">
     <cfRule type="duplicateValues" dxfId="172" priority="181"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B49">
+  <conditionalFormatting sqref="B51">
     <cfRule type="duplicateValues" dxfId="171" priority="180"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B51">
+  <conditionalFormatting sqref="B52">
     <cfRule type="duplicateValues" dxfId="170" priority="179"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B52">
-    <cfRule type="duplicateValues" dxfId="169" priority="178"/>
-  </conditionalFormatting>
   <conditionalFormatting sqref="B58">
-    <cfRule type="duplicateValues" dxfId="168" priority="176"/>
+    <cfRule type="duplicateValues" dxfId="169" priority="177"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B59">
+    <cfRule type="duplicateValues" dxfId="168" priority="175"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B63">
     <cfRule type="duplicateValues" dxfId="167" priority="174"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B63">
-    <cfRule type="duplicateValues" dxfId="166" priority="173"/>
+  <conditionalFormatting sqref="B64">
+    <cfRule type="duplicateValues" dxfId="166" priority="172"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B64">
+  <conditionalFormatting sqref="B66">
     <cfRule type="duplicateValues" dxfId="165" priority="171"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B66">
+  <conditionalFormatting sqref="B67">
     <cfRule type="duplicateValues" dxfId="164" priority="170"/>
+    <cfRule type="duplicateValues" dxfId="163" priority="169"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B67">
-    <cfRule type="duplicateValues" dxfId="163" priority="169"/>
+  <conditionalFormatting sqref="B68">
     <cfRule type="duplicateValues" dxfId="162" priority="168"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B68">
+  <conditionalFormatting sqref="B69">
     <cfRule type="duplicateValues" dxfId="161" priority="167"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B69">
-    <cfRule type="duplicateValues" dxfId="160" priority="166"/>
+  <conditionalFormatting sqref="B70">
+    <cfRule type="duplicateValues" dxfId="160" priority="165"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B70">
+  <conditionalFormatting sqref="B72">
     <cfRule type="duplicateValues" dxfId="159" priority="164"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B72">
-    <cfRule type="duplicateValues" dxfId="158" priority="163"/>
+  <conditionalFormatting sqref="B73">
+    <cfRule type="duplicateValues" dxfId="158" priority="162"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B73">
+  <conditionalFormatting sqref="B74">
     <cfRule type="duplicateValues" dxfId="157" priority="161"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B74">
+  <conditionalFormatting sqref="B75">
     <cfRule type="duplicateValues" dxfId="156" priority="160"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B75">
+  <conditionalFormatting sqref="B76">
     <cfRule type="duplicateValues" dxfId="155" priority="159"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B76">
-    <cfRule type="duplicateValues" dxfId="154" priority="158"/>
+  <conditionalFormatting sqref="B77">
+    <cfRule type="duplicateValues" dxfId="154" priority="157"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B77">
+  <conditionalFormatting sqref="B78">
     <cfRule type="duplicateValues" dxfId="153" priority="156"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B78">
+  <conditionalFormatting sqref="B83">
     <cfRule type="duplicateValues" dxfId="152" priority="155"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B83">
+  <conditionalFormatting sqref="B84">
     <cfRule type="duplicateValues" dxfId="151" priority="154"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B84">
+  <conditionalFormatting sqref="B85">
     <cfRule type="duplicateValues" dxfId="150" priority="153"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B85">
+  <conditionalFormatting sqref="B87">
     <cfRule type="duplicateValues" dxfId="149" priority="152"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B87">
+  <conditionalFormatting sqref="B88">
     <cfRule type="duplicateValues" dxfId="148" priority="151"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B88">
+  <conditionalFormatting sqref="B89">
     <cfRule type="duplicateValues" dxfId="147" priority="150"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B89">
+  <conditionalFormatting sqref="B90">
     <cfRule type="duplicateValues" dxfId="146" priority="149"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B90">
+  <conditionalFormatting sqref="B91">
     <cfRule type="duplicateValues" dxfId="145" priority="148"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B91">
+  <conditionalFormatting sqref="B92">
     <cfRule type="duplicateValues" dxfId="144" priority="147"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B92">
+  <conditionalFormatting sqref="B93">
     <cfRule type="duplicateValues" dxfId="143" priority="146"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B93">
+  <conditionalFormatting sqref="B94">
     <cfRule type="duplicateValues" dxfId="142" priority="145"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B94">
+  <conditionalFormatting sqref="B95">
     <cfRule type="duplicateValues" dxfId="141" priority="144"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B95">
+  <conditionalFormatting sqref="B96">
     <cfRule type="duplicateValues" dxfId="140" priority="143"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B96">
+  <conditionalFormatting sqref="B97">
     <cfRule type="duplicateValues" dxfId="139" priority="142"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B97">
+  <conditionalFormatting sqref="B98">
     <cfRule type="duplicateValues" dxfId="138" priority="141"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B98">
+  <conditionalFormatting sqref="B99">
     <cfRule type="duplicateValues" dxfId="137" priority="140"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B99">
+  <conditionalFormatting sqref="B100">
     <cfRule type="duplicateValues" dxfId="136" priority="139"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B100">
+  <conditionalFormatting sqref="B101">
     <cfRule type="duplicateValues" dxfId="135" priority="138"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B101">
-    <cfRule type="duplicateValues" dxfId="134" priority="137"/>
-  </conditionalFormatting>
   <conditionalFormatting sqref="B104">
-    <cfRule type="duplicateValues" dxfId="133" priority="135"/>
-    <cfRule type="duplicateValues" dxfId="132" priority="136"/>
+    <cfRule type="duplicateValues" dxfId="134" priority="136"/>
+    <cfRule type="duplicateValues" dxfId="133" priority="137"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B105:B106">
+    <cfRule type="duplicateValues" dxfId="132" priority="135"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B107">
     <cfRule type="duplicateValues" dxfId="131" priority="134"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B107">
+  <conditionalFormatting sqref="B108">
     <cfRule type="duplicateValues" dxfId="130" priority="133"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B108">
+  <conditionalFormatting sqref="B109">
     <cfRule type="duplicateValues" dxfId="129" priority="132"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B109">
+  <conditionalFormatting sqref="B110">
     <cfRule type="duplicateValues" dxfId="128" priority="131"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B110">
+  <conditionalFormatting sqref="B111">
     <cfRule type="duplicateValues" dxfId="127" priority="130"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B111">
+  <conditionalFormatting sqref="B112">
     <cfRule type="duplicateValues" dxfId="126" priority="129"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B112">
+  <conditionalFormatting sqref="B113">
     <cfRule type="duplicateValues" dxfId="125" priority="128"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B113">
+  <conditionalFormatting sqref="B114">
     <cfRule type="duplicateValues" dxfId="124" priority="127"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B114">
+  <conditionalFormatting sqref="B115">
     <cfRule type="duplicateValues" dxfId="123" priority="126"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B115">
+  <conditionalFormatting sqref="B116">
     <cfRule type="duplicateValues" dxfId="122" priority="125"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B116">
+  <conditionalFormatting sqref="B117">
     <cfRule type="duplicateValues" dxfId="121" priority="124"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B117">
+  <conditionalFormatting sqref="B118">
     <cfRule type="duplicateValues" dxfId="120" priority="123"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B118">
+  <conditionalFormatting sqref="B119">
     <cfRule type="duplicateValues" dxfId="119" priority="122"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B119">
+  <conditionalFormatting sqref="B120">
     <cfRule type="duplicateValues" dxfId="118" priority="121"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B120">
+  <conditionalFormatting sqref="B121">
     <cfRule type="duplicateValues" dxfId="117" priority="120"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B121">
+  <conditionalFormatting sqref="B122">
     <cfRule type="duplicateValues" dxfId="116" priority="119"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B122">
+  <conditionalFormatting sqref="B126">
     <cfRule type="duplicateValues" dxfId="115" priority="118"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B126">
+  <conditionalFormatting sqref="B127">
     <cfRule type="duplicateValues" dxfId="114" priority="117"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B127">
+  <conditionalFormatting sqref="B128">
     <cfRule type="duplicateValues" dxfId="113" priority="116"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B128">
+  <conditionalFormatting sqref="B129">
     <cfRule type="duplicateValues" dxfId="112" priority="115"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B129">
+  <conditionalFormatting sqref="B130">
     <cfRule type="duplicateValues" dxfId="111" priority="114"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B130">
+  <conditionalFormatting sqref="B131">
     <cfRule type="duplicateValues" dxfId="110" priority="113"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B131">
+  <conditionalFormatting sqref="B132">
     <cfRule type="duplicateValues" dxfId="109" priority="112"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B132">
+  <conditionalFormatting sqref="B133">
     <cfRule type="duplicateValues" dxfId="108" priority="111"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B133">
+  <conditionalFormatting sqref="B136">
     <cfRule type="duplicateValues" dxfId="107" priority="110"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B136">
+  <conditionalFormatting sqref="B137">
     <cfRule type="duplicateValues" dxfId="106" priority="109"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B137">
+  <conditionalFormatting sqref="B138">
     <cfRule type="duplicateValues" dxfId="105" priority="108"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B138">
+  <conditionalFormatting sqref="B139">
     <cfRule type="duplicateValues" dxfId="104" priority="107"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B139">
+  <conditionalFormatting sqref="B140">
     <cfRule type="duplicateValues" dxfId="103" priority="106"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B140">
+  <conditionalFormatting sqref="B141">
     <cfRule type="duplicateValues" dxfId="102" priority="105"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B141">
+  <conditionalFormatting sqref="B142">
     <cfRule type="duplicateValues" dxfId="101" priority="104"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B142">
+  <conditionalFormatting sqref="B143">
     <cfRule type="duplicateValues" dxfId="100" priority="103"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B143">
+  <conditionalFormatting sqref="B144">
     <cfRule type="duplicateValues" dxfId="99" priority="102"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B144">
+  <conditionalFormatting sqref="B145">
     <cfRule type="duplicateValues" dxfId="98" priority="101"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B145">
+  <conditionalFormatting sqref="B147">
     <cfRule type="duplicateValues" dxfId="97" priority="100"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B147">
+  <conditionalFormatting sqref="B148">
     <cfRule type="duplicateValues" dxfId="96" priority="99"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B148">
+  <conditionalFormatting sqref="B149">
     <cfRule type="duplicateValues" dxfId="95" priority="98"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B149">
+  <conditionalFormatting sqref="B150">
     <cfRule type="duplicateValues" dxfId="94" priority="97"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B150">
+  <conditionalFormatting sqref="B151">
     <cfRule type="duplicateValues" dxfId="93" priority="96"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B151">
+  <conditionalFormatting sqref="B152">
     <cfRule type="duplicateValues" dxfId="92" priority="95"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B152">
+  <conditionalFormatting sqref="B153">
     <cfRule type="duplicateValues" dxfId="91" priority="94"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B153">
+  <conditionalFormatting sqref="B154">
     <cfRule type="duplicateValues" dxfId="90" priority="93"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B154">
+  <conditionalFormatting sqref="B155">
     <cfRule type="duplicateValues" dxfId="89" priority="92"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B155">
+  <conditionalFormatting sqref="B156">
     <cfRule type="duplicateValues" dxfId="88" priority="91"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B156">
+  <conditionalFormatting sqref="B157">
     <cfRule type="duplicateValues" dxfId="87" priority="90"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B157">
+  <conditionalFormatting sqref="B171">
     <cfRule type="duplicateValues" dxfId="86" priority="89"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B171">
+  <conditionalFormatting sqref="B172">
     <cfRule type="duplicateValues" dxfId="85" priority="88"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B172">
+  <conditionalFormatting sqref="B174">
     <cfRule type="duplicateValues" dxfId="84" priority="87"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B174">
+  <conditionalFormatting sqref="B177:B178">
     <cfRule type="duplicateValues" dxfId="83" priority="86"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B177:B178">
+  <conditionalFormatting sqref="B181">
     <cfRule type="duplicateValues" dxfId="82" priority="85"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B181">
+  <conditionalFormatting sqref="B182">
     <cfRule type="duplicateValues" dxfId="81" priority="84"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B182">
+  <conditionalFormatting sqref="B183">
     <cfRule type="duplicateValues" dxfId="80" priority="83"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B183">
+  <conditionalFormatting sqref="B184">
     <cfRule type="duplicateValues" dxfId="79" priority="82"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B184">
+  <conditionalFormatting sqref="B185">
     <cfRule type="duplicateValues" dxfId="78" priority="81"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B185">
+  <conditionalFormatting sqref="B186">
     <cfRule type="duplicateValues" dxfId="77" priority="80"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B186">
+  <conditionalFormatting sqref="B188">
     <cfRule type="duplicateValues" dxfId="76" priority="79"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B188">
+  <conditionalFormatting sqref="B189">
     <cfRule type="duplicateValues" dxfId="75" priority="78"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B189">
+  <conditionalFormatting sqref="B190">
     <cfRule type="duplicateValues" dxfId="74" priority="77"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B190">
+  <conditionalFormatting sqref="B191">
     <cfRule type="duplicateValues" dxfId="73" priority="76"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B191">
+  <conditionalFormatting sqref="B192">
     <cfRule type="duplicateValues" dxfId="72" priority="75"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B192">
+  <conditionalFormatting sqref="B193">
     <cfRule type="duplicateValues" dxfId="71" priority="74"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B193">
+  <conditionalFormatting sqref="B195">
     <cfRule type="duplicateValues" dxfId="70" priority="73"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B195">
+  <conditionalFormatting sqref="B196">
     <cfRule type="duplicateValues" dxfId="69" priority="72"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B196">
+  <conditionalFormatting sqref="B197">
     <cfRule type="duplicateValues" dxfId="68" priority="71"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B197">
+  <conditionalFormatting sqref="B198">
     <cfRule type="duplicateValues" dxfId="67" priority="70"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B198">
+  <conditionalFormatting sqref="B199">
     <cfRule type="duplicateValues" dxfId="66" priority="69"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B199">
+  <conditionalFormatting sqref="B200">
     <cfRule type="duplicateValues" dxfId="65" priority="68"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B200">
+  <conditionalFormatting sqref="B201">
     <cfRule type="duplicateValues" dxfId="64" priority="67"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B201">
+  <conditionalFormatting sqref="B202">
     <cfRule type="duplicateValues" dxfId="63" priority="66"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B202">
+  <conditionalFormatting sqref="B203">
     <cfRule type="duplicateValues" dxfId="62" priority="65"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B203">
+  <conditionalFormatting sqref="B204">
     <cfRule type="duplicateValues" dxfId="61" priority="64"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B204">
+  <conditionalFormatting sqref="B205">
     <cfRule type="duplicateValues" dxfId="60" priority="63"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B205">
+  <conditionalFormatting sqref="B206">
     <cfRule type="duplicateValues" dxfId="59" priority="62"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B206">
+  <conditionalFormatting sqref="B207">
     <cfRule type="duplicateValues" dxfId="58" priority="61"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B207">
+  <conditionalFormatting sqref="B215">
     <cfRule type="duplicateValues" dxfId="57" priority="60"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B215">
+  <conditionalFormatting sqref="B218">
     <cfRule type="duplicateValues" dxfId="56" priority="59"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B218">
+  <conditionalFormatting sqref="B220">
     <cfRule type="duplicateValues" dxfId="55" priority="58"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B220">
+  <conditionalFormatting sqref="B222">
     <cfRule type="duplicateValues" dxfId="54" priority="57"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B222">
+  <conditionalFormatting sqref="B223">
     <cfRule type="duplicateValues" dxfId="53" priority="56"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B223">
+  <conditionalFormatting sqref="B224">
     <cfRule type="duplicateValues" dxfId="52" priority="55"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B224">
+  <conditionalFormatting sqref="B225">
     <cfRule type="duplicateValues" dxfId="51" priority="54"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B225">
+  <conditionalFormatting sqref="B227">
     <cfRule type="duplicateValues" dxfId="50" priority="53"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B227">
+  <conditionalFormatting sqref="B229">
     <cfRule type="duplicateValues" dxfId="49" priority="52"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B229">
+  <conditionalFormatting sqref="B230">
     <cfRule type="duplicateValues" dxfId="48" priority="51"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B230">
+  <conditionalFormatting sqref="B232">
     <cfRule type="duplicateValues" dxfId="47" priority="50"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B232">
+  <conditionalFormatting sqref="B233">
     <cfRule type="duplicateValues" dxfId="46" priority="49"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B233">
+  <conditionalFormatting sqref="B234">
     <cfRule type="duplicateValues" dxfId="45" priority="48"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B234">
+  <conditionalFormatting sqref="B235">
     <cfRule type="duplicateValues" dxfId="44" priority="47"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B235">
+  <conditionalFormatting sqref="B236">
     <cfRule type="duplicateValues" dxfId="43" priority="46"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B236">
+  <conditionalFormatting sqref="B237">
     <cfRule type="duplicateValues" dxfId="42" priority="45"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B237">
-    <cfRule type="duplicateValues" dxfId="41" priority="44"/>
+  <conditionalFormatting sqref="B239">
+    <cfRule type="duplicateValues" dxfId="41" priority="43"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B239">
+  <conditionalFormatting sqref="B240">
     <cfRule type="duplicateValues" dxfId="40" priority="42"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B240">
+  <conditionalFormatting sqref="B241">
     <cfRule type="duplicateValues" dxfId="39" priority="41"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B241">
+  <conditionalFormatting sqref="B242">
     <cfRule type="duplicateValues" dxfId="38" priority="40"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B242">
+  <conditionalFormatting sqref="B243">
     <cfRule type="duplicateValues" dxfId="37" priority="39"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B243">
+  <conditionalFormatting sqref="B250">
     <cfRule type="duplicateValues" dxfId="36" priority="38"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B250">
+  <conditionalFormatting sqref="B251">
     <cfRule type="duplicateValues" dxfId="35" priority="37"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B251">
+  <conditionalFormatting sqref="B253">
     <cfRule type="duplicateValues" dxfId="34" priority="36"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B253">
+  <conditionalFormatting sqref="B255">
     <cfRule type="duplicateValues" dxfId="33" priority="35"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B255">
+  <conditionalFormatting sqref="B258:B259">
     <cfRule type="duplicateValues" dxfId="32" priority="34"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B258:B259">
+  <conditionalFormatting sqref="B260">
     <cfRule type="duplicateValues" dxfId="31" priority="33"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B260">
+  <conditionalFormatting sqref="B265:B267 B269">
     <cfRule type="duplicateValues" dxfId="30" priority="32"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B265:B267 B269">
+  <conditionalFormatting sqref="B268">
     <cfRule type="duplicateValues" dxfId="29" priority="31"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B268">
+  <conditionalFormatting sqref="B270">
     <cfRule type="duplicateValues" dxfId="28" priority="30"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B270">
+  <conditionalFormatting sqref="B271">
     <cfRule type="duplicateValues" dxfId="27" priority="29"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B271">
+  <conditionalFormatting sqref="B273">
     <cfRule type="duplicateValues" dxfId="26" priority="28"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B273">
+  <conditionalFormatting sqref="B275">
     <cfRule type="duplicateValues" dxfId="25" priority="27"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B275">
+  <conditionalFormatting sqref="B278">
     <cfRule type="duplicateValues" dxfId="24" priority="26"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B278">
+  <conditionalFormatting sqref="B279">
     <cfRule type="duplicateValues" dxfId="23" priority="25"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B279">
+  <conditionalFormatting sqref="B280">
     <cfRule type="duplicateValues" dxfId="22" priority="24"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B280">
+  <conditionalFormatting sqref="B281">
     <cfRule type="duplicateValues" dxfId="21" priority="23"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B281">
+  <conditionalFormatting sqref="B282">
     <cfRule type="duplicateValues" dxfId="20" priority="22"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B282">
-    <cfRule type="duplicateValues" dxfId="19" priority="21"/>
+  <conditionalFormatting sqref="B283">
+    <cfRule type="duplicateValues" dxfId="19" priority="20"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B283">
+  <conditionalFormatting sqref="B284:B286">
     <cfRule type="duplicateValues" dxfId="18" priority="19"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B284:B286">
+  <conditionalFormatting sqref="B287">
     <cfRule type="duplicateValues" dxfId="17" priority="18"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B287">
+  <conditionalFormatting sqref="B288">
     <cfRule type="duplicateValues" dxfId="16" priority="17"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B288">
+  <conditionalFormatting sqref="B291">
     <cfRule type="duplicateValues" dxfId="15" priority="16"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B291">
+  <conditionalFormatting sqref="B292">
     <cfRule type="duplicateValues" dxfId="14" priority="15"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B292">
+  <conditionalFormatting sqref="B293">
     <cfRule type="duplicateValues" dxfId="13" priority="14"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B293">
+  <conditionalFormatting sqref="B294">
     <cfRule type="duplicateValues" dxfId="12" priority="13"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B294">
+  <conditionalFormatting sqref="B295">
     <cfRule type="duplicateValues" dxfId="11" priority="12"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B295">
+  <conditionalFormatting sqref="B296">
     <cfRule type="duplicateValues" dxfId="10" priority="11"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B296">
+  <conditionalFormatting sqref="B297">
     <cfRule type="duplicateValues" dxfId="9" priority="10"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B297">
+  <conditionalFormatting sqref="B298">
     <cfRule type="duplicateValues" dxfId="8" priority="9"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B298">
+  <conditionalFormatting sqref="B299">
     <cfRule type="duplicateValues" dxfId="7" priority="8"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B299">
+  <conditionalFormatting sqref="B300">
     <cfRule type="duplicateValues" dxfId="6" priority="7"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B300">
+  <conditionalFormatting sqref="B301">
     <cfRule type="duplicateValues" dxfId="5" priority="6"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B301">
+  <conditionalFormatting sqref="B302">
     <cfRule type="duplicateValues" dxfId="4" priority="5"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B302">
+  <conditionalFormatting sqref="B303">
     <cfRule type="duplicateValues" dxfId="3" priority="4"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B303">
+  <conditionalFormatting sqref="B304">
     <cfRule type="duplicateValues" dxfId="2" priority="3"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B304">
+  <conditionalFormatting sqref="B306">
     <cfRule type="duplicateValues" dxfId="1" priority="2"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B306">
+  <conditionalFormatting sqref="B309">
     <cfRule type="duplicateValues" dxfId="0" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -53560,11 +53606,11 @@
       </c>
       <c r="B6" s="16">
         <f>COUNTIFS(sum!J:J,"no news")</f>
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="C6" s="10">
         <f>B6/$B$5</f>
-        <v>0.92363636363636359</v>
+        <v>0.91636363636363638</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.4">
@@ -53573,11 +53619,11 @@
       </c>
       <c r="B7" s="16">
         <f>COUNTIFS(sum!J:J,"rejected")</f>
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="C7" s="10">
         <f t="shared" ref="C7:C10" si="0">B7/$B$5</f>
-        <v>5.8181818181818182E-2</v>
+        <v>6.545454545454546E-2</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.4">

</xml_diff>

<commit_message>
add some new thought into the write-up
</commit_message>
<xml_diff>
--- a/EconJM_status.xlsx
+++ b/EconJM_status.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\javie\Dropbox\Work\Job Search\2025 EconJM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{80043ACE-4A8F-4F83-A536-3C3D456B89FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{851EE1F0-9E31-4B99-A62B-5757413AF67B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="14620" xr2:uid="{6FE48536-7E5C-BF4C-9490-2A6392576298}"/>
   </bookViews>
@@ -428,7 +428,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2928" uniqueCount="891">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3025" uniqueCount="919">
   <si>
     <t>add_id</t>
   </si>
@@ -3103,9 +3103,6 @@
     <t>Ireland</t>
   </si>
   <si>
-    <t>*may be not updated. See timeline for accurate status of applications</t>
-  </si>
-  <si>
     <t>purdue_post_sloan</t>
   </si>
   <si>
@@ -3137,6 +3134,93 @@
   </si>
   <si>
     <t>zurich_post_dig</t>
+  </si>
+  <si>
+    <t>andres_bello</t>
+  </si>
+  <si>
+    <t>https://www.aeaweb.org/joe/listing.php?JOE_ID=2026-01_111477201&amp;q=eNplj1EKwkAMRO-Sb4Uq6EcPIAjeYYm7sa7GbEm2lVwi3t0oFgT_wpvMJPOAQ7aapbNd0Ru0D8gSMNY8ErTQwAKuNN2LpmCEGs8OnRn5RhFoZWBewIV4HrPZ8Haum_V22ax8t2jusiDv_5RYBqk6BaXuXCfMcKQUToUTqc0woqScsFKwqHg7Ms2KUiSpoQhPM-Jvo-Bvk4ajC_Dx9sWqZ6Pf5r53unkX7LH7pj2fL5LLXFyZ</t>
+  </si>
+  <si>
+    <t>Universidad Andres Bello</t>
+  </si>
+  <si>
+    <t>hec_ine</t>
+  </si>
+  <si>
+    <t>generating docs</t>
+  </si>
+  <si>
+    <t>wheterall</t>
+  </si>
+  <si>
+    <t>Queens University</t>
+  </si>
+  <si>
+    <t>porto</t>
+  </si>
+  <si>
+    <t>University of Porto</t>
+  </si>
+  <si>
+    <t>lyon_post</t>
+  </si>
+  <si>
+    <t>École Normale Superieure de Lyon</t>
+  </si>
+  <si>
+    <t>uciii_post</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Carlos III </t>
+  </si>
+  <si>
+    <t>added some other job postings</t>
+  </si>
+  <si>
+    <t>*may be not updated because I forgot to update the "sum" page. See timeline for accurate status of applications</t>
+  </si>
+  <si>
+    <t>fiu_teaching</t>
+  </si>
+  <si>
+    <t>https://search.careers.fiu.edu/?q=536746</t>
+  </si>
+  <si>
+    <t>reading</t>
+  </si>
+  <si>
+    <t>University of Reading</t>
+  </si>
+  <si>
+    <t>Simonetta Longhi (s.longhi@reading.ac.uk)</t>
+  </si>
+  <si>
+    <t>https://jobs.reading.ac.uk/Job/JobDetail?JobId=25073</t>
+  </si>
+  <si>
+    <t>n_iowa_teaching</t>
+  </si>
+  <si>
+    <t>https://uni.wd5.myworkdayjobs.com/en-US/UNI/job/Assistant-Professor-of-Instruction-or-Practice---Economics_JR1009</t>
+  </si>
+  <si>
+    <t>University of North Iowa</t>
+  </si>
+  <si>
+    <t>toronto_limited</t>
+  </si>
+  <si>
+    <t>https://jobs.utoronto.ca/job/Toronto-Assistant-Professor-Contractually-Limited-Term-Appointment-%28CLTA%29-EconomicsApplied-Economics-ON/599485817/</t>
+  </si>
+  <si>
+    <t>north_western</t>
+  </si>
+  <si>
+    <t>https://www.nwciowa.edu/employment/openings/402/visiting-faculty---economics</t>
+  </si>
+  <si>
+    <t>Northwestern College</t>
   </si>
 </sst>
 </file>
@@ -3328,27 +3412,7 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Percent" xfId="2" builtinId="5"/>
   </cellStyles>
-  <dxfs count="263">
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="252">
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -3356,16 +3420,6 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -3383,85 +3437,11 @@
       <font>
         <color rgb="FF9C0006"/>
       </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <color theme="8" tint="-0.24994659260841701"/>
-      </font>
       <fill>
-        <patternFill patternType="none">
-          <bgColor auto="1"/>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="8" tint="-0.24994659260841701"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="3" tint="0.24994659260841701"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left style="hair">
-          <color auto="1"/>
-        </left>
-        <right style="hair">
-          <color auto="1"/>
-        </right>
-        <top style="hair">
-          <color auto="1"/>
-        </top>
-        <bottom style="hair">
-          <color auto="1"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="2" tint="-0.24994659260841701"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i/>
-        <color theme="0" tint="-0.24994659260841701"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="5" tint="0.79998168889431442"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
     </dxf>
     <dxf>
       <font>
@@ -36177,7 +36157,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F7772053-9363-CA4A-A53F-040B7C700753}">
-  <dimension ref="A1:W283"/>
+  <dimension ref="A1:W294"/>
   <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="16" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="19.6640625" customWidth="1"/>
@@ -37622,7 +37602,7 @@
         <v>95</v>
       </c>
       <c r="J29" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="M29" t="s">
         <v>477</v>
@@ -48558,7 +48538,7 @@
         <v>95</v>
       </c>
       <c r="J251" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="M251" t="s">
         <v>719</v>
@@ -49791,13 +49771,13 @@
     </row>
     <row r="277" spans="1:23" x14ac:dyDescent="0.4">
       <c r="A277" t="s">
-        <v>880</v>
+        <v>879</v>
       </c>
       <c r="D277" s="1">
         <v>46068</v>
       </c>
       <c r="F277" t="s">
-        <v>881</v>
+        <v>880</v>
       </c>
       <c r="I277" t="s">
         <v>95</v>
@@ -49836,13 +49816,13 @@
     </row>
     <row r="278" spans="1:23" x14ac:dyDescent="0.4">
       <c r="A278" t="s">
-        <v>882</v>
+        <v>881</v>
       </c>
       <c r="D278" s="1">
         <v>46054</v>
       </c>
       <c r="F278" t="s">
-        <v>883</v>
+        <v>882</v>
       </c>
       <c r="I278" t="s">
         <v>95</v>
@@ -49881,7 +49861,7 @@
     </row>
     <row r="279" spans="1:23" x14ac:dyDescent="0.4">
       <c r="A279" t="s">
-        <v>884</v>
+        <v>883</v>
       </c>
       <c r="D279" s="1">
         <v>46052</v>
@@ -49926,7 +49906,7 @@
     </row>
     <row r="280" spans="1:23" x14ac:dyDescent="0.4">
       <c r="A280" t="s">
-        <v>885</v>
+        <v>884</v>
       </c>
       <c r="D280" s="1">
         <v>46054</v>
@@ -49941,7 +49921,7 @@
         <v>401</v>
       </c>
       <c r="M280" t="s">
-        <v>886</v>
+        <v>885</v>
       </c>
       <c r="N280" t="e" vm="12">
         <v>#VALUE!</v>
@@ -49971,7 +49951,7 @@
     </row>
     <row r="281" spans="1:23" x14ac:dyDescent="0.4">
       <c r="A281" t="s">
-        <v>887</v>
+        <v>886</v>
       </c>
       <c r="D281" s="1">
         <v>46054</v>
@@ -49986,7 +49966,7 @@
         <v>401</v>
       </c>
       <c r="M281" t="s">
-        <v>888</v>
+        <v>887</v>
       </c>
       <c r="N281" t="e" vm="1">
         <v>#VALUE!</v>
@@ -50016,7 +49996,7 @@
     </row>
     <row r="282" spans="1:23" x14ac:dyDescent="0.4">
       <c r="A282" t="s">
-        <v>889</v>
+        <v>888</v>
       </c>
       <c r="D282" s="1">
         <v>46054</v>
@@ -50061,7 +50041,7 @@
     </row>
     <row r="283" spans="1:23" x14ac:dyDescent="0.4">
       <c r="A283" t="s">
-        <v>890</v>
+        <v>889</v>
       </c>
       <c r="D283" s="1">
         <v>46054</v>
@@ -50101,6 +50081,482 @@
         <v>0</v>
       </c>
       <c r="W283">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="284" spans="1:23" x14ac:dyDescent="0.4">
+      <c r="A284" t="s">
+        <v>890</v>
+      </c>
+      <c r="D284" s="1">
+        <v>46054</v>
+      </c>
+      <c r="E284" t="s">
+        <v>39</v>
+      </c>
+      <c r="F284" t="s">
+        <v>891</v>
+      </c>
+      <c r="I284" t="s">
+        <v>95</v>
+      </c>
+      <c r="J284" t="s">
+        <v>401</v>
+      </c>
+      <c r="M284" t="s">
+        <v>892</v>
+      </c>
+      <c r="N284" t="e" vm="5">
+        <v>#VALUE!</v>
+      </c>
+      <c r="O284" t="str" cm="1">
+        <f t="array" aca="1" ref="O284" ca="1">_FV(N284,"Name")</f>
+        <v>Chile</v>
+      </c>
+      <c r="P284" t="s">
+        <v>11</v>
+      </c>
+      <c r="R284" t="s">
+        <v>775</v>
+      </c>
+      <c r="S284" s="1">
+        <v>46054</v>
+      </c>
+      <c r="U284">
+        <v>1</v>
+      </c>
+      <c r="V284">
+        <v>0</v>
+      </c>
+      <c r="W284">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="285" spans="1:23" x14ac:dyDescent="0.4">
+      <c r="A285" t="s">
+        <v>893</v>
+      </c>
+      <c r="D285" s="1">
+        <v>46082</v>
+      </c>
+      <c r="E285" t="s">
+        <v>15</v>
+      </c>
+      <c r="I285" t="s">
+        <v>894</v>
+      </c>
+      <c r="J285" t="s">
+        <v>401</v>
+      </c>
+      <c r="M285" t="s">
+        <v>807</v>
+      </c>
+      <c r="N285" t="e" vm="4">
+        <v>#VALUE!</v>
+      </c>
+      <c r="P285" t="s">
+        <v>25</v>
+      </c>
+      <c r="R285" t="s">
+        <v>775</v>
+      </c>
+      <c r="S285" s="1">
+        <v>46113</v>
+      </c>
+      <c r="U285">
+        <v>1</v>
+      </c>
+      <c r="V285">
+        <v>0</v>
+      </c>
+      <c r="W285">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="286" spans="1:23" x14ac:dyDescent="0.4">
+      <c r="A286" t="s">
+        <v>895</v>
+      </c>
+      <c r="D286" s="1">
+        <v>46069</v>
+      </c>
+      <c r="E286" t="s">
+        <v>15</v>
+      </c>
+      <c r="I286" t="s">
+        <v>894</v>
+      </c>
+      <c r="J286" t="s">
+        <v>401</v>
+      </c>
+      <c r="M286" t="s">
+        <v>896</v>
+      </c>
+      <c r="N286" t="e" vm="10">
+        <v>#VALUE!</v>
+      </c>
+      <c r="P286" t="s">
+        <v>25</v>
+      </c>
+      <c r="R286" t="s">
+        <v>775</v>
+      </c>
+      <c r="S286" s="1">
+        <v>46107</v>
+      </c>
+      <c r="U286">
+        <v>1</v>
+      </c>
+      <c r="V286">
+        <v>0</v>
+      </c>
+      <c r="W286">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="287" spans="1:23" x14ac:dyDescent="0.4">
+      <c r="A287" t="s">
+        <v>897</v>
+      </c>
+      <c r="D287" s="1">
+        <v>46081</v>
+      </c>
+      <c r="E287" t="s">
+        <v>15</v>
+      </c>
+      <c r="I287" t="s">
+        <v>894</v>
+      </c>
+      <c r="J287" t="s">
+        <v>401</v>
+      </c>
+      <c r="M287" t="s">
+        <v>898</v>
+      </c>
+      <c r="N287" t="e" vm="22">
+        <v>#VALUE!</v>
+      </c>
+      <c r="P287" t="s">
+        <v>11</v>
+      </c>
+      <c r="R287" t="s">
+        <v>775</v>
+      </c>
+      <c r="S287" s="1">
+        <v>46081</v>
+      </c>
+      <c r="U287">
+        <v>1</v>
+      </c>
+      <c r="V287">
+        <v>0</v>
+      </c>
+      <c r="W287">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="288" spans="1:23" x14ac:dyDescent="0.4">
+      <c r="A288" t="s">
+        <v>899</v>
+      </c>
+      <c r="D288" s="1">
+        <v>46069</v>
+      </c>
+      <c r="E288" t="s">
+        <v>15</v>
+      </c>
+      <c r="I288" t="s">
+        <v>894</v>
+      </c>
+      <c r="J288" t="s">
+        <v>401</v>
+      </c>
+      <c r="M288" t="s">
+        <v>900</v>
+      </c>
+      <c r="N288" t="e" vm="4">
+        <v>#VALUE!</v>
+      </c>
+      <c r="P288" t="s">
+        <v>25</v>
+      </c>
+      <c r="R288" t="s">
+        <v>775</v>
+      </c>
+      <c r="S288" s="1">
+        <v>46082</v>
+      </c>
+      <c r="U288">
+        <v>1</v>
+      </c>
+      <c r="V288">
+        <v>0</v>
+      </c>
+      <c r="W288">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="289" spans="1:23" x14ac:dyDescent="0.4">
+      <c r="A289" t="s">
+        <v>901</v>
+      </c>
+      <c r="D289" s="1">
+        <v>46069</v>
+      </c>
+      <c r="E289" t="s">
+        <v>15</v>
+      </c>
+      <c r="I289" t="s">
+        <v>894</v>
+      </c>
+      <c r="J289" t="s">
+        <v>401</v>
+      </c>
+      <c r="M289" t="s">
+        <v>902</v>
+      </c>
+      <c r="N289" t="e" vm="2">
+        <v>#VALUE!</v>
+      </c>
+      <c r="P289" t="s">
+        <v>25</v>
+      </c>
+      <c r="R289" t="s">
+        <v>775</v>
+      </c>
+      <c r="S289" s="1">
+        <v>46073</v>
+      </c>
+      <c r="U289">
+        <v>1</v>
+      </c>
+      <c r="V289">
+        <v>0</v>
+      </c>
+      <c r="W289">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="290" spans="1:23" x14ac:dyDescent="0.4">
+      <c r="A290" t="s">
+        <v>905</v>
+      </c>
+      <c r="D290" s="1">
+        <v>46063</v>
+      </c>
+      <c r="E290" t="s">
+        <v>39</v>
+      </c>
+      <c r="F290" t="s">
+        <v>906</v>
+      </c>
+      <c r="I290" t="s">
+        <v>894</v>
+      </c>
+      <c r="J290" t="s">
+        <v>401</v>
+      </c>
+      <c r="M290" t="s">
+        <v>831</v>
+      </c>
+      <c r="N290" t="e" vm="1">
+        <v>#VALUE!</v>
+      </c>
+      <c r="P290" t="s">
+        <v>19</v>
+      </c>
+      <c r="R290" t="s">
+        <v>19</v>
+      </c>
+      <c r="S290" s="1">
+        <v>46055</v>
+      </c>
+      <c r="U290">
+        <v>1</v>
+      </c>
+      <c r="V290">
+        <v>0</v>
+      </c>
+      <c r="W290">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="291" spans="1:23" x14ac:dyDescent="0.4">
+      <c r="A291" t="s">
+        <v>907</v>
+      </c>
+      <c r="D291" s="1">
+        <v>46068</v>
+      </c>
+      <c r="E291" t="s">
+        <v>39</v>
+      </c>
+      <c r="F291" s="2" t="s">
+        <v>910</v>
+      </c>
+      <c r="H291" t="s">
+        <v>909</v>
+      </c>
+      <c r="I291" t="s">
+        <v>894</v>
+      </c>
+      <c r="J291" t="s">
+        <v>401</v>
+      </c>
+      <c r="M291" t="s">
+        <v>908</v>
+      </c>
+      <c r="N291" t="e" vm="21">
+        <v>#VALUE!</v>
+      </c>
+      <c r="P291" t="s">
+        <v>11</v>
+      </c>
+      <c r="R291" t="s">
+        <v>775</v>
+      </c>
+      <c r="S291" s="1">
+        <v>46068</v>
+      </c>
+      <c r="U291">
+        <v>1</v>
+      </c>
+      <c r="V291">
+        <v>0</v>
+      </c>
+      <c r="W291">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="292" spans="1:23" x14ac:dyDescent="0.4">
+      <c r="A292" t="s">
+        <v>911</v>
+      </c>
+      <c r="D292" s="1">
+        <v>46069</v>
+      </c>
+      <c r="E292" t="s">
+        <v>39</v>
+      </c>
+      <c r="F292" t="s">
+        <v>912</v>
+      </c>
+      <c r="I292" t="s">
+        <v>894</v>
+      </c>
+      <c r="J292" t="s">
+        <v>401</v>
+      </c>
+      <c r="M292" t="s">
+        <v>913</v>
+      </c>
+      <c r="N292" t="e" vm="1">
+        <v>#VALUE!</v>
+      </c>
+      <c r="P292" t="s">
+        <v>11</v>
+      </c>
+      <c r="R292" t="s">
+        <v>19</v>
+      </c>
+      <c r="S292" s="1">
+        <v>46080</v>
+      </c>
+      <c r="U292">
+        <v>1</v>
+      </c>
+      <c r="V292">
+        <v>0</v>
+      </c>
+      <c r="W292">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="293" spans="1:23" x14ac:dyDescent="0.4">
+      <c r="A293" t="s">
+        <v>914</v>
+      </c>
+      <c r="D293" s="1">
+        <v>46069</v>
+      </c>
+      <c r="E293" t="s">
+        <v>39</v>
+      </c>
+      <c r="F293" t="s">
+        <v>915</v>
+      </c>
+      <c r="I293" t="s">
+        <v>894</v>
+      </c>
+      <c r="J293" t="s">
+        <v>401</v>
+      </c>
+      <c r="M293" t="s">
+        <v>198</v>
+      </c>
+      <c r="N293" t="e" vm="10">
+        <v>#VALUE!</v>
+      </c>
+      <c r="P293" t="s">
+        <v>11</v>
+      </c>
+      <c r="R293" t="s">
+        <v>19</v>
+      </c>
+      <c r="S293" s="1">
+        <v>46082</v>
+      </c>
+      <c r="U293">
+        <v>1</v>
+      </c>
+      <c r="V293">
+        <v>0</v>
+      </c>
+      <c r="W293">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="294" spans="1:23" x14ac:dyDescent="0.4">
+      <c r="A294" t="s">
+        <v>916</v>
+      </c>
+      <c r="D294" s="1">
+        <v>46063</v>
+      </c>
+      <c r="E294" t="s">
+        <v>39</v>
+      </c>
+      <c r="F294" t="s">
+        <v>917</v>
+      </c>
+      <c r="I294" t="s">
+        <v>894</v>
+      </c>
+      <c r="J294" t="s">
+        <v>401</v>
+      </c>
+      <c r="M294" t="s">
+        <v>918</v>
+      </c>
+      <c r="N294" t="e" vm="1">
+        <v>#VALUE!</v>
+      </c>
+      <c r="P294" t="s">
+        <v>11</v>
+      </c>
+      <c r="R294" t="s">
+        <v>775</v>
+      </c>
+      <c r="S294" s="1">
+        <v>46082</v>
+      </c>
+      <c r="U294">
+        <v>1</v>
+      </c>
+      <c r="V294">
+        <v>0</v>
+      </c>
+      <c r="W294">
         <v>0</v>
       </c>
     </row>
@@ -50110,64 +50566,64 @@
       <sortCondition ref="D1:D267"/>
     </sortState>
   </autoFilter>
-  <conditionalFormatting sqref="A1:B208 A210:B1048576">
-    <cfRule type="duplicateValues" dxfId="262" priority="23"/>
+  <conditionalFormatting sqref="A1:B208 A210:B283 A285:B1048576 B284">
+    <cfRule type="duplicateValues" dxfId="251" priority="23"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A2:B22">
-    <cfRule type="duplicateValues" dxfId="261" priority="24"/>
+    <cfRule type="duplicateValues" dxfId="250" priority="24"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A61:B61">
-    <cfRule type="duplicateValues" dxfId="260" priority="22"/>
+    <cfRule type="duplicateValues" dxfId="249" priority="22"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="I1:I1048576">
-    <cfRule type="containsText" dxfId="259" priority="15" operator="containsText" text="closed">
+    <cfRule type="containsText" dxfId="248" priority="15" operator="containsText" text="closed">
       <formula>NOT(ISERROR(SEARCH("closed",I1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="258" priority="16" operator="containsText" text="abandoned">
+    <cfRule type="containsText" dxfId="247" priority="16" operator="containsText" text="abandoned">
       <formula>NOT(ISERROR(SEARCH("abandoned",I1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="257" priority="18" operator="containsText" text="late app">
+    <cfRule type="containsText" dxfId="246" priority="18" operator="containsText" text="late app">
       <formula>NOT(ISERROR(SEARCH("late app",I1)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P78:P80 P83:P89 P92:P112 P115:P124 P126:P181 S136 S153 S159 S166 S173 S178 P183:P205 P208:P211 P213:P218 P220:P233 S225 P235:P237 P239:P248 I1:J1 P276:P283 R276:R283 I2:L1048576">
-    <cfRule type="containsText" dxfId="256" priority="21" operator="containsText" text="completed">
+  <conditionalFormatting sqref="I2:L1048576 P78:P80 P83:P89 P92:P112 P115:P124 P126:P181 S136 S153 S159 S166 S173 S178 P183:P205 P208:P211 P213:P218 P220:P233 S225 P235:P237 P239:P248 N284:N285 I1:J1 N291:N293 P276:P294 R276:R294">
+    <cfRule type="containsText" dxfId="245" priority="21" operator="containsText" text="completed">
       <formula>NOT(ISERROR(SEARCH("completed",I1)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J1:J1048576">
-    <cfRule type="containsText" dxfId="255" priority="10" operator="containsText" text="no news">
+    <cfRule type="containsText" dxfId="244" priority="10" operator="containsText" text="no news">
       <formula>NOT(ISERROR(SEARCH("no news",J1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="254" priority="11" operator="containsText" text="offer">
+    <cfRule type="containsText" dxfId="243" priority="11" operator="containsText" text="offer">
       <formula>NOT(ISERROR(SEARCH("offer",J1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="253" priority="12" operator="containsText" text="fly out">
+    <cfRule type="containsText" dxfId="242" priority="12" operator="containsText" text="fly out">
       <formula>NOT(ISERROR(SEARCH("fly out",J1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="252" priority="13" operator="containsText" text="interview">
+    <cfRule type="containsText" dxfId="241" priority="13" operator="containsText" text="interview">
       <formula>NOT(ISERROR(SEARCH("interview",J1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="251" priority="14" operator="containsText" text="rejected">
+    <cfRule type="containsText" dxfId="240" priority="14" operator="containsText" text="rejected">
       <formula>NOT(ISERROR(SEARCH("rejected",J1)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K1:L1048576 P78:P80 P83:P89 P92:P112 P115:P124 P126:P181 S136 S153 S159 S166 S173 S178 P183:P205 P208:P211 P213:P218 P220:P233 S225 P235:P237 P239:P248 P276:P283 R276:R283">
-    <cfRule type="containsText" dxfId="250" priority="19" operator="containsText" text="NO">
+  <conditionalFormatting sqref="K1:L1048576 P78:P80 P83:P89 P92:P112 P115:P124 P126:P181 S136 S153 S159 S166 S173 S178 P183:P205 P208:P211 P213:P218 P220:P233 S225 P235:P237 P239:P248 N284:N285 N291:N293 P276:P294 R276:R294">
+    <cfRule type="containsText" dxfId="239" priority="19" operator="containsText" text="NO">
       <formula>NOT(ISERROR(SEARCH("NO",K1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="249" priority="20" operator="containsText" text="YES">
+    <cfRule type="containsText" dxfId="238" priority="20" operator="containsText" text="YES">
       <formula>NOT(ISERROR(SEARCH("YES",K1)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="P250:P267">
-    <cfRule type="containsText" dxfId="248" priority="1" operator="containsText" text="NO">
+    <cfRule type="containsText" dxfId="237" priority="1" operator="containsText" text="NO">
       <formula>NOT(ISERROR(SEARCH("NO",P250)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="247" priority="2" operator="containsText" text="YES">
+    <cfRule type="containsText" dxfId="236" priority="2" operator="containsText" text="YES">
       <formula>NOT(ISERROR(SEARCH("YES",P250)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="246" priority="3" operator="containsText" text="completed">
+    <cfRule type="containsText" dxfId="235" priority="3" operator="containsText" text="completed">
       <formula>NOT(ISERROR(SEARCH("completed",P250)))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -50282,19 +50738,20 @@
     <hyperlink ref="F272" r:id="rId108" xr:uid="{34317180-A8EC-4C92-AB27-7AD534355822}"/>
     <hyperlink ref="F246" r:id="rId109" xr:uid="{81F56FF4-6BEE-4876-B897-D914C7668775}"/>
     <hyperlink ref="E275" r:id="rId110" xr:uid="{ACFEBBD7-5100-486E-81B2-AD29703033C3}"/>
+    <hyperlink ref="F291" r:id="rId111" xr:uid="{311A156E-3561-465E-A136-460E4C083957}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId111"/>
+  <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId112"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{923E81FA-B875-3C4E-A189-1A21268FA086}">
-  <dimension ref="A1:C341"/>
+  <dimension ref="A1:C348"/>
   <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="16" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="32.83203125" customWidth="1"/>
-    <col min="2" max="2" width="17.25" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.1640625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="21" customWidth="1"/>
   </cols>
   <sheetData>
@@ -53894,7 +54351,7 @@
         <v>46049</v>
       </c>
       <c r="B334" t="s">
-        <v>882</v>
+        <v>881</v>
       </c>
       <c r="C334" t="s">
         <v>96</v>
@@ -53905,7 +54362,7 @@
         <v>46049</v>
       </c>
       <c r="B335" t="s">
-        <v>880</v>
+        <v>879</v>
       </c>
       <c r="C335" t="s">
         <v>96</v>
@@ -53927,7 +54384,7 @@
         <v>46052</v>
       </c>
       <c r="B337" t="s">
-        <v>884</v>
+        <v>883</v>
       </c>
       <c r="C337" t="s">
         <v>96</v>
@@ -53938,7 +54395,7 @@
         <v>46052</v>
       </c>
       <c r="B338" t="s">
-        <v>885</v>
+        <v>884</v>
       </c>
       <c r="C338" t="s">
         <v>96</v>
@@ -53949,7 +54406,7 @@
         <v>46052</v>
       </c>
       <c r="B339" t="s">
-        <v>887</v>
+        <v>886</v>
       </c>
       <c r="C339" t="s">
         <v>96</v>
@@ -53960,7 +54417,7 @@
         <v>46052</v>
       </c>
       <c r="B340" t="s">
-        <v>889</v>
+        <v>888</v>
       </c>
       <c r="C340" t="s">
         <v>96</v>
@@ -53971,669 +54428,759 @@
         <v>46052</v>
       </c>
       <c r="B341" t="s">
-        <v>890</v>
+        <v>889</v>
       </c>
       <c r="C341" t="s">
         <v>96</v>
       </c>
     </row>
+    <row r="342" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A342" s="1">
+        <v>46055</v>
+      </c>
+      <c r="B342" t="s">
+        <v>721</v>
+      </c>
+      <c r="C342" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="343" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A343" s="1">
+        <v>46056</v>
+      </c>
+      <c r="B343" t="s">
+        <v>889</v>
+      </c>
+      <c r="C343" t="s">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="344" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A344" s="1">
+        <v>46056</v>
+      </c>
+      <c r="B344" t="s">
+        <v>224</v>
+      </c>
+      <c r="C344" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="345" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A345" s="1">
+        <v>46058</v>
+      </c>
+      <c r="B345" t="s">
+        <v>738</v>
+      </c>
+      <c r="C345" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="346" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A346" s="1">
+        <v>46058</v>
+      </c>
+      <c r="B346" t="s">
+        <v>478</v>
+      </c>
+      <c r="C346" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="347" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A347" s="1">
+        <v>46058</v>
+      </c>
+      <c r="B347" t="s">
+        <v>890</v>
+      </c>
+      <c r="C347" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="348" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A348" s="1">
+        <v>46059</v>
+      </c>
+      <c r="C348" t="s">
+        <v>903</v>
+      </c>
+    </row>
   </sheetData>
   <conditionalFormatting sqref="B5">
-    <cfRule type="duplicateValues" dxfId="245" priority="237"/>
-    <cfRule type="duplicateValues" dxfId="244" priority="238"/>
+    <cfRule type="duplicateValues" dxfId="234" priority="243"/>
+    <cfRule type="duplicateValues" dxfId="233" priority="244"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B10">
-    <cfRule type="duplicateValues" dxfId="243" priority="236"/>
-    <cfRule type="duplicateValues" dxfId="242" priority="235"/>
+    <cfRule type="duplicateValues" dxfId="232" priority="242"/>
+    <cfRule type="duplicateValues" dxfId="231" priority="241"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B11">
-    <cfRule type="duplicateValues" dxfId="241" priority="233"/>
-    <cfRule type="duplicateValues" dxfId="240" priority="234"/>
+    <cfRule type="duplicateValues" dxfId="230" priority="239"/>
+    <cfRule type="duplicateValues" dxfId="229" priority="240"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B12">
-    <cfRule type="duplicateValues" dxfId="239" priority="232"/>
-    <cfRule type="duplicateValues" dxfId="238" priority="231"/>
+    <cfRule type="duplicateValues" dxfId="228" priority="238"/>
+    <cfRule type="duplicateValues" dxfId="227" priority="237"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B15">
-    <cfRule type="duplicateValues" dxfId="237" priority="230"/>
-    <cfRule type="duplicateValues" dxfId="236" priority="229"/>
+    <cfRule type="duplicateValues" dxfId="226" priority="236"/>
+    <cfRule type="duplicateValues" dxfId="225" priority="235"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B16">
-    <cfRule type="duplicateValues" dxfId="235" priority="228"/>
+    <cfRule type="duplicateValues" dxfId="224" priority="234"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B17">
-    <cfRule type="duplicateValues" dxfId="234" priority="227"/>
-    <cfRule type="duplicateValues" dxfId="233" priority="226"/>
+    <cfRule type="duplicateValues" dxfId="223" priority="233"/>
+    <cfRule type="duplicateValues" dxfId="222" priority="232"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B18">
-    <cfRule type="duplicateValues" dxfId="232" priority="225"/>
-    <cfRule type="duplicateValues" dxfId="231" priority="224"/>
+    <cfRule type="duplicateValues" dxfId="221" priority="230"/>
+    <cfRule type="duplicateValues" dxfId="220" priority="231"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B19">
-    <cfRule type="duplicateValues" dxfId="230" priority="223"/>
+    <cfRule type="duplicateValues" dxfId="219" priority="229"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B22:B23">
-    <cfRule type="duplicateValues" dxfId="229" priority="222"/>
-    <cfRule type="duplicateValues" dxfId="228" priority="221"/>
+    <cfRule type="duplicateValues" dxfId="218" priority="228"/>
+    <cfRule type="duplicateValues" dxfId="217" priority="227"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B24">
-    <cfRule type="duplicateValues" dxfId="227" priority="220"/>
-    <cfRule type="duplicateValues" dxfId="226" priority="219"/>
+    <cfRule type="duplicateValues" dxfId="216" priority="226"/>
+    <cfRule type="duplicateValues" dxfId="215" priority="225"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B27">
-    <cfRule type="duplicateValues" dxfId="225" priority="218"/>
-    <cfRule type="duplicateValues" dxfId="224" priority="217"/>
+    <cfRule type="duplicateValues" dxfId="214" priority="224"/>
+    <cfRule type="duplicateValues" dxfId="213" priority="223"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B28">
-    <cfRule type="duplicateValues" dxfId="223" priority="216"/>
+    <cfRule type="duplicateValues" dxfId="212" priority="222"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B29">
-    <cfRule type="duplicateValues" dxfId="222" priority="215"/>
-    <cfRule type="duplicateValues" dxfId="221" priority="214"/>
+    <cfRule type="duplicateValues" dxfId="211" priority="221"/>
+    <cfRule type="duplicateValues" dxfId="210" priority="220"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B30">
-    <cfRule type="duplicateValues" dxfId="220" priority="213"/>
+    <cfRule type="duplicateValues" dxfId="209" priority="219"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B31">
-    <cfRule type="duplicateValues" dxfId="219" priority="212"/>
+    <cfRule type="duplicateValues" dxfId="208" priority="218"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B32">
-    <cfRule type="duplicateValues" dxfId="218" priority="211"/>
+    <cfRule type="duplicateValues" dxfId="207" priority="217"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B33">
-    <cfRule type="duplicateValues" dxfId="217" priority="210"/>
+    <cfRule type="duplicateValues" dxfId="206" priority="216"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B34">
-    <cfRule type="duplicateValues" dxfId="216" priority="209"/>
+    <cfRule type="duplicateValues" dxfId="205" priority="215"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B35">
-    <cfRule type="duplicateValues" dxfId="215" priority="208"/>
+    <cfRule type="duplicateValues" dxfId="204" priority="214"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B37">
-    <cfRule type="duplicateValues" dxfId="214" priority="207"/>
+    <cfRule type="duplicateValues" dxfId="203" priority="213"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B38">
-    <cfRule type="duplicateValues" dxfId="213" priority="206"/>
+    <cfRule type="duplicateValues" dxfId="202" priority="212"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B42">
-    <cfRule type="duplicateValues" dxfId="212" priority="205"/>
+    <cfRule type="duplicateValues" dxfId="201" priority="211"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B43">
-    <cfRule type="duplicateValues" dxfId="211" priority="204"/>
+    <cfRule type="duplicateValues" dxfId="200" priority="210"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B44:B45">
-    <cfRule type="duplicateValues" dxfId="210" priority="203"/>
+    <cfRule type="duplicateValues" dxfId="199" priority="209"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B46">
-    <cfRule type="duplicateValues" dxfId="209" priority="202"/>
+    <cfRule type="duplicateValues" dxfId="198" priority="208"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B48">
-    <cfRule type="duplicateValues" dxfId="208" priority="201"/>
+    <cfRule type="duplicateValues" dxfId="197" priority="207"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B49">
-    <cfRule type="duplicateValues" dxfId="207" priority="200"/>
+    <cfRule type="duplicateValues" dxfId="196" priority="206"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B51">
-    <cfRule type="duplicateValues" dxfId="206" priority="199"/>
+    <cfRule type="duplicateValues" dxfId="195" priority="205"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B52">
-    <cfRule type="duplicateValues" dxfId="205" priority="198"/>
+    <cfRule type="duplicateValues" dxfId="194" priority="204"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B58">
-    <cfRule type="duplicateValues" dxfId="204" priority="196"/>
+    <cfRule type="duplicateValues" dxfId="193" priority="202"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B59">
-    <cfRule type="duplicateValues" dxfId="203" priority="194"/>
+    <cfRule type="duplicateValues" dxfId="192" priority="200"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B63">
-    <cfRule type="duplicateValues" dxfId="202" priority="193"/>
+    <cfRule type="duplicateValues" dxfId="191" priority="199"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B64">
-    <cfRule type="duplicateValues" dxfId="201" priority="191"/>
+    <cfRule type="duplicateValues" dxfId="190" priority="197"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B66">
-    <cfRule type="duplicateValues" dxfId="200" priority="190"/>
+    <cfRule type="duplicateValues" dxfId="189" priority="196"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B67">
-    <cfRule type="duplicateValues" dxfId="199" priority="189"/>
-    <cfRule type="duplicateValues" dxfId="198" priority="188"/>
+    <cfRule type="duplicateValues" dxfId="188" priority="195"/>
+    <cfRule type="duplicateValues" dxfId="187" priority="194"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B68">
-    <cfRule type="duplicateValues" dxfId="197" priority="187"/>
+    <cfRule type="duplicateValues" dxfId="186" priority="193"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B69">
-    <cfRule type="duplicateValues" dxfId="196" priority="186"/>
+    <cfRule type="duplicateValues" dxfId="185" priority="192"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B70">
-    <cfRule type="duplicateValues" dxfId="195" priority="184"/>
+    <cfRule type="duplicateValues" dxfId="184" priority="190"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B72">
-    <cfRule type="duplicateValues" dxfId="194" priority="183"/>
+    <cfRule type="duplicateValues" dxfId="183" priority="189"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B73">
-    <cfRule type="duplicateValues" dxfId="193" priority="181"/>
+    <cfRule type="duplicateValues" dxfId="182" priority="187"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B74">
-    <cfRule type="duplicateValues" dxfId="192" priority="180"/>
+    <cfRule type="duplicateValues" dxfId="181" priority="186"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B75">
-    <cfRule type="duplicateValues" dxfId="191" priority="179"/>
+    <cfRule type="duplicateValues" dxfId="180" priority="185"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B76">
-    <cfRule type="duplicateValues" dxfId="190" priority="178"/>
+    <cfRule type="duplicateValues" dxfId="179" priority="184"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B77">
-    <cfRule type="duplicateValues" dxfId="189" priority="176"/>
+    <cfRule type="duplicateValues" dxfId="178" priority="182"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B78">
-    <cfRule type="duplicateValues" dxfId="188" priority="175"/>
+    <cfRule type="duplicateValues" dxfId="177" priority="181"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B83">
-    <cfRule type="duplicateValues" dxfId="187" priority="174"/>
+    <cfRule type="duplicateValues" dxfId="176" priority="180"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B84">
-    <cfRule type="duplicateValues" dxfId="186" priority="173"/>
+    <cfRule type="duplicateValues" dxfId="175" priority="179"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B85">
-    <cfRule type="duplicateValues" dxfId="185" priority="172"/>
+    <cfRule type="duplicateValues" dxfId="174" priority="178"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B87">
-    <cfRule type="duplicateValues" dxfId="184" priority="171"/>
+    <cfRule type="duplicateValues" dxfId="173" priority="177"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B88">
-    <cfRule type="duplicateValues" dxfId="183" priority="170"/>
+    <cfRule type="duplicateValues" dxfId="172" priority="176"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B89">
-    <cfRule type="duplicateValues" dxfId="182" priority="169"/>
+    <cfRule type="duplicateValues" dxfId="171" priority="175"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B90">
-    <cfRule type="duplicateValues" dxfId="181" priority="168"/>
+    <cfRule type="duplicateValues" dxfId="170" priority="174"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B91">
-    <cfRule type="duplicateValues" dxfId="180" priority="167"/>
+    <cfRule type="duplicateValues" dxfId="169" priority="173"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B92">
-    <cfRule type="duplicateValues" dxfId="179" priority="166"/>
+    <cfRule type="duplicateValues" dxfId="168" priority="172"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B93">
-    <cfRule type="duplicateValues" dxfId="178" priority="165"/>
+    <cfRule type="duplicateValues" dxfId="167" priority="171"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B94">
-    <cfRule type="duplicateValues" dxfId="177" priority="164"/>
+    <cfRule type="duplicateValues" dxfId="166" priority="170"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B95">
-    <cfRule type="duplicateValues" dxfId="176" priority="163"/>
+    <cfRule type="duplicateValues" dxfId="165" priority="169"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B96">
-    <cfRule type="duplicateValues" dxfId="175" priority="162"/>
+    <cfRule type="duplicateValues" dxfId="164" priority="168"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B97">
-    <cfRule type="duplicateValues" dxfId="174" priority="161"/>
+    <cfRule type="duplicateValues" dxfId="163" priority="167"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B98">
-    <cfRule type="duplicateValues" dxfId="173" priority="160"/>
+    <cfRule type="duplicateValues" dxfId="162" priority="166"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B99">
-    <cfRule type="duplicateValues" dxfId="172" priority="159"/>
+    <cfRule type="duplicateValues" dxfId="161" priority="165"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B100">
-    <cfRule type="duplicateValues" dxfId="171" priority="158"/>
+    <cfRule type="duplicateValues" dxfId="160" priority="164"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B101">
-    <cfRule type="duplicateValues" dxfId="170" priority="157"/>
+    <cfRule type="duplicateValues" dxfId="159" priority="163"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B104">
-    <cfRule type="duplicateValues" dxfId="169" priority="156"/>
-    <cfRule type="duplicateValues" dxfId="168" priority="155"/>
+    <cfRule type="duplicateValues" dxfId="158" priority="162"/>
+    <cfRule type="duplicateValues" dxfId="157" priority="161"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B105:B106">
-    <cfRule type="duplicateValues" dxfId="167" priority="154"/>
+    <cfRule type="duplicateValues" dxfId="156" priority="160"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B107">
-    <cfRule type="duplicateValues" dxfId="166" priority="153"/>
+    <cfRule type="duplicateValues" dxfId="155" priority="159"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B108">
-    <cfRule type="duplicateValues" dxfId="165" priority="152"/>
+    <cfRule type="duplicateValues" dxfId="154" priority="158"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B109">
-    <cfRule type="duplicateValues" dxfId="164" priority="151"/>
+    <cfRule type="duplicateValues" dxfId="153" priority="157"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B110">
-    <cfRule type="duplicateValues" dxfId="163" priority="150"/>
+    <cfRule type="duplicateValues" dxfId="152" priority="156"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B111">
-    <cfRule type="duplicateValues" dxfId="162" priority="149"/>
+    <cfRule type="duplicateValues" dxfId="151" priority="155"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B112">
-    <cfRule type="duplicateValues" dxfId="161" priority="148"/>
+    <cfRule type="duplicateValues" dxfId="150" priority="154"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B113">
-    <cfRule type="duplicateValues" dxfId="160" priority="147"/>
+    <cfRule type="duplicateValues" dxfId="149" priority="153"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B114">
-    <cfRule type="duplicateValues" dxfId="159" priority="146"/>
+    <cfRule type="duplicateValues" dxfId="148" priority="152"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B115">
-    <cfRule type="duplicateValues" dxfId="158" priority="145"/>
+    <cfRule type="duplicateValues" dxfId="147" priority="151"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B116">
-    <cfRule type="duplicateValues" dxfId="157" priority="144"/>
+    <cfRule type="duplicateValues" dxfId="146" priority="150"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B117">
-    <cfRule type="duplicateValues" dxfId="156" priority="143"/>
+    <cfRule type="duplicateValues" dxfId="145" priority="149"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B118">
-    <cfRule type="duplicateValues" dxfId="155" priority="142"/>
+    <cfRule type="duplicateValues" dxfId="144" priority="148"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B119">
-    <cfRule type="duplicateValues" dxfId="154" priority="141"/>
+    <cfRule type="duplicateValues" dxfId="143" priority="147"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B120">
-    <cfRule type="duplicateValues" dxfId="153" priority="140"/>
+    <cfRule type="duplicateValues" dxfId="142" priority="146"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B121">
-    <cfRule type="duplicateValues" dxfId="152" priority="139"/>
+    <cfRule type="duplicateValues" dxfId="141" priority="145"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B122">
-    <cfRule type="duplicateValues" dxfId="151" priority="138"/>
+    <cfRule type="duplicateValues" dxfId="140" priority="144"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B126">
-    <cfRule type="duplicateValues" dxfId="150" priority="137"/>
+    <cfRule type="duplicateValues" dxfId="139" priority="143"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B127">
-    <cfRule type="duplicateValues" dxfId="149" priority="136"/>
+    <cfRule type="duplicateValues" dxfId="138" priority="142"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B128">
-    <cfRule type="duplicateValues" dxfId="148" priority="135"/>
+    <cfRule type="duplicateValues" dxfId="137" priority="141"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B129">
-    <cfRule type="duplicateValues" dxfId="147" priority="134"/>
+    <cfRule type="duplicateValues" dxfId="136" priority="140"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B130">
-    <cfRule type="duplicateValues" dxfId="146" priority="133"/>
+    <cfRule type="duplicateValues" dxfId="135" priority="139"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B131">
-    <cfRule type="duplicateValues" dxfId="145" priority="132"/>
+    <cfRule type="duplicateValues" dxfId="134" priority="138"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B132">
-    <cfRule type="duplicateValues" dxfId="144" priority="131"/>
+    <cfRule type="duplicateValues" dxfId="133" priority="137"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B133">
-    <cfRule type="duplicateValues" dxfId="143" priority="130"/>
+    <cfRule type="duplicateValues" dxfId="132" priority="136"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B136">
-    <cfRule type="duplicateValues" dxfId="142" priority="129"/>
+    <cfRule type="duplicateValues" dxfId="131" priority="135"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B137">
-    <cfRule type="duplicateValues" dxfId="141" priority="128"/>
+    <cfRule type="duplicateValues" dxfId="130" priority="134"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B138">
-    <cfRule type="duplicateValues" dxfId="140" priority="127"/>
+    <cfRule type="duplicateValues" dxfId="129" priority="133"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B139">
-    <cfRule type="duplicateValues" dxfId="139" priority="126"/>
+    <cfRule type="duplicateValues" dxfId="128" priority="132"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B140">
-    <cfRule type="duplicateValues" dxfId="138" priority="125"/>
+    <cfRule type="duplicateValues" dxfId="127" priority="131"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B141">
-    <cfRule type="duplicateValues" dxfId="137" priority="124"/>
+    <cfRule type="duplicateValues" dxfId="126" priority="130"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B142">
-    <cfRule type="duplicateValues" dxfId="136" priority="123"/>
+    <cfRule type="duplicateValues" dxfId="125" priority="129"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B143">
-    <cfRule type="duplicateValues" dxfId="135" priority="122"/>
+    <cfRule type="duplicateValues" dxfId="124" priority="128"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B144">
-    <cfRule type="duplicateValues" dxfId="134" priority="121"/>
+    <cfRule type="duplicateValues" dxfId="123" priority="127"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B145">
-    <cfRule type="duplicateValues" dxfId="133" priority="120"/>
+    <cfRule type="duplicateValues" dxfId="122" priority="126"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B147">
-    <cfRule type="duplicateValues" dxfId="132" priority="119"/>
+    <cfRule type="duplicateValues" dxfId="121" priority="125"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B148">
-    <cfRule type="duplicateValues" dxfId="131" priority="118"/>
+    <cfRule type="duplicateValues" dxfId="120" priority="124"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B149">
-    <cfRule type="duplicateValues" dxfId="130" priority="117"/>
+    <cfRule type="duplicateValues" dxfId="119" priority="123"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B150">
-    <cfRule type="duplicateValues" dxfId="129" priority="116"/>
+    <cfRule type="duplicateValues" dxfId="118" priority="122"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B151">
-    <cfRule type="duplicateValues" dxfId="128" priority="115"/>
+    <cfRule type="duplicateValues" dxfId="117" priority="121"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B152">
-    <cfRule type="duplicateValues" dxfId="127" priority="114"/>
+    <cfRule type="duplicateValues" dxfId="116" priority="120"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B153">
-    <cfRule type="duplicateValues" dxfId="126" priority="113"/>
+    <cfRule type="duplicateValues" dxfId="115" priority="119"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B154">
-    <cfRule type="duplicateValues" dxfId="125" priority="112"/>
+    <cfRule type="duplicateValues" dxfId="114" priority="118"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B155">
-    <cfRule type="duplicateValues" dxfId="124" priority="111"/>
+    <cfRule type="duplicateValues" dxfId="113" priority="117"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B156">
-    <cfRule type="duplicateValues" dxfId="123" priority="110"/>
+    <cfRule type="duplicateValues" dxfId="112" priority="116"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B157">
-    <cfRule type="duplicateValues" dxfId="122" priority="109"/>
+    <cfRule type="duplicateValues" dxfId="111" priority="115"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B171">
-    <cfRule type="duplicateValues" dxfId="121" priority="108"/>
+    <cfRule type="duplicateValues" dxfId="110" priority="114"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B172">
-    <cfRule type="duplicateValues" dxfId="120" priority="107"/>
+    <cfRule type="duplicateValues" dxfId="109" priority="113"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B174">
-    <cfRule type="duplicateValues" dxfId="119" priority="106"/>
+    <cfRule type="duplicateValues" dxfId="108" priority="112"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B177:B178">
-    <cfRule type="duplicateValues" dxfId="118" priority="105"/>
+    <cfRule type="duplicateValues" dxfId="107" priority="111"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B181">
-    <cfRule type="duplicateValues" dxfId="117" priority="104"/>
+    <cfRule type="duplicateValues" dxfId="106" priority="110"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B182">
-    <cfRule type="duplicateValues" dxfId="116" priority="103"/>
+    <cfRule type="duplicateValues" dxfId="105" priority="109"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B183">
-    <cfRule type="duplicateValues" dxfId="115" priority="102"/>
+    <cfRule type="duplicateValues" dxfId="104" priority="108"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B184">
-    <cfRule type="duplicateValues" dxfId="114" priority="101"/>
+    <cfRule type="duplicateValues" dxfId="103" priority="107"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B185">
-    <cfRule type="duplicateValues" dxfId="113" priority="100"/>
+    <cfRule type="duplicateValues" dxfId="102" priority="106"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B186">
-    <cfRule type="duplicateValues" dxfId="112" priority="99"/>
+    <cfRule type="duplicateValues" dxfId="101" priority="105"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B188">
-    <cfRule type="duplicateValues" dxfId="111" priority="98"/>
+    <cfRule type="duplicateValues" dxfId="100" priority="104"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B189">
-    <cfRule type="duplicateValues" dxfId="110" priority="97"/>
+    <cfRule type="duplicateValues" dxfId="99" priority="103"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B190">
-    <cfRule type="duplicateValues" dxfId="109" priority="96"/>
+    <cfRule type="duplicateValues" dxfId="98" priority="102"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B191">
-    <cfRule type="duplicateValues" dxfId="108" priority="95"/>
+    <cfRule type="duplicateValues" dxfId="97" priority="101"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B192">
-    <cfRule type="duplicateValues" dxfId="107" priority="94"/>
+    <cfRule type="duplicateValues" dxfId="96" priority="100"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B193">
-    <cfRule type="duplicateValues" dxfId="106" priority="93"/>
+    <cfRule type="duplicateValues" dxfId="95" priority="99"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B195">
-    <cfRule type="duplicateValues" dxfId="105" priority="92"/>
+    <cfRule type="duplicateValues" dxfId="94" priority="98"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B196">
-    <cfRule type="duplicateValues" dxfId="104" priority="91"/>
+    <cfRule type="duplicateValues" dxfId="93" priority="97"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B197">
-    <cfRule type="duplicateValues" dxfId="103" priority="90"/>
+    <cfRule type="duplicateValues" dxfId="92" priority="96"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B198">
-    <cfRule type="duplicateValues" dxfId="102" priority="89"/>
+    <cfRule type="duplicateValues" dxfId="91" priority="95"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B199">
-    <cfRule type="duplicateValues" dxfId="101" priority="88"/>
+    <cfRule type="duplicateValues" dxfId="90" priority="94"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B200">
-    <cfRule type="duplicateValues" dxfId="100" priority="87"/>
+    <cfRule type="duplicateValues" dxfId="89" priority="93"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B201">
-    <cfRule type="duplicateValues" dxfId="99" priority="86"/>
+    <cfRule type="duplicateValues" dxfId="88" priority="92"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B202">
-    <cfRule type="duplicateValues" dxfId="98" priority="85"/>
+    <cfRule type="duplicateValues" dxfId="87" priority="91"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B203">
-    <cfRule type="duplicateValues" dxfId="97" priority="84"/>
+    <cfRule type="duplicateValues" dxfId="86" priority="90"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B204">
-    <cfRule type="duplicateValues" dxfId="96" priority="83"/>
+    <cfRule type="duplicateValues" dxfId="85" priority="89"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B205">
-    <cfRule type="duplicateValues" dxfId="95" priority="82"/>
+    <cfRule type="duplicateValues" dxfId="84" priority="88"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B206">
-    <cfRule type="duplicateValues" dxfId="94" priority="81"/>
+    <cfRule type="duplicateValues" dxfId="83" priority="87"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B207">
-    <cfRule type="duplicateValues" dxfId="93" priority="80"/>
+    <cfRule type="duplicateValues" dxfId="82" priority="86"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B215">
-    <cfRule type="duplicateValues" dxfId="92" priority="79"/>
+    <cfRule type="duplicateValues" dxfId="81" priority="85"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B218">
-    <cfRule type="duplicateValues" dxfId="91" priority="78"/>
+    <cfRule type="duplicateValues" dxfId="80" priority="84"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B220">
-    <cfRule type="duplicateValues" dxfId="90" priority="77"/>
+    <cfRule type="duplicateValues" dxfId="79" priority="83"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B222">
-    <cfRule type="duplicateValues" dxfId="89" priority="76"/>
+    <cfRule type="duplicateValues" dxfId="78" priority="82"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B223">
-    <cfRule type="duplicateValues" dxfId="88" priority="75"/>
+    <cfRule type="duplicateValues" dxfId="77" priority="81"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B224">
-    <cfRule type="duplicateValues" dxfId="87" priority="74"/>
+    <cfRule type="duplicateValues" dxfId="76" priority="80"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B225">
-    <cfRule type="duplicateValues" dxfId="86" priority="73"/>
+    <cfRule type="duplicateValues" dxfId="75" priority="79"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B227">
-    <cfRule type="duplicateValues" dxfId="85" priority="72"/>
+    <cfRule type="duplicateValues" dxfId="74" priority="78"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B229">
-    <cfRule type="duplicateValues" dxfId="84" priority="71"/>
+    <cfRule type="duplicateValues" dxfId="73" priority="77"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B230">
-    <cfRule type="duplicateValues" dxfId="83" priority="70"/>
+    <cfRule type="duplicateValues" dxfId="72" priority="76"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B232">
-    <cfRule type="duplicateValues" dxfId="82" priority="69"/>
+    <cfRule type="duplicateValues" dxfId="71" priority="75"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B233">
-    <cfRule type="duplicateValues" dxfId="81" priority="68"/>
+    <cfRule type="duplicateValues" dxfId="70" priority="74"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B234">
-    <cfRule type="duplicateValues" dxfId="80" priority="67"/>
+    <cfRule type="duplicateValues" dxfId="69" priority="73"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B235">
-    <cfRule type="duplicateValues" dxfId="79" priority="66"/>
+    <cfRule type="duplicateValues" dxfId="68" priority="72"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B236">
-    <cfRule type="duplicateValues" dxfId="78" priority="65"/>
+    <cfRule type="duplicateValues" dxfId="67" priority="71"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B237">
-    <cfRule type="duplicateValues" dxfId="77" priority="64"/>
+    <cfRule type="duplicateValues" dxfId="66" priority="70"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B239">
-    <cfRule type="duplicateValues" dxfId="76" priority="62"/>
+    <cfRule type="duplicateValues" dxfId="65" priority="68"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B240">
-    <cfRule type="duplicateValues" dxfId="75" priority="61"/>
+    <cfRule type="duplicateValues" dxfId="64" priority="67"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B241">
-    <cfRule type="duplicateValues" dxfId="74" priority="60"/>
+    <cfRule type="duplicateValues" dxfId="63" priority="66"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B242">
-    <cfRule type="duplicateValues" dxfId="73" priority="59"/>
+    <cfRule type="duplicateValues" dxfId="62" priority="65"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B243">
-    <cfRule type="duplicateValues" dxfId="72" priority="58"/>
+    <cfRule type="duplicateValues" dxfId="61" priority="64"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B250">
-    <cfRule type="duplicateValues" dxfId="71" priority="57"/>
+    <cfRule type="duplicateValues" dxfId="60" priority="63"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B251">
-    <cfRule type="duplicateValues" dxfId="70" priority="56"/>
+    <cfRule type="duplicateValues" dxfId="59" priority="62"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B253">
-    <cfRule type="duplicateValues" dxfId="69" priority="55"/>
+    <cfRule type="duplicateValues" dxfId="58" priority="61"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B255">
-    <cfRule type="duplicateValues" dxfId="68" priority="54"/>
+    <cfRule type="duplicateValues" dxfId="57" priority="60"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B258:B259">
-    <cfRule type="duplicateValues" dxfId="67" priority="53"/>
+    <cfRule type="duplicateValues" dxfId="56" priority="59"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B260">
-    <cfRule type="duplicateValues" dxfId="66" priority="52"/>
+    <cfRule type="duplicateValues" dxfId="55" priority="58"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B265:B267 B269">
-    <cfRule type="duplicateValues" dxfId="65" priority="51"/>
+    <cfRule type="duplicateValues" dxfId="54" priority="57"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B268">
-    <cfRule type="duplicateValues" dxfId="64" priority="50"/>
+    <cfRule type="duplicateValues" dxfId="53" priority="56"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B270">
-    <cfRule type="duplicateValues" dxfId="63" priority="49"/>
+    <cfRule type="duplicateValues" dxfId="52" priority="55"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B271">
-    <cfRule type="duplicateValues" dxfId="62" priority="48"/>
+    <cfRule type="duplicateValues" dxfId="51" priority="54"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B273">
-    <cfRule type="duplicateValues" dxfId="61" priority="47"/>
+    <cfRule type="duplicateValues" dxfId="50" priority="53"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B275">
-    <cfRule type="duplicateValues" dxfId="60" priority="46"/>
+    <cfRule type="duplicateValues" dxfId="49" priority="52"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B278">
-    <cfRule type="duplicateValues" dxfId="59" priority="45"/>
+    <cfRule type="duplicateValues" dxfId="48" priority="51"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B279">
-    <cfRule type="duplicateValues" dxfId="58" priority="44"/>
+    <cfRule type="duplicateValues" dxfId="47" priority="50"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B280">
-    <cfRule type="duplicateValues" dxfId="57" priority="43"/>
+    <cfRule type="duplicateValues" dxfId="46" priority="49"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B281">
-    <cfRule type="duplicateValues" dxfId="56" priority="42"/>
+    <cfRule type="duplicateValues" dxfId="45" priority="48"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B282">
-    <cfRule type="duplicateValues" dxfId="55" priority="41"/>
+    <cfRule type="duplicateValues" dxfId="44" priority="47"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B283">
-    <cfRule type="duplicateValues" dxfId="54" priority="39"/>
+    <cfRule type="duplicateValues" dxfId="43" priority="45"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B284:B286">
-    <cfRule type="duplicateValues" dxfId="53" priority="38"/>
+    <cfRule type="duplicateValues" dxfId="42" priority="44"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B287">
-    <cfRule type="duplicateValues" dxfId="52" priority="37"/>
+    <cfRule type="duplicateValues" dxfId="41" priority="43"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B288">
-    <cfRule type="duplicateValues" dxfId="51" priority="36"/>
+    <cfRule type="duplicateValues" dxfId="40" priority="42"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B291">
-    <cfRule type="duplicateValues" dxfId="50" priority="35"/>
+    <cfRule type="duplicateValues" dxfId="39" priority="41"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B292">
-    <cfRule type="duplicateValues" dxfId="49" priority="34"/>
+    <cfRule type="duplicateValues" dxfId="38" priority="40"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B293">
-    <cfRule type="duplicateValues" dxfId="48" priority="33"/>
+    <cfRule type="duplicateValues" dxfId="37" priority="39"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B294">
-    <cfRule type="duplicateValues" dxfId="47" priority="32"/>
+    <cfRule type="duplicateValues" dxfId="36" priority="38"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B295">
-    <cfRule type="duplicateValues" dxfId="46" priority="31"/>
+    <cfRule type="duplicateValues" dxfId="35" priority="37"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B296">
-    <cfRule type="duplicateValues" dxfId="45" priority="30"/>
+    <cfRule type="duplicateValues" dxfId="34" priority="36"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B297">
-    <cfRule type="duplicateValues" dxfId="44" priority="29"/>
+    <cfRule type="duplicateValues" dxfId="33" priority="35"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B298">
-    <cfRule type="duplicateValues" dxfId="43" priority="28"/>
+    <cfRule type="duplicateValues" dxfId="32" priority="34"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B299">
-    <cfRule type="duplicateValues" dxfId="42" priority="27"/>
+    <cfRule type="duplicateValues" dxfId="31" priority="33"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B300">
-    <cfRule type="duplicateValues" dxfId="41" priority="26"/>
+    <cfRule type="duplicateValues" dxfId="30" priority="32"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B301">
-    <cfRule type="duplicateValues" dxfId="40" priority="25"/>
+    <cfRule type="duplicateValues" dxfId="29" priority="31"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B302">
-    <cfRule type="duplicateValues" dxfId="39" priority="24"/>
+    <cfRule type="duplicateValues" dxfId="28" priority="30"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B303">
-    <cfRule type="duplicateValues" dxfId="38" priority="23"/>
+    <cfRule type="duplicateValues" dxfId="27" priority="29"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B304">
-    <cfRule type="duplicateValues" dxfId="37" priority="22"/>
+    <cfRule type="duplicateValues" dxfId="26" priority="28"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B306">
-    <cfRule type="duplicateValues" dxfId="36" priority="21"/>
+    <cfRule type="duplicateValues" dxfId="25" priority="27"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B309">
-    <cfRule type="duplicateValues" dxfId="35" priority="20"/>
+    <cfRule type="duplicateValues" dxfId="24" priority="26"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B310">
-    <cfRule type="duplicateValues" dxfId="34" priority="19"/>
+    <cfRule type="duplicateValues" dxfId="23" priority="25"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B313">
-    <cfRule type="duplicateValues" dxfId="33" priority="18"/>
-    <cfRule type="duplicateValues" dxfId="32" priority="17"/>
+    <cfRule type="duplicateValues" dxfId="22" priority="24"/>
+    <cfRule type="duplicateValues" dxfId="21" priority="23"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B314">
-    <cfRule type="duplicateValues" dxfId="31" priority="16"/>
+    <cfRule type="duplicateValues" dxfId="20" priority="22"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B316">
-    <cfRule type="duplicateValues" dxfId="30" priority="15"/>
+    <cfRule type="duplicateValues" dxfId="19" priority="21"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B319">
-    <cfRule type="duplicateValues" dxfId="29" priority="14"/>
+    <cfRule type="duplicateValues" dxfId="18" priority="20"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B321">
-    <cfRule type="duplicateValues" dxfId="28" priority="12"/>
+    <cfRule type="duplicateValues" dxfId="17" priority="18"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B322">
-    <cfRule type="duplicateValues" dxfId="27" priority="11"/>
+    <cfRule type="duplicateValues" dxfId="16" priority="17"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B325">
-    <cfRule type="duplicateValues" dxfId="26" priority="10"/>
+    <cfRule type="duplicateValues" dxfId="15" priority="16"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B327">
-    <cfRule type="duplicateValues" dxfId="25" priority="9"/>
+    <cfRule type="duplicateValues" dxfId="14" priority="15"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B329">
-    <cfRule type="duplicateValues" dxfId="24" priority="8"/>
+    <cfRule type="duplicateValues" dxfId="13" priority="14"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B330">
-    <cfRule type="duplicateValues" dxfId="23" priority="7"/>
+    <cfRule type="duplicateValues" dxfId="12" priority="13"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B332">
-    <cfRule type="duplicateValues" dxfId="22" priority="6"/>
+    <cfRule type="duplicateValues" dxfId="11" priority="12"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B333">
-    <cfRule type="duplicateValues" dxfId="21" priority="5"/>
-    <cfRule type="duplicateValues" dxfId="20" priority="4"/>
+    <cfRule type="duplicateValues" dxfId="10" priority="10"/>
+    <cfRule type="duplicateValues" dxfId="9" priority="11"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B334">
-    <cfRule type="duplicateValues" dxfId="19" priority="3"/>
+    <cfRule type="duplicateValues" dxfId="8" priority="9"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B335">
-    <cfRule type="duplicateValues" dxfId="18" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="7" priority="8"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B337:B341">
-    <cfRule type="duplicateValues" dxfId="17" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="6" priority="7"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B342">
+    <cfRule type="duplicateValues" dxfId="5" priority="6"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B343">
+    <cfRule type="duplicateValues" dxfId="4" priority="5"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B344">
+    <cfRule type="duplicateValues" dxfId="3" priority="4"/>
+    <cfRule type="duplicateValues" dxfId="2" priority="3"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B345">
+    <cfRule type="duplicateValues" dxfId="1" priority="2"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B346">
+    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -54655,15 +55202,15 @@
       </c>
       <c r="B1" s="15">
         <f>COUNTA(sum!A:A) -1</f>
-        <v>282</v>
+        <v>293</v>
       </c>
       <c r="C1" s="22">
         <f>COUNTIF(sum!I:I, "completed")/(B1-COUNTIF(sum!I:I, "abandoned")-COUNTIF(sum!I:I, "late app"))</f>
-        <v>1</v>
+        <v>0.96478873239436624</v>
       </c>
       <c r="D1" s="21">
         <f>COUNTIF(sum!I:I, "completed")</f>
-        <v>273</v>
+        <v>274</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="22" customHeight="1" x14ac:dyDescent="0.4">
@@ -54698,7 +55245,7 @@
       </c>
       <c r="B5" s="15">
         <f>COUNTA(sum!J:J) -1</f>
-        <v>282</v>
+        <v>293</v>
       </c>
       <c r="C5" s="14">
         <f>B5/B1</f>
@@ -54711,11 +55258,11 @@
       </c>
       <c r="B6" s="16">
         <f>COUNTIFS(sum!J:J,"no news")</f>
-        <v>248</v>
+        <v>257</v>
       </c>
       <c r="C6" s="10">
         <f>B6/$B$5</f>
-        <v>0.87943262411347523</v>
+        <v>0.87713310580204773</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.4">
@@ -54724,11 +55271,11 @@
       </c>
       <c r="B7" s="16">
         <f>COUNTIFS(sum!J:J,"rejected")</f>
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="C7" s="10">
         <f t="shared" ref="C7:C10" si="0">B7/$B$5</f>
-        <v>9.2198581560283682E-2</v>
+        <v>9.556313993174062E-2</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.4">
@@ -54741,7 +55288,7 @@
       </c>
       <c r="C8" s="10">
         <f t="shared" si="0"/>
-        <v>2.8368794326241134E-2</v>
+        <v>2.7303754266211604E-2</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.4">
@@ -54754,7 +55301,7 @@
       </c>
       <c r="C9" s="10">
         <f t="shared" si="0"/>
-        <v>3.5460992907801418E-3</v>
+        <v>3.4129692832764505E-3</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.4">
@@ -54772,7 +55319,7 @@
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A11" s="23" t="s">
-        <v>879</v>
+        <v>904</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
new round of applications
</commit_message>
<xml_diff>
--- a/EconJM_status.xlsx
+++ b/EconJM_status.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\javie\Dropbox\Work\Job Search\2025 EconJM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{851EE1F0-9E31-4B99-A62B-5757413AF67B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4CB7AFDA-2E68-45BA-8FD0-E8E046281AFB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="14620" xr2:uid="{6FE48536-7E5C-BF4C-9490-2A6392576298}"/>
   </bookViews>
@@ -428,7 +428,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3025" uniqueCount="919">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3063" uniqueCount="925">
   <si>
     <t>add_id</t>
   </si>
@@ -3221,6 +3221,24 @@
   </si>
   <si>
     <t>Northwestern College</t>
+  </si>
+  <si>
+    <t>tilurg_postdoc</t>
+  </si>
+  <si>
+    <t>Tilurg University</t>
+  </si>
+  <si>
+    <t>south_denmark</t>
+  </si>
+  <si>
+    <t>https://fa-eosd-saasfaprod1.fa.ocs.oraclecloud.com/hcmUI/CandidateExperience/en/sites/CX_1001/job/3205</t>
+  </si>
+  <si>
+    <t>Danish Institute for Advanced Study</t>
+  </si>
+  <si>
+    <t>full</t>
   </si>
 </sst>
 </file>
@@ -3412,7 +3430,67 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Percent" xfId="2" builtinId="5"/>
   </cellStyles>
-  <dxfs count="252">
+  <dxfs count="258">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -36157,7 +36235,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F7772053-9363-CA4A-A53F-040B7C700753}">
-  <dimension ref="A1:W294"/>
+  <dimension ref="A1:W296"/>
   <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="16" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="19.6640625" customWidth="1"/>
@@ -50143,7 +50221,7 @@
         <v>15</v>
       </c>
       <c r="I285" t="s">
-        <v>894</v>
+        <v>95</v>
       </c>
       <c r="J285" t="s">
         <v>401</v>
@@ -50153,6 +50231,10 @@
       </c>
       <c r="N285" t="e" vm="4">
         <v>#VALUE!</v>
+      </c>
+      <c r="O285" t="str" cm="1">
+        <f t="array" aca="1" ref="O285" ca="1">_FV(N285,"Name")</f>
+        <v>France</v>
       </c>
       <c r="P285" t="s">
         <v>25</v>
@@ -50184,7 +50266,7 @@
         <v>15</v>
       </c>
       <c r="I286" t="s">
-        <v>894</v>
+        <v>95</v>
       </c>
       <c r="J286" t="s">
         <v>401</v>
@@ -50194,6 +50276,10 @@
       </c>
       <c r="N286" t="e" vm="10">
         <v>#VALUE!</v>
+      </c>
+      <c r="O286" t="str" cm="1">
+        <f t="array" aca="1" ref="O286" ca="1">_FV(N286,"Name")</f>
+        <v>Canada</v>
       </c>
       <c r="P286" t="s">
         <v>25</v>
@@ -50225,7 +50311,7 @@
         <v>15</v>
       </c>
       <c r="I287" t="s">
-        <v>894</v>
+        <v>95</v>
       </c>
       <c r="J287" t="s">
         <v>401</v>
@@ -50235,6 +50321,10 @@
       </c>
       <c r="N287" t="e" vm="22">
         <v>#VALUE!</v>
+      </c>
+      <c r="O287" t="str" cm="1">
+        <f t="array" aca="1" ref="O287" ca="1">_FV(N287,"Name")</f>
+        <v>Portugal</v>
       </c>
       <c r="P287" t="s">
         <v>11</v>
@@ -50266,7 +50356,7 @@
         <v>15</v>
       </c>
       <c r="I288" t="s">
-        <v>894</v>
+        <v>95</v>
       </c>
       <c r="J288" t="s">
         <v>401</v>
@@ -50276,6 +50366,10 @@
       </c>
       <c r="N288" t="e" vm="4">
         <v>#VALUE!</v>
+      </c>
+      <c r="O288" t="str" cm="1">
+        <f t="array" aca="1" ref="O288" ca="1">_FV(N288,"Name")</f>
+        <v>France</v>
       </c>
       <c r="P288" t="s">
         <v>25</v>
@@ -50307,7 +50401,7 @@
         <v>15</v>
       </c>
       <c r="I289" t="s">
-        <v>894</v>
+        <v>95</v>
       </c>
       <c r="J289" t="s">
         <v>401</v>
@@ -50317,6 +50411,10 @@
       </c>
       <c r="N289" t="e" vm="2">
         <v>#VALUE!</v>
+      </c>
+      <c r="O289" t="str" cm="1">
+        <f t="array" aca="1" ref="O289" ca="1">_FV(N289,"Name")</f>
+        <v>Spain</v>
       </c>
       <c r="P289" t="s">
         <v>25</v>
@@ -50351,7 +50449,7 @@
         <v>906</v>
       </c>
       <c r="I290" t="s">
-        <v>894</v>
+        <v>95</v>
       </c>
       <c r="J290" t="s">
         <v>401</v>
@@ -50361,6 +50459,10 @@
       </c>
       <c r="N290" t="e" vm="1">
         <v>#VALUE!</v>
+      </c>
+      <c r="O290" t="str" cm="1">
+        <f t="array" aca="1" ref="O290" ca="1">_FV(N290,"Name")</f>
+        <v>United States</v>
       </c>
       <c r="P290" t="s">
         <v>19</v>
@@ -50398,7 +50500,7 @@
         <v>909</v>
       </c>
       <c r="I291" t="s">
-        <v>894</v>
+        <v>95</v>
       </c>
       <c r="J291" t="s">
         <v>401</v>
@@ -50408,6 +50510,10 @@
       </c>
       <c r="N291" t="e" vm="21">
         <v>#VALUE!</v>
+      </c>
+      <c r="O291" t="str" cm="1">
+        <f t="array" aca="1" ref="O291" ca="1">_FV(N291,"Name")</f>
+        <v>United Kingdom</v>
       </c>
       <c r="P291" t="s">
         <v>11</v>
@@ -50453,6 +50559,10 @@
       <c r="N292" t="e" vm="1">
         <v>#VALUE!</v>
       </c>
+      <c r="O292" t="str" cm="1">
+        <f t="array" aca="1" ref="O292" ca="1">_FV(N292,"Name")</f>
+        <v>United States</v>
+      </c>
       <c r="P292" t="s">
         <v>11</v>
       </c>
@@ -50497,6 +50607,10 @@
       <c r="N293" t="e" vm="10">
         <v>#VALUE!</v>
       </c>
+      <c r="O293" t="str" cm="1">
+        <f t="array" aca="1" ref="O293" ca="1">_FV(N293,"Name")</f>
+        <v>Canada</v>
+      </c>
       <c r="P293" t="s">
         <v>11</v>
       </c>
@@ -50541,6 +50655,10 @@
       <c r="N294" t="e" vm="1">
         <v>#VALUE!</v>
       </c>
+      <c r="O294" t="str" cm="1">
+        <f t="array" aca="1" ref="O294" ca="1">_FV(N294,"Name")</f>
+        <v>United States</v>
+      </c>
       <c r="P294" t="s">
         <v>11</v>
       </c>
@@ -50557,6 +50675,96 @@
         <v>0</v>
       </c>
       <c r="W294">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="295" spans="1:23" x14ac:dyDescent="0.4">
+      <c r="A295" t="s">
+        <v>919</v>
+      </c>
+      <c r="D295" s="1">
+        <v>46068</v>
+      </c>
+      <c r="E295" t="s">
+        <v>15</v>
+      </c>
+      <c r="I295" t="s">
+        <v>95</v>
+      </c>
+      <c r="J295" t="s">
+        <v>401</v>
+      </c>
+      <c r="M295" t="s">
+        <v>920</v>
+      </c>
+      <c r="N295" t="e" vm="6">
+        <v>#VALUE!</v>
+      </c>
+      <c r="O295" t="str" cm="1">
+        <f t="array" aca="1" ref="O295" ca="1">_FV(N295,"Name")</f>
+        <v>Netherlands</v>
+      </c>
+      <c r="P295" t="s">
+        <v>25</v>
+      </c>
+      <c r="R295" t="s">
+        <v>775</v>
+      </c>
+      <c r="S295" s="1">
+        <v>46068</v>
+      </c>
+      <c r="U295">
+        <v>1</v>
+      </c>
+      <c r="V295">
+        <v>0</v>
+      </c>
+      <c r="W295">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="296" spans="1:23" x14ac:dyDescent="0.4">
+      <c r="A296" t="s">
+        <v>921</v>
+      </c>
+      <c r="D296" s="1">
+        <v>46069</v>
+      </c>
+      <c r="F296" s="2" t="s">
+        <v>922</v>
+      </c>
+      <c r="I296" t="s">
+        <v>95</v>
+      </c>
+      <c r="J296" t="s">
+        <v>401</v>
+      </c>
+      <c r="M296" t="s">
+        <v>923</v>
+      </c>
+      <c r="N296" t="e" vm="20">
+        <v>#VALUE!</v>
+      </c>
+      <c r="O296" t="str" cm="1">
+        <f t="array" aca="1" ref="O296" ca="1">_FV(N296,"Name")</f>
+        <v>Denmark</v>
+      </c>
+      <c r="P296" t="s">
+        <v>924</v>
+      </c>
+      <c r="R296" t="s">
+        <v>775</v>
+      </c>
+      <c r="S296" s="1">
+        <v>46082</v>
+      </c>
+      <c r="U296">
+        <v>1</v>
+      </c>
+      <c r="V296">
+        <v>0</v>
+      </c>
+      <c r="W296">
         <v>0</v>
       </c>
     </row>
@@ -50567,63 +50775,63 @@
     </sortState>
   </autoFilter>
   <conditionalFormatting sqref="A1:B208 A210:B283 A285:B1048576 B284">
-    <cfRule type="duplicateValues" dxfId="251" priority="23"/>
+    <cfRule type="duplicateValues" dxfId="257" priority="23"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A2:B22">
-    <cfRule type="duplicateValues" dxfId="250" priority="24"/>
+    <cfRule type="duplicateValues" dxfId="256" priority="24"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A61:B61">
-    <cfRule type="duplicateValues" dxfId="249" priority="22"/>
+    <cfRule type="duplicateValues" dxfId="255" priority="22"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="I1:I1048576">
-    <cfRule type="containsText" dxfId="248" priority="15" operator="containsText" text="closed">
+    <cfRule type="containsText" dxfId="254" priority="15" operator="containsText" text="closed">
       <formula>NOT(ISERROR(SEARCH("closed",I1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="247" priority="16" operator="containsText" text="abandoned">
+    <cfRule type="containsText" dxfId="253" priority="16" operator="containsText" text="abandoned">
       <formula>NOT(ISERROR(SEARCH("abandoned",I1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="246" priority="18" operator="containsText" text="late app">
+    <cfRule type="containsText" dxfId="252" priority="18" operator="containsText" text="late app">
       <formula>NOT(ISERROR(SEARCH("late app",I1)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I2:L1048576 P78:P80 P83:P89 P92:P112 P115:P124 P126:P181 S136 S153 S159 S166 S173 S178 P183:P205 P208:P211 P213:P218 P220:P233 S225 P235:P237 P239:P248 N284:N285 I1:J1 N291:N293 P276:P294 R276:R294">
-    <cfRule type="containsText" dxfId="245" priority="21" operator="containsText" text="completed">
+  <conditionalFormatting sqref="P78:P80 P83:P89 P92:P112 P115:P124 P126:P181 S136 S153 S159 S166 S173 S178 P183:P205 P208:P211 P213:P218 P220:P233 S225 P235:P237 P239:P248 N284:N285 N291:N293 I1:J1 N295:N296 P276:P296 R276:R296 I2:L1048576">
+    <cfRule type="containsText" dxfId="251" priority="21" operator="containsText" text="completed">
       <formula>NOT(ISERROR(SEARCH("completed",I1)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J1:J1048576">
-    <cfRule type="containsText" dxfId="244" priority="10" operator="containsText" text="no news">
+    <cfRule type="containsText" dxfId="250" priority="10" operator="containsText" text="no news">
       <formula>NOT(ISERROR(SEARCH("no news",J1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="243" priority="11" operator="containsText" text="offer">
+    <cfRule type="containsText" dxfId="249" priority="11" operator="containsText" text="offer">
       <formula>NOT(ISERROR(SEARCH("offer",J1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="242" priority="12" operator="containsText" text="fly out">
+    <cfRule type="containsText" dxfId="248" priority="12" operator="containsText" text="fly out">
       <formula>NOT(ISERROR(SEARCH("fly out",J1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="241" priority="13" operator="containsText" text="interview">
+    <cfRule type="containsText" dxfId="247" priority="13" operator="containsText" text="interview">
       <formula>NOT(ISERROR(SEARCH("interview",J1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="240" priority="14" operator="containsText" text="rejected">
+    <cfRule type="containsText" dxfId="246" priority="14" operator="containsText" text="rejected">
       <formula>NOT(ISERROR(SEARCH("rejected",J1)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K1:L1048576 P78:P80 P83:P89 P92:P112 P115:P124 P126:P181 S136 S153 S159 S166 S173 S178 P183:P205 P208:P211 P213:P218 P220:P233 S225 P235:P237 P239:P248 N284:N285 N291:N293 P276:P294 R276:R294">
-    <cfRule type="containsText" dxfId="239" priority="19" operator="containsText" text="NO">
+  <conditionalFormatting sqref="K1:L1048576 P78:P80 P83:P89 P92:P112 P115:P124 P126:P181 S136 S153 S159 S166 S173 S178 P183:P205 P208:P211 P213:P218 P220:P233 S225 P235:P237 P239:P248 N284:N285 N291:N293 N295:N296 P276:P296 R276:R296">
+    <cfRule type="containsText" dxfId="245" priority="19" operator="containsText" text="NO">
       <formula>NOT(ISERROR(SEARCH("NO",K1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="238" priority="20" operator="containsText" text="YES">
+    <cfRule type="containsText" dxfId="244" priority="20" operator="containsText" text="YES">
       <formula>NOT(ISERROR(SEARCH("YES",K1)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="P250:P267">
-    <cfRule type="containsText" dxfId="237" priority="1" operator="containsText" text="NO">
+    <cfRule type="containsText" dxfId="243" priority="1" operator="containsText" text="NO">
       <formula>NOT(ISERROR(SEARCH("NO",P250)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="236" priority="2" operator="containsText" text="YES">
+    <cfRule type="containsText" dxfId="242" priority="2" operator="containsText" text="YES">
       <formula>NOT(ISERROR(SEARCH("YES",P250)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="235" priority="3" operator="containsText" text="completed">
+    <cfRule type="containsText" dxfId="241" priority="3" operator="containsText" text="completed">
       <formula>NOT(ISERROR(SEARCH("completed",P250)))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -50739,15 +50947,16 @@
     <hyperlink ref="F246" r:id="rId109" xr:uid="{81F56FF4-6BEE-4876-B897-D914C7668775}"/>
     <hyperlink ref="E275" r:id="rId110" xr:uid="{ACFEBBD7-5100-486E-81B2-AD29703033C3}"/>
     <hyperlink ref="F291" r:id="rId111" xr:uid="{311A156E-3561-465E-A136-460E4C083957}"/>
+    <hyperlink ref="F296" r:id="rId112" xr:uid="{6122D6CC-37C2-48AE-B198-BBEB4D956A30}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId112"/>
+  <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId113"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{923E81FA-B875-3C4E-A189-1A21268FA086}">
-  <dimension ref="A1:C348"/>
+  <dimension ref="A1:C360"/>
   <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="16" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="32.83203125" customWidth="1"/>
@@ -54508,678 +54717,828 @@
         <v>903</v>
       </c>
     </row>
+    <row r="349" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A349" s="1">
+        <v>46062</v>
+      </c>
+      <c r="B349" t="s">
+        <v>893</v>
+      </c>
+      <c r="C349" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="350" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A350" s="1">
+        <v>46062</v>
+      </c>
+      <c r="B350" t="s">
+        <v>895</v>
+      </c>
+      <c r="C350" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="351" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A351" s="1">
+        <v>46062</v>
+      </c>
+      <c r="B351" t="s">
+        <v>897</v>
+      </c>
+      <c r="C351" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="352" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A352" s="1">
+        <v>46062</v>
+      </c>
+      <c r="B352" t="s">
+        <v>899</v>
+      </c>
+      <c r="C352" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="353" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A353" s="1">
+        <v>46062</v>
+      </c>
+      <c r="B353" t="s">
+        <v>901</v>
+      </c>
+      <c r="C353" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="354" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A354" s="1">
+        <v>46062</v>
+      </c>
+      <c r="B354" t="s">
+        <v>919</v>
+      </c>
+      <c r="C354" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="355" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A355" s="1">
+        <v>46062</v>
+      </c>
+      <c r="B355" t="s">
+        <v>905</v>
+      </c>
+      <c r="C355" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="356" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A356" s="1">
+        <v>46062</v>
+      </c>
+      <c r="B356" t="s">
+        <v>907</v>
+      </c>
+      <c r="C356" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="357" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A357" s="1">
+        <v>46062</v>
+      </c>
+      <c r="B357" t="s">
+        <v>911</v>
+      </c>
+      <c r="C357" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="358" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A358" s="1">
+        <v>46062</v>
+      </c>
+      <c r="B358" t="s">
+        <v>914</v>
+      </c>
+      <c r="C358" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="359" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A359" s="1">
+        <v>46062</v>
+      </c>
+      <c r="B359" t="s">
+        <v>916</v>
+      </c>
+      <c r="C359" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="360" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A360" s="1">
+        <v>46062</v>
+      </c>
+      <c r="B360" t="s">
+        <v>921</v>
+      </c>
+      <c r="C360" t="s">
+        <v>96</v>
+      </c>
+    </row>
   </sheetData>
   <conditionalFormatting sqref="B5">
-    <cfRule type="duplicateValues" dxfId="234" priority="243"/>
-    <cfRule type="duplicateValues" dxfId="233" priority="244"/>
+    <cfRule type="duplicateValues" dxfId="240" priority="249"/>
+    <cfRule type="duplicateValues" dxfId="239" priority="250"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B10">
+    <cfRule type="duplicateValues" dxfId="238" priority="248"/>
+    <cfRule type="duplicateValues" dxfId="237" priority="247"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B11">
+    <cfRule type="duplicateValues" dxfId="236" priority="245"/>
+    <cfRule type="duplicateValues" dxfId="235" priority="246"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B12">
+    <cfRule type="duplicateValues" dxfId="234" priority="244"/>
+    <cfRule type="duplicateValues" dxfId="233" priority="243"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B15">
     <cfRule type="duplicateValues" dxfId="232" priority="242"/>
     <cfRule type="duplicateValues" dxfId="231" priority="241"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B11">
-    <cfRule type="duplicateValues" dxfId="230" priority="239"/>
-    <cfRule type="duplicateValues" dxfId="229" priority="240"/>
+  <conditionalFormatting sqref="B16">
+    <cfRule type="duplicateValues" dxfId="230" priority="240"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B12">
+  <conditionalFormatting sqref="B17">
+    <cfRule type="duplicateValues" dxfId="229" priority="239"/>
     <cfRule type="duplicateValues" dxfId="228" priority="238"/>
-    <cfRule type="duplicateValues" dxfId="227" priority="237"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B15">
-    <cfRule type="duplicateValues" dxfId="226" priority="236"/>
+  <conditionalFormatting sqref="B18">
+    <cfRule type="duplicateValues" dxfId="227" priority="236"/>
+    <cfRule type="duplicateValues" dxfId="226" priority="237"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B19">
     <cfRule type="duplicateValues" dxfId="225" priority="235"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B16">
+  <conditionalFormatting sqref="B22:B23">
     <cfRule type="duplicateValues" dxfId="224" priority="234"/>
+    <cfRule type="duplicateValues" dxfId="223" priority="233"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B17">
-    <cfRule type="duplicateValues" dxfId="223" priority="233"/>
+  <conditionalFormatting sqref="B24">
     <cfRule type="duplicateValues" dxfId="222" priority="232"/>
+    <cfRule type="duplicateValues" dxfId="221" priority="231"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B18">
-    <cfRule type="duplicateValues" dxfId="221" priority="230"/>
-    <cfRule type="duplicateValues" dxfId="220" priority="231"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B19">
+  <conditionalFormatting sqref="B27">
+    <cfRule type="duplicateValues" dxfId="220" priority="230"/>
     <cfRule type="duplicateValues" dxfId="219" priority="229"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B22:B23">
+  <conditionalFormatting sqref="B28">
     <cfRule type="duplicateValues" dxfId="218" priority="228"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B29">
     <cfRule type="duplicateValues" dxfId="217" priority="227"/>
+    <cfRule type="duplicateValues" dxfId="216" priority="226"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B24">
-    <cfRule type="duplicateValues" dxfId="216" priority="226"/>
+  <conditionalFormatting sqref="B30">
     <cfRule type="duplicateValues" dxfId="215" priority="225"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B27">
+  <conditionalFormatting sqref="B31">
     <cfRule type="duplicateValues" dxfId="214" priority="224"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B32">
     <cfRule type="duplicateValues" dxfId="213" priority="223"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B28">
+  <conditionalFormatting sqref="B33">
     <cfRule type="duplicateValues" dxfId="212" priority="222"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B29">
+  <conditionalFormatting sqref="B34">
     <cfRule type="duplicateValues" dxfId="211" priority="221"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B35">
     <cfRule type="duplicateValues" dxfId="210" priority="220"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B30">
+  <conditionalFormatting sqref="B37">
     <cfRule type="duplicateValues" dxfId="209" priority="219"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B31">
+  <conditionalFormatting sqref="B38">
     <cfRule type="duplicateValues" dxfId="208" priority="218"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B32">
+  <conditionalFormatting sqref="B42">
     <cfRule type="duplicateValues" dxfId="207" priority="217"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B33">
+  <conditionalFormatting sqref="B43">
     <cfRule type="duplicateValues" dxfId="206" priority="216"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B34">
+  <conditionalFormatting sqref="B44:B45">
     <cfRule type="duplicateValues" dxfId="205" priority="215"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B35">
+  <conditionalFormatting sqref="B46">
     <cfRule type="duplicateValues" dxfId="204" priority="214"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B37">
+  <conditionalFormatting sqref="B48">
     <cfRule type="duplicateValues" dxfId="203" priority="213"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B38">
+  <conditionalFormatting sqref="B49">
     <cfRule type="duplicateValues" dxfId="202" priority="212"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B42">
+  <conditionalFormatting sqref="B51">
     <cfRule type="duplicateValues" dxfId="201" priority="211"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B43">
+  <conditionalFormatting sqref="B52">
     <cfRule type="duplicateValues" dxfId="200" priority="210"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B44:B45">
-    <cfRule type="duplicateValues" dxfId="199" priority="209"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B46">
-    <cfRule type="duplicateValues" dxfId="198" priority="208"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B48">
-    <cfRule type="duplicateValues" dxfId="197" priority="207"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B49">
-    <cfRule type="duplicateValues" dxfId="196" priority="206"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B51">
-    <cfRule type="duplicateValues" dxfId="195" priority="205"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B52">
-    <cfRule type="duplicateValues" dxfId="194" priority="204"/>
-  </conditionalFormatting>
   <conditionalFormatting sqref="B58">
-    <cfRule type="duplicateValues" dxfId="193" priority="202"/>
+    <cfRule type="duplicateValues" dxfId="199" priority="208"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B59">
-    <cfRule type="duplicateValues" dxfId="192" priority="200"/>
+    <cfRule type="duplicateValues" dxfId="198" priority="206"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B63">
-    <cfRule type="duplicateValues" dxfId="191" priority="199"/>
+    <cfRule type="duplicateValues" dxfId="197" priority="205"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B64">
-    <cfRule type="duplicateValues" dxfId="190" priority="197"/>
+    <cfRule type="duplicateValues" dxfId="196" priority="203"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B66">
-    <cfRule type="duplicateValues" dxfId="189" priority="196"/>
+    <cfRule type="duplicateValues" dxfId="195" priority="202"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B67">
-    <cfRule type="duplicateValues" dxfId="188" priority="195"/>
-    <cfRule type="duplicateValues" dxfId="187" priority="194"/>
+    <cfRule type="duplicateValues" dxfId="194" priority="201"/>
+    <cfRule type="duplicateValues" dxfId="193" priority="200"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B68">
-    <cfRule type="duplicateValues" dxfId="186" priority="193"/>
+    <cfRule type="duplicateValues" dxfId="192" priority="199"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B69">
-    <cfRule type="duplicateValues" dxfId="185" priority="192"/>
+    <cfRule type="duplicateValues" dxfId="191" priority="198"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B70">
-    <cfRule type="duplicateValues" dxfId="184" priority="190"/>
+    <cfRule type="duplicateValues" dxfId="190" priority="196"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B72">
-    <cfRule type="duplicateValues" dxfId="183" priority="189"/>
+    <cfRule type="duplicateValues" dxfId="189" priority="195"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B73">
-    <cfRule type="duplicateValues" dxfId="182" priority="187"/>
+    <cfRule type="duplicateValues" dxfId="188" priority="193"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B74">
-    <cfRule type="duplicateValues" dxfId="181" priority="186"/>
+    <cfRule type="duplicateValues" dxfId="187" priority="192"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B75">
-    <cfRule type="duplicateValues" dxfId="180" priority="185"/>
+    <cfRule type="duplicateValues" dxfId="186" priority="191"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B76">
-    <cfRule type="duplicateValues" dxfId="179" priority="184"/>
+    <cfRule type="duplicateValues" dxfId="185" priority="190"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B77">
+    <cfRule type="duplicateValues" dxfId="184" priority="188"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B78">
+    <cfRule type="duplicateValues" dxfId="183" priority="187"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B83">
+    <cfRule type="duplicateValues" dxfId="182" priority="186"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B84">
+    <cfRule type="duplicateValues" dxfId="181" priority="185"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B85">
+    <cfRule type="duplicateValues" dxfId="180" priority="184"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B87">
+    <cfRule type="duplicateValues" dxfId="179" priority="183"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B88">
     <cfRule type="duplicateValues" dxfId="178" priority="182"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B78">
+  <conditionalFormatting sqref="B89">
     <cfRule type="duplicateValues" dxfId="177" priority="181"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B83">
+  <conditionalFormatting sqref="B90">
     <cfRule type="duplicateValues" dxfId="176" priority="180"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B84">
+  <conditionalFormatting sqref="B91">
     <cfRule type="duplicateValues" dxfId="175" priority="179"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B85">
+  <conditionalFormatting sqref="B92">
     <cfRule type="duplicateValues" dxfId="174" priority="178"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B87">
+  <conditionalFormatting sqref="B93">
     <cfRule type="duplicateValues" dxfId="173" priority="177"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B88">
+  <conditionalFormatting sqref="B94">
     <cfRule type="duplicateValues" dxfId="172" priority="176"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B89">
+  <conditionalFormatting sqref="B95">
     <cfRule type="duplicateValues" dxfId="171" priority="175"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B90">
+  <conditionalFormatting sqref="B96">
     <cfRule type="duplicateValues" dxfId="170" priority="174"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B91">
+  <conditionalFormatting sqref="B97">
     <cfRule type="duplicateValues" dxfId="169" priority="173"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B92">
+  <conditionalFormatting sqref="B98">
     <cfRule type="duplicateValues" dxfId="168" priority="172"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B93">
+  <conditionalFormatting sqref="B99">
     <cfRule type="duplicateValues" dxfId="167" priority="171"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B94">
+  <conditionalFormatting sqref="B100">
     <cfRule type="duplicateValues" dxfId="166" priority="170"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B95">
+  <conditionalFormatting sqref="B101">
     <cfRule type="duplicateValues" dxfId="165" priority="169"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B96">
+  <conditionalFormatting sqref="B104">
     <cfRule type="duplicateValues" dxfId="164" priority="168"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B97">
     <cfRule type="duplicateValues" dxfId="163" priority="167"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B98">
+  <conditionalFormatting sqref="B105:B106">
     <cfRule type="duplicateValues" dxfId="162" priority="166"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B99">
+  <conditionalFormatting sqref="B107">
     <cfRule type="duplicateValues" dxfId="161" priority="165"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B100">
+  <conditionalFormatting sqref="B108">
     <cfRule type="duplicateValues" dxfId="160" priority="164"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B101">
+  <conditionalFormatting sqref="B109">
     <cfRule type="duplicateValues" dxfId="159" priority="163"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B104">
+  <conditionalFormatting sqref="B110">
     <cfRule type="duplicateValues" dxfId="158" priority="162"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B111">
     <cfRule type="duplicateValues" dxfId="157" priority="161"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B105:B106">
+  <conditionalFormatting sqref="B112">
     <cfRule type="duplicateValues" dxfId="156" priority="160"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B107">
+  <conditionalFormatting sqref="B113">
     <cfRule type="duplicateValues" dxfId="155" priority="159"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B108">
+  <conditionalFormatting sqref="B114">
     <cfRule type="duplicateValues" dxfId="154" priority="158"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B109">
+  <conditionalFormatting sqref="B115">
     <cfRule type="duplicateValues" dxfId="153" priority="157"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B110">
+  <conditionalFormatting sqref="B116">
     <cfRule type="duplicateValues" dxfId="152" priority="156"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B111">
+  <conditionalFormatting sqref="B117">
     <cfRule type="duplicateValues" dxfId="151" priority="155"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B112">
+  <conditionalFormatting sqref="B118">
     <cfRule type="duplicateValues" dxfId="150" priority="154"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B113">
+  <conditionalFormatting sqref="B119">
     <cfRule type="duplicateValues" dxfId="149" priority="153"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B114">
+  <conditionalFormatting sqref="B120">
     <cfRule type="duplicateValues" dxfId="148" priority="152"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B115">
+  <conditionalFormatting sqref="B121">
     <cfRule type="duplicateValues" dxfId="147" priority="151"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B116">
+  <conditionalFormatting sqref="B122">
     <cfRule type="duplicateValues" dxfId="146" priority="150"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B117">
+  <conditionalFormatting sqref="B126">
     <cfRule type="duplicateValues" dxfId="145" priority="149"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B118">
+  <conditionalFormatting sqref="B127">
     <cfRule type="duplicateValues" dxfId="144" priority="148"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B119">
+  <conditionalFormatting sqref="B128">
     <cfRule type="duplicateValues" dxfId="143" priority="147"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B120">
+  <conditionalFormatting sqref="B129">
     <cfRule type="duplicateValues" dxfId="142" priority="146"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B121">
+  <conditionalFormatting sqref="B130">
     <cfRule type="duplicateValues" dxfId="141" priority="145"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B122">
+  <conditionalFormatting sqref="B131">
     <cfRule type="duplicateValues" dxfId="140" priority="144"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B126">
+  <conditionalFormatting sqref="B132">
     <cfRule type="duplicateValues" dxfId="139" priority="143"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B127">
+  <conditionalFormatting sqref="B133">
     <cfRule type="duplicateValues" dxfId="138" priority="142"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B128">
+  <conditionalFormatting sqref="B136">
     <cfRule type="duplicateValues" dxfId="137" priority="141"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B129">
+  <conditionalFormatting sqref="B137">
     <cfRule type="duplicateValues" dxfId="136" priority="140"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B130">
+  <conditionalFormatting sqref="B138">
     <cfRule type="duplicateValues" dxfId="135" priority="139"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B131">
+  <conditionalFormatting sqref="B139">
     <cfRule type="duplicateValues" dxfId="134" priority="138"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B132">
+  <conditionalFormatting sqref="B140">
     <cfRule type="duplicateValues" dxfId="133" priority="137"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B133">
+  <conditionalFormatting sqref="B141">
     <cfRule type="duplicateValues" dxfId="132" priority="136"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B136">
+  <conditionalFormatting sqref="B142">
     <cfRule type="duplicateValues" dxfId="131" priority="135"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B137">
+  <conditionalFormatting sqref="B143">
     <cfRule type="duplicateValues" dxfId="130" priority="134"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B138">
+  <conditionalFormatting sqref="B144">
     <cfRule type="duplicateValues" dxfId="129" priority="133"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B139">
+  <conditionalFormatting sqref="B145">
     <cfRule type="duplicateValues" dxfId="128" priority="132"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B140">
+  <conditionalFormatting sqref="B147">
     <cfRule type="duplicateValues" dxfId="127" priority="131"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B141">
+  <conditionalFormatting sqref="B148">
     <cfRule type="duplicateValues" dxfId="126" priority="130"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B142">
+  <conditionalFormatting sqref="B149">
     <cfRule type="duplicateValues" dxfId="125" priority="129"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B143">
+  <conditionalFormatting sqref="B150">
     <cfRule type="duplicateValues" dxfId="124" priority="128"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B144">
+  <conditionalFormatting sqref="B151">
     <cfRule type="duplicateValues" dxfId="123" priority="127"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B145">
+  <conditionalFormatting sqref="B152">
     <cfRule type="duplicateValues" dxfId="122" priority="126"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B147">
+  <conditionalFormatting sqref="B153">
     <cfRule type="duplicateValues" dxfId="121" priority="125"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B148">
+  <conditionalFormatting sqref="B154">
     <cfRule type="duplicateValues" dxfId="120" priority="124"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B149">
+  <conditionalFormatting sqref="B155">
     <cfRule type="duplicateValues" dxfId="119" priority="123"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B150">
+  <conditionalFormatting sqref="B156">
     <cfRule type="duplicateValues" dxfId="118" priority="122"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B151">
+  <conditionalFormatting sqref="B157">
     <cfRule type="duplicateValues" dxfId="117" priority="121"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B152">
+  <conditionalFormatting sqref="B171">
     <cfRule type="duplicateValues" dxfId="116" priority="120"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B153">
+  <conditionalFormatting sqref="B172">
     <cfRule type="duplicateValues" dxfId="115" priority="119"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B154">
+  <conditionalFormatting sqref="B174">
     <cfRule type="duplicateValues" dxfId="114" priority="118"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B155">
+  <conditionalFormatting sqref="B177:B178">
     <cfRule type="duplicateValues" dxfId="113" priority="117"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B156">
+  <conditionalFormatting sqref="B181">
     <cfRule type="duplicateValues" dxfId="112" priority="116"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B157">
+  <conditionalFormatting sqref="B182">
     <cfRule type="duplicateValues" dxfId="111" priority="115"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B171">
+  <conditionalFormatting sqref="B183">
     <cfRule type="duplicateValues" dxfId="110" priority="114"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B172">
+  <conditionalFormatting sqref="B184">
     <cfRule type="duplicateValues" dxfId="109" priority="113"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B174">
+  <conditionalFormatting sqref="B185">
     <cfRule type="duplicateValues" dxfId="108" priority="112"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B177:B178">
+  <conditionalFormatting sqref="B186">
     <cfRule type="duplicateValues" dxfId="107" priority="111"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B181">
+  <conditionalFormatting sqref="B188">
     <cfRule type="duplicateValues" dxfId="106" priority="110"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B182">
+  <conditionalFormatting sqref="B189">
     <cfRule type="duplicateValues" dxfId="105" priority="109"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B183">
+  <conditionalFormatting sqref="B190">
     <cfRule type="duplicateValues" dxfId="104" priority="108"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B184">
+  <conditionalFormatting sqref="B191">
     <cfRule type="duplicateValues" dxfId="103" priority="107"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B185">
+  <conditionalFormatting sqref="B192">
     <cfRule type="duplicateValues" dxfId="102" priority="106"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B186">
+  <conditionalFormatting sqref="B193">
     <cfRule type="duplicateValues" dxfId="101" priority="105"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B188">
+  <conditionalFormatting sqref="B195">
     <cfRule type="duplicateValues" dxfId="100" priority="104"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B189">
+  <conditionalFormatting sqref="B196">
     <cfRule type="duplicateValues" dxfId="99" priority="103"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B190">
+  <conditionalFormatting sqref="B197">
     <cfRule type="duplicateValues" dxfId="98" priority="102"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B191">
+  <conditionalFormatting sqref="B198">
     <cfRule type="duplicateValues" dxfId="97" priority="101"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B192">
+  <conditionalFormatting sqref="B199">
     <cfRule type="duplicateValues" dxfId="96" priority="100"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B193">
+  <conditionalFormatting sqref="B200">
     <cfRule type="duplicateValues" dxfId="95" priority="99"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B195">
+  <conditionalFormatting sqref="B201">
     <cfRule type="duplicateValues" dxfId="94" priority="98"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B196">
+  <conditionalFormatting sqref="B202">
     <cfRule type="duplicateValues" dxfId="93" priority="97"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B197">
+  <conditionalFormatting sqref="B203">
     <cfRule type="duplicateValues" dxfId="92" priority="96"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B198">
+  <conditionalFormatting sqref="B204">
     <cfRule type="duplicateValues" dxfId="91" priority="95"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B199">
+  <conditionalFormatting sqref="B205">
     <cfRule type="duplicateValues" dxfId="90" priority="94"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B200">
+  <conditionalFormatting sqref="B206">
     <cfRule type="duplicateValues" dxfId="89" priority="93"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B201">
+  <conditionalFormatting sqref="B207">
     <cfRule type="duplicateValues" dxfId="88" priority="92"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B202">
+  <conditionalFormatting sqref="B215">
     <cfRule type="duplicateValues" dxfId="87" priority="91"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B203">
+  <conditionalFormatting sqref="B218">
     <cfRule type="duplicateValues" dxfId="86" priority="90"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B204">
+  <conditionalFormatting sqref="B220">
     <cfRule type="duplicateValues" dxfId="85" priority="89"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B205">
+  <conditionalFormatting sqref="B222">
     <cfRule type="duplicateValues" dxfId="84" priority="88"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B206">
+  <conditionalFormatting sqref="B223">
     <cfRule type="duplicateValues" dxfId="83" priority="87"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B207">
+  <conditionalFormatting sqref="B224">
     <cfRule type="duplicateValues" dxfId="82" priority="86"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B215">
+  <conditionalFormatting sqref="B225">
     <cfRule type="duplicateValues" dxfId="81" priority="85"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B218">
+  <conditionalFormatting sqref="B227">
     <cfRule type="duplicateValues" dxfId="80" priority="84"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B220">
+  <conditionalFormatting sqref="B229">
     <cfRule type="duplicateValues" dxfId="79" priority="83"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B222">
+  <conditionalFormatting sqref="B230">
     <cfRule type="duplicateValues" dxfId="78" priority="82"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B223">
+  <conditionalFormatting sqref="B232">
     <cfRule type="duplicateValues" dxfId="77" priority="81"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B224">
+  <conditionalFormatting sqref="B233">
     <cfRule type="duplicateValues" dxfId="76" priority="80"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B225">
+  <conditionalFormatting sqref="B234">
     <cfRule type="duplicateValues" dxfId="75" priority="79"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B227">
+  <conditionalFormatting sqref="B235">
     <cfRule type="duplicateValues" dxfId="74" priority="78"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B229">
+  <conditionalFormatting sqref="B236">
     <cfRule type="duplicateValues" dxfId="73" priority="77"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B230">
+  <conditionalFormatting sqref="B237">
     <cfRule type="duplicateValues" dxfId="72" priority="76"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B232">
-    <cfRule type="duplicateValues" dxfId="71" priority="75"/>
+  <conditionalFormatting sqref="B239">
+    <cfRule type="duplicateValues" dxfId="71" priority="74"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B233">
-    <cfRule type="duplicateValues" dxfId="70" priority="74"/>
+  <conditionalFormatting sqref="B240">
+    <cfRule type="duplicateValues" dxfId="70" priority="73"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B234">
-    <cfRule type="duplicateValues" dxfId="69" priority="73"/>
+  <conditionalFormatting sqref="B241">
+    <cfRule type="duplicateValues" dxfId="69" priority="72"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B235">
-    <cfRule type="duplicateValues" dxfId="68" priority="72"/>
+  <conditionalFormatting sqref="B242">
+    <cfRule type="duplicateValues" dxfId="68" priority="71"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B236">
-    <cfRule type="duplicateValues" dxfId="67" priority="71"/>
+  <conditionalFormatting sqref="B243">
+    <cfRule type="duplicateValues" dxfId="67" priority="70"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B237">
-    <cfRule type="duplicateValues" dxfId="66" priority="70"/>
+  <conditionalFormatting sqref="B250">
+    <cfRule type="duplicateValues" dxfId="66" priority="69"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B239">
+  <conditionalFormatting sqref="B251">
     <cfRule type="duplicateValues" dxfId="65" priority="68"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B240">
+  <conditionalFormatting sqref="B253">
     <cfRule type="duplicateValues" dxfId="64" priority="67"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B241">
+  <conditionalFormatting sqref="B255">
     <cfRule type="duplicateValues" dxfId="63" priority="66"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B242">
+  <conditionalFormatting sqref="B258:B259">
     <cfRule type="duplicateValues" dxfId="62" priority="65"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B243">
+  <conditionalFormatting sqref="B260">
     <cfRule type="duplicateValues" dxfId="61" priority="64"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B250">
+  <conditionalFormatting sqref="B265:B267 B269">
     <cfRule type="duplicateValues" dxfId="60" priority="63"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B251">
+  <conditionalFormatting sqref="B268">
     <cfRule type="duplicateValues" dxfId="59" priority="62"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B253">
+  <conditionalFormatting sqref="B270">
     <cfRule type="duplicateValues" dxfId="58" priority="61"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B255">
+  <conditionalFormatting sqref="B271">
     <cfRule type="duplicateValues" dxfId="57" priority="60"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B258:B259">
+  <conditionalFormatting sqref="B273">
     <cfRule type="duplicateValues" dxfId="56" priority="59"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B260">
+  <conditionalFormatting sqref="B275">
     <cfRule type="duplicateValues" dxfId="55" priority="58"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B265:B267 B269">
+  <conditionalFormatting sqref="B278">
     <cfRule type="duplicateValues" dxfId="54" priority="57"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B268">
+  <conditionalFormatting sqref="B279">
     <cfRule type="duplicateValues" dxfId="53" priority="56"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B270">
+  <conditionalFormatting sqref="B280">
     <cfRule type="duplicateValues" dxfId="52" priority="55"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B271">
+  <conditionalFormatting sqref="B281">
     <cfRule type="duplicateValues" dxfId="51" priority="54"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B273">
+  <conditionalFormatting sqref="B282">
     <cfRule type="duplicateValues" dxfId="50" priority="53"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B275">
-    <cfRule type="duplicateValues" dxfId="49" priority="52"/>
+  <conditionalFormatting sqref="B283">
+    <cfRule type="duplicateValues" dxfId="49" priority="51"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B278">
-    <cfRule type="duplicateValues" dxfId="48" priority="51"/>
+  <conditionalFormatting sqref="B284:B286">
+    <cfRule type="duplicateValues" dxfId="48" priority="50"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B279">
-    <cfRule type="duplicateValues" dxfId="47" priority="50"/>
+  <conditionalFormatting sqref="B287">
+    <cfRule type="duplicateValues" dxfId="47" priority="49"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B280">
-    <cfRule type="duplicateValues" dxfId="46" priority="49"/>
+  <conditionalFormatting sqref="B288">
+    <cfRule type="duplicateValues" dxfId="46" priority="48"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B281">
-    <cfRule type="duplicateValues" dxfId="45" priority="48"/>
+  <conditionalFormatting sqref="B291">
+    <cfRule type="duplicateValues" dxfId="45" priority="47"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B282">
-    <cfRule type="duplicateValues" dxfId="44" priority="47"/>
+  <conditionalFormatting sqref="B292">
+    <cfRule type="duplicateValues" dxfId="44" priority="46"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B283">
+  <conditionalFormatting sqref="B293">
     <cfRule type="duplicateValues" dxfId="43" priority="45"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B284:B286">
+  <conditionalFormatting sqref="B294">
     <cfRule type="duplicateValues" dxfId="42" priority="44"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B287">
+  <conditionalFormatting sqref="B295">
     <cfRule type="duplicateValues" dxfId="41" priority="43"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B288">
+  <conditionalFormatting sqref="B296">
     <cfRule type="duplicateValues" dxfId="40" priority="42"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B291">
+  <conditionalFormatting sqref="B297">
     <cfRule type="duplicateValues" dxfId="39" priority="41"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B292">
+  <conditionalFormatting sqref="B298">
     <cfRule type="duplicateValues" dxfId="38" priority="40"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B293">
+  <conditionalFormatting sqref="B299">
     <cfRule type="duplicateValues" dxfId="37" priority="39"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B294">
+  <conditionalFormatting sqref="B300">
     <cfRule type="duplicateValues" dxfId="36" priority="38"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B295">
+  <conditionalFormatting sqref="B301">
     <cfRule type="duplicateValues" dxfId="35" priority="37"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B296">
+  <conditionalFormatting sqref="B302">
     <cfRule type="duplicateValues" dxfId="34" priority="36"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B297">
+  <conditionalFormatting sqref="B303">
     <cfRule type="duplicateValues" dxfId="33" priority="35"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B298">
+  <conditionalFormatting sqref="B304">
     <cfRule type="duplicateValues" dxfId="32" priority="34"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B299">
+  <conditionalFormatting sqref="B306">
     <cfRule type="duplicateValues" dxfId="31" priority="33"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B300">
+  <conditionalFormatting sqref="B309">
     <cfRule type="duplicateValues" dxfId="30" priority="32"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B301">
+  <conditionalFormatting sqref="B310">
     <cfRule type="duplicateValues" dxfId="29" priority="31"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B302">
+  <conditionalFormatting sqref="B313">
     <cfRule type="duplicateValues" dxfId="28" priority="30"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B303">
     <cfRule type="duplicateValues" dxfId="27" priority="29"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B304">
+  <conditionalFormatting sqref="B314">
     <cfRule type="duplicateValues" dxfId="26" priority="28"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B306">
+  <conditionalFormatting sqref="B316">
     <cfRule type="duplicateValues" dxfId="25" priority="27"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B309">
+  <conditionalFormatting sqref="B319">
     <cfRule type="duplicateValues" dxfId="24" priority="26"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B310">
-    <cfRule type="duplicateValues" dxfId="23" priority="25"/>
+  <conditionalFormatting sqref="B321">
+    <cfRule type="duplicateValues" dxfId="23" priority="24"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B313">
-    <cfRule type="duplicateValues" dxfId="22" priority="24"/>
-    <cfRule type="duplicateValues" dxfId="21" priority="23"/>
+  <conditionalFormatting sqref="B322">
+    <cfRule type="duplicateValues" dxfId="22" priority="23"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B314">
-    <cfRule type="duplicateValues" dxfId="20" priority="22"/>
+  <conditionalFormatting sqref="B325">
+    <cfRule type="duplicateValues" dxfId="21" priority="22"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B316">
-    <cfRule type="duplicateValues" dxfId="19" priority="21"/>
+  <conditionalFormatting sqref="B327">
+    <cfRule type="duplicateValues" dxfId="20" priority="21"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B319">
-    <cfRule type="duplicateValues" dxfId="18" priority="20"/>
+  <conditionalFormatting sqref="B329">
+    <cfRule type="duplicateValues" dxfId="19" priority="20"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B321">
+  <conditionalFormatting sqref="B330">
+    <cfRule type="duplicateValues" dxfId="18" priority="19"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B332">
     <cfRule type="duplicateValues" dxfId="17" priority="18"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B322">
-    <cfRule type="duplicateValues" dxfId="16" priority="17"/>
+  <conditionalFormatting sqref="B333">
+    <cfRule type="duplicateValues" dxfId="16" priority="16"/>
+    <cfRule type="duplicateValues" dxfId="15" priority="17"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B325">
-    <cfRule type="duplicateValues" dxfId="15" priority="16"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B327">
+  <conditionalFormatting sqref="B334">
     <cfRule type="duplicateValues" dxfId="14" priority="15"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B329">
+  <conditionalFormatting sqref="B335">
     <cfRule type="duplicateValues" dxfId="13" priority="14"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B330">
+  <conditionalFormatting sqref="B337:B341">
     <cfRule type="duplicateValues" dxfId="12" priority="13"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B332">
+  <conditionalFormatting sqref="B342">
     <cfRule type="duplicateValues" dxfId="11" priority="12"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B333">
-    <cfRule type="duplicateValues" dxfId="10" priority="10"/>
-    <cfRule type="duplicateValues" dxfId="9" priority="11"/>
+  <conditionalFormatting sqref="B343">
+    <cfRule type="duplicateValues" dxfId="10" priority="11"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B334">
+  <conditionalFormatting sqref="B344">
+    <cfRule type="duplicateValues" dxfId="9" priority="10"/>
     <cfRule type="duplicateValues" dxfId="8" priority="9"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B335">
+  <conditionalFormatting sqref="B345">
     <cfRule type="duplicateValues" dxfId="7" priority="8"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B337:B341">
+  <conditionalFormatting sqref="B346">
     <cfRule type="duplicateValues" dxfId="6" priority="7"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B342">
+  <conditionalFormatting sqref="B349:B350">
     <cfRule type="duplicateValues" dxfId="5" priority="6"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B343">
+  <conditionalFormatting sqref="B351:B353">
     <cfRule type="duplicateValues" dxfId="4" priority="5"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B344">
+  <conditionalFormatting sqref="B354">
     <cfRule type="duplicateValues" dxfId="3" priority="4"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B355">
     <cfRule type="duplicateValues" dxfId="2" priority="3"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B345">
+  <conditionalFormatting sqref="B356:B359">
     <cfRule type="duplicateValues" dxfId="1" priority="2"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B346">
+  <conditionalFormatting sqref="B360">
     <cfRule type="duplicateValues" dxfId="0" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -55202,15 +55561,15 @@
       </c>
       <c r="B1" s="15">
         <f>COUNTA(sum!A:A) -1</f>
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="C1" s="22">
         <f>COUNTIF(sum!I:I, "completed")/(B1-COUNTIF(sum!I:I, "abandoned")-COUNTIF(sum!I:I, "late app"))</f>
-        <v>0.96478873239436624</v>
+        <v>0.98951048951048948</v>
       </c>
       <c r="D1" s="21">
         <f>COUNTIF(sum!I:I, "completed")</f>
-        <v>274</v>
+        <v>283</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="22" customHeight="1" x14ac:dyDescent="0.4">
@@ -55245,7 +55604,7 @@
       </c>
       <c r="B5" s="15">
         <f>COUNTA(sum!J:J) -1</f>
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="C5" s="14">
         <f>B5/B1</f>
@@ -55258,11 +55617,11 @@
       </c>
       <c r="B6" s="16">
         <f>COUNTIFS(sum!J:J,"no news")</f>
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="C6" s="10">
         <f>B6/$B$5</f>
-        <v>0.87713310580204773</v>
+        <v>0.87796610169491529</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.4">
@@ -55275,7 +55634,7 @@
       </c>
       <c r="C7" s="10">
         <f t="shared" ref="C7:C10" si="0">B7/$B$5</f>
-        <v>9.556313993174062E-2</v>
+        <v>9.4915254237288138E-2</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.4">
@@ -55288,7 +55647,7 @@
       </c>
       <c r="C8" s="10">
         <f t="shared" si="0"/>
-        <v>2.7303754266211604E-2</v>
+        <v>2.7118644067796609E-2</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.4">
@@ -55301,7 +55660,7 @@
       </c>
       <c r="C9" s="10">
         <f t="shared" si="0"/>
-        <v>3.4129692832764505E-3</v>
+        <v>3.3898305084745762E-3</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.4">

</xml_diff>

<commit_message>
updated excel + thoughs
</commit_message>
<xml_diff>
--- a/EconJM_status.xlsx
+++ b/EconJM_status.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\javie\Dropbox\Work\Job Search\2025 EconJM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1CDF8CA5-636E-4A97-BC79-CC6E28A305ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0065D0FC-DCA2-451B-BC93-36394C3F0ADD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="14620" activeTab="1" xr2:uid="{6FE48536-7E5C-BF4C-9490-2A6392576298}"/>
   </bookViews>
@@ -438,7 +438,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3211" uniqueCount="967">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3227" uniqueCount="967">
   <si>
     <t>add_id</t>
   </si>
@@ -3566,7 +3566,67 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Percent" xfId="2" builtinId="5"/>
   </cellStyles>
-  <dxfs count="17">
+  <dxfs count="23">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF006100"/>
@@ -49737,63 +49797,63 @@
     </sortState>
   </autoFilter>
   <conditionalFormatting sqref="A1:B208 A210:B283 A285:B1048576 B284">
-    <cfRule type="duplicateValues" dxfId="16" priority="23"/>
+    <cfRule type="duplicateValues" dxfId="22" priority="23"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A2:B22">
-    <cfRule type="duplicateValues" dxfId="15" priority="24"/>
+    <cfRule type="duplicateValues" dxfId="21" priority="24"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A61:B61">
-    <cfRule type="duplicateValues" dxfId="14" priority="22"/>
+    <cfRule type="duplicateValues" dxfId="20" priority="22"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="I1:I1048576">
-    <cfRule type="containsText" dxfId="13" priority="15" operator="containsText" text="closed">
+    <cfRule type="containsText" dxfId="19" priority="15" operator="containsText" text="closed">
       <formula>NOT(ISERROR(SEARCH("closed",I1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="12" priority="16" operator="containsText" text="abandoned">
+    <cfRule type="containsText" dxfId="18" priority="16" operator="containsText" text="abandoned">
       <formula>NOT(ISERROR(SEARCH("abandoned",I1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="11" priority="18" operator="containsText" text="late app">
+    <cfRule type="containsText" dxfId="17" priority="18" operator="containsText" text="late app">
       <formula>NOT(ISERROR(SEARCH("late app",I1)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I2:L1048576 P78:P80 P83:P89 P92:P112 P115:P124 P126:P181 S136 S153 S159 S166 S173 S178 P183:P205 P208:P211 P213:P218 P220:P233 S225 P235:P237 P239:P248 P276:P309 R276:R309 I1:J1">
-    <cfRule type="containsText" dxfId="10" priority="21" operator="containsText" text="completed">
+    <cfRule type="containsText" dxfId="16" priority="21" operator="containsText" text="completed">
       <formula>NOT(ISERROR(SEARCH("completed",I1)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J1:J1048576">
-    <cfRule type="containsText" dxfId="9" priority="10" operator="containsText" text="no news">
+    <cfRule type="containsText" dxfId="15" priority="10" operator="containsText" text="no news">
       <formula>NOT(ISERROR(SEARCH("no news",J1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="8" priority="11" operator="containsText" text="offer">
+    <cfRule type="containsText" dxfId="14" priority="11" operator="containsText" text="offer">
       <formula>NOT(ISERROR(SEARCH("offer",J1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="7" priority="12" operator="containsText" text="fly out">
+    <cfRule type="containsText" dxfId="13" priority="12" operator="containsText" text="fly out">
       <formula>NOT(ISERROR(SEARCH("fly out",J1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="6" priority="13" operator="containsText" text="interview">
+    <cfRule type="containsText" dxfId="12" priority="13" operator="containsText" text="interview">
       <formula>NOT(ISERROR(SEARCH("interview",J1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="5" priority="14" operator="containsText" text="rejected">
+    <cfRule type="containsText" dxfId="11" priority="14" operator="containsText" text="rejected">
       <formula>NOT(ISERROR(SEARCH("rejected",J1)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K1:L1048576 P78:P80 P83:P89 P92:P112 P115:P124 P126:P181 S136 S153 S159 S166 S173 S178 P183:P205 P208:P211 P213:P218 P220:P233 S225 P235:P237 P239:P248 P276:P309 R276:R309">
-    <cfRule type="containsText" dxfId="4" priority="19" operator="containsText" text="NO">
+    <cfRule type="containsText" dxfId="10" priority="19" operator="containsText" text="NO">
       <formula>NOT(ISERROR(SEARCH("NO",K1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="3" priority="20" operator="containsText" text="YES">
+    <cfRule type="containsText" dxfId="9" priority="20" operator="containsText" text="YES">
       <formula>NOT(ISERROR(SEARCH("YES",K1)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="P250:P267">
-    <cfRule type="containsText" dxfId="2" priority="1" operator="containsText" text="NO">
+    <cfRule type="containsText" dxfId="8" priority="1" operator="containsText" text="NO">
       <formula>NOT(ISERROR(SEARCH("NO",P250)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="YES">
+    <cfRule type="containsText" dxfId="7" priority="2" operator="containsText" text="YES">
       <formula>NOT(ISERROR(SEARCH("YES",P250)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="0" priority="3" operator="containsText" text="completed">
+    <cfRule type="containsText" dxfId="6" priority="3" operator="containsText" text="completed">
       <formula>NOT(ISERROR(SEARCH("completed",P250)))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -49923,7 +49983,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{923E81FA-B875-3C4E-A189-1A21268FA086}">
-  <dimension ref="A1:C382"/>
+  <dimension ref="A1:C390"/>
   <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="16" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="32.83203125" customWidth="1"/>
@@ -54055,7 +54115,113 @@
         <v>405</v>
       </c>
     </row>
+    <row r="383" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A383" s="1">
+        <v>46076</v>
+      </c>
+      <c r="B383" t="s">
+        <v>598</v>
+      </c>
+      <c r="C383" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="384" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A384" s="1">
+        <v>46076</v>
+      </c>
+      <c r="B384" t="s">
+        <v>825</v>
+      </c>
+      <c r="C384" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="385" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A385" s="1">
+        <v>46076</v>
+      </c>
+      <c r="B385" t="s">
+        <v>88</v>
+      </c>
+      <c r="C385" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="386" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A386" s="1">
+        <v>46079</v>
+      </c>
+      <c r="B386" t="s">
+        <v>277</v>
+      </c>
+      <c r="C386" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="387" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A387" s="1">
+        <v>46079</v>
+      </c>
+      <c r="B387" t="s">
+        <v>65</v>
+      </c>
+      <c r="C387" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="388" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A388" s="1">
+        <v>46080</v>
+      </c>
+      <c r="B388" t="s">
+        <v>723</v>
+      </c>
+      <c r="C388" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="389" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A389" s="1">
+        <v>46083</v>
+      </c>
+      <c r="B389" t="s">
+        <v>593</v>
+      </c>
+      <c r="C389" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="390" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A390" s="1">
+        <v>46083</v>
+      </c>
+      <c r="B390" t="s">
+        <v>855</v>
+      </c>
+      <c r="C390" t="s">
+        <v>402</v>
+      </c>
+    </row>
   </sheetData>
+  <conditionalFormatting sqref="B383">
+    <cfRule type="duplicateValues" dxfId="5" priority="6"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B384">
+    <cfRule type="duplicateValues" dxfId="4" priority="5"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B385">
+    <cfRule type="duplicateValues" dxfId="3" priority="4"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B387">
+    <cfRule type="duplicateValues" dxfId="2" priority="3"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B389">
+    <cfRule type="duplicateValues" dxfId="1" priority="2"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B390">
+    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
+  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
fixed mayor phrasing and grammar errors
</commit_message>
<xml_diff>
--- a/EconJM_status.xlsx
+++ b/EconJM_status.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\javie\Dropbox\Work\Job Search\2025 EconJM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0065D0FC-DCA2-451B-BC93-36394C3F0ADD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B14633BD-299C-40C7-B140-944B478BAF0A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="14620" activeTab="1" xr2:uid="{6FE48536-7E5C-BF4C-9490-2A6392576298}"/>
   </bookViews>
@@ -438,7 +438,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3227" uniqueCount="967">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3231" uniqueCount="967">
   <si>
     <t>add_id</t>
   </si>
@@ -3566,7 +3566,27 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Percent" xfId="2" builtinId="5"/>
   </cellStyles>
-  <dxfs count="23">
+  <dxfs count="25">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -49797,63 +49817,63 @@
     </sortState>
   </autoFilter>
   <conditionalFormatting sqref="A1:B208 A210:B283 A285:B1048576 B284">
-    <cfRule type="duplicateValues" dxfId="22" priority="23"/>
+    <cfRule type="duplicateValues" dxfId="24" priority="23"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A2:B22">
-    <cfRule type="duplicateValues" dxfId="21" priority="24"/>
+    <cfRule type="duplicateValues" dxfId="23" priority="24"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A61:B61">
-    <cfRule type="duplicateValues" dxfId="20" priority="22"/>
+    <cfRule type="duplicateValues" dxfId="22" priority="22"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="I1:I1048576">
-    <cfRule type="containsText" dxfId="19" priority="15" operator="containsText" text="closed">
+    <cfRule type="containsText" dxfId="21" priority="15" operator="containsText" text="closed">
       <formula>NOT(ISERROR(SEARCH("closed",I1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="18" priority="16" operator="containsText" text="abandoned">
+    <cfRule type="containsText" dxfId="20" priority="16" operator="containsText" text="abandoned">
       <formula>NOT(ISERROR(SEARCH("abandoned",I1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="17" priority="18" operator="containsText" text="late app">
+    <cfRule type="containsText" dxfId="19" priority="18" operator="containsText" text="late app">
       <formula>NOT(ISERROR(SEARCH("late app",I1)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I2:L1048576 P78:P80 P83:P89 P92:P112 P115:P124 P126:P181 S136 S153 S159 S166 S173 S178 P183:P205 P208:P211 P213:P218 P220:P233 S225 P235:P237 P239:P248 P276:P309 R276:R309 I1:J1">
-    <cfRule type="containsText" dxfId="16" priority="21" operator="containsText" text="completed">
+    <cfRule type="containsText" dxfId="18" priority="21" operator="containsText" text="completed">
       <formula>NOT(ISERROR(SEARCH("completed",I1)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J1:J1048576">
-    <cfRule type="containsText" dxfId="15" priority="10" operator="containsText" text="no news">
+    <cfRule type="containsText" dxfId="17" priority="10" operator="containsText" text="no news">
       <formula>NOT(ISERROR(SEARCH("no news",J1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="14" priority="11" operator="containsText" text="offer">
+    <cfRule type="containsText" dxfId="16" priority="11" operator="containsText" text="offer">
       <formula>NOT(ISERROR(SEARCH("offer",J1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="13" priority="12" operator="containsText" text="fly out">
+    <cfRule type="containsText" dxfId="15" priority="12" operator="containsText" text="fly out">
       <formula>NOT(ISERROR(SEARCH("fly out",J1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="12" priority="13" operator="containsText" text="interview">
+    <cfRule type="containsText" dxfId="14" priority="13" operator="containsText" text="interview">
       <formula>NOT(ISERROR(SEARCH("interview",J1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="11" priority="14" operator="containsText" text="rejected">
+    <cfRule type="containsText" dxfId="13" priority="14" operator="containsText" text="rejected">
       <formula>NOT(ISERROR(SEARCH("rejected",J1)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K1:L1048576 P78:P80 P83:P89 P92:P112 P115:P124 P126:P181 S136 S153 S159 S166 S173 S178 P183:P205 P208:P211 P213:P218 P220:P233 S225 P235:P237 P239:P248 P276:P309 R276:R309">
-    <cfRule type="containsText" dxfId="10" priority="19" operator="containsText" text="NO">
+    <cfRule type="containsText" dxfId="12" priority="19" operator="containsText" text="NO">
       <formula>NOT(ISERROR(SEARCH("NO",K1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="9" priority="20" operator="containsText" text="YES">
+    <cfRule type="containsText" dxfId="11" priority="20" operator="containsText" text="YES">
       <formula>NOT(ISERROR(SEARCH("YES",K1)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="P250:P267">
-    <cfRule type="containsText" dxfId="8" priority="1" operator="containsText" text="NO">
+    <cfRule type="containsText" dxfId="10" priority="1" operator="containsText" text="NO">
       <formula>NOT(ISERROR(SEARCH("NO",P250)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="7" priority="2" operator="containsText" text="YES">
+    <cfRule type="containsText" dxfId="9" priority="2" operator="containsText" text="YES">
       <formula>NOT(ISERROR(SEARCH("YES",P250)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="6" priority="3" operator="containsText" text="completed">
+    <cfRule type="containsText" dxfId="8" priority="3" operator="containsText" text="completed">
       <formula>NOT(ISERROR(SEARCH("completed",P250)))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -49983,7 +50003,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{923E81FA-B875-3C4E-A189-1A21268FA086}">
-  <dimension ref="A1:C390"/>
+  <dimension ref="A1:C392"/>
   <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="16" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="32.83203125" customWidth="1"/>
@@ -54203,23 +54223,51 @@
         <v>402</v>
       </c>
     </row>
+    <row r="391" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A391" s="1">
+        <v>46084</v>
+      </c>
+      <c r="B391" t="s">
+        <v>721</v>
+      </c>
+      <c r="C391" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="392" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A392" s="1">
+        <v>46084</v>
+      </c>
+      <c r="B392" t="s">
+        <v>619</v>
+      </c>
+      <c r="C392" t="s">
+        <v>402</v>
+      </c>
+    </row>
   </sheetData>
   <conditionalFormatting sqref="B383">
+    <cfRule type="duplicateValues" dxfId="7" priority="8"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B384">
+    <cfRule type="duplicateValues" dxfId="6" priority="7"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B385">
     <cfRule type="duplicateValues" dxfId="5" priority="6"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B384">
+  <conditionalFormatting sqref="B387">
     <cfRule type="duplicateValues" dxfId="4" priority="5"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B385">
+  <conditionalFormatting sqref="B389">
     <cfRule type="duplicateValues" dxfId="3" priority="4"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B387">
+  <conditionalFormatting sqref="B390">
     <cfRule type="duplicateValues" dxfId="2" priority="3"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B389">
+  <conditionalFormatting sqref="B391">
     <cfRule type="duplicateValues" dxfId="1" priority="2"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B390">
+  <conditionalFormatting sqref="B392">
     <cfRule type="duplicateValues" dxfId="0" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
new link to repo on pdf
</commit_message>
<xml_diff>
--- a/EconJM_status.xlsx
+++ b/EconJM_status.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\javie\Dropbox\Work\Job Search\2025 EconJM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B14633BD-299C-40C7-B140-944B478BAF0A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F04C0E7-4484-4656-9AE9-6822A5AFDD1E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="14620" activeTab="1" xr2:uid="{6FE48536-7E5C-BF4C-9490-2A6392576298}"/>
   </bookViews>
@@ -438,7 +438,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3231" uniqueCount="967">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3235" uniqueCount="967">
   <si>
     <t>add_id</t>
   </si>
@@ -3566,7 +3566,27 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Percent" xfId="2" builtinId="5"/>
   </cellStyles>
-  <dxfs count="25">
+  <dxfs count="27">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -49817,63 +49837,63 @@
     </sortState>
   </autoFilter>
   <conditionalFormatting sqref="A1:B208 A210:B283 A285:B1048576 B284">
-    <cfRule type="duplicateValues" dxfId="24" priority="23"/>
+    <cfRule type="duplicateValues" dxfId="26" priority="23"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A2:B22">
-    <cfRule type="duplicateValues" dxfId="23" priority="24"/>
+    <cfRule type="duplicateValues" dxfId="25" priority="24"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A61:B61">
-    <cfRule type="duplicateValues" dxfId="22" priority="22"/>
+    <cfRule type="duplicateValues" dxfId="24" priority="22"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="I1:I1048576">
-    <cfRule type="containsText" dxfId="21" priority="15" operator="containsText" text="closed">
+    <cfRule type="containsText" dxfId="23" priority="15" operator="containsText" text="closed">
       <formula>NOT(ISERROR(SEARCH("closed",I1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="20" priority="16" operator="containsText" text="abandoned">
+    <cfRule type="containsText" dxfId="22" priority="16" operator="containsText" text="abandoned">
       <formula>NOT(ISERROR(SEARCH("abandoned",I1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="19" priority="18" operator="containsText" text="late app">
+    <cfRule type="containsText" dxfId="21" priority="18" operator="containsText" text="late app">
       <formula>NOT(ISERROR(SEARCH("late app",I1)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I2:L1048576 P78:P80 P83:P89 P92:P112 P115:P124 P126:P181 S136 S153 S159 S166 S173 S178 P183:P205 P208:P211 P213:P218 P220:P233 S225 P235:P237 P239:P248 P276:P309 R276:R309 I1:J1">
-    <cfRule type="containsText" dxfId="18" priority="21" operator="containsText" text="completed">
+    <cfRule type="containsText" dxfId="20" priority="21" operator="containsText" text="completed">
       <formula>NOT(ISERROR(SEARCH("completed",I1)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J1:J1048576">
-    <cfRule type="containsText" dxfId="17" priority="10" operator="containsText" text="no news">
+    <cfRule type="containsText" dxfId="19" priority="10" operator="containsText" text="no news">
       <formula>NOT(ISERROR(SEARCH("no news",J1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="16" priority="11" operator="containsText" text="offer">
+    <cfRule type="containsText" dxfId="18" priority="11" operator="containsText" text="offer">
       <formula>NOT(ISERROR(SEARCH("offer",J1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="15" priority="12" operator="containsText" text="fly out">
+    <cfRule type="containsText" dxfId="17" priority="12" operator="containsText" text="fly out">
       <formula>NOT(ISERROR(SEARCH("fly out",J1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="14" priority="13" operator="containsText" text="interview">
+    <cfRule type="containsText" dxfId="16" priority="13" operator="containsText" text="interview">
       <formula>NOT(ISERROR(SEARCH("interview",J1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="13" priority="14" operator="containsText" text="rejected">
+    <cfRule type="containsText" dxfId="15" priority="14" operator="containsText" text="rejected">
       <formula>NOT(ISERROR(SEARCH("rejected",J1)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K1:L1048576 P78:P80 P83:P89 P92:P112 P115:P124 P126:P181 S136 S153 S159 S166 S173 S178 P183:P205 P208:P211 P213:P218 P220:P233 S225 P235:P237 P239:P248 P276:P309 R276:R309">
-    <cfRule type="containsText" dxfId="12" priority="19" operator="containsText" text="NO">
+    <cfRule type="containsText" dxfId="14" priority="19" operator="containsText" text="NO">
       <formula>NOT(ISERROR(SEARCH("NO",K1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="11" priority="20" operator="containsText" text="YES">
+    <cfRule type="containsText" dxfId="13" priority="20" operator="containsText" text="YES">
       <formula>NOT(ISERROR(SEARCH("YES",K1)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="P250:P267">
-    <cfRule type="containsText" dxfId="10" priority="1" operator="containsText" text="NO">
+    <cfRule type="containsText" dxfId="12" priority="1" operator="containsText" text="NO">
       <formula>NOT(ISERROR(SEARCH("NO",P250)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="9" priority="2" operator="containsText" text="YES">
+    <cfRule type="containsText" dxfId="11" priority="2" operator="containsText" text="YES">
       <formula>NOT(ISERROR(SEARCH("YES",P250)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="8" priority="3" operator="containsText" text="completed">
+    <cfRule type="containsText" dxfId="10" priority="3" operator="containsText" text="completed">
       <formula>NOT(ISERROR(SEARCH("completed",P250)))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -50003,7 +50023,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{923E81FA-B875-3C4E-A189-1A21268FA086}">
-  <dimension ref="A1:C392"/>
+  <dimension ref="A1:C394"/>
   <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="16" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="32.83203125" customWidth="1"/>
@@ -54245,29 +54265,57 @@
         <v>402</v>
       </c>
     </row>
+    <row r="393" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A393" s="1">
+        <v>46086</v>
+      </c>
+      <c r="B393" t="s">
+        <v>820</v>
+      </c>
+      <c r="C393" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="394" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A394" s="1">
+        <v>46086</v>
+      </c>
+      <c r="B394" t="s">
+        <v>808</v>
+      </c>
+      <c r="C394" t="s">
+        <v>402</v>
+      </c>
+    </row>
   </sheetData>
   <conditionalFormatting sqref="B383">
+    <cfRule type="duplicateValues" dxfId="9" priority="10"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B384">
+    <cfRule type="duplicateValues" dxfId="8" priority="9"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B385">
     <cfRule type="duplicateValues" dxfId="7" priority="8"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B384">
+  <conditionalFormatting sqref="B387">
     <cfRule type="duplicateValues" dxfId="6" priority="7"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B385">
+  <conditionalFormatting sqref="B389">
     <cfRule type="duplicateValues" dxfId="5" priority="6"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B387">
+  <conditionalFormatting sqref="B390">
     <cfRule type="duplicateValues" dxfId="4" priority="5"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B389">
+  <conditionalFormatting sqref="B391">
     <cfRule type="duplicateValues" dxfId="3" priority="4"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B390">
+  <conditionalFormatting sqref="B392">
     <cfRule type="duplicateValues" dxfId="2" priority="3"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B391">
+  <conditionalFormatting sqref="B393">
     <cfRule type="duplicateValues" dxfId="1" priority="2"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B392">
+  <conditionalFormatting sqref="B394">
     <cfRule type="duplicateValues" dxfId="0" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
update the JMP thoughs
</commit_message>
<xml_diff>
--- a/EconJM_status.xlsx
+++ b/EconJM_status.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\javie\Dropbox\Work\Job Search\2025 EconJM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F04C0E7-4484-4656-9AE9-6822A5AFDD1E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF0415E7-3901-434A-91EB-A78A4840DAF5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="14620" activeTab="1" xr2:uid="{6FE48536-7E5C-BF4C-9490-2A6392576298}"/>
   </bookViews>
@@ -438,7 +438,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3235" uniqueCount="967">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3248" uniqueCount="967">
   <si>
     <t>add_id</t>
   </si>
@@ -3566,7 +3566,67 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Percent" xfId="2" builtinId="5"/>
   </cellStyles>
-  <dxfs count="27">
+  <dxfs count="33">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -49837,63 +49897,63 @@
     </sortState>
   </autoFilter>
   <conditionalFormatting sqref="A1:B208 A210:B283 A285:B1048576 B284">
-    <cfRule type="duplicateValues" dxfId="26" priority="23"/>
+    <cfRule type="duplicateValues" dxfId="32" priority="23"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A2:B22">
-    <cfRule type="duplicateValues" dxfId="25" priority="24"/>
+    <cfRule type="duplicateValues" dxfId="31" priority="24"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A61:B61">
-    <cfRule type="duplicateValues" dxfId="24" priority="22"/>
+    <cfRule type="duplicateValues" dxfId="30" priority="22"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="I1:I1048576">
-    <cfRule type="containsText" dxfId="23" priority="15" operator="containsText" text="closed">
+    <cfRule type="containsText" dxfId="29" priority="15" operator="containsText" text="closed">
       <formula>NOT(ISERROR(SEARCH("closed",I1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="22" priority="16" operator="containsText" text="abandoned">
+    <cfRule type="containsText" dxfId="28" priority="16" operator="containsText" text="abandoned">
       <formula>NOT(ISERROR(SEARCH("abandoned",I1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="21" priority="18" operator="containsText" text="late app">
+    <cfRule type="containsText" dxfId="27" priority="18" operator="containsText" text="late app">
       <formula>NOT(ISERROR(SEARCH("late app",I1)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I2:L1048576 P78:P80 P83:P89 P92:P112 P115:P124 P126:P181 S136 S153 S159 S166 S173 S178 P183:P205 P208:P211 P213:P218 P220:P233 S225 P235:P237 P239:P248 P276:P309 R276:R309 I1:J1">
-    <cfRule type="containsText" dxfId="20" priority="21" operator="containsText" text="completed">
+    <cfRule type="containsText" dxfId="26" priority="21" operator="containsText" text="completed">
       <formula>NOT(ISERROR(SEARCH("completed",I1)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J1:J1048576">
-    <cfRule type="containsText" dxfId="19" priority="10" operator="containsText" text="no news">
+    <cfRule type="containsText" dxfId="25" priority="10" operator="containsText" text="no news">
       <formula>NOT(ISERROR(SEARCH("no news",J1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="18" priority="11" operator="containsText" text="offer">
+    <cfRule type="containsText" dxfId="24" priority="11" operator="containsText" text="offer">
       <formula>NOT(ISERROR(SEARCH("offer",J1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="17" priority="12" operator="containsText" text="fly out">
+    <cfRule type="containsText" dxfId="23" priority="12" operator="containsText" text="fly out">
       <formula>NOT(ISERROR(SEARCH("fly out",J1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="16" priority="13" operator="containsText" text="interview">
+    <cfRule type="containsText" dxfId="22" priority="13" operator="containsText" text="interview">
       <formula>NOT(ISERROR(SEARCH("interview",J1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="15" priority="14" operator="containsText" text="rejected">
+    <cfRule type="containsText" dxfId="21" priority="14" operator="containsText" text="rejected">
       <formula>NOT(ISERROR(SEARCH("rejected",J1)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K1:L1048576 P78:P80 P83:P89 P92:P112 P115:P124 P126:P181 S136 S153 S159 S166 S173 S178 P183:P205 P208:P211 P213:P218 P220:P233 S225 P235:P237 P239:P248 P276:P309 R276:R309">
-    <cfRule type="containsText" dxfId="14" priority="19" operator="containsText" text="NO">
+    <cfRule type="containsText" dxfId="20" priority="19" operator="containsText" text="NO">
       <formula>NOT(ISERROR(SEARCH("NO",K1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="13" priority="20" operator="containsText" text="YES">
+    <cfRule type="containsText" dxfId="19" priority="20" operator="containsText" text="YES">
       <formula>NOT(ISERROR(SEARCH("YES",K1)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="P250:P267">
-    <cfRule type="containsText" dxfId="12" priority="1" operator="containsText" text="NO">
+    <cfRule type="containsText" dxfId="18" priority="1" operator="containsText" text="NO">
       <formula>NOT(ISERROR(SEARCH("NO",P250)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="11" priority="2" operator="containsText" text="YES">
+    <cfRule type="containsText" dxfId="17" priority="2" operator="containsText" text="YES">
       <formula>NOT(ISERROR(SEARCH("YES",P250)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="10" priority="3" operator="containsText" text="completed">
+    <cfRule type="containsText" dxfId="16" priority="3" operator="containsText" text="completed">
       <formula>NOT(ISERROR(SEARCH("completed",P250)))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -50023,7 +50083,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{923E81FA-B875-3C4E-A189-1A21268FA086}">
-  <dimension ref="A1:C394"/>
+  <dimension ref="A1:C401"/>
   <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="16" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="32.83203125" customWidth="1"/>
@@ -54287,35 +54347,125 @@
         <v>402</v>
       </c>
     </row>
+    <row r="395" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A395" s="1">
+        <v>46091</v>
+      </c>
+      <c r="B395" t="s">
+        <v>635</v>
+      </c>
+      <c r="C395" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="396" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A396" s="1">
+        <v>46091</v>
+      </c>
+      <c r="B396" t="s">
+        <v>487</v>
+      </c>
+      <c r="C396" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="397" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A397" s="1">
+        <v>46094</v>
+      </c>
+      <c r="B397" t="s">
+        <v>440</v>
+      </c>
+      <c r="C397" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="398" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A398" s="1">
+        <v>46094</v>
+      </c>
+      <c r="B398" t="s">
+        <v>496</v>
+      </c>
+      <c r="C398" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="399" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A399" s="1">
+        <v>46094</v>
+      </c>
+      <c r="C399" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="400" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A400" s="1">
+        <v>46099</v>
+      </c>
+      <c r="B400" t="s">
+        <v>920</v>
+      </c>
+      <c r="C400" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="401" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A401" s="1">
+        <v>46100</v>
+      </c>
+      <c r="B401" t="s">
+        <v>906</v>
+      </c>
+      <c r="C401" t="s">
+        <v>402</v>
+      </c>
+    </row>
   </sheetData>
   <conditionalFormatting sqref="B383">
+    <cfRule type="duplicateValues" dxfId="15" priority="16"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B384">
+    <cfRule type="duplicateValues" dxfId="14" priority="15"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B385">
+    <cfRule type="duplicateValues" dxfId="13" priority="14"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B387">
+    <cfRule type="duplicateValues" dxfId="12" priority="13"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B389">
+    <cfRule type="duplicateValues" dxfId="11" priority="12"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B390">
+    <cfRule type="duplicateValues" dxfId="10" priority="11"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B391">
     <cfRule type="duplicateValues" dxfId="9" priority="10"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B384">
+  <conditionalFormatting sqref="B392">
     <cfRule type="duplicateValues" dxfId="8" priority="9"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B385">
+  <conditionalFormatting sqref="B393">
     <cfRule type="duplicateValues" dxfId="7" priority="8"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B387">
+  <conditionalFormatting sqref="B394">
     <cfRule type="duplicateValues" dxfId="6" priority="7"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B389">
+  <conditionalFormatting sqref="B396">
     <cfRule type="duplicateValues" dxfId="5" priority="6"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B390">
-    <cfRule type="duplicateValues" dxfId="4" priority="5"/>
+  <conditionalFormatting sqref="B397">
+    <cfRule type="duplicateValues" dxfId="4" priority="4"/>
+    <cfRule type="duplicateValues" dxfId="3" priority="5"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B391">
-    <cfRule type="duplicateValues" dxfId="3" priority="4"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B392">
+  <conditionalFormatting sqref="B398">
     <cfRule type="duplicateValues" dxfId="2" priority="3"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B393">
+  <conditionalFormatting sqref="B400">
     <cfRule type="duplicateValues" dxfId="1" priority="2"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B394">
+  <conditionalFormatting sqref="B401">
     <cfRule type="duplicateValues" dxfId="0" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
update the econ thoughs with Alex Albright blog post
</commit_message>
<xml_diff>
--- a/EconJM_status.xlsx
+++ b/EconJM_status.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\javie\Dropbox\Work\Job Search\2025 EconJM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E6D2ABF-EA20-49C4-A64E-8C8901E19753}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C0073BD6-B0F7-4D8C-953D-AEFAB13E4FEC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="14620" activeTab="1" xr2:uid="{6FE48536-7E5C-BF4C-9490-2A6392576298}"/>
   </bookViews>
@@ -438,7 +438,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3264" uniqueCount="967">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3272" uniqueCount="968">
   <si>
     <t>add_id</t>
   </si>
@@ -3375,6 +3375,9 @@
   </si>
   <si>
     <t>Brown University</t>
+  </si>
+  <si>
+    <t>viena</t>
   </si>
 </sst>
 </file>
@@ -3566,7 +3569,37 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Percent" xfId="2" builtinId="5"/>
   </cellStyles>
-  <dxfs count="40">
+  <dxfs count="43">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -49967,63 +50000,63 @@
     </sortState>
   </autoFilter>
   <conditionalFormatting sqref="A1:B208 A210:B283 A285:B1048576 B284">
-    <cfRule type="duplicateValues" dxfId="39" priority="23"/>
+    <cfRule type="duplicateValues" dxfId="42" priority="23"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A2:B22">
-    <cfRule type="duplicateValues" dxfId="38" priority="24"/>
+    <cfRule type="duplicateValues" dxfId="41" priority="24"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A61:B61">
-    <cfRule type="duplicateValues" dxfId="37" priority="22"/>
+    <cfRule type="duplicateValues" dxfId="40" priority="22"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="I1:I1048576">
-    <cfRule type="containsText" dxfId="36" priority="15" operator="containsText" text="closed">
+    <cfRule type="containsText" dxfId="39" priority="15" operator="containsText" text="closed">
       <formula>NOT(ISERROR(SEARCH("closed",I1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="35" priority="16" operator="containsText" text="abandoned">
+    <cfRule type="containsText" dxfId="38" priority="16" operator="containsText" text="abandoned">
       <formula>NOT(ISERROR(SEARCH("abandoned",I1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="34" priority="18" operator="containsText" text="late app">
+    <cfRule type="containsText" dxfId="37" priority="18" operator="containsText" text="late app">
       <formula>NOT(ISERROR(SEARCH("late app",I1)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I2:L1048576 P78:P80 P83:P89 P92:P112 P115:P124 P126:P181 S136 S153 S159 S166 S173 S178 P183:P205 P208:P211 P213:P218 P220:P233 S225 P235:P237 P239:P248 P276:P309 R276:R309 I1:J1">
-    <cfRule type="containsText" dxfId="33" priority="21" operator="containsText" text="completed">
+    <cfRule type="containsText" dxfId="36" priority="21" operator="containsText" text="completed">
       <formula>NOT(ISERROR(SEARCH("completed",I1)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J1:J1048576">
-    <cfRule type="containsText" dxfId="32" priority="10" operator="containsText" text="no news">
+    <cfRule type="containsText" dxfId="35" priority="10" operator="containsText" text="no news">
       <formula>NOT(ISERROR(SEARCH("no news",J1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="31" priority="11" operator="containsText" text="offer">
+    <cfRule type="containsText" dxfId="34" priority="11" operator="containsText" text="offer">
       <formula>NOT(ISERROR(SEARCH("offer",J1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="30" priority="12" operator="containsText" text="fly out">
+    <cfRule type="containsText" dxfId="33" priority="12" operator="containsText" text="fly out">
       <formula>NOT(ISERROR(SEARCH("fly out",J1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="29" priority="13" operator="containsText" text="interview">
+    <cfRule type="containsText" dxfId="32" priority="13" operator="containsText" text="interview">
       <formula>NOT(ISERROR(SEARCH("interview",J1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="28" priority="14" operator="containsText" text="rejected">
+    <cfRule type="containsText" dxfId="31" priority="14" operator="containsText" text="rejected">
       <formula>NOT(ISERROR(SEARCH("rejected",J1)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K1:L1048576 P78:P80 P83:P89 P92:P112 P115:P124 P126:P181 S136 S153 S159 S166 S173 S178 P183:P205 P208:P211 P213:P218 P220:P233 S225 P235:P237 P239:P248 P276:P309 R276:R309">
-    <cfRule type="containsText" dxfId="27" priority="19" operator="containsText" text="NO">
+    <cfRule type="containsText" dxfId="30" priority="19" operator="containsText" text="NO">
       <formula>NOT(ISERROR(SEARCH("NO",K1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="26" priority="20" operator="containsText" text="YES">
+    <cfRule type="containsText" dxfId="29" priority="20" operator="containsText" text="YES">
       <formula>NOT(ISERROR(SEARCH("YES",K1)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="P250:P267">
-    <cfRule type="containsText" dxfId="25" priority="1" operator="containsText" text="NO">
+    <cfRule type="containsText" dxfId="28" priority="1" operator="containsText" text="NO">
       <formula>NOT(ISERROR(SEARCH("NO",P250)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="24" priority="2" operator="containsText" text="YES">
+    <cfRule type="containsText" dxfId="27" priority="2" operator="containsText" text="YES">
       <formula>NOT(ISERROR(SEARCH("YES",P250)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="23" priority="3" operator="containsText" text="completed">
+    <cfRule type="containsText" dxfId="26" priority="3" operator="containsText" text="completed">
       <formula>NOT(ISERROR(SEARCH("completed",P250)))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -50153,7 +50186,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{923E81FA-B875-3C4E-A189-1A21268FA086}">
-  <dimension ref="A1:C409"/>
+  <dimension ref="A1:C413"/>
   <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="16" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="32.83203125" customWidth="1"/>
@@ -54579,70 +54612,123 @@
         <v>402</v>
       </c>
     </row>
+    <row r="410" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A410" s="1">
+        <v>46122</v>
+      </c>
+      <c r="B410" t="s">
+        <v>913</v>
+      </c>
+      <c r="C410" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="411" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A411" s="1">
+        <v>46122</v>
+      </c>
+      <c r="B411" t="s">
+        <v>621</v>
+      </c>
+      <c r="C411" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="412" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A412" s="1">
+        <v>46125</v>
+      </c>
+      <c r="B412" t="s">
+        <v>431</v>
+      </c>
+      <c r="C412" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="413" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A413" s="1">
+        <v>46125</v>
+      </c>
+      <c r="B413" t="s">
+        <v>967</v>
+      </c>
+      <c r="C413" t="s">
+        <v>402</v>
+      </c>
+    </row>
   </sheetData>
   <conditionalFormatting sqref="B383">
+    <cfRule type="duplicateValues" dxfId="25" priority="26"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B384">
+    <cfRule type="duplicateValues" dxfId="24" priority="25"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B385">
+    <cfRule type="duplicateValues" dxfId="23" priority="24"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B387">
     <cfRule type="duplicateValues" dxfId="22" priority="23"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B384">
+  <conditionalFormatting sqref="B389">
     <cfRule type="duplicateValues" dxfId="21" priority="22"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B385">
+  <conditionalFormatting sqref="B390">
     <cfRule type="duplicateValues" dxfId="20" priority="21"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B387">
+  <conditionalFormatting sqref="B391">
     <cfRule type="duplicateValues" dxfId="19" priority="20"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B389">
+  <conditionalFormatting sqref="B392">
     <cfRule type="duplicateValues" dxfId="18" priority="19"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B390">
+  <conditionalFormatting sqref="B393">
     <cfRule type="duplicateValues" dxfId="17" priority="18"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B391">
+  <conditionalFormatting sqref="B394">
     <cfRule type="duplicateValues" dxfId="16" priority="17"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B392">
+  <conditionalFormatting sqref="B396">
     <cfRule type="duplicateValues" dxfId="15" priority="16"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B393">
-    <cfRule type="duplicateValues" dxfId="14" priority="15"/>
+  <conditionalFormatting sqref="B397">
+    <cfRule type="duplicateValues" dxfId="14" priority="14"/>
+    <cfRule type="duplicateValues" dxfId="13" priority="15"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B394">
-    <cfRule type="duplicateValues" dxfId="13" priority="14"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B396">
+  <conditionalFormatting sqref="B398">
     <cfRule type="duplicateValues" dxfId="12" priority="13"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B397">
-    <cfRule type="duplicateValues" dxfId="11" priority="11"/>
-    <cfRule type="duplicateValues" dxfId="10" priority="12"/>
+  <conditionalFormatting sqref="B400">
+    <cfRule type="duplicateValues" dxfId="11" priority="12"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B398">
+  <conditionalFormatting sqref="B401">
+    <cfRule type="duplicateValues" dxfId="10" priority="11"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B402">
     <cfRule type="duplicateValues" dxfId="9" priority="10"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B400">
+  <conditionalFormatting sqref="B404">
     <cfRule type="duplicateValues" dxfId="8" priority="9"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B401">
+  <conditionalFormatting sqref="B405">
     <cfRule type="duplicateValues" dxfId="7" priority="8"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B402">
+  <conditionalFormatting sqref="B406">
     <cfRule type="duplicateValues" dxfId="6" priority="7"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B404">
-    <cfRule type="duplicateValues" dxfId="5" priority="6"/>
+  <conditionalFormatting sqref="B407">
+    <cfRule type="duplicateValues" dxfId="5" priority="5"/>
+    <cfRule type="duplicateValues" dxfId="4" priority="6"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B405">
-    <cfRule type="duplicateValues" dxfId="4" priority="5"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B406">
+  <conditionalFormatting sqref="B408">
     <cfRule type="duplicateValues" dxfId="3" priority="4"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B407">
-    <cfRule type="duplicateValues" dxfId="2" priority="2"/>
-    <cfRule type="duplicateValues" dxfId="1" priority="3"/>
+  <conditionalFormatting sqref="B410">
+    <cfRule type="duplicateValues" dxfId="2" priority="3"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B408">
+  <conditionalFormatting sqref="B411">
+    <cfRule type="duplicateValues" dxfId="1" priority="2"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B412">
     <cfRule type="duplicateValues" dxfId="0" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>